<commit_message>
sync: resultados automáticos openfootball
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -5963,8 +5963,12 @@
           <t>Cabo Verde</t>
         </is>
       </c>
-      <c r="F16" s="27" t="n"/>
-      <c r="G16" s="27" t="n"/>
+      <c r="F16" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="H16" s="16">
         <f>IF(AND(ISNUMBER(F16),ISNUMBER(G16)),"Finalizado","Pendiente")</f>
         <v/>
@@ -6007,8 +6011,12 @@
           <t>Egipto</t>
         </is>
       </c>
-      <c r="F17" s="27" t="n"/>
-      <c r="G17" s="27" t="n"/>
+      <c r="F17" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H17" s="16">
         <f>IF(AND(ISNUMBER(F17),ISNUMBER(G17)),"Finalizado","Pendiente")</f>
         <v/>

</xml_diff>

<commit_message>
fix: sync resultados pendientes y disparar sync en push a main
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="1" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Partidos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Pronosticos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Helpers &gt;&gt;" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Álvaro" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Papá" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Diego" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Puntuacion" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="_Helpers" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="_Lists" sheetId="12" state="hidden" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partidos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pronosticos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Helpers &gt;&gt;" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Álvaro" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papá" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diego" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puntuacion" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Helpers" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="12" state="hidden" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Partidos'!$A$3:$K$107</definedName>
@@ -507,14 +507,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -540,10 +540,10 @@
             <v>Puntos</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="051C2C"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="051C2C"/>
               </a:solidFill>
@@ -553,8 +553,8 @@
           <invertIfNegative val="1"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -625,9 +625,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -674,14 +674,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -715,10 +715,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="0066CC"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="0066CC"/>
               </a:solidFill>
@@ -760,10 +760,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="C5A028"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="C5A028"/>
               </a:solidFill>
@@ -805,10 +805,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="051C2C"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="051C2C"/>
               </a:solidFill>
@@ -858,9 +858,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -910,14 +910,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -949,7 +949,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="C5A028"/>
               </a:solidFill>
@@ -959,7 +959,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1035,7 +1035,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="0066CC"/>
               </a:solidFill>
@@ -1045,7 +1045,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1121,7 +1121,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="2E7D32"/>
               </a:solidFill>
@@ -1131,7 +1131,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1214,9 +1214,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1248,9 +1248,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1282,14 +1282,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1314,10 +1314,10 @@
             <v>Exactos</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2E7D32"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="2E7D32"/>
               </a:solidFill>
@@ -1351,10 +1351,10 @@
             <v>Parciales</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="C5A028"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="C5A028"/>
               </a:solidFill>
@@ -1388,10 +1388,10 @@
             <v>Fallos</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="B71C1C"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="B71C1C"/>
               </a:solidFill>
@@ -1441,9 +1441,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1492,7 +1492,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -1510,24 +1510,24 @@
       <nvPicPr>
         <cNvPr id="4" name="Picture 3"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="0" y="0"/>
           <a:ext cx="11469077" cy="4395889"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -1538,7 +1538,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -1553,9 +1553,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1575,9 +1575,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1597,9 +1597,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1619,9 +1619,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -6059,8 +6059,12 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="F18" s="27" t="n"/>
-      <c r="G18" s="27" t="n"/>
+      <c r="F18" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H18" s="16">
         <f>IF(AND(ISNUMBER(F18),ISNUMBER(G18)),"Finalizado","Pendiente")</f>
         <v/>
@@ -6103,8 +6107,12 @@
           <t>Nueva Zelanda</t>
         </is>
       </c>
-      <c r="F19" s="27" t="n"/>
-      <c r="G19" s="27" t="n"/>
+      <c r="F19" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="27" t="n">
+        <v>2</v>
+      </c>
       <c r="H19" s="16">
         <f>IF(AND(ISNUMBER(F19),ISNUMBER(G19)),"Finalizado","Pendiente")</f>
         <v/>

</xml_diff>

<commit_message>
fix: sync diario 00:00 y 06:00 hora España + resultados noche 16/06
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -6155,8 +6155,12 @@
           <t>Senegal</t>
         </is>
       </c>
-      <c r="F20" s="27" t="n"/>
-      <c r="G20" s="27" t="n"/>
+      <c r="F20" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H20" s="16">
         <f>IF(AND(ISNUMBER(F20),ISNUMBER(G20)),"Finalizado","Pendiente")</f>
         <v/>
@@ -6199,8 +6203,12 @@
           <t>Noruega</t>
         </is>
       </c>
-      <c r="F21" s="27" t="n"/>
-      <c r="G21" s="27" t="n"/>
+      <c r="F21" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="27" t="n">
+        <v>4</v>
+      </c>
       <c r="H21" s="16">
         <f>IF(AND(ISNUMBER(F21),ISNUMBER(G21)),"Finalizado","Pendiente")</f>
         <v/>
@@ -6243,8 +6251,12 @@
           <t>Argelia</t>
         </is>
       </c>
-      <c r="F22" s="27" t="n"/>
-      <c r="G22" s="27" t="n"/>
+      <c r="F22" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="H22" s="16">
         <f>IF(AND(ISNUMBER(F22),ISNUMBER(G22)),"Finalizado","Pendiente")</f>
         <v/>
@@ -6287,8 +6299,12 @@
           <t>Jordania</t>
         </is>
       </c>
-      <c r="F23" s="27" t="n"/>
-      <c r="G23" s="27" t="n"/>
+      <c r="F23" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H23" s="16">
         <f>IF(AND(ISNUMBER(F23),ISNUMBER(G23)),"Finalizado","Pendiente")</f>
         <v/>

</xml_diff>

<commit_message>
Habilitar sync 24h y aplicar resultados Canadá/México.
El cron anterior dejaba un hueco de 08:00 a 18:00 hora peninsular; ahora corre cada 30 min sin parar.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="1" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Partidos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Pronosticos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Helpers &gt;&gt;" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Álvaro" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Papá" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Diego" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Puntuacion" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="_Helpers" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="_Lists" sheetId="12" state="hidden" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partidos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pronosticos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Helpers &gt;&gt;" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Álvaro" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papá" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diego" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puntuacion" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Helpers" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="12" state="hidden" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Partidos'!$A$3:$K$107</definedName>
@@ -507,14 +507,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -540,10 +540,10 @@
             <v>Puntos</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="051C2C"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="051C2C"/>
               </a:solidFill>
@@ -553,8 +553,8 @@
           <invertIfNegative val="1"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -625,9 +625,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -674,14 +674,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -715,10 +715,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="0066CC"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="0066CC"/>
               </a:solidFill>
@@ -760,10 +760,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="C5A028"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="C5A028"/>
               </a:solidFill>
@@ -805,10 +805,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="051C2C"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="051C2C"/>
               </a:solidFill>
@@ -858,9 +858,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -910,14 +910,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -949,7 +949,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="C5A028"/>
               </a:solidFill>
@@ -959,7 +959,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1035,7 +1035,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="0066CC"/>
               </a:solidFill>
@@ -1045,7 +1045,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1121,7 +1121,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="2E7D32"/>
               </a:solidFill>
@@ -1131,7 +1131,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1214,9 +1214,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1248,9 +1248,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1282,14 +1282,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1314,10 +1314,10 @@
             <v>Exactos</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2E7D32"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="2E7D32"/>
               </a:solidFill>
@@ -1351,10 +1351,10 @@
             <v>Parciales</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="C5A028"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="C5A028"/>
               </a:solidFill>
@@ -1388,10 +1388,10 @@
             <v>Fallos</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="B71C1C"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="B71C1C"/>
               </a:solidFill>
@@ -1441,9 +1441,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1492,7 +1492,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -1510,24 +1510,24 @@
       <nvPicPr>
         <cNvPr id="4" name="Picture 3"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="0" y="0"/>
           <a:ext cx="11469077" cy="4395889"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -1538,7 +1538,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -1553,9 +1553,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1575,9 +1575,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1597,9 +1597,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1619,9 +1619,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -6635,8 +6635,12 @@
           <t>Catar</t>
         </is>
       </c>
-      <c r="F30" s="27" t="n"/>
-      <c r="G30" s="27" t="n"/>
+      <c r="F30" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="G30" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="H30" s="16">
         <f>IF(AND(ISNUMBER(F30),ISNUMBER(G30)),"Finalizado","Pendiente")</f>
         <v/>
@@ -6679,8 +6683,12 @@
           <t>República de Corea</t>
         </is>
       </c>
-      <c r="F31" s="27" t="n"/>
-      <c r="G31" s="27" t="n"/>
+      <c r="F31" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="H31" s="16">
         <f>IF(AND(ISNUMBER(F31),ISNUMBER(G31)),"Finalizado","Pendiente")</f>
         <v/>

</xml_diff>

<commit_message>
Dieciseisavos con equipos reales y puntuacion KO con empates.
Actualiza partidos 73-88, nueva logica de scoring, parches Excel y dashboards regenerados.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -2436,7 +2436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2562,21 +2562,44 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Empate exacto, fallo clasificado</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>pts</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>BONUS RONDA PERFECTA</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Empate dif., acierto clasificado</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>pts</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Octavos (8 clasificados)</t>
-        </is>
-      </c>
-      <c r="B14" s="32" t="n">
-        <v>15</v>
+          <t>Empate dif., fallo clasificado</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -2585,24 +2608,16 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Cuartos (4 clasificados)</t>
-        </is>
-      </c>
-      <c r="B15" s="32" t="n">
-        <v>15</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>pts</t>
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>BONUS RONDA PERFECTA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Semifinales (2 clasificados)</t>
+          <t>Octavos (8 clasificados)</t>
         </is>
       </c>
       <c r="B16" s="32" t="n">
@@ -2614,23 +2629,53 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Cuartos (4 clasificados)</t>
+        </is>
+      </c>
+      <c r="B17" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>pts</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Semifinales (2 clasificados)</t>
+        </is>
+      </c>
+      <c r="B18" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>APUESTAS ESPECIALES</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Cada acierto</t>
         </is>
       </c>
-      <c r="B19" s="32" t="n">
+      <c r="B21" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>pts</t>
         </is>
@@ -2724,7 +2769,7 @@
         <v/>
       </c>
       <c r="D2">
-        <f>IF(AND(Resumen!$B$34&lt;&gt;"",Álvaro!$B$111&lt;&gt;"",Álvaro!$B$111=Resumen!$B$34),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$35&lt;&gt;"",Álvaro!$B$112&lt;&gt;"",Álvaro!$B$112=Resumen!$B$35),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$36&lt;&gt;"",Álvaro!$B$113&lt;&gt;"",Álvaro!$B$113=Resumen!$B$36),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$37&lt;&gt;"",Álvaro!$B$114&lt;&gt;"",Álvaro!$B$114=Resumen!$B$37),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$38&lt;&gt;"",Álvaro!$B$115&lt;&gt;"",Álvaro!$B$115=Resumen!$B$38),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$39&lt;&gt;"",Álvaro!$B$116&lt;&gt;"",Álvaro!$B$116=Resumen!$B$39),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$40&lt;&gt;"",Álvaro!$B$117&lt;&gt;"",Álvaro!$B$117=Resumen!$B$40),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$41&lt;&gt;"",Álvaro!$B$118&lt;&gt;"",Álvaro!$B$118=Resumen!$B$41),Puntuacion!$B$19,0)</f>
+        <f>IF(AND(Resumen!$B$34&lt;&gt;"",Álvaro!$B$111&lt;&gt;"",Álvaro!$B$111=Resumen!$B$34),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$35&lt;&gt;"",Álvaro!$B$112&lt;&gt;"",Álvaro!$B$112=Resumen!$B$35),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$36&lt;&gt;"",Álvaro!$B$113&lt;&gt;"",Álvaro!$B$113=Resumen!$B$36),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$37&lt;&gt;"",Álvaro!$B$114&lt;&gt;"",Álvaro!$B$114=Resumen!$B$37),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$38&lt;&gt;"",Álvaro!$B$115&lt;&gt;"",Álvaro!$B$115=Resumen!$B$38),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$39&lt;&gt;"",Álvaro!$B$116&lt;&gt;"",Álvaro!$B$116=Resumen!$B$39),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$40&lt;&gt;"",Álvaro!$B$117&lt;&gt;"",Álvaro!$B$117=Resumen!$B$40),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$41&lt;&gt;"",Álvaro!$B$118&lt;&gt;"",Álvaro!$B$118=Resumen!$B$41),Puntuacion!$B$22,0)</f>
         <v/>
       </c>
       <c r="E2">
@@ -2752,15 +2797,15 @@
         <v/>
       </c>
       <c r="K2">
-        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Octavos",Partidos!$H$4:$H$107,"Finalizado")=8,COUNTIFS(Partidos!$J$4:$J$107,"Octavos",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A2,Pronosticos!$I$4:$I$315,"Octavos")=8),Puntuacion!$B$14,0)</f>
+        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Octavos",Partidos!$H$4:$H$107,"Finalizado")=8,COUNTIFS(Partidos!$J$4:$J$107,"Octavos",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A2,Pronosticos!$I$4:$I$315,"Octavos")=8),Puntuacion!$B$17,0)</f>
         <v/>
       </c>
       <c r="L2">
-        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Cuartos",Partidos!$H$4:$H$107,"Finalizado")=4,COUNTIFS(Partidos!$J$4:$J$107,"Cuartos",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A2,Pronosticos!$I$4:$I$315,"Cuartos")=4),Puntuacion!$B$15,0)</f>
+        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Cuartos",Partidos!$H$4:$H$107,"Finalizado")=4,COUNTIFS(Partidos!$J$4:$J$107,"Cuartos",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A2,Pronosticos!$I$4:$I$315,"Cuartos")=4),Puntuacion!$B$18,0)</f>
         <v/>
       </c>
       <c r="M2">
-        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Semifinal",Partidos!$H$4:$H$107,"Finalizado")=2,COUNTIFS(Partidos!$J$4:$J$107,"Semifinal",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A2,Pronosticos!$I$4:$I$315,"Semifinal")=2),Puntuacion!$B$16,0)</f>
+        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Semifinal",Partidos!$H$4:$H$107,"Finalizado")=2,COUNTIFS(Partidos!$J$4:$J$107,"Semifinal",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A2,Pronosticos!$I$4:$I$315,"Semifinal")=2),Puntuacion!$B$19,0)</f>
         <v/>
       </c>
     </row>
@@ -2779,7 +2824,7 @@
         <v/>
       </c>
       <c r="D3">
-        <f>IF(AND(Resumen!$B$34&lt;&gt;"",Papá!$B$111&lt;&gt;"",Papá!$B$111=Resumen!$B$34),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$35&lt;&gt;"",Papá!$B$112&lt;&gt;"",Papá!$B$112=Resumen!$B$35),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$36&lt;&gt;"",Papá!$B$113&lt;&gt;"",Papá!$B$113=Resumen!$B$36),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$37&lt;&gt;"",Papá!$B$114&lt;&gt;"",Papá!$B$114=Resumen!$B$37),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$38&lt;&gt;"",Papá!$B$115&lt;&gt;"",Papá!$B$115=Resumen!$B$38),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$39&lt;&gt;"",Papá!$B$116&lt;&gt;"",Papá!$B$116=Resumen!$B$39),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$40&lt;&gt;"",Papá!$B$117&lt;&gt;"",Papá!$B$117=Resumen!$B$40),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$41&lt;&gt;"",Papá!$B$118&lt;&gt;"",Papá!$B$118=Resumen!$B$41),Puntuacion!$B$19,0)</f>
+        <f>IF(AND(Resumen!$B$34&lt;&gt;"",Papá!$B$111&lt;&gt;"",Papá!$B$111=Resumen!$B$34),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$35&lt;&gt;"",Papá!$B$112&lt;&gt;"",Papá!$B$112=Resumen!$B$35),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$36&lt;&gt;"",Papá!$B$113&lt;&gt;"",Papá!$B$113=Resumen!$B$36),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$37&lt;&gt;"",Papá!$B$114&lt;&gt;"",Papá!$B$114=Resumen!$B$37),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$38&lt;&gt;"",Papá!$B$115&lt;&gt;"",Papá!$B$115=Resumen!$B$38),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$39&lt;&gt;"",Papá!$B$116&lt;&gt;"",Papá!$B$116=Resumen!$B$39),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$40&lt;&gt;"",Papá!$B$117&lt;&gt;"",Papá!$B$117=Resumen!$B$40),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$41&lt;&gt;"",Papá!$B$118&lt;&gt;"",Papá!$B$118=Resumen!$B$41),Puntuacion!$B$22,0)</f>
         <v/>
       </c>
       <c r="E3">
@@ -2807,15 +2852,15 @@
         <v/>
       </c>
       <c r="K3">
-        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Octavos",Partidos!$H$4:$H$107,"Finalizado")=8,COUNTIFS(Partidos!$J$4:$J$107,"Octavos",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A3,Pronosticos!$I$4:$I$315,"Octavos")=8),Puntuacion!$B$14,0)</f>
+        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Octavos",Partidos!$H$4:$H$107,"Finalizado")=8,COUNTIFS(Partidos!$J$4:$J$107,"Octavos",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A3,Pronosticos!$I$4:$I$315,"Octavos")=8),Puntuacion!$B$17,0)</f>
         <v/>
       </c>
       <c r="L3">
-        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Cuartos",Partidos!$H$4:$H$107,"Finalizado")=4,COUNTIFS(Partidos!$J$4:$J$107,"Cuartos",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A3,Pronosticos!$I$4:$I$315,"Cuartos")=4),Puntuacion!$B$15,0)</f>
+        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Cuartos",Partidos!$H$4:$H$107,"Finalizado")=4,COUNTIFS(Partidos!$J$4:$J$107,"Cuartos",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A3,Pronosticos!$I$4:$I$315,"Cuartos")=4),Puntuacion!$B$18,0)</f>
         <v/>
       </c>
       <c r="M3">
-        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Semifinal",Partidos!$H$4:$H$107,"Finalizado")=2,COUNTIFS(Partidos!$J$4:$J$107,"Semifinal",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A3,Pronosticos!$I$4:$I$315,"Semifinal")=2),Puntuacion!$B$16,0)</f>
+        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Semifinal",Partidos!$H$4:$H$107,"Finalizado")=2,COUNTIFS(Partidos!$J$4:$J$107,"Semifinal",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A3,Pronosticos!$I$4:$I$315,"Semifinal")=2),Puntuacion!$B$19,0)</f>
         <v/>
       </c>
     </row>
@@ -2834,7 +2879,7 @@
         <v/>
       </c>
       <c r="D4">
-        <f>IF(AND(Resumen!$B$34&lt;&gt;"",Diego!$B$111&lt;&gt;"",Diego!$B$111=Resumen!$B$34),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$35&lt;&gt;"",Diego!$B$112&lt;&gt;"",Diego!$B$112=Resumen!$B$35),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$36&lt;&gt;"",Diego!$B$113&lt;&gt;"",Diego!$B$113=Resumen!$B$36),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$37&lt;&gt;"",Diego!$B$114&lt;&gt;"",Diego!$B$114=Resumen!$B$37),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$38&lt;&gt;"",Diego!$B$115&lt;&gt;"",Diego!$B$115=Resumen!$B$38),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$39&lt;&gt;"",Diego!$B$116&lt;&gt;"",Diego!$B$116=Resumen!$B$39),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$40&lt;&gt;"",Diego!$B$117&lt;&gt;"",Diego!$B$117=Resumen!$B$40),Puntuacion!$B$19,0)+IF(AND(Resumen!$B$41&lt;&gt;"",Diego!$B$118&lt;&gt;"",Diego!$B$118=Resumen!$B$41),Puntuacion!$B$19,0)</f>
+        <f>IF(AND(Resumen!$B$34&lt;&gt;"",Diego!$B$111&lt;&gt;"",Diego!$B$111=Resumen!$B$34),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$35&lt;&gt;"",Diego!$B$112&lt;&gt;"",Diego!$B$112=Resumen!$B$35),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$36&lt;&gt;"",Diego!$B$113&lt;&gt;"",Diego!$B$113=Resumen!$B$36),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$37&lt;&gt;"",Diego!$B$114&lt;&gt;"",Diego!$B$114=Resumen!$B$37),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$38&lt;&gt;"",Diego!$B$115&lt;&gt;"",Diego!$B$115=Resumen!$B$38),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$39&lt;&gt;"",Diego!$B$116&lt;&gt;"",Diego!$B$116=Resumen!$B$39),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$40&lt;&gt;"",Diego!$B$117&lt;&gt;"",Diego!$B$117=Resumen!$B$40),Puntuacion!$B$22,0)+IF(AND(Resumen!$B$41&lt;&gt;"",Diego!$B$118&lt;&gt;"",Diego!$B$118=Resumen!$B$41),Puntuacion!$B$22,0)</f>
         <v/>
       </c>
       <c r="E4">
@@ -2862,15 +2907,15 @@
         <v/>
       </c>
       <c r="K4">
-        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Octavos",Partidos!$H$4:$H$107,"Finalizado")=8,COUNTIFS(Partidos!$J$4:$J$107,"Octavos",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A4,Pronosticos!$I$4:$I$315,"Octavos")=8),Puntuacion!$B$14,0)</f>
+        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Octavos",Partidos!$H$4:$H$107,"Finalizado")=8,COUNTIFS(Partidos!$J$4:$J$107,"Octavos",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A4,Pronosticos!$I$4:$I$315,"Octavos")=8),Puntuacion!$B$17,0)</f>
         <v/>
       </c>
       <c r="L4">
-        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Cuartos",Partidos!$H$4:$H$107,"Finalizado")=4,COUNTIFS(Partidos!$J$4:$J$107,"Cuartos",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A4,Pronosticos!$I$4:$I$315,"Cuartos")=4),Puntuacion!$B$15,0)</f>
+        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Cuartos",Partidos!$H$4:$H$107,"Finalizado")=4,COUNTIFS(Partidos!$J$4:$J$107,"Cuartos",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A4,Pronosticos!$I$4:$I$315,"Cuartos")=4),Puntuacion!$B$18,0)</f>
         <v/>
       </c>
       <c r="M4">
-        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Semifinal",Partidos!$H$4:$H$107,"Finalizado")=2,COUNTIFS(Partidos!$J$4:$J$107,"Semifinal",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A4,Pronosticos!$I$4:$I$315,"Semifinal")=2),Puntuacion!$B$16,0)</f>
+        <f>IF(AND(COUNTIFS(Partidos!$J$4:$J$107,"Semifinal",Partidos!$H$4:$H$107,"Finalizado")=2,COUNTIFS(Partidos!$J$4:$J$107,"Semifinal",Partidos!$H$4:$H$107,"Finalizado")&gt;0,SUMIFS(Pronosticos!$J$4:$J$315,Pronosticos!$D$4:$D$315,A4,Pronosticos!$I$4:$I$315,"Semifinal")=2),Puntuacion!$B$19,0)</f>
         <v/>
       </c>
     </row>
@@ -5060,11 +5105,11 @@
         <v/>
       </c>
       <c r="H34" s="17">
-        <f>IF(Puntuacion!$B$19=0,0,G34/Puntuacion!$B$19)</f>
+        <f>IF(Puntuacion!$B$22=0,0,G34/Puntuacion!$B$22)</f>
         <v/>
       </c>
       <c r="I34" s="17">
-        <f>Puntuacion!$B$19</f>
+        <f>Puntuacion!$B$22</f>
         <v/>
       </c>
     </row>
@@ -5092,11 +5137,11 @@
         <v/>
       </c>
       <c r="H35" s="17">
-        <f>IF(Puntuacion!$B$19=0,0,G35/Puntuacion!$B$19)</f>
+        <f>IF(Puntuacion!$B$22=0,0,G35/Puntuacion!$B$22)</f>
         <v/>
       </c>
       <c r="I35" s="17">
-        <f>Puntuacion!$B$19</f>
+        <f>Puntuacion!$B$22</f>
         <v/>
       </c>
     </row>
@@ -5124,11 +5169,11 @@
         <v/>
       </c>
       <c r="H36" s="17">
-        <f>IF(Puntuacion!$B$19=0,0,G36/Puntuacion!$B$19)</f>
+        <f>IF(Puntuacion!$B$22=0,0,G36/Puntuacion!$B$22)</f>
         <v/>
       </c>
       <c r="I36" s="17">
-        <f>Puntuacion!$B$19</f>
+        <f>Puntuacion!$B$22</f>
         <v/>
       </c>
     </row>
@@ -8659,12 +8704,12 @@
       </c>
       <c r="D76" s="19" t="inlineStr">
         <is>
-          <t>Ganador 1A</t>
+          <t>Sudáfrica</t>
         </is>
       </c>
       <c r="E76" s="19" t="inlineStr">
         <is>
-          <t>Ganador 2B</t>
+          <t>Canadá</t>
         </is>
       </c>
       <c r="F76" s="27" t="n"/>
@@ -8699,12 +8744,12 @@
       </c>
       <c r="D77" s="19" t="inlineStr">
         <is>
-          <t>Ganador 1C</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="E77" s="19" t="inlineStr">
         <is>
-          <t>Ganador 2D</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="F77" s="27" t="n"/>
@@ -8739,12 +8784,12 @@
       </c>
       <c r="D78" s="19" t="inlineStr">
         <is>
-          <t>Ganador 1E</t>
+          <t>Países Bajos</t>
         </is>
       </c>
       <c r="E78" s="19" t="inlineStr">
         <is>
-          <t>Ganador 2F</t>
+          <t>Marruecos</t>
         </is>
       </c>
       <c r="F78" s="27" t="n"/>
@@ -8779,12 +8824,12 @@
       </c>
       <c r="D79" s="19" t="inlineStr">
         <is>
-          <t>Ganador 1G</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E79" s="19" t="inlineStr">
         <is>
-          <t>Ganador 2H</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F79" s="27" t="n"/>
@@ -8819,12 +8864,12 @@
       </c>
       <c r="D80" s="19" t="inlineStr">
         <is>
-          <t>Ganador 1I</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="E80" s="19" t="inlineStr">
         <is>
-          <t>Ganador 2J</t>
+          <t>Suecia</t>
         </is>
       </c>
       <c r="F80" s="27" t="n"/>
@@ -8859,12 +8904,12 @@
       </c>
       <c r="D81" s="19" t="inlineStr">
         <is>
-          <t>Ganador 1K</t>
+          <t>Costa de Marfil</t>
         </is>
       </c>
       <c r="E81" s="19" t="inlineStr">
         <is>
-          <t>Ganador 2L</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F81" s="27" t="n"/>
@@ -8899,12 +8944,12 @@
       </c>
       <c r="D82" s="19" t="inlineStr">
         <is>
-          <t>Ganador 1B</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E82" s="19" t="inlineStr">
         <is>
-          <t>Ganador 2A</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="F82" s="27" t="n"/>
@@ -8939,12 +8984,12 @@
       </c>
       <c r="D83" s="19" t="inlineStr">
         <is>
-          <t>Ganador 1D</t>
+          <t>Inglaterra</t>
         </is>
       </c>
       <c r="E83" s="19" t="inlineStr">
         <is>
-          <t>Ganador 2C</t>
+          <t>RD Congo</t>
         </is>
       </c>
       <c r="F83" s="27" t="n"/>
@@ -8979,12 +9024,12 @@
       </c>
       <c r="D84" s="19" t="inlineStr">
         <is>
-          <t>Ganador 1F</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E84" s="19" t="inlineStr">
         <is>
-          <t>Ganador 2E</t>
+          <t>Bosnia y Herzegovina</t>
         </is>
       </c>
       <c r="F84" s="27" t="n"/>
@@ -9019,12 +9064,12 @@
       </c>
       <c r="D85" s="19" t="inlineStr">
         <is>
-          <t>Ganador 1H</t>
+          <t>Bélgica</t>
         </is>
       </c>
       <c r="E85" s="19" t="inlineStr">
         <is>
-          <t>Ganador 2G</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="F85" s="27" t="n"/>
@@ -9059,12 +9104,12 @@
       </c>
       <c r="D86" s="19" t="inlineStr">
         <is>
-          <t>Ganador 1J</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E86" s="19" t="inlineStr">
         <is>
-          <t>Ganador 2I</t>
+          <t>Croacia</t>
         </is>
       </c>
       <c r="F86" s="27" t="n"/>
@@ -9099,12 +9144,12 @@
       </c>
       <c r="D87" s="19" t="inlineStr">
         <is>
-          <t>Ganador 1L</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E87" s="19" t="inlineStr">
         <is>
-          <t>Ganador 2K</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="F87" s="27" t="n"/>
@@ -9139,12 +9184,12 @@
       </c>
       <c r="D88" s="19" t="inlineStr">
         <is>
-          <t>Ganador 3A</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="E88" s="19" t="inlineStr">
         <is>
-          <t>Ganador 3B</t>
+          <t>Argelia</t>
         </is>
       </c>
       <c r="F88" s="27" t="n"/>
@@ -9179,12 +9224,12 @@
       </c>
       <c r="D89" s="19" t="inlineStr">
         <is>
-          <t>Ganador 3C</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E89" s="19" t="inlineStr">
         <is>
-          <t>Ganador 3D</t>
+          <t>Cabo Verde</t>
         </is>
       </c>
       <c r="F89" s="27" t="n"/>
@@ -9219,12 +9264,12 @@
       </c>
       <c r="D90" s="19" t="inlineStr">
         <is>
-          <t>Ganador 3E</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E90" s="19" t="inlineStr">
         <is>
-          <t>Ganador 3F</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="F90" s="27" t="n"/>
@@ -9259,12 +9304,12 @@
       </c>
       <c r="D91" s="19" t="inlineStr">
         <is>
-          <t>Ganador 3G</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="E91" s="19" t="inlineStr">
         <is>
-          <t>Ganador 3H</t>
+          <t>Egipto</t>
         </is>
       </c>
       <c r="F91" s="27" t="n"/>
@@ -10067,7 +10112,7 @@
         <v/>
       </c>
       <c r="G4" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A4,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E4)),NOT(ISNUMBER($F4))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A4,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E4=INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0)),$F4=INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E4-$F4)=(INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E4&gt;$F4,INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),AND($E4=$F4,INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),AND($E4&lt;$F4,INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E4=INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0)),$F4=INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E4-$F4)=(INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H4&lt;&gt;"",$H4=INDEX(Partidos!$K$4:$K$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A4,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E4)),NOT(ISNUMBER($F4))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A4,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E4=INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0)),$F4=INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E4-$F4)=(INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E4&gt;$F4,INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),AND($E4=$F4,INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),AND($E4&lt;$F4,INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0)),IF(AND($E4=INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0)),$F4=INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),IF(AND($H4&lt;&gt;"",$H4=INDEX(Partidos!$K$4:$K$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E4=$F4,($E4-$F4)=(INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0)))),IF(AND($H4&lt;&gt;"",$H4=INDEX(Partidos!$K$4:$K$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H4&lt;&gt;"",$H4=INDEX(Partidos!$K$4:$K$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E4=INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0)),$F4=INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E4-$F4)=(INDEX(Partidos!$F$4:$F$107,MATCH($A4,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H4&lt;&gt;"",$H4=INDEX(Partidos!$K$4:$K$107,MATCH($A4,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H4" s="19">
@@ -10109,7 +10154,7 @@
         <v/>
       </c>
       <c r="G5" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A5,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E5)),NOT(ISNUMBER($F5))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A5,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E5=INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0)),$F5=INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E5-$F5)=(INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E5&gt;$F5,INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),AND($E5=$F5,INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),AND($E5&lt;$F5,INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E5=INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0)),$F5=INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E5-$F5)=(INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H5&lt;&gt;"",$H5=INDEX(Partidos!$K$4:$K$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A5,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E5)),NOT(ISNUMBER($F5))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A5,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E5=INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0)),$F5=INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E5-$F5)=(INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E5&gt;$F5,INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),AND($E5=$F5,INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),AND($E5&lt;$F5,INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0)),IF(AND($E5=INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0)),$F5=INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),IF(AND($H5&lt;&gt;"",$H5=INDEX(Partidos!$K$4:$K$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E5=$F5,($E5-$F5)=(INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0)))),IF(AND($H5&lt;&gt;"",$H5=INDEX(Partidos!$K$4:$K$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H5&lt;&gt;"",$H5=INDEX(Partidos!$K$4:$K$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E5=INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0)),$F5=INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E5-$F5)=(INDEX(Partidos!$F$4:$F$107,MATCH($A5,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H5&lt;&gt;"",$H5=INDEX(Partidos!$K$4:$K$107,MATCH($A5,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H5" s="19">
@@ -10151,7 +10196,7 @@
         <v/>
       </c>
       <c r="G6" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A6,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E6)),NOT(ISNUMBER($F6))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A6,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E6=INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0)),$F6=INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E6-$F6)=(INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E6&gt;$F6,INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),AND($E6=$F6,INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),AND($E6&lt;$F6,INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E6=INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0)),$F6=INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E6-$F6)=(INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H6&lt;&gt;"",$H6=INDEX(Partidos!$K$4:$K$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A6,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E6)),NOT(ISNUMBER($F6))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A6,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E6=INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0)),$F6=INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E6-$F6)=(INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E6&gt;$F6,INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),AND($E6=$F6,INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),AND($E6&lt;$F6,INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0)),IF(AND($E6=INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0)),$F6=INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),IF(AND($H6&lt;&gt;"",$H6=INDEX(Partidos!$K$4:$K$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E6=$F6,($E6-$F6)=(INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0)))),IF(AND($H6&lt;&gt;"",$H6=INDEX(Partidos!$K$4:$K$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H6&lt;&gt;"",$H6=INDEX(Partidos!$K$4:$K$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E6=INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0)),$F6=INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E6-$F6)=(INDEX(Partidos!$F$4:$F$107,MATCH($A6,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H6&lt;&gt;"",$H6=INDEX(Partidos!$K$4:$K$107,MATCH($A6,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H6" s="19">
@@ -10193,7 +10238,7 @@
         <v/>
       </c>
       <c r="G7" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A7,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E7)),NOT(ISNUMBER($F7))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A7,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E7=INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0)),$F7=INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E7-$F7)=(INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E7&gt;$F7,INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),AND($E7=$F7,INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),AND($E7&lt;$F7,INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E7=INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0)),$F7=INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E7-$F7)=(INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H7&lt;&gt;"",$H7=INDEX(Partidos!$K$4:$K$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A7,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E7)),NOT(ISNUMBER($F7))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A7,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E7=INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0)),$F7=INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E7-$F7)=(INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E7&gt;$F7,INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),AND($E7=$F7,INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),AND($E7&lt;$F7,INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0)),IF(AND($E7=INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0)),$F7=INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),IF(AND($H7&lt;&gt;"",$H7=INDEX(Partidos!$K$4:$K$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E7=$F7,($E7-$F7)=(INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0)))),IF(AND($H7&lt;&gt;"",$H7=INDEX(Partidos!$K$4:$K$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H7&lt;&gt;"",$H7=INDEX(Partidos!$K$4:$K$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E7=INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0)),$F7=INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E7-$F7)=(INDEX(Partidos!$F$4:$F$107,MATCH($A7,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H7&lt;&gt;"",$H7=INDEX(Partidos!$K$4:$K$107,MATCH($A7,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H7" s="19">
@@ -10235,7 +10280,7 @@
         <v/>
       </c>
       <c r="G8" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A8,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E8)),NOT(ISNUMBER($F8))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A8,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E8=INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0)),$F8=INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E8-$F8)=(INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E8&gt;$F8,INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),AND($E8=$F8,INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),AND($E8&lt;$F8,INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E8=INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0)),$F8=INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E8-$F8)=(INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H8&lt;&gt;"",$H8=INDEX(Partidos!$K$4:$K$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A8,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E8)),NOT(ISNUMBER($F8))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A8,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E8=INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0)),$F8=INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E8-$F8)=(INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E8&gt;$F8,INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),AND($E8=$F8,INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),AND($E8&lt;$F8,INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0)),IF(AND($E8=INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0)),$F8=INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),IF(AND($H8&lt;&gt;"",$H8=INDEX(Partidos!$K$4:$K$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E8=$F8,($E8-$F8)=(INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0)))),IF(AND($H8&lt;&gt;"",$H8=INDEX(Partidos!$K$4:$K$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H8&lt;&gt;"",$H8=INDEX(Partidos!$K$4:$K$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E8=INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0)),$F8=INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E8-$F8)=(INDEX(Partidos!$F$4:$F$107,MATCH($A8,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H8&lt;&gt;"",$H8=INDEX(Partidos!$K$4:$K$107,MATCH($A8,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H8" s="19">
@@ -10277,7 +10322,7 @@
         <v/>
       </c>
       <c r="G9" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A9,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E9)),NOT(ISNUMBER($F9))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A9,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E9=INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0)),$F9=INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E9-$F9)=(INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E9&gt;$F9,INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),AND($E9=$F9,INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),AND($E9&lt;$F9,INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E9=INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0)),$F9=INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E9-$F9)=(INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H9&lt;&gt;"",$H9=INDEX(Partidos!$K$4:$K$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A9,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E9)),NOT(ISNUMBER($F9))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A9,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E9=INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0)),$F9=INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E9-$F9)=(INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E9&gt;$F9,INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),AND($E9=$F9,INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),AND($E9&lt;$F9,INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0)),IF(AND($E9=INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0)),$F9=INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),IF(AND($H9&lt;&gt;"",$H9=INDEX(Partidos!$K$4:$K$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E9=$F9,($E9-$F9)=(INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0)))),IF(AND($H9&lt;&gt;"",$H9=INDEX(Partidos!$K$4:$K$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H9&lt;&gt;"",$H9=INDEX(Partidos!$K$4:$K$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E9=INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0)),$F9=INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E9-$F9)=(INDEX(Partidos!$F$4:$F$107,MATCH($A9,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H9&lt;&gt;"",$H9=INDEX(Partidos!$K$4:$K$107,MATCH($A9,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H9" s="19">
@@ -10319,7 +10364,7 @@
         <v/>
       </c>
       <c r="G10" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A10,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E10)),NOT(ISNUMBER($F10))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A10,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E10=INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0)),$F10=INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E10-$F10)=(INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E10&gt;$F10,INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),AND($E10=$F10,INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),AND($E10&lt;$F10,INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E10=INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0)),$F10=INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E10-$F10)=(INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H10&lt;&gt;"",$H10=INDEX(Partidos!$K$4:$K$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A10,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E10)),NOT(ISNUMBER($F10))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A10,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E10=INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0)),$F10=INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E10-$F10)=(INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E10&gt;$F10,INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),AND($E10=$F10,INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),AND($E10&lt;$F10,INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0)),IF(AND($E10=INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0)),$F10=INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),IF(AND($H10&lt;&gt;"",$H10=INDEX(Partidos!$K$4:$K$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E10=$F10,($E10-$F10)=(INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0)))),IF(AND($H10&lt;&gt;"",$H10=INDEX(Partidos!$K$4:$K$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H10&lt;&gt;"",$H10=INDEX(Partidos!$K$4:$K$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E10=INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0)),$F10=INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E10-$F10)=(INDEX(Partidos!$F$4:$F$107,MATCH($A10,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H10&lt;&gt;"",$H10=INDEX(Partidos!$K$4:$K$107,MATCH($A10,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H10" s="19">
@@ -10361,7 +10406,7 @@
         <v/>
       </c>
       <c r="G11" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A11,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E11)),NOT(ISNUMBER($F11))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A11,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E11=INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0)),$F11=INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E11-$F11)=(INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E11&gt;$F11,INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),AND($E11=$F11,INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),AND($E11&lt;$F11,INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E11=INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0)),$F11=INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E11-$F11)=(INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H11&lt;&gt;"",$H11=INDEX(Partidos!$K$4:$K$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A11,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E11)),NOT(ISNUMBER($F11))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A11,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E11=INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0)),$F11=INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E11-$F11)=(INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E11&gt;$F11,INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),AND($E11=$F11,INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),AND($E11&lt;$F11,INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0)),IF(AND($E11=INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0)),$F11=INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),IF(AND($H11&lt;&gt;"",$H11=INDEX(Partidos!$K$4:$K$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E11=$F11,($E11-$F11)=(INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0)))),IF(AND($H11&lt;&gt;"",$H11=INDEX(Partidos!$K$4:$K$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H11&lt;&gt;"",$H11=INDEX(Partidos!$K$4:$K$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E11=INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0)),$F11=INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E11-$F11)=(INDEX(Partidos!$F$4:$F$107,MATCH($A11,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H11&lt;&gt;"",$H11=INDEX(Partidos!$K$4:$K$107,MATCH($A11,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H11" s="19">
@@ -10403,7 +10448,7 @@
         <v/>
       </c>
       <c r="G12" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A12,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E12)),NOT(ISNUMBER($F12))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A12,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E12=INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0)),$F12=INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E12-$F12)=(INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E12&gt;$F12,INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),AND($E12=$F12,INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),AND($E12&lt;$F12,INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E12=INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0)),$F12=INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E12-$F12)=(INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H12&lt;&gt;"",$H12=INDEX(Partidos!$K$4:$K$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A12,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E12)),NOT(ISNUMBER($F12))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A12,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E12=INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0)),$F12=INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E12-$F12)=(INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E12&gt;$F12,INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),AND($E12=$F12,INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),AND($E12&lt;$F12,INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0)),IF(AND($E12=INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0)),$F12=INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),IF(AND($H12&lt;&gt;"",$H12=INDEX(Partidos!$K$4:$K$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E12=$F12,($E12-$F12)=(INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0)))),IF(AND($H12&lt;&gt;"",$H12=INDEX(Partidos!$K$4:$K$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H12&lt;&gt;"",$H12=INDEX(Partidos!$K$4:$K$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E12=INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0)),$F12=INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E12-$F12)=(INDEX(Partidos!$F$4:$F$107,MATCH($A12,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H12&lt;&gt;"",$H12=INDEX(Partidos!$K$4:$K$107,MATCH($A12,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H12" s="19">
@@ -10445,7 +10490,7 @@
         <v/>
       </c>
       <c r="G13" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A13,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E13)),NOT(ISNUMBER($F13))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A13,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E13=INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0)),$F13=INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E13-$F13)=(INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E13&gt;$F13,INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),AND($E13=$F13,INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),AND($E13&lt;$F13,INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E13=INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0)),$F13=INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E13-$F13)=(INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H13&lt;&gt;"",$H13=INDEX(Partidos!$K$4:$K$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A13,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E13)),NOT(ISNUMBER($F13))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A13,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E13=INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0)),$F13=INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E13-$F13)=(INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E13&gt;$F13,INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),AND($E13=$F13,INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),AND($E13&lt;$F13,INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0)),IF(AND($E13=INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0)),$F13=INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),IF(AND($H13&lt;&gt;"",$H13=INDEX(Partidos!$K$4:$K$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E13=$F13,($E13-$F13)=(INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0)))),IF(AND($H13&lt;&gt;"",$H13=INDEX(Partidos!$K$4:$K$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H13&lt;&gt;"",$H13=INDEX(Partidos!$K$4:$K$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E13=INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0)),$F13=INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E13-$F13)=(INDEX(Partidos!$F$4:$F$107,MATCH($A13,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H13&lt;&gt;"",$H13=INDEX(Partidos!$K$4:$K$107,MATCH($A13,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H13" s="19">
@@ -10487,7 +10532,7 @@
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A14,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E14)),NOT(ISNUMBER($F14))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A14,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E14=INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0)),$F14=INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E14-$F14)=(INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E14&gt;$F14,INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),AND($E14=$F14,INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),AND($E14&lt;$F14,INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E14=INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0)),$F14=INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E14-$F14)=(INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H14&lt;&gt;"",$H14=INDEX(Partidos!$K$4:$K$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A14,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E14)),NOT(ISNUMBER($F14))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A14,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E14=INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0)),$F14=INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E14-$F14)=(INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E14&gt;$F14,INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),AND($E14=$F14,INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),AND($E14&lt;$F14,INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0)),IF(AND($E14=INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0)),$F14=INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),IF(AND($H14&lt;&gt;"",$H14=INDEX(Partidos!$K$4:$K$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E14=$F14,($E14-$F14)=(INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0)))),IF(AND($H14&lt;&gt;"",$H14=INDEX(Partidos!$K$4:$K$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H14&lt;&gt;"",$H14=INDEX(Partidos!$K$4:$K$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E14=INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0)),$F14=INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E14-$F14)=(INDEX(Partidos!$F$4:$F$107,MATCH($A14,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H14&lt;&gt;"",$H14=INDEX(Partidos!$K$4:$K$107,MATCH($A14,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H14" s="19">
@@ -10529,7 +10574,7 @@
         <v/>
       </c>
       <c r="G15" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A15,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E15)),NOT(ISNUMBER($F15))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A15,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E15=INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0)),$F15=INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E15-$F15)=(INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E15&gt;$F15,INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),AND($E15=$F15,INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),AND($E15&lt;$F15,INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E15=INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0)),$F15=INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E15-$F15)=(INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H15&lt;&gt;"",$H15=INDEX(Partidos!$K$4:$K$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A15,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E15)),NOT(ISNUMBER($F15))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A15,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E15=INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0)),$F15=INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E15-$F15)=(INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E15&gt;$F15,INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),AND($E15=$F15,INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),AND($E15&lt;$F15,INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0)),IF(AND($E15=INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0)),$F15=INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),IF(AND($H15&lt;&gt;"",$H15=INDEX(Partidos!$K$4:$K$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E15=$F15,($E15-$F15)=(INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0)))),IF(AND($H15&lt;&gt;"",$H15=INDEX(Partidos!$K$4:$K$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H15&lt;&gt;"",$H15=INDEX(Partidos!$K$4:$K$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E15=INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0)),$F15=INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E15-$F15)=(INDEX(Partidos!$F$4:$F$107,MATCH($A15,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H15&lt;&gt;"",$H15=INDEX(Partidos!$K$4:$K$107,MATCH($A15,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H15" s="19">
@@ -10571,7 +10616,7 @@
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A16,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E16)),NOT(ISNUMBER($F16))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A16,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E16=INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0)),$F16=INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E16-$F16)=(INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E16&gt;$F16,INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),AND($E16=$F16,INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),AND($E16&lt;$F16,INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E16=INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0)),$F16=INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E16-$F16)=(INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H16&lt;&gt;"",$H16=INDEX(Partidos!$K$4:$K$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A16,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E16)),NOT(ISNUMBER($F16))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A16,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E16=INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0)),$F16=INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E16-$F16)=(INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E16&gt;$F16,INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),AND($E16=$F16,INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),AND($E16&lt;$F16,INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0)),IF(AND($E16=INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0)),$F16=INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),IF(AND($H16&lt;&gt;"",$H16=INDEX(Partidos!$K$4:$K$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E16=$F16,($E16-$F16)=(INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0)))),IF(AND($H16&lt;&gt;"",$H16=INDEX(Partidos!$K$4:$K$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H16&lt;&gt;"",$H16=INDEX(Partidos!$K$4:$K$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E16=INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0)),$F16=INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E16-$F16)=(INDEX(Partidos!$F$4:$F$107,MATCH($A16,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H16&lt;&gt;"",$H16=INDEX(Partidos!$K$4:$K$107,MATCH($A16,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H16" s="19">
@@ -10613,7 +10658,7 @@
         <v/>
       </c>
       <c r="G17" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A17,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E17)),NOT(ISNUMBER($F17))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A17,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E17=INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0)),$F17=INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E17-$F17)=(INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E17&gt;$F17,INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),AND($E17=$F17,INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),AND($E17&lt;$F17,INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E17=INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0)),$F17=INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E17-$F17)=(INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H17&lt;&gt;"",$H17=INDEX(Partidos!$K$4:$K$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A17,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E17)),NOT(ISNUMBER($F17))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A17,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E17=INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0)),$F17=INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E17-$F17)=(INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E17&gt;$F17,INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),AND($E17=$F17,INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),AND($E17&lt;$F17,INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0)),IF(AND($E17=INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0)),$F17=INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),IF(AND($H17&lt;&gt;"",$H17=INDEX(Partidos!$K$4:$K$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E17=$F17,($E17-$F17)=(INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0)))),IF(AND($H17&lt;&gt;"",$H17=INDEX(Partidos!$K$4:$K$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H17&lt;&gt;"",$H17=INDEX(Partidos!$K$4:$K$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E17=INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0)),$F17=INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E17-$F17)=(INDEX(Partidos!$F$4:$F$107,MATCH($A17,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H17&lt;&gt;"",$H17=INDEX(Partidos!$K$4:$K$107,MATCH($A17,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H17" s="19">
@@ -10655,7 +10700,7 @@
         <v/>
       </c>
       <c r="G18" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A18,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E18)),NOT(ISNUMBER($F18))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A18,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E18=INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0)),$F18=INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E18-$F18)=(INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E18&gt;$F18,INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),AND($E18=$F18,INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),AND($E18&lt;$F18,INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E18=INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0)),$F18=INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E18-$F18)=(INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H18&lt;&gt;"",$H18=INDEX(Partidos!$K$4:$K$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A18,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E18)),NOT(ISNUMBER($F18))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A18,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E18=INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0)),$F18=INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E18-$F18)=(INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E18&gt;$F18,INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),AND($E18=$F18,INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),AND($E18&lt;$F18,INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0)),IF(AND($E18=INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0)),$F18=INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),IF(AND($H18&lt;&gt;"",$H18=INDEX(Partidos!$K$4:$K$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E18=$F18,($E18-$F18)=(INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0)))),IF(AND($H18&lt;&gt;"",$H18=INDEX(Partidos!$K$4:$K$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H18&lt;&gt;"",$H18=INDEX(Partidos!$K$4:$K$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E18=INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0)),$F18=INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E18-$F18)=(INDEX(Partidos!$F$4:$F$107,MATCH($A18,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H18&lt;&gt;"",$H18=INDEX(Partidos!$K$4:$K$107,MATCH($A18,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H18" s="19">
@@ -10697,7 +10742,7 @@
         <v/>
       </c>
       <c r="G19" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A19,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E19)),NOT(ISNUMBER($F19))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A19,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E19=INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0)),$F19=INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E19-$F19)=(INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E19&gt;$F19,INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),AND($E19=$F19,INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),AND($E19&lt;$F19,INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E19=INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0)),$F19=INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E19-$F19)=(INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H19&lt;&gt;"",$H19=INDEX(Partidos!$K$4:$K$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A19,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E19)),NOT(ISNUMBER($F19))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A19,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E19=INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0)),$F19=INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E19-$F19)=(INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E19&gt;$F19,INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),AND($E19=$F19,INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),AND($E19&lt;$F19,INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0)),IF(AND($E19=INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0)),$F19=INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),IF(AND($H19&lt;&gt;"",$H19=INDEX(Partidos!$K$4:$K$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E19=$F19,($E19-$F19)=(INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0)))),IF(AND($H19&lt;&gt;"",$H19=INDEX(Partidos!$K$4:$K$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H19&lt;&gt;"",$H19=INDEX(Partidos!$K$4:$K$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E19=INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0)),$F19=INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E19-$F19)=(INDEX(Partidos!$F$4:$F$107,MATCH($A19,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H19&lt;&gt;"",$H19=INDEX(Partidos!$K$4:$K$107,MATCH($A19,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H19" s="19">
@@ -10739,7 +10784,7 @@
         <v/>
       </c>
       <c r="G20" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A20,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E20)),NOT(ISNUMBER($F20))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A20,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E20=INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0)),$F20=INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E20-$F20)=(INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E20&gt;$F20,INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),AND($E20=$F20,INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),AND($E20&lt;$F20,INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E20=INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0)),$F20=INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E20-$F20)=(INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H20&lt;&gt;"",$H20=INDEX(Partidos!$K$4:$K$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A20,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E20)),NOT(ISNUMBER($F20))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A20,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E20=INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0)),$F20=INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E20-$F20)=(INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E20&gt;$F20,INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),AND($E20=$F20,INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),AND($E20&lt;$F20,INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0)),IF(AND($E20=INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0)),$F20=INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),IF(AND($H20&lt;&gt;"",$H20=INDEX(Partidos!$K$4:$K$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E20=$F20,($E20-$F20)=(INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0)))),IF(AND($H20&lt;&gt;"",$H20=INDEX(Partidos!$K$4:$K$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H20&lt;&gt;"",$H20=INDEX(Partidos!$K$4:$K$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E20=INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0)),$F20=INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E20-$F20)=(INDEX(Partidos!$F$4:$F$107,MATCH($A20,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H20&lt;&gt;"",$H20=INDEX(Partidos!$K$4:$K$107,MATCH($A20,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H20" s="19">
@@ -10781,7 +10826,7 @@
         <v/>
       </c>
       <c r="G21" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A21,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E21)),NOT(ISNUMBER($F21))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A21,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E21=INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0)),$F21=INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E21-$F21)=(INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E21&gt;$F21,INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),AND($E21=$F21,INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),AND($E21&lt;$F21,INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E21=INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0)),$F21=INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E21-$F21)=(INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H21&lt;&gt;"",$H21=INDEX(Partidos!$K$4:$K$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A21,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E21)),NOT(ISNUMBER($F21))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A21,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E21=INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0)),$F21=INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E21-$F21)=(INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E21&gt;$F21,INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),AND($E21=$F21,INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),AND($E21&lt;$F21,INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0)),IF(AND($E21=INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0)),$F21=INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),IF(AND($H21&lt;&gt;"",$H21=INDEX(Partidos!$K$4:$K$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E21=$F21,($E21-$F21)=(INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0)))),IF(AND($H21&lt;&gt;"",$H21=INDEX(Partidos!$K$4:$K$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H21&lt;&gt;"",$H21=INDEX(Partidos!$K$4:$K$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E21=INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0)),$F21=INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E21-$F21)=(INDEX(Partidos!$F$4:$F$107,MATCH($A21,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H21&lt;&gt;"",$H21=INDEX(Partidos!$K$4:$K$107,MATCH($A21,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H21" s="19">
@@ -10823,7 +10868,7 @@
         <v/>
       </c>
       <c r="G22" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A22,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E22)),NOT(ISNUMBER($F22))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A22,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E22=INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0)),$F22=INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E22-$F22)=(INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E22&gt;$F22,INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),AND($E22=$F22,INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),AND($E22&lt;$F22,INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E22=INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0)),$F22=INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E22-$F22)=(INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H22&lt;&gt;"",$H22=INDEX(Partidos!$K$4:$K$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A22,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E22)),NOT(ISNUMBER($F22))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A22,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E22=INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0)),$F22=INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E22-$F22)=(INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E22&gt;$F22,INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),AND($E22=$F22,INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),AND($E22&lt;$F22,INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0)),IF(AND($E22=INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0)),$F22=INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),IF(AND($H22&lt;&gt;"",$H22=INDEX(Partidos!$K$4:$K$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E22=$F22,($E22-$F22)=(INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0)))),IF(AND($H22&lt;&gt;"",$H22=INDEX(Partidos!$K$4:$K$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H22&lt;&gt;"",$H22=INDEX(Partidos!$K$4:$K$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E22=INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0)),$F22=INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E22-$F22)=(INDEX(Partidos!$F$4:$F$107,MATCH($A22,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H22&lt;&gt;"",$H22=INDEX(Partidos!$K$4:$K$107,MATCH($A22,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H22" s="19">
@@ -10865,7 +10910,7 @@
         <v/>
       </c>
       <c r="G23" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A23,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E23)),NOT(ISNUMBER($F23))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A23,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E23=INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0)),$F23=INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E23-$F23)=(INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E23&gt;$F23,INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),AND($E23=$F23,INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),AND($E23&lt;$F23,INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E23=INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0)),$F23=INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E23-$F23)=(INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H23&lt;&gt;"",$H23=INDEX(Partidos!$K$4:$K$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A23,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E23)),NOT(ISNUMBER($F23))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A23,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E23=INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0)),$F23=INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E23-$F23)=(INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E23&gt;$F23,INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),AND($E23=$F23,INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),AND($E23&lt;$F23,INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0)),IF(AND($E23=INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0)),$F23=INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),IF(AND($H23&lt;&gt;"",$H23=INDEX(Partidos!$K$4:$K$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E23=$F23,($E23-$F23)=(INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0)))),IF(AND($H23&lt;&gt;"",$H23=INDEX(Partidos!$K$4:$K$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H23&lt;&gt;"",$H23=INDEX(Partidos!$K$4:$K$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E23=INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0)),$F23=INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E23-$F23)=(INDEX(Partidos!$F$4:$F$107,MATCH($A23,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H23&lt;&gt;"",$H23=INDEX(Partidos!$K$4:$K$107,MATCH($A23,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H23" s="19">
@@ -10907,7 +10952,7 @@
         <v/>
       </c>
       <c r="G24" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A24,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E24)),NOT(ISNUMBER($F24))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A24,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E24=INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0)),$F24=INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E24-$F24)=(INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E24&gt;$F24,INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),AND($E24=$F24,INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),AND($E24&lt;$F24,INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E24=INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0)),$F24=INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E24-$F24)=(INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H24&lt;&gt;"",$H24=INDEX(Partidos!$K$4:$K$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A24,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E24)),NOT(ISNUMBER($F24))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A24,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E24=INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0)),$F24=INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E24-$F24)=(INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E24&gt;$F24,INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),AND($E24=$F24,INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),AND($E24&lt;$F24,INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0)),IF(AND($E24=INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0)),$F24=INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),IF(AND($H24&lt;&gt;"",$H24=INDEX(Partidos!$K$4:$K$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E24=$F24,($E24-$F24)=(INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0)))),IF(AND($H24&lt;&gt;"",$H24=INDEX(Partidos!$K$4:$K$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H24&lt;&gt;"",$H24=INDEX(Partidos!$K$4:$K$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E24=INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0)),$F24=INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E24-$F24)=(INDEX(Partidos!$F$4:$F$107,MATCH($A24,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H24&lt;&gt;"",$H24=INDEX(Partidos!$K$4:$K$107,MATCH($A24,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H24" s="19">
@@ -10949,7 +10994,7 @@
         <v/>
       </c>
       <c r="G25" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A25,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E25)),NOT(ISNUMBER($F25))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A25,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E25=INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0)),$F25=INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E25-$F25)=(INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E25&gt;$F25,INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),AND($E25=$F25,INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),AND($E25&lt;$F25,INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E25=INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0)),$F25=INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E25-$F25)=(INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H25&lt;&gt;"",$H25=INDEX(Partidos!$K$4:$K$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A25,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E25)),NOT(ISNUMBER($F25))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A25,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E25=INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0)),$F25=INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E25-$F25)=(INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E25&gt;$F25,INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),AND($E25=$F25,INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),AND($E25&lt;$F25,INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0)),IF(AND($E25=INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0)),$F25=INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),IF(AND($H25&lt;&gt;"",$H25=INDEX(Partidos!$K$4:$K$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E25=$F25,($E25-$F25)=(INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0)))),IF(AND($H25&lt;&gt;"",$H25=INDEX(Partidos!$K$4:$K$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H25&lt;&gt;"",$H25=INDEX(Partidos!$K$4:$K$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E25=INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0)),$F25=INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E25-$F25)=(INDEX(Partidos!$F$4:$F$107,MATCH($A25,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H25&lt;&gt;"",$H25=INDEX(Partidos!$K$4:$K$107,MATCH($A25,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H25" s="19">
@@ -10991,7 +11036,7 @@
         <v/>
       </c>
       <c r="G26" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A26,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E26)),NOT(ISNUMBER($F26))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A26,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E26=INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0)),$F26=INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E26-$F26)=(INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E26&gt;$F26,INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),AND($E26=$F26,INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),AND($E26&lt;$F26,INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E26=INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0)),$F26=INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E26-$F26)=(INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H26&lt;&gt;"",$H26=INDEX(Partidos!$K$4:$K$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A26,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E26)),NOT(ISNUMBER($F26))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A26,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E26=INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0)),$F26=INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E26-$F26)=(INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E26&gt;$F26,INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),AND($E26=$F26,INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),AND($E26&lt;$F26,INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0)),IF(AND($E26=INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0)),$F26=INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),IF(AND($H26&lt;&gt;"",$H26=INDEX(Partidos!$K$4:$K$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E26=$F26,($E26-$F26)=(INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0)))),IF(AND($H26&lt;&gt;"",$H26=INDEX(Partidos!$K$4:$K$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H26&lt;&gt;"",$H26=INDEX(Partidos!$K$4:$K$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E26=INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0)),$F26=INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E26-$F26)=(INDEX(Partidos!$F$4:$F$107,MATCH($A26,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H26&lt;&gt;"",$H26=INDEX(Partidos!$K$4:$K$107,MATCH($A26,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H26" s="19">
@@ -11033,7 +11078,7 @@
         <v/>
       </c>
       <c r="G27" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A27,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E27)),NOT(ISNUMBER($F27))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A27,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E27=INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0)),$F27=INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E27-$F27)=(INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E27&gt;$F27,INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),AND($E27=$F27,INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),AND($E27&lt;$F27,INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E27=INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0)),$F27=INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E27-$F27)=(INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H27&lt;&gt;"",$H27=INDEX(Partidos!$K$4:$K$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A27,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E27)),NOT(ISNUMBER($F27))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A27,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E27=INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0)),$F27=INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E27-$F27)=(INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E27&gt;$F27,INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),AND($E27=$F27,INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),AND($E27&lt;$F27,INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0)),IF(AND($E27=INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0)),$F27=INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),IF(AND($H27&lt;&gt;"",$H27=INDEX(Partidos!$K$4:$K$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E27=$F27,($E27-$F27)=(INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0)))),IF(AND($H27&lt;&gt;"",$H27=INDEX(Partidos!$K$4:$K$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H27&lt;&gt;"",$H27=INDEX(Partidos!$K$4:$K$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E27=INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0)),$F27=INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E27-$F27)=(INDEX(Partidos!$F$4:$F$107,MATCH($A27,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H27&lt;&gt;"",$H27=INDEX(Partidos!$K$4:$K$107,MATCH($A27,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H27" s="19">
@@ -11075,7 +11120,7 @@
         <v/>
       </c>
       <c r="G28" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A28,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E28)),NOT(ISNUMBER($F28))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A28,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E28=INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0)),$F28=INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E28-$F28)=(INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E28&gt;$F28,INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),AND($E28=$F28,INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),AND($E28&lt;$F28,INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E28=INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0)),$F28=INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E28-$F28)=(INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H28&lt;&gt;"",$H28=INDEX(Partidos!$K$4:$K$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A28,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E28)),NOT(ISNUMBER($F28))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A28,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E28=INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0)),$F28=INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E28-$F28)=(INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E28&gt;$F28,INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),AND($E28=$F28,INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),AND($E28&lt;$F28,INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0)),IF(AND($E28=INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0)),$F28=INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),IF(AND($H28&lt;&gt;"",$H28=INDEX(Partidos!$K$4:$K$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E28=$F28,($E28-$F28)=(INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0)))),IF(AND($H28&lt;&gt;"",$H28=INDEX(Partidos!$K$4:$K$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H28&lt;&gt;"",$H28=INDEX(Partidos!$K$4:$K$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E28=INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0)),$F28=INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E28-$F28)=(INDEX(Partidos!$F$4:$F$107,MATCH($A28,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H28&lt;&gt;"",$H28=INDEX(Partidos!$K$4:$K$107,MATCH($A28,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H28" s="19">
@@ -11117,7 +11162,7 @@
         <v/>
       </c>
       <c r="G29" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A29,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E29)),NOT(ISNUMBER($F29))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A29,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E29=INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0)),$F29=INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E29-$F29)=(INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E29&gt;$F29,INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),AND($E29=$F29,INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),AND($E29&lt;$F29,INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E29=INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0)),$F29=INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E29-$F29)=(INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H29&lt;&gt;"",$H29=INDEX(Partidos!$K$4:$K$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A29,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E29)),NOT(ISNUMBER($F29))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A29,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E29=INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0)),$F29=INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E29-$F29)=(INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E29&gt;$F29,INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),AND($E29=$F29,INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),AND($E29&lt;$F29,INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0)),IF(AND($E29=INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0)),$F29=INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),IF(AND($H29&lt;&gt;"",$H29=INDEX(Partidos!$K$4:$K$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E29=$F29,($E29-$F29)=(INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0)))),IF(AND($H29&lt;&gt;"",$H29=INDEX(Partidos!$K$4:$K$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H29&lt;&gt;"",$H29=INDEX(Partidos!$K$4:$K$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E29=INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0)),$F29=INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E29-$F29)=(INDEX(Partidos!$F$4:$F$107,MATCH($A29,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H29&lt;&gt;"",$H29=INDEX(Partidos!$K$4:$K$107,MATCH($A29,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H29" s="19">
@@ -11159,7 +11204,7 @@
         <v/>
       </c>
       <c r="G30" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A30,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E30)),NOT(ISNUMBER($F30))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A30,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E30=INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0)),$F30=INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E30-$F30)=(INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E30&gt;$F30,INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),AND($E30=$F30,INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),AND($E30&lt;$F30,INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E30=INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0)),$F30=INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E30-$F30)=(INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H30&lt;&gt;"",$H30=INDEX(Partidos!$K$4:$K$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A30,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E30)),NOT(ISNUMBER($F30))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A30,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E30=INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0)),$F30=INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E30-$F30)=(INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E30&gt;$F30,INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),AND($E30=$F30,INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),AND($E30&lt;$F30,INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0)),IF(AND($E30=INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0)),$F30=INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),IF(AND($H30&lt;&gt;"",$H30=INDEX(Partidos!$K$4:$K$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E30=$F30,($E30-$F30)=(INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0)))),IF(AND($H30&lt;&gt;"",$H30=INDEX(Partidos!$K$4:$K$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H30&lt;&gt;"",$H30=INDEX(Partidos!$K$4:$K$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E30=INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0)),$F30=INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E30-$F30)=(INDEX(Partidos!$F$4:$F$107,MATCH($A30,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H30&lt;&gt;"",$H30=INDEX(Partidos!$K$4:$K$107,MATCH($A30,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H30" s="19">
@@ -11201,7 +11246,7 @@
         <v/>
       </c>
       <c r="G31" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A31,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E31)),NOT(ISNUMBER($F31))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A31,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E31=INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0)),$F31=INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E31-$F31)=(INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E31&gt;$F31,INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),AND($E31=$F31,INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),AND($E31&lt;$F31,INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E31=INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0)),$F31=INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E31-$F31)=(INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H31&lt;&gt;"",$H31=INDEX(Partidos!$K$4:$K$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A31,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E31)),NOT(ISNUMBER($F31))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A31,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E31=INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0)),$F31=INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E31-$F31)=(INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E31&gt;$F31,INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),AND($E31=$F31,INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),AND($E31&lt;$F31,INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0)),IF(AND($E31=INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0)),$F31=INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),IF(AND($H31&lt;&gt;"",$H31=INDEX(Partidos!$K$4:$K$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E31=$F31,($E31-$F31)=(INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0)))),IF(AND($H31&lt;&gt;"",$H31=INDEX(Partidos!$K$4:$K$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H31&lt;&gt;"",$H31=INDEX(Partidos!$K$4:$K$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E31=INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0)),$F31=INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E31-$F31)=(INDEX(Partidos!$F$4:$F$107,MATCH($A31,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H31&lt;&gt;"",$H31=INDEX(Partidos!$K$4:$K$107,MATCH($A31,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H31" s="19">
@@ -11243,7 +11288,7 @@
         <v/>
       </c>
       <c r="G32" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A32,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E32)),NOT(ISNUMBER($F32))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A32,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E32=INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0)),$F32=INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E32-$F32)=(INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E32&gt;$F32,INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),AND($E32=$F32,INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),AND($E32&lt;$F32,INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E32=INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0)),$F32=INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E32-$F32)=(INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H32&lt;&gt;"",$H32=INDEX(Partidos!$K$4:$K$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A32,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E32)),NOT(ISNUMBER($F32))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A32,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E32=INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0)),$F32=INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E32-$F32)=(INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E32&gt;$F32,INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),AND($E32=$F32,INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),AND($E32&lt;$F32,INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0)),IF(AND($E32=INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0)),$F32=INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),IF(AND($H32&lt;&gt;"",$H32=INDEX(Partidos!$K$4:$K$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E32=$F32,($E32-$F32)=(INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0)))),IF(AND($H32&lt;&gt;"",$H32=INDEX(Partidos!$K$4:$K$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H32&lt;&gt;"",$H32=INDEX(Partidos!$K$4:$K$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E32=INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0)),$F32=INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E32-$F32)=(INDEX(Partidos!$F$4:$F$107,MATCH($A32,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H32&lt;&gt;"",$H32=INDEX(Partidos!$K$4:$K$107,MATCH($A32,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H32" s="19">
@@ -11285,7 +11330,7 @@
         <v/>
       </c>
       <c r="G33" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A33,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E33)),NOT(ISNUMBER($F33))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A33,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E33=INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0)),$F33=INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E33-$F33)=(INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E33&gt;$F33,INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),AND($E33=$F33,INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),AND($E33&lt;$F33,INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E33=INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0)),$F33=INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E33-$F33)=(INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H33&lt;&gt;"",$H33=INDEX(Partidos!$K$4:$K$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A33,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E33)),NOT(ISNUMBER($F33))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A33,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E33=INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0)),$F33=INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E33-$F33)=(INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E33&gt;$F33,INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),AND($E33=$F33,INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),AND($E33&lt;$F33,INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0)),IF(AND($E33=INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0)),$F33=INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),IF(AND($H33&lt;&gt;"",$H33=INDEX(Partidos!$K$4:$K$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E33=$F33,($E33-$F33)=(INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0)))),IF(AND($H33&lt;&gt;"",$H33=INDEX(Partidos!$K$4:$K$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H33&lt;&gt;"",$H33=INDEX(Partidos!$K$4:$K$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E33=INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0)),$F33=INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E33-$F33)=(INDEX(Partidos!$F$4:$F$107,MATCH($A33,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H33&lt;&gt;"",$H33=INDEX(Partidos!$K$4:$K$107,MATCH($A33,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H33" s="19">
@@ -11327,7 +11372,7 @@
         <v/>
       </c>
       <c r="G34" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A34,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E34)),NOT(ISNUMBER($F34))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A34,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E34=INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0)),$F34=INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E34-$F34)=(INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E34&gt;$F34,INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),AND($E34=$F34,INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),AND($E34&lt;$F34,INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E34=INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0)),$F34=INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E34-$F34)=(INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H34&lt;&gt;"",$H34=INDEX(Partidos!$K$4:$K$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A34,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E34)),NOT(ISNUMBER($F34))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A34,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E34=INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0)),$F34=INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E34-$F34)=(INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E34&gt;$F34,INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),AND($E34=$F34,INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),AND($E34&lt;$F34,INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0)),IF(AND($E34=INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0)),$F34=INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),IF(AND($H34&lt;&gt;"",$H34=INDEX(Partidos!$K$4:$K$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E34=$F34,($E34-$F34)=(INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0)))),IF(AND($H34&lt;&gt;"",$H34=INDEX(Partidos!$K$4:$K$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H34&lt;&gt;"",$H34=INDEX(Partidos!$K$4:$K$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E34=INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0)),$F34=INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E34-$F34)=(INDEX(Partidos!$F$4:$F$107,MATCH($A34,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H34&lt;&gt;"",$H34=INDEX(Partidos!$K$4:$K$107,MATCH($A34,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H34" s="19">
@@ -11369,7 +11414,7 @@
         <v/>
       </c>
       <c r="G35" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A35,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E35)),NOT(ISNUMBER($F35))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A35,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E35=INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0)),$F35=INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E35-$F35)=(INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E35&gt;$F35,INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),AND($E35=$F35,INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),AND($E35&lt;$F35,INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E35=INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0)),$F35=INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E35-$F35)=(INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H35&lt;&gt;"",$H35=INDEX(Partidos!$K$4:$K$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A35,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E35)),NOT(ISNUMBER($F35))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A35,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E35=INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0)),$F35=INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E35-$F35)=(INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E35&gt;$F35,INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),AND($E35=$F35,INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),AND($E35&lt;$F35,INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0)),IF(AND($E35=INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0)),$F35=INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),IF(AND($H35&lt;&gt;"",$H35=INDEX(Partidos!$K$4:$K$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E35=$F35,($E35-$F35)=(INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0)))),IF(AND($H35&lt;&gt;"",$H35=INDEX(Partidos!$K$4:$K$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H35&lt;&gt;"",$H35=INDEX(Partidos!$K$4:$K$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E35=INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0)),$F35=INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E35-$F35)=(INDEX(Partidos!$F$4:$F$107,MATCH($A35,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H35&lt;&gt;"",$H35=INDEX(Partidos!$K$4:$K$107,MATCH($A35,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H35" s="19">
@@ -11411,7 +11456,7 @@
         <v/>
       </c>
       <c r="G36" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A36,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E36)),NOT(ISNUMBER($F36))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A36,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E36=INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0)),$F36=INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E36-$F36)=(INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E36&gt;$F36,INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),AND($E36=$F36,INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),AND($E36&lt;$F36,INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E36=INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0)),$F36=INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E36-$F36)=(INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H36&lt;&gt;"",$H36=INDEX(Partidos!$K$4:$K$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A36,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E36)),NOT(ISNUMBER($F36))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A36,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E36=INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0)),$F36=INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E36-$F36)=(INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E36&gt;$F36,INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),AND($E36=$F36,INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),AND($E36&lt;$F36,INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0)),IF(AND($E36=INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0)),$F36=INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),IF(AND($H36&lt;&gt;"",$H36=INDEX(Partidos!$K$4:$K$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E36=$F36,($E36-$F36)=(INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0)))),IF(AND($H36&lt;&gt;"",$H36=INDEX(Partidos!$K$4:$K$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H36&lt;&gt;"",$H36=INDEX(Partidos!$K$4:$K$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E36=INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0)),$F36=INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E36-$F36)=(INDEX(Partidos!$F$4:$F$107,MATCH($A36,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H36&lt;&gt;"",$H36=INDEX(Partidos!$K$4:$K$107,MATCH($A36,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H36" s="19">
@@ -11453,7 +11498,7 @@
         <v/>
       </c>
       <c r="G37" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A37,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E37)),NOT(ISNUMBER($F37))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A37,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E37=INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0)),$F37=INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E37-$F37)=(INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E37&gt;$F37,INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),AND($E37=$F37,INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),AND($E37&lt;$F37,INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E37=INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0)),$F37=INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E37-$F37)=(INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H37&lt;&gt;"",$H37=INDEX(Partidos!$K$4:$K$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A37,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E37)),NOT(ISNUMBER($F37))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A37,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E37=INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0)),$F37=INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E37-$F37)=(INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E37&gt;$F37,INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),AND($E37=$F37,INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),AND($E37&lt;$F37,INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0)),IF(AND($E37=INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0)),$F37=INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),IF(AND($H37&lt;&gt;"",$H37=INDEX(Partidos!$K$4:$K$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E37=$F37,($E37-$F37)=(INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0)))),IF(AND($H37&lt;&gt;"",$H37=INDEX(Partidos!$K$4:$K$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H37&lt;&gt;"",$H37=INDEX(Partidos!$K$4:$K$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E37=INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0)),$F37=INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E37-$F37)=(INDEX(Partidos!$F$4:$F$107,MATCH($A37,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H37&lt;&gt;"",$H37=INDEX(Partidos!$K$4:$K$107,MATCH($A37,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H37" s="19">
@@ -11495,7 +11540,7 @@
         <v/>
       </c>
       <c r="G38" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A38,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E38)),NOT(ISNUMBER($F38))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A38,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E38=INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0)),$F38=INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E38-$F38)=(INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E38&gt;$F38,INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),AND($E38=$F38,INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),AND($E38&lt;$F38,INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E38=INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0)),$F38=INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E38-$F38)=(INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H38&lt;&gt;"",$H38=INDEX(Partidos!$K$4:$K$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A38,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E38)),NOT(ISNUMBER($F38))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A38,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E38=INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0)),$F38=INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E38-$F38)=(INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E38&gt;$F38,INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),AND($E38=$F38,INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),AND($E38&lt;$F38,INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0)),IF(AND($E38=INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0)),$F38=INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),IF(AND($H38&lt;&gt;"",$H38=INDEX(Partidos!$K$4:$K$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E38=$F38,($E38-$F38)=(INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0)))),IF(AND($H38&lt;&gt;"",$H38=INDEX(Partidos!$K$4:$K$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H38&lt;&gt;"",$H38=INDEX(Partidos!$K$4:$K$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E38=INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0)),$F38=INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E38-$F38)=(INDEX(Partidos!$F$4:$F$107,MATCH($A38,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H38&lt;&gt;"",$H38=INDEX(Partidos!$K$4:$K$107,MATCH($A38,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H38" s="19">
@@ -11537,7 +11582,7 @@
         <v/>
       </c>
       <c r="G39" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A39,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E39)),NOT(ISNUMBER($F39))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A39,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E39=INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0)),$F39=INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E39-$F39)=(INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E39&gt;$F39,INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),AND($E39=$F39,INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),AND($E39&lt;$F39,INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E39=INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0)),$F39=INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E39-$F39)=(INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H39&lt;&gt;"",$H39=INDEX(Partidos!$K$4:$K$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A39,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E39)),NOT(ISNUMBER($F39))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A39,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E39=INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0)),$F39=INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E39-$F39)=(INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E39&gt;$F39,INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),AND($E39=$F39,INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),AND($E39&lt;$F39,INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0)),IF(AND($E39=INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0)),$F39=INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),IF(AND($H39&lt;&gt;"",$H39=INDEX(Partidos!$K$4:$K$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E39=$F39,($E39-$F39)=(INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0)))),IF(AND($H39&lt;&gt;"",$H39=INDEX(Partidos!$K$4:$K$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H39&lt;&gt;"",$H39=INDEX(Partidos!$K$4:$K$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E39=INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0)),$F39=INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E39-$F39)=(INDEX(Partidos!$F$4:$F$107,MATCH($A39,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H39&lt;&gt;"",$H39=INDEX(Partidos!$K$4:$K$107,MATCH($A39,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H39" s="19">
@@ -11579,7 +11624,7 @@
         <v/>
       </c>
       <c r="G40" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A40,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E40)),NOT(ISNUMBER($F40))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A40,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E40=INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0)),$F40=INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E40-$F40)=(INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E40&gt;$F40,INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),AND($E40=$F40,INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),AND($E40&lt;$F40,INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E40=INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0)),$F40=INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E40-$F40)=(INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H40&lt;&gt;"",$H40=INDEX(Partidos!$K$4:$K$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A40,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E40)),NOT(ISNUMBER($F40))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A40,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E40=INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0)),$F40=INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E40-$F40)=(INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E40&gt;$F40,INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),AND($E40=$F40,INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),AND($E40&lt;$F40,INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0)),IF(AND($E40=INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0)),$F40=INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),IF(AND($H40&lt;&gt;"",$H40=INDEX(Partidos!$K$4:$K$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E40=$F40,($E40-$F40)=(INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0)))),IF(AND($H40&lt;&gt;"",$H40=INDEX(Partidos!$K$4:$K$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H40&lt;&gt;"",$H40=INDEX(Partidos!$K$4:$K$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E40=INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0)),$F40=INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E40-$F40)=(INDEX(Partidos!$F$4:$F$107,MATCH($A40,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H40&lt;&gt;"",$H40=INDEX(Partidos!$K$4:$K$107,MATCH($A40,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H40" s="19">
@@ -11621,7 +11666,7 @@
         <v/>
       </c>
       <c r="G41" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A41,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E41)),NOT(ISNUMBER($F41))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A41,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E41=INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0)),$F41=INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E41-$F41)=(INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E41&gt;$F41,INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),AND($E41=$F41,INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),AND($E41&lt;$F41,INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E41=INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0)),$F41=INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E41-$F41)=(INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H41&lt;&gt;"",$H41=INDEX(Partidos!$K$4:$K$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A41,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E41)),NOT(ISNUMBER($F41))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A41,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E41=INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0)),$F41=INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E41-$F41)=(INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E41&gt;$F41,INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),AND($E41=$F41,INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),AND($E41&lt;$F41,INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0)),IF(AND($E41=INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0)),$F41=INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),IF(AND($H41&lt;&gt;"",$H41=INDEX(Partidos!$K$4:$K$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E41=$F41,($E41-$F41)=(INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0)))),IF(AND($H41&lt;&gt;"",$H41=INDEX(Partidos!$K$4:$K$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H41&lt;&gt;"",$H41=INDEX(Partidos!$K$4:$K$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E41=INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0)),$F41=INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E41-$F41)=(INDEX(Partidos!$F$4:$F$107,MATCH($A41,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H41&lt;&gt;"",$H41=INDEX(Partidos!$K$4:$K$107,MATCH($A41,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H41" s="19">
@@ -11663,7 +11708,7 @@
         <v/>
       </c>
       <c r="G42" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A42,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E42)),NOT(ISNUMBER($F42))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A42,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E42=INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0)),$F42=INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E42-$F42)=(INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E42&gt;$F42,INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),AND($E42=$F42,INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),AND($E42&lt;$F42,INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E42=INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0)),$F42=INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E42-$F42)=(INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H42&lt;&gt;"",$H42=INDEX(Partidos!$K$4:$K$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A42,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E42)),NOT(ISNUMBER($F42))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A42,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E42=INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0)),$F42=INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E42-$F42)=(INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E42&gt;$F42,INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),AND($E42=$F42,INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),AND($E42&lt;$F42,INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0)),IF(AND($E42=INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0)),$F42=INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),IF(AND($H42&lt;&gt;"",$H42=INDEX(Partidos!$K$4:$K$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E42=$F42,($E42-$F42)=(INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0)))),IF(AND($H42&lt;&gt;"",$H42=INDEX(Partidos!$K$4:$K$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H42&lt;&gt;"",$H42=INDEX(Partidos!$K$4:$K$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E42=INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0)),$F42=INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E42-$F42)=(INDEX(Partidos!$F$4:$F$107,MATCH($A42,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H42&lt;&gt;"",$H42=INDEX(Partidos!$K$4:$K$107,MATCH($A42,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H42" s="19">
@@ -11705,7 +11750,7 @@
         <v/>
       </c>
       <c r="G43" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A43,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E43)),NOT(ISNUMBER($F43))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A43,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E43=INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0)),$F43=INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E43-$F43)=(INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E43&gt;$F43,INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),AND($E43=$F43,INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),AND($E43&lt;$F43,INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E43=INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0)),$F43=INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E43-$F43)=(INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H43&lt;&gt;"",$H43=INDEX(Partidos!$K$4:$K$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A43,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E43)),NOT(ISNUMBER($F43))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A43,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E43=INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0)),$F43=INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E43-$F43)=(INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E43&gt;$F43,INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),AND($E43=$F43,INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),AND($E43&lt;$F43,INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0)),IF(AND($E43=INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0)),$F43=INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),IF(AND($H43&lt;&gt;"",$H43=INDEX(Partidos!$K$4:$K$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E43=$F43,($E43-$F43)=(INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0)))),IF(AND($H43&lt;&gt;"",$H43=INDEX(Partidos!$K$4:$K$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H43&lt;&gt;"",$H43=INDEX(Partidos!$K$4:$K$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E43=INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0)),$F43=INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E43-$F43)=(INDEX(Partidos!$F$4:$F$107,MATCH($A43,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H43&lt;&gt;"",$H43=INDEX(Partidos!$K$4:$K$107,MATCH($A43,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H43" s="19">
@@ -11747,7 +11792,7 @@
         <v/>
       </c>
       <c r="G44" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A44,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E44)),NOT(ISNUMBER($F44))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A44,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E44=INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0)),$F44=INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E44-$F44)=(INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E44&gt;$F44,INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),AND($E44=$F44,INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),AND($E44&lt;$F44,INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E44=INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0)),$F44=INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E44-$F44)=(INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H44&lt;&gt;"",$H44=INDEX(Partidos!$K$4:$K$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A44,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E44)),NOT(ISNUMBER($F44))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A44,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E44=INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0)),$F44=INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E44-$F44)=(INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E44&gt;$F44,INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),AND($E44=$F44,INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),AND($E44&lt;$F44,INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0)),IF(AND($E44=INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0)),$F44=INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),IF(AND($H44&lt;&gt;"",$H44=INDEX(Partidos!$K$4:$K$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E44=$F44,($E44-$F44)=(INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0)))),IF(AND($H44&lt;&gt;"",$H44=INDEX(Partidos!$K$4:$K$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H44&lt;&gt;"",$H44=INDEX(Partidos!$K$4:$K$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E44=INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0)),$F44=INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E44-$F44)=(INDEX(Partidos!$F$4:$F$107,MATCH($A44,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H44&lt;&gt;"",$H44=INDEX(Partidos!$K$4:$K$107,MATCH($A44,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H44" s="19">
@@ -11789,7 +11834,7 @@
         <v/>
       </c>
       <c r="G45" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A45,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E45)),NOT(ISNUMBER($F45))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A45,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E45=INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0)),$F45=INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E45-$F45)=(INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E45&gt;$F45,INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),AND($E45=$F45,INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),AND($E45&lt;$F45,INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E45=INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0)),$F45=INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E45-$F45)=(INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H45&lt;&gt;"",$H45=INDEX(Partidos!$K$4:$K$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A45,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E45)),NOT(ISNUMBER($F45))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A45,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E45=INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0)),$F45=INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E45-$F45)=(INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E45&gt;$F45,INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),AND($E45=$F45,INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),AND($E45&lt;$F45,INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0)),IF(AND($E45=INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0)),$F45=INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),IF(AND($H45&lt;&gt;"",$H45=INDEX(Partidos!$K$4:$K$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E45=$F45,($E45-$F45)=(INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0)))),IF(AND($H45&lt;&gt;"",$H45=INDEX(Partidos!$K$4:$K$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H45&lt;&gt;"",$H45=INDEX(Partidos!$K$4:$K$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E45=INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0)),$F45=INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E45-$F45)=(INDEX(Partidos!$F$4:$F$107,MATCH($A45,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H45&lt;&gt;"",$H45=INDEX(Partidos!$K$4:$K$107,MATCH($A45,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H45" s="19">
@@ -11831,7 +11876,7 @@
         <v/>
       </c>
       <c r="G46" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A46,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E46)),NOT(ISNUMBER($F46))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A46,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E46=INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0)),$F46=INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E46-$F46)=(INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E46&gt;$F46,INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),AND($E46=$F46,INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),AND($E46&lt;$F46,INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E46=INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0)),$F46=INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E46-$F46)=(INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H46&lt;&gt;"",$H46=INDEX(Partidos!$K$4:$K$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A46,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E46)),NOT(ISNUMBER($F46))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A46,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E46=INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0)),$F46=INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E46-$F46)=(INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E46&gt;$F46,INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),AND($E46=$F46,INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),AND($E46&lt;$F46,INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0)),IF(AND($E46=INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0)),$F46=INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),IF(AND($H46&lt;&gt;"",$H46=INDEX(Partidos!$K$4:$K$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E46=$F46,($E46-$F46)=(INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0)))),IF(AND($H46&lt;&gt;"",$H46=INDEX(Partidos!$K$4:$K$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H46&lt;&gt;"",$H46=INDEX(Partidos!$K$4:$K$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E46=INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0)),$F46=INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E46-$F46)=(INDEX(Partidos!$F$4:$F$107,MATCH($A46,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H46&lt;&gt;"",$H46=INDEX(Partidos!$K$4:$K$107,MATCH($A46,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H46" s="19">
@@ -11873,7 +11918,7 @@
         <v/>
       </c>
       <c r="G47" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A47,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E47)),NOT(ISNUMBER($F47))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A47,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E47=INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0)),$F47=INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E47-$F47)=(INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E47&gt;$F47,INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),AND($E47=$F47,INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),AND($E47&lt;$F47,INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E47=INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0)),$F47=INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E47-$F47)=(INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H47&lt;&gt;"",$H47=INDEX(Partidos!$K$4:$K$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A47,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E47)),NOT(ISNUMBER($F47))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A47,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E47=INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0)),$F47=INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E47-$F47)=(INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E47&gt;$F47,INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),AND($E47=$F47,INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),AND($E47&lt;$F47,INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0)),IF(AND($E47=INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0)),$F47=INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),IF(AND($H47&lt;&gt;"",$H47=INDEX(Partidos!$K$4:$K$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E47=$F47,($E47-$F47)=(INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0)))),IF(AND($H47&lt;&gt;"",$H47=INDEX(Partidos!$K$4:$K$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H47&lt;&gt;"",$H47=INDEX(Partidos!$K$4:$K$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E47=INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0)),$F47=INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E47-$F47)=(INDEX(Partidos!$F$4:$F$107,MATCH($A47,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H47&lt;&gt;"",$H47=INDEX(Partidos!$K$4:$K$107,MATCH($A47,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H47" s="19">
@@ -11915,7 +11960,7 @@
         <v/>
       </c>
       <c r="G48" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A48,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E48)),NOT(ISNUMBER($F48))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A48,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E48=INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0)),$F48=INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E48-$F48)=(INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E48&gt;$F48,INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),AND($E48=$F48,INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),AND($E48&lt;$F48,INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E48=INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0)),$F48=INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E48-$F48)=(INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H48&lt;&gt;"",$H48=INDEX(Partidos!$K$4:$K$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A48,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E48)),NOT(ISNUMBER($F48))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A48,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E48=INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0)),$F48=INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E48-$F48)=(INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E48&gt;$F48,INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),AND($E48=$F48,INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),AND($E48&lt;$F48,INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0)),IF(AND($E48=INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0)),$F48=INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),IF(AND($H48&lt;&gt;"",$H48=INDEX(Partidos!$K$4:$K$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E48=$F48,($E48-$F48)=(INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0)))),IF(AND($H48&lt;&gt;"",$H48=INDEX(Partidos!$K$4:$K$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H48&lt;&gt;"",$H48=INDEX(Partidos!$K$4:$K$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E48=INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0)),$F48=INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E48-$F48)=(INDEX(Partidos!$F$4:$F$107,MATCH($A48,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H48&lt;&gt;"",$H48=INDEX(Partidos!$K$4:$K$107,MATCH($A48,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H48" s="19">
@@ -11957,7 +12002,7 @@
         <v/>
       </c>
       <c r="G49" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A49,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E49)),NOT(ISNUMBER($F49))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A49,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E49=INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0)),$F49=INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E49-$F49)=(INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E49&gt;$F49,INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),AND($E49=$F49,INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),AND($E49&lt;$F49,INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E49=INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0)),$F49=INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E49-$F49)=(INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H49&lt;&gt;"",$H49=INDEX(Partidos!$K$4:$K$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A49,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E49)),NOT(ISNUMBER($F49))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A49,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E49=INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0)),$F49=INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E49-$F49)=(INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E49&gt;$F49,INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),AND($E49=$F49,INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),AND($E49&lt;$F49,INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0)),IF(AND($E49=INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0)),$F49=INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),IF(AND($H49&lt;&gt;"",$H49=INDEX(Partidos!$K$4:$K$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E49=$F49,($E49-$F49)=(INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0)))),IF(AND($H49&lt;&gt;"",$H49=INDEX(Partidos!$K$4:$K$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H49&lt;&gt;"",$H49=INDEX(Partidos!$K$4:$K$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E49=INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0)),$F49=INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E49-$F49)=(INDEX(Partidos!$F$4:$F$107,MATCH($A49,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H49&lt;&gt;"",$H49=INDEX(Partidos!$K$4:$K$107,MATCH($A49,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H49" s="19">
@@ -11999,7 +12044,7 @@
         <v/>
       </c>
       <c r="G50" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A50,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E50)),NOT(ISNUMBER($F50))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A50,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E50=INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0)),$F50=INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E50-$F50)=(INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E50&gt;$F50,INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),AND($E50=$F50,INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),AND($E50&lt;$F50,INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E50=INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0)),$F50=INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E50-$F50)=(INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H50&lt;&gt;"",$H50=INDEX(Partidos!$K$4:$K$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A50,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E50)),NOT(ISNUMBER($F50))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A50,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E50=INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0)),$F50=INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E50-$F50)=(INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E50&gt;$F50,INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),AND($E50=$F50,INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),AND($E50&lt;$F50,INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0)),IF(AND($E50=INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0)),$F50=INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),IF(AND($H50&lt;&gt;"",$H50=INDEX(Partidos!$K$4:$K$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E50=$F50,($E50-$F50)=(INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0)))),IF(AND($H50&lt;&gt;"",$H50=INDEX(Partidos!$K$4:$K$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H50&lt;&gt;"",$H50=INDEX(Partidos!$K$4:$K$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E50=INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0)),$F50=INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E50-$F50)=(INDEX(Partidos!$F$4:$F$107,MATCH($A50,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H50&lt;&gt;"",$H50=INDEX(Partidos!$K$4:$K$107,MATCH($A50,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H50" s="19">
@@ -12041,7 +12086,7 @@
         <v/>
       </c>
       <c r="G51" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A51,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E51)),NOT(ISNUMBER($F51))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A51,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E51=INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0)),$F51=INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E51-$F51)=(INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E51&gt;$F51,INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),AND($E51=$F51,INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),AND($E51&lt;$F51,INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E51=INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0)),$F51=INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E51-$F51)=(INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H51&lt;&gt;"",$H51=INDEX(Partidos!$K$4:$K$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A51,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E51)),NOT(ISNUMBER($F51))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A51,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E51=INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0)),$F51=INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E51-$F51)=(INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E51&gt;$F51,INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),AND($E51=$F51,INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),AND($E51&lt;$F51,INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0)),IF(AND($E51=INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0)),$F51=INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),IF(AND($H51&lt;&gt;"",$H51=INDEX(Partidos!$K$4:$K$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E51=$F51,($E51-$F51)=(INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0)))),IF(AND($H51&lt;&gt;"",$H51=INDEX(Partidos!$K$4:$K$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H51&lt;&gt;"",$H51=INDEX(Partidos!$K$4:$K$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E51=INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0)),$F51=INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E51-$F51)=(INDEX(Partidos!$F$4:$F$107,MATCH($A51,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H51&lt;&gt;"",$H51=INDEX(Partidos!$K$4:$K$107,MATCH($A51,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H51" s="19">
@@ -12083,7 +12128,7 @@
         <v/>
       </c>
       <c r="G52" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A52,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E52)),NOT(ISNUMBER($F52))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A52,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E52=INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0)),$F52=INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E52-$F52)=(INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E52&gt;$F52,INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),AND($E52=$F52,INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),AND($E52&lt;$F52,INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E52=INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0)),$F52=INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E52-$F52)=(INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H52&lt;&gt;"",$H52=INDEX(Partidos!$K$4:$K$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A52,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E52)),NOT(ISNUMBER($F52))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A52,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E52=INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0)),$F52=INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E52-$F52)=(INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E52&gt;$F52,INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),AND($E52=$F52,INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),AND($E52&lt;$F52,INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0)),IF(AND($E52=INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0)),$F52=INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),IF(AND($H52&lt;&gt;"",$H52=INDEX(Partidos!$K$4:$K$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E52=$F52,($E52-$F52)=(INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0)))),IF(AND($H52&lt;&gt;"",$H52=INDEX(Partidos!$K$4:$K$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H52&lt;&gt;"",$H52=INDEX(Partidos!$K$4:$K$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E52=INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0)),$F52=INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E52-$F52)=(INDEX(Partidos!$F$4:$F$107,MATCH($A52,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H52&lt;&gt;"",$H52=INDEX(Partidos!$K$4:$K$107,MATCH($A52,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H52" s="19">
@@ -12125,7 +12170,7 @@
         <v/>
       </c>
       <c r="G53" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A53,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E53)),NOT(ISNUMBER($F53))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A53,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E53=INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0)),$F53=INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E53-$F53)=(INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E53&gt;$F53,INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),AND($E53=$F53,INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),AND($E53&lt;$F53,INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E53=INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0)),$F53=INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E53-$F53)=(INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H53&lt;&gt;"",$H53=INDEX(Partidos!$K$4:$K$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A53,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E53)),NOT(ISNUMBER($F53))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A53,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E53=INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0)),$F53=INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E53-$F53)=(INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E53&gt;$F53,INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),AND($E53=$F53,INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),AND($E53&lt;$F53,INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0)),IF(AND($E53=INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0)),$F53=INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),IF(AND($H53&lt;&gt;"",$H53=INDEX(Partidos!$K$4:$K$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E53=$F53,($E53-$F53)=(INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0)))),IF(AND($H53&lt;&gt;"",$H53=INDEX(Partidos!$K$4:$K$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H53&lt;&gt;"",$H53=INDEX(Partidos!$K$4:$K$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E53=INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0)),$F53=INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E53-$F53)=(INDEX(Partidos!$F$4:$F$107,MATCH($A53,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H53&lt;&gt;"",$H53=INDEX(Partidos!$K$4:$K$107,MATCH($A53,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H53" s="19">
@@ -12167,7 +12212,7 @@
         <v/>
       </c>
       <c r="G54" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A54,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E54)),NOT(ISNUMBER($F54))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A54,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E54=INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0)),$F54=INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E54-$F54)=(INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E54&gt;$F54,INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),AND($E54=$F54,INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),AND($E54&lt;$F54,INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E54=INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0)),$F54=INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E54-$F54)=(INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H54&lt;&gt;"",$H54=INDEX(Partidos!$K$4:$K$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A54,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E54)),NOT(ISNUMBER($F54))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A54,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E54=INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0)),$F54=INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E54-$F54)=(INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E54&gt;$F54,INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),AND($E54=$F54,INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),AND($E54&lt;$F54,INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0)),IF(AND($E54=INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0)),$F54=INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),IF(AND($H54&lt;&gt;"",$H54=INDEX(Partidos!$K$4:$K$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E54=$F54,($E54-$F54)=(INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0)))),IF(AND($H54&lt;&gt;"",$H54=INDEX(Partidos!$K$4:$K$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H54&lt;&gt;"",$H54=INDEX(Partidos!$K$4:$K$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E54=INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0)),$F54=INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E54-$F54)=(INDEX(Partidos!$F$4:$F$107,MATCH($A54,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H54&lt;&gt;"",$H54=INDEX(Partidos!$K$4:$K$107,MATCH($A54,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H54" s="19">
@@ -12209,7 +12254,7 @@
         <v/>
       </c>
       <c r="G55" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A55,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E55)),NOT(ISNUMBER($F55))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A55,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E55=INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0)),$F55=INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E55-$F55)=(INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E55&gt;$F55,INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),AND($E55=$F55,INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),AND($E55&lt;$F55,INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E55=INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0)),$F55=INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E55-$F55)=(INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H55&lt;&gt;"",$H55=INDEX(Partidos!$K$4:$K$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A55,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E55)),NOT(ISNUMBER($F55))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A55,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E55=INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0)),$F55=INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E55-$F55)=(INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E55&gt;$F55,INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),AND($E55=$F55,INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),AND($E55&lt;$F55,INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0)),IF(AND($E55=INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0)),$F55=INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),IF(AND($H55&lt;&gt;"",$H55=INDEX(Partidos!$K$4:$K$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E55=$F55,($E55-$F55)=(INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0)))),IF(AND($H55&lt;&gt;"",$H55=INDEX(Partidos!$K$4:$K$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H55&lt;&gt;"",$H55=INDEX(Partidos!$K$4:$K$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E55=INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0)),$F55=INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E55-$F55)=(INDEX(Partidos!$F$4:$F$107,MATCH($A55,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H55&lt;&gt;"",$H55=INDEX(Partidos!$K$4:$K$107,MATCH($A55,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H55" s="19">
@@ -12251,7 +12296,7 @@
         <v/>
       </c>
       <c r="G56" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A56,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E56)),NOT(ISNUMBER($F56))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A56,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E56=INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0)),$F56=INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E56-$F56)=(INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E56&gt;$F56,INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),AND($E56=$F56,INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),AND($E56&lt;$F56,INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E56=INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0)),$F56=INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E56-$F56)=(INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H56&lt;&gt;"",$H56=INDEX(Partidos!$K$4:$K$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A56,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E56)),NOT(ISNUMBER($F56))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A56,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E56=INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0)),$F56=INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E56-$F56)=(INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E56&gt;$F56,INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),AND($E56=$F56,INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),AND($E56&lt;$F56,INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0)),IF(AND($E56=INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0)),$F56=INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),IF(AND($H56&lt;&gt;"",$H56=INDEX(Partidos!$K$4:$K$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E56=$F56,($E56-$F56)=(INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0)))),IF(AND($H56&lt;&gt;"",$H56=INDEX(Partidos!$K$4:$K$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H56&lt;&gt;"",$H56=INDEX(Partidos!$K$4:$K$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E56=INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0)),$F56=INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E56-$F56)=(INDEX(Partidos!$F$4:$F$107,MATCH($A56,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H56&lt;&gt;"",$H56=INDEX(Partidos!$K$4:$K$107,MATCH($A56,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H56" s="19">
@@ -12293,7 +12338,7 @@
         <v/>
       </c>
       <c r="G57" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A57,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E57)),NOT(ISNUMBER($F57))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A57,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E57=INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0)),$F57=INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E57-$F57)=(INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E57&gt;$F57,INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),AND($E57=$F57,INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),AND($E57&lt;$F57,INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E57=INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0)),$F57=INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E57-$F57)=(INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H57&lt;&gt;"",$H57=INDEX(Partidos!$K$4:$K$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A57,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E57)),NOT(ISNUMBER($F57))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A57,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E57=INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0)),$F57=INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E57-$F57)=(INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E57&gt;$F57,INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),AND($E57=$F57,INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),AND($E57&lt;$F57,INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0)),IF(AND($E57=INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0)),$F57=INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),IF(AND($H57&lt;&gt;"",$H57=INDEX(Partidos!$K$4:$K$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E57=$F57,($E57-$F57)=(INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0)))),IF(AND($H57&lt;&gt;"",$H57=INDEX(Partidos!$K$4:$K$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H57&lt;&gt;"",$H57=INDEX(Partidos!$K$4:$K$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E57=INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0)),$F57=INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E57-$F57)=(INDEX(Partidos!$F$4:$F$107,MATCH($A57,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H57&lt;&gt;"",$H57=INDEX(Partidos!$K$4:$K$107,MATCH($A57,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H57" s="19">
@@ -12335,7 +12380,7 @@
         <v/>
       </c>
       <c r="G58" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A58,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E58)),NOT(ISNUMBER($F58))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A58,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E58=INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0)),$F58=INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E58-$F58)=(INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E58&gt;$F58,INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),AND($E58=$F58,INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),AND($E58&lt;$F58,INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E58=INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0)),$F58=INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E58-$F58)=(INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H58&lt;&gt;"",$H58=INDEX(Partidos!$K$4:$K$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A58,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E58)),NOT(ISNUMBER($F58))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A58,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E58=INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0)),$F58=INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E58-$F58)=(INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E58&gt;$F58,INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),AND($E58=$F58,INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),AND($E58&lt;$F58,INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0)),IF(AND($E58=INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0)),$F58=INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),IF(AND($H58&lt;&gt;"",$H58=INDEX(Partidos!$K$4:$K$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E58=$F58,($E58-$F58)=(INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0)))),IF(AND($H58&lt;&gt;"",$H58=INDEX(Partidos!$K$4:$K$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H58&lt;&gt;"",$H58=INDEX(Partidos!$K$4:$K$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E58=INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0)),$F58=INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E58-$F58)=(INDEX(Partidos!$F$4:$F$107,MATCH($A58,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H58&lt;&gt;"",$H58=INDEX(Partidos!$K$4:$K$107,MATCH($A58,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H58" s="19">
@@ -12377,7 +12422,7 @@
         <v/>
       </c>
       <c r="G59" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A59,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E59)),NOT(ISNUMBER($F59))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A59,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E59=INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0)),$F59=INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E59-$F59)=(INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E59&gt;$F59,INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),AND($E59=$F59,INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),AND($E59&lt;$F59,INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E59=INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0)),$F59=INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E59-$F59)=(INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H59&lt;&gt;"",$H59=INDEX(Partidos!$K$4:$K$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A59,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E59)),NOT(ISNUMBER($F59))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A59,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E59=INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0)),$F59=INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E59-$F59)=(INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E59&gt;$F59,INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),AND($E59=$F59,INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),AND($E59&lt;$F59,INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0)),IF(AND($E59=INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0)),$F59=INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),IF(AND($H59&lt;&gt;"",$H59=INDEX(Partidos!$K$4:$K$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E59=$F59,($E59-$F59)=(INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0)))),IF(AND($H59&lt;&gt;"",$H59=INDEX(Partidos!$K$4:$K$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H59&lt;&gt;"",$H59=INDEX(Partidos!$K$4:$K$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E59=INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0)),$F59=INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E59-$F59)=(INDEX(Partidos!$F$4:$F$107,MATCH($A59,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H59&lt;&gt;"",$H59=INDEX(Partidos!$K$4:$K$107,MATCH($A59,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H59" s="19">
@@ -12419,7 +12464,7 @@
         <v/>
       </c>
       <c r="G60" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A60,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E60)),NOT(ISNUMBER($F60))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A60,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E60=INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0)),$F60=INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E60-$F60)=(INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E60&gt;$F60,INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),AND($E60=$F60,INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),AND($E60&lt;$F60,INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E60=INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0)),$F60=INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E60-$F60)=(INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H60&lt;&gt;"",$H60=INDEX(Partidos!$K$4:$K$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A60,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E60)),NOT(ISNUMBER($F60))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A60,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E60=INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0)),$F60=INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E60-$F60)=(INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E60&gt;$F60,INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),AND($E60=$F60,INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),AND($E60&lt;$F60,INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0)),IF(AND($E60=INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0)),$F60=INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),IF(AND($H60&lt;&gt;"",$H60=INDEX(Partidos!$K$4:$K$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E60=$F60,($E60-$F60)=(INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0)))),IF(AND($H60&lt;&gt;"",$H60=INDEX(Partidos!$K$4:$K$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H60&lt;&gt;"",$H60=INDEX(Partidos!$K$4:$K$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E60=INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0)),$F60=INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E60-$F60)=(INDEX(Partidos!$F$4:$F$107,MATCH($A60,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H60&lt;&gt;"",$H60=INDEX(Partidos!$K$4:$K$107,MATCH($A60,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H60" s="19">
@@ -12461,7 +12506,7 @@
         <v/>
       </c>
       <c r="G61" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A61,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E61)),NOT(ISNUMBER($F61))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A61,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E61=INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0)),$F61=INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E61-$F61)=(INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E61&gt;$F61,INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),AND($E61=$F61,INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),AND($E61&lt;$F61,INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E61=INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0)),$F61=INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E61-$F61)=(INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H61&lt;&gt;"",$H61=INDEX(Partidos!$K$4:$K$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A61,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E61)),NOT(ISNUMBER($F61))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A61,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E61=INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0)),$F61=INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E61-$F61)=(INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E61&gt;$F61,INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),AND($E61=$F61,INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),AND($E61&lt;$F61,INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0)),IF(AND($E61=INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0)),$F61=INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),IF(AND($H61&lt;&gt;"",$H61=INDEX(Partidos!$K$4:$K$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E61=$F61,($E61-$F61)=(INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0)))),IF(AND($H61&lt;&gt;"",$H61=INDEX(Partidos!$K$4:$K$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H61&lt;&gt;"",$H61=INDEX(Partidos!$K$4:$K$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E61=INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0)),$F61=INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E61-$F61)=(INDEX(Partidos!$F$4:$F$107,MATCH($A61,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H61&lt;&gt;"",$H61=INDEX(Partidos!$K$4:$K$107,MATCH($A61,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H61" s="19">
@@ -12503,7 +12548,7 @@
         <v/>
       </c>
       <c r="G62" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A62,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E62)),NOT(ISNUMBER($F62))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A62,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E62=INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0)),$F62=INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E62-$F62)=(INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E62&gt;$F62,INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),AND($E62=$F62,INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),AND($E62&lt;$F62,INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E62=INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0)),$F62=INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E62-$F62)=(INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H62&lt;&gt;"",$H62=INDEX(Partidos!$K$4:$K$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A62,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E62)),NOT(ISNUMBER($F62))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A62,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E62=INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0)),$F62=INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E62-$F62)=(INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E62&gt;$F62,INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),AND($E62=$F62,INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),AND($E62&lt;$F62,INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0)),IF(AND($E62=INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0)),$F62=INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),IF(AND($H62&lt;&gt;"",$H62=INDEX(Partidos!$K$4:$K$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E62=$F62,($E62-$F62)=(INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0)))),IF(AND($H62&lt;&gt;"",$H62=INDEX(Partidos!$K$4:$K$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H62&lt;&gt;"",$H62=INDEX(Partidos!$K$4:$K$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E62=INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0)),$F62=INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E62-$F62)=(INDEX(Partidos!$F$4:$F$107,MATCH($A62,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H62&lt;&gt;"",$H62=INDEX(Partidos!$K$4:$K$107,MATCH($A62,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H62" s="19">
@@ -12545,7 +12590,7 @@
         <v/>
       </c>
       <c r="G63" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A63,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E63)),NOT(ISNUMBER($F63))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A63,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E63=INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0)),$F63=INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E63-$F63)=(INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E63&gt;$F63,INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),AND($E63=$F63,INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),AND($E63&lt;$F63,INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E63=INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0)),$F63=INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E63-$F63)=(INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H63&lt;&gt;"",$H63=INDEX(Partidos!$K$4:$K$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A63,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E63)),NOT(ISNUMBER($F63))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A63,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E63=INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0)),$F63=INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E63-$F63)=(INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E63&gt;$F63,INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),AND($E63=$F63,INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),AND($E63&lt;$F63,INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0)),IF(AND($E63=INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0)),$F63=INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),IF(AND($H63&lt;&gt;"",$H63=INDEX(Partidos!$K$4:$K$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E63=$F63,($E63-$F63)=(INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0)))),IF(AND($H63&lt;&gt;"",$H63=INDEX(Partidos!$K$4:$K$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H63&lt;&gt;"",$H63=INDEX(Partidos!$K$4:$K$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E63=INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0)),$F63=INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E63-$F63)=(INDEX(Partidos!$F$4:$F$107,MATCH($A63,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H63&lt;&gt;"",$H63=INDEX(Partidos!$K$4:$K$107,MATCH($A63,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H63" s="19">
@@ -12587,7 +12632,7 @@
         <v/>
       </c>
       <c r="G64" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A64,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E64)),NOT(ISNUMBER($F64))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A64,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E64=INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0)),$F64=INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E64-$F64)=(INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E64&gt;$F64,INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),AND($E64=$F64,INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),AND($E64&lt;$F64,INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E64=INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0)),$F64=INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E64-$F64)=(INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H64&lt;&gt;"",$H64=INDEX(Partidos!$K$4:$K$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A64,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E64)),NOT(ISNUMBER($F64))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A64,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E64=INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0)),$F64=INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E64-$F64)=(INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E64&gt;$F64,INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),AND($E64=$F64,INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),AND($E64&lt;$F64,INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0)),IF(AND($E64=INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0)),$F64=INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),IF(AND($H64&lt;&gt;"",$H64=INDEX(Partidos!$K$4:$K$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E64=$F64,($E64-$F64)=(INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0)))),IF(AND($H64&lt;&gt;"",$H64=INDEX(Partidos!$K$4:$K$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H64&lt;&gt;"",$H64=INDEX(Partidos!$K$4:$K$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E64=INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0)),$F64=INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E64-$F64)=(INDEX(Partidos!$F$4:$F$107,MATCH($A64,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H64&lt;&gt;"",$H64=INDEX(Partidos!$K$4:$K$107,MATCH($A64,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H64" s="19">
@@ -12629,7 +12674,7 @@
         <v/>
       </c>
       <c r="G65" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A65,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E65)),NOT(ISNUMBER($F65))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A65,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E65=INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0)),$F65=INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E65-$F65)=(INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E65&gt;$F65,INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),AND($E65=$F65,INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),AND($E65&lt;$F65,INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E65=INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0)),$F65=INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E65-$F65)=(INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H65&lt;&gt;"",$H65=INDEX(Partidos!$K$4:$K$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A65,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E65)),NOT(ISNUMBER($F65))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A65,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E65=INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0)),$F65=INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E65-$F65)=(INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E65&gt;$F65,INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),AND($E65=$F65,INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),AND($E65&lt;$F65,INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0)),IF(AND($E65=INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0)),$F65=INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),IF(AND($H65&lt;&gt;"",$H65=INDEX(Partidos!$K$4:$K$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E65=$F65,($E65-$F65)=(INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0)))),IF(AND($H65&lt;&gt;"",$H65=INDEX(Partidos!$K$4:$K$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H65&lt;&gt;"",$H65=INDEX(Partidos!$K$4:$K$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E65=INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0)),$F65=INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E65-$F65)=(INDEX(Partidos!$F$4:$F$107,MATCH($A65,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H65&lt;&gt;"",$H65=INDEX(Partidos!$K$4:$K$107,MATCH($A65,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H65" s="19">
@@ -12671,7 +12716,7 @@
         <v/>
       </c>
       <c r="G66" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A66,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E66)),NOT(ISNUMBER($F66))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A66,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E66=INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0)),$F66=INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E66-$F66)=(INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E66&gt;$F66,INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),AND($E66=$F66,INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),AND($E66&lt;$F66,INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E66=INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0)),$F66=INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E66-$F66)=(INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H66&lt;&gt;"",$H66=INDEX(Partidos!$K$4:$K$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A66,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E66)),NOT(ISNUMBER($F66))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A66,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E66=INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0)),$F66=INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E66-$F66)=(INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E66&gt;$F66,INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),AND($E66=$F66,INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),AND($E66&lt;$F66,INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0)),IF(AND($E66=INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0)),$F66=INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),IF(AND($H66&lt;&gt;"",$H66=INDEX(Partidos!$K$4:$K$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E66=$F66,($E66-$F66)=(INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0)))),IF(AND($H66&lt;&gt;"",$H66=INDEX(Partidos!$K$4:$K$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H66&lt;&gt;"",$H66=INDEX(Partidos!$K$4:$K$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E66=INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0)),$F66=INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E66-$F66)=(INDEX(Partidos!$F$4:$F$107,MATCH($A66,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H66&lt;&gt;"",$H66=INDEX(Partidos!$K$4:$K$107,MATCH($A66,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H66" s="19">
@@ -12713,7 +12758,7 @@
         <v/>
       </c>
       <c r="G67" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A67,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E67)),NOT(ISNUMBER($F67))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A67,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E67=INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0)),$F67=INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E67-$F67)=(INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E67&gt;$F67,INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),AND($E67=$F67,INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),AND($E67&lt;$F67,INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E67=INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0)),$F67=INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E67-$F67)=(INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H67&lt;&gt;"",$H67=INDEX(Partidos!$K$4:$K$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A67,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E67)),NOT(ISNUMBER($F67))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A67,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E67=INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0)),$F67=INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E67-$F67)=(INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E67&gt;$F67,INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),AND($E67=$F67,INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),AND($E67&lt;$F67,INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0)),IF(AND($E67=INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0)),$F67=INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),IF(AND($H67&lt;&gt;"",$H67=INDEX(Partidos!$K$4:$K$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E67=$F67,($E67-$F67)=(INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0)))),IF(AND($H67&lt;&gt;"",$H67=INDEX(Partidos!$K$4:$K$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H67&lt;&gt;"",$H67=INDEX(Partidos!$K$4:$K$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E67=INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0)),$F67=INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E67-$F67)=(INDEX(Partidos!$F$4:$F$107,MATCH($A67,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H67&lt;&gt;"",$H67=INDEX(Partidos!$K$4:$K$107,MATCH($A67,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H67" s="19">
@@ -12755,7 +12800,7 @@
         <v/>
       </c>
       <c r="G68" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A68,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E68)),NOT(ISNUMBER($F68))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A68,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E68=INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0)),$F68=INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E68-$F68)=(INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E68&gt;$F68,INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),AND($E68=$F68,INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),AND($E68&lt;$F68,INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E68=INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0)),$F68=INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E68-$F68)=(INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H68&lt;&gt;"",$H68=INDEX(Partidos!$K$4:$K$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A68,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E68)),NOT(ISNUMBER($F68))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A68,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E68=INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0)),$F68=INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E68-$F68)=(INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E68&gt;$F68,INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),AND($E68=$F68,INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),AND($E68&lt;$F68,INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0)),IF(AND($E68=INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0)),$F68=INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),IF(AND($H68&lt;&gt;"",$H68=INDEX(Partidos!$K$4:$K$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E68=$F68,($E68-$F68)=(INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0)))),IF(AND($H68&lt;&gt;"",$H68=INDEX(Partidos!$K$4:$K$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H68&lt;&gt;"",$H68=INDEX(Partidos!$K$4:$K$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E68=INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0)),$F68=INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E68-$F68)=(INDEX(Partidos!$F$4:$F$107,MATCH($A68,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H68&lt;&gt;"",$H68=INDEX(Partidos!$K$4:$K$107,MATCH($A68,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H68" s="19">
@@ -12797,7 +12842,7 @@
         <v/>
       </c>
       <c r="G69" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A69,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E69)),NOT(ISNUMBER($F69))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A69,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E69=INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0)),$F69=INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E69-$F69)=(INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E69&gt;$F69,INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),AND($E69=$F69,INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),AND($E69&lt;$F69,INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E69=INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0)),$F69=INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E69-$F69)=(INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H69&lt;&gt;"",$H69=INDEX(Partidos!$K$4:$K$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A69,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E69)),NOT(ISNUMBER($F69))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A69,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E69=INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0)),$F69=INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E69-$F69)=(INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E69&gt;$F69,INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),AND($E69=$F69,INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),AND($E69&lt;$F69,INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0)),IF(AND($E69=INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0)),$F69=INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),IF(AND($H69&lt;&gt;"",$H69=INDEX(Partidos!$K$4:$K$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E69=$F69,($E69-$F69)=(INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0)))),IF(AND($H69&lt;&gt;"",$H69=INDEX(Partidos!$K$4:$K$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H69&lt;&gt;"",$H69=INDEX(Partidos!$K$4:$K$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E69=INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0)),$F69=INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E69-$F69)=(INDEX(Partidos!$F$4:$F$107,MATCH($A69,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H69&lt;&gt;"",$H69=INDEX(Partidos!$K$4:$K$107,MATCH($A69,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H69" s="19">
@@ -12839,7 +12884,7 @@
         <v/>
       </c>
       <c r="G70" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A70,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E70)),NOT(ISNUMBER($F70))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A70,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E70=INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0)),$F70=INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E70-$F70)=(INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E70&gt;$F70,INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),AND($E70=$F70,INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),AND($E70&lt;$F70,INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E70=INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0)),$F70=INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E70-$F70)=(INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H70&lt;&gt;"",$H70=INDEX(Partidos!$K$4:$K$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A70,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E70)),NOT(ISNUMBER($F70))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A70,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E70=INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0)),$F70=INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E70-$F70)=(INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E70&gt;$F70,INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),AND($E70=$F70,INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),AND($E70&lt;$F70,INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0)),IF(AND($E70=INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0)),$F70=INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),IF(AND($H70&lt;&gt;"",$H70=INDEX(Partidos!$K$4:$K$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E70=$F70,($E70-$F70)=(INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0)))),IF(AND($H70&lt;&gt;"",$H70=INDEX(Partidos!$K$4:$K$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H70&lt;&gt;"",$H70=INDEX(Partidos!$K$4:$K$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E70=INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0)),$F70=INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E70-$F70)=(INDEX(Partidos!$F$4:$F$107,MATCH($A70,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H70&lt;&gt;"",$H70=INDEX(Partidos!$K$4:$K$107,MATCH($A70,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H70" s="19">
@@ -12881,7 +12926,7 @@
         <v/>
       </c>
       <c r="G71" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A71,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E71)),NOT(ISNUMBER($F71))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A71,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E71=INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0)),$F71=INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E71-$F71)=(INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E71&gt;$F71,INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),AND($E71=$F71,INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),AND($E71&lt;$F71,INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E71=INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0)),$F71=INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E71-$F71)=(INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H71&lt;&gt;"",$H71=INDEX(Partidos!$K$4:$K$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A71,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E71)),NOT(ISNUMBER($F71))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A71,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E71=INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0)),$F71=INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E71-$F71)=(INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E71&gt;$F71,INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),AND($E71=$F71,INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),AND($E71&lt;$F71,INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0)),IF(AND($E71=INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0)),$F71=INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),IF(AND($H71&lt;&gt;"",$H71=INDEX(Partidos!$K$4:$K$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E71=$F71,($E71-$F71)=(INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0)))),IF(AND($H71&lt;&gt;"",$H71=INDEX(Partidos!$K$4:$K$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H71&lt;&gt;"",$H71=INDEX(Partidos!$K$4:$K$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E71=INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0)),$F71=INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E71-$F71)=(INDEX(Partidos!$F$4:$F$107,MATCH($A71,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H71&lt;&gt;"",$H71=INDEX(Partidos!$K$4:$K$107,MATCH($A71,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H71" s="19">
@@ -12923,7 +12968,7 @@
         <v/>
       </c>
       <c r="G72" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A72,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E72)),NOT(ISNUMBER($F72))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A72,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E72=INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0)),$F72=INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E72-$F72)=(INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E72&gt;$F72,INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),AND($E72=$F72,INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),AND($E72&lt;$F72,INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E72=INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0)),$F72=INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E72-$F72)=(INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H72&lt;&gt;"",$H72=INDEX(Partidos!$K$4:$K$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A72,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E72)),NOT(ISNUMBER($F72))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A72,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E72=INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0)),$F72=INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E72-$F72)=(INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E72&gt;$F72,INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),AND($E72=$F72,INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),AND($E72&lt;$F72,INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0)),IF(AND($E72=INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0)),$F72=INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),IF(AND($H72&lt;&gt;"",$H72=INDEX(Partidos!$K$4:$K$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E72=$F72,($E72-$F72)=(INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0)))),IF(AND($H72&lt;&gt;"",$H72=INDEX(Partidos!$K$4:$K$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H72&lt;&gt;"",$H72=INDEX(Partidos!$K$4:$K$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E72=INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0)),$F72=INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E72-$F72)=(INDEX(Partidos!$F$4:$F$107,MATCH($A72,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H72&lt;&gt;"",$H72=INDEX(Partidos!$K$4:$K$107,MATCH($A72,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H72" s="19">
@@ -12965,7 +13010,7 @@
         <v/>
       </c>
       <c r="G73" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A73,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E73)),NOT(ISNUMBER($F73))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A73,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E73=INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0)),$F73=INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E73-$F73)=(INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E73&gt;$F73,INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),AND($E73=$F73,INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),AND($E73&lt;$F73,INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E73=INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0)),$F73=INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E73-$F73)=(INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H73&lt;&gt;"",$H73=INDEX(Partidos!$K$4:$K$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A73,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E73)),NOT(ISNUMBER($F73))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A73,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E73=INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0)),$F73=INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E73-$F73)=(INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E73&gt;$F73,INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),AND($E73=$F73,INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),AND($E73&lt;$F73,INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0)),IF(AND($E73=INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0)),$F73=INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),IF(AND($H73&lt;&gt;"",$H73=INDEX(Partidos!$K$4:$K$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E73=$F73,($E73-$F73)=(INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0)))),IF(AND($H73&lt;&gt;"",$H73=INDEX(Partidos!$K$4:$K$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H73&lt;&gt;"",$H73=INDEX(Partidos!$K$4:$K$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E73=INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0)),$F73=INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E73-$F73)=(INDEX(Partidos!$F$4:$F$107,MATCH($A73,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H73&lt;&gt;"",$H73=INDEX(Partidos!$K$4:$K$107,MATCH($A73,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H73" s="19">
@@ -13007,7 +13052,7 @@
         <v/>
       </c>
       <c r="G74" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A74,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E74)),NOT(ISNUMBER($F74))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A74,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E74=INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0)),$F74=INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E74-$F74)=(INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E74&gt;$F74,INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),AND($E74=$F74,INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),AND($E74&lt;$F74,INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E74=INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0)),$F74=INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E74-$F74)=(INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H74&lt;&gt;"",$H74=INDEX(Partidos!$K$4:$K$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A74,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E74)),NOT(ISNUMBER($F74))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A74,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E74=INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0)),$F74=INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E74-$F74)=(INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E74&gt;$F74,INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),AND($E74=$F74,INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),AND($E74&lt;$F74,INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0)),IF(AND($E74=INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0)),$F74=INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),IF(AND($H74&lt;&gt;"",$H74=INDEX(Partidos!$K$4:$K$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E74=$F74,($E74-$F74)=(INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0)))),IF(AND($H74&lt;&gt;"",$H74=INDEX(Partidos!$K$4:$K$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H74&lt;&gt;"",$H74=INDEX(Partidos!$K$4:$K$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E74=INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0)),$F74=INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E74-$F74)=(INDEX(Partidos!$F$4:$F$107,MATCH($A74,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H74&lt;&gt;"",$H74=INDEX(Partidos!$K$4:$K$107,MATCH($A74,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H74" s="19">
@@ -13049,7 +13094,7 @@
         <v/>
       </c>
       <c r="G75" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A75,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E75)),NOT(ISNUMBER($F75))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A75,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E75=INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0)),$F75=INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E75-$F75)=(INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E75&gt;$F75,INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),AND($E75=$F75,INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),AND($E75&lt;$F75,INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E75=INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0)),$F75=INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E75-$F75)=(INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H75&lt;&gt;"",$H75=INDEX(Partidos!$K$4:$K$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A75,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E75)),NOT(ISNUMBER($F75))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A75,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E75=INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0)),$F75=INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E75-$F75)=(INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E75&gt;$F75,INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),AND($E75=$F75,INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),AND($E75&lt;$F75,INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0)),IF(AND($E75=INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0)),$F75=INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),IF(AND($H75&lt;&gt;"",$H75=INDEX(Partidos!$K$4:$K$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E75=$F75,($E75-$F75)=(INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0)))),IF(AND($H75&lt;&gt;"",$H75=INDEX(Partidos!$K$4:$K$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H75&lt;&gt;"",$H75=INDEX(Partidos!$K$4:$K$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E75=INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0)),$F75=INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E75-$F75)=(INDEX(Partidos!$F$4:$F$107,MATCH($A75,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H75&lt;&gt;"",$H75=INDEX(Partidos!$K$4:$K$107,MATCH($A75,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H75" s="19">
@@ -13091,7 +13136,7 @@
         <v/>
       </c>
       <c r="G76" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A76,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E76)),NOT(ISNUMBER($F76))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A76,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E76=INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0)),$F76=INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E76-$F76)=(INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E76&gt;$F76,INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),AND($E76=$F76,INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),AND($E76&lt;$F76,INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E76=INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0)),$F76=INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E76-$F76)=(INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H76&lt;&gt;"",$H76=INDEX(Partidos!$K$4:$K$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A76,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E76)),NOT(ISNUMBER($F76))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A76,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E76=INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0)),$F76=INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E76-$F76)=(INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E76&gt;$F76,INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),AND($E76=$F76,INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),AND($E76&lt;$F76,INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0)),IF(AND($E76=INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0)),$F76=INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),IF(AND($H76&lt;&gt;"",$H76=INDEX(Partidos!$K$4:$K$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E76=$F76,($E76-$F76)=(INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0)))),IF(AND($H76&lt;&gt;"",$H76=INDEX(Partidos!$K$4:$K$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H76&lt;&gt;"",$H76=INDEX(Partidos!$K$4:$K$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E76=INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0)),$F76=INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E76-$F76)=(INDEX(Partidos!$F$4:$F$107,MATCH($A76,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H76&lt;&gt;"",$H76=INDEX(Partidos!$K$4:$K$107,MATCH($A76,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H76" s="19">
@@ -13133,7 +13178,7 @@
         <v/>
       </c>
       <c r="G77" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A77,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E77)),NOT(ISNUMBER($F77))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A77,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E77=INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0)),$F77=INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E77-$F77)=(INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E77&gt;$F77,INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),AND($E77=$F77,INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),AND($E77&lt;$F77,INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E77=INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0)),$F77=INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E77-$F77)=(INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H77&lt;&gt;"",$H77=INDEX(Partidos!$K$4:$K$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A77,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E77)),NOT(ISNUMBER($F77))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A77,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E77=INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0)),$F77=INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E77-$F77)=(INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E77&gt;$F77,INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),AND($E77=$F77,INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),AND($E77&lt;$F77,INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0)),IF(AND($E77=INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0)),$F77=INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),IF(AND($H77&lt;&gt;"",$H77=INDEX(Partidos!$K$4:$K$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E77=$F77,($E77-$F77)=(INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0)))),IF(AND($H77&lt;&gt;"",$H77=INDEX(Partidos!$K$4:$K$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H77&lt;&gt;"",$H77=INDEX(Partidos!$K$4:$K$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E77=INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0)),$F77=INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E77-$F77)=(INDEX(Partidos!$F$4:$F$107,MATCH($A77,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H77&lt;&gt;"",$H77=INDEX(Partidos!$K$4:$K$107,MATCH($A77,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H77" s="19">
@@ -13175,7 +13220,7 @@
         <v/>
       </c>
       <c r="G78" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A78,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E78)),NOT(ISNUMBER($F78))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A78,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E78=INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0)),$F78=INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E78-$F78)=(INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E78&gt;$F78,INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),AND($E78=$F78,INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),AND($E78&lt;$F78,INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E78=INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0)),$F78=INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E78-$F78)=(INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H78&lt;&gt;"",$H78=INDEX(Partidos!$K$4:$K$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A78,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E78)),NOT(ISNUMBER($F78))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A78,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E78=INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0)),$F78=INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E78-$F78)=(INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E78&gt;$F78,INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),AND($E78=$F78,INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),AND($E78&lt;$F78,INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0)),IF(AND($E78=INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0)),$F78=INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),IF(AND($H78&lt;&gt;"",$H78=INDEX(Partidos!$K$4:$K$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E78=$F78,($E78-$F78)=(INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0)))),IF(AND($H78&lt;&gt;"",$H78=INDEX(Partidos!$K$4:$K$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H78&lt;&gt;"",$H78=INDEX(Partidos!$K$4:$K$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E78=INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0)),$F78=INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E78-$F78)=(INDEX(Partidos!$F$4:$F$107,MATCH($A78,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H78&lt;&gt;"",$H78=INDEX(Partidos!$K$4:$K$107,MATCH($A78,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H78" s="19">
@@ -13217,7 +13262,7 @@
         <v/>
       </c>
       <c r="G79" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A79,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E79)),NOT(ISNUMBER($F79))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A79,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E79=INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0)),$F79=INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E79-$F79)=(INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E79&gt;$F79,INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),AND($E79=$F79,INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),AND($E79&lt;$F79,INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E79=INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0)),$F79=INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E79-$F79)=(INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H79&lt;&gt;"",$H79=INDEX(Partidos!$K$4:$K$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A79,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E79)),NOT(ISNUMBER($F79))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A79,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E79=INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0)),$F79=INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E79-$F79)=(INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E79&gt;$F79,INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),AND($E79=$F79,INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),AND($E79&lt;$F79,INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0)),IF(AND($E79=INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0)),$F79=INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),IF(AND($H79&lt;&gt;"",$H79=INDEX(Partidos!$K$4:$K$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E79=$F79,($E79-$F79)=(INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0)))),IF(AND($H79&lt;&gt;"",$H79=INDEX(Partidos!$K$4:$K$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H79&lt;&gt;"",$H79=INDEX(Partidos!$K$4:$K$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E79=INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0)),$F79=INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E79-$F79)=(INDEX(Partidos!$F$4:$F$107,MATCH($A79,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H79&lt;&gt;"",$H79=INDEX(Partidos!$K$4:$K$107,MATCH($A79,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H79" s="19">
@@ -13259,7 +13304,7 @@
         <v/>
       </c>
       <c r="G80" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A80,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E80)),NOT(ISNUMBER($F80))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A80,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E80=INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0)),$F80=INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E80-$F80)=(INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E80&gt;$F80,INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),AND($E80=$F80,INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),AND($E80&lt;$F80,INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E80=INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0)),$F80=INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E80-$F80)=(INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H80&lt;&gt;"",$H80=INDEX(Partidos!$K$4:$K$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A80,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E80)),NOT(ISNUMBER($F80))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A80,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E80=INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0)),$F80=INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E80-$F80)=(INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E80&gt;$F80,INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),AND($E80=$F80,INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),AND($E80&lt;$F80,INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0)),IF(AND($E80=INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0)),$F80=INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),IF(AND($H80&lt;&gt;"",$H80=INDEX(Partidos!$K$4:$K$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E80=$F80,($E80-$F80)=(INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0)))),IF(AND($H80&lt;&gt;"",$H80=INDEX(Partidos!$K$4:$K$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H80&lt;&gt;"",$H80=INDEX(Partidos!$K$4:$K$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E80=INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0)),$F80=INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E80-$F80)=(INDEX(Partidos!$F$4:$F$107,MATCH($A80,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H80&lt;&gt;"",$H80=INDEX(Partidos!$K$4:$K$107,MATCH($A80,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H80" s="19">
@@ -13301,7 +13346,7 @@
         <v/>
       </c>
       <c r="G81" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A81,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E81)),NOT(ISNUMBER($F81))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A81,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E81=INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0)),$F81=INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E81-$F81)=(INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E81&gt;$F81,INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),AND($E81=$F81,INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),AND($E81&lt;$F81,INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E81=INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0)),$F81=INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E81-$F81)=(INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H81&lt;&gt;"",$H81=INDEX(Partidos!$K$4:$K$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A81,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E81)),NOT(ISNUMBER($F81))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A81,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E81=INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0)),$F81=INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E81-$F81)=(INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E81&gt;$F81,INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),AND($E81=$F81,INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),AND($E81&lt;$F81,INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0)),IF(AND($E81=INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0)),$F81=INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),IF(AND($H81&lt;&gt;"",$H81=INDEX(Partidos!$K$4:$K$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E81=$F81,($E81-$F81)=(INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0)))),IF(AND($H81&lt;&gt;"",$H81=INDEX(Partidos!$K$4:$K$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H81&lt;&gt;"",$H81=INDEX(Partidos!$K$4:$K$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E81=INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0)),$F81=INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E81-$F81)=(INDEX(Partidos!$F$4:$F$107,MATCH($A81,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H81&lt;&gt;"",$H81=INDEX(Partidos!$K$4:$K$107,MATCH($A81,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H81" s="19">
@@ -13343,7 +13388,7 @@
         <v/>
       </c>
       <c r="G82" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A82,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E82)),NOT(ISNUMBER($F82))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A82,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E82=INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0)),$F82=INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E82-$F82)=(INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E82&gt;$F82,INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),AND($E82=$F82,INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),AND($E82&lt;$F82,INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E82=INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0)),$F82=INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E82-$F82)=(INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H82&lt;&gt;"",$H82=INDEX(Partidos!$K$4:$K$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A82,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E82)),NOT(ISNUMBER($F82))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A82,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E82=INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0)),$F82=INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E82-$F82)=(INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E82&gt;$F82,INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),AND($E82=$F82,INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),AND($E82&lt;$F82,INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0)),IF(AND($E82=INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0)),$F82=INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),IF(AND($H82&lt;&gt;"",$H82=INDEX(Partidos!$K$4:$K$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E82=$F82,($E82-$F82)=(INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0)))),IF(AND($H82&lt;&gt;"",$H82=INDEX(Partidos!$K$4:$K$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H82&lt;&gt;"",$H82=INDEX(Partidos!$K$4:$K$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E82=INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0)),$F82=INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E82-$F82)=(INDEX(Partidos!$F$4:$F$107,MATCH($A82,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H82&lt;&gt;"",$H82=INDEX(Partidos!$K$4:$K$107,MATCH($A82,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H82" s="19">
@@ -13385,7 +13430,7 @@
         <v/>
       </c>
       <c r="G83" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A83,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E83)),NOT(ISNUMBER($F83))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A83,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E83=INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0)),$F83=INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E83-$F83)=(INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E83&gt;$F83,INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),AND($E83=$F83,INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),AND($E83&lt;$F83,INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E83=INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0)),$F83=INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E83-$F83)=(INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H83&lt;&gt;"",$H83=INDEX(Partidos!$K$4:$K$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A83,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E83)),NOT(ISNUMBER($F83))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A83,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E83=INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0)),$F83=INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E83-$F83)=(INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E83&gt;$F83,INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),AND($E83=$F83,INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),AND($E83&lt;$F83,INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0)),IF(AND($E83=INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0)),$F83=INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),IF(AND($H83&lt;&gt;"",$H83=INDEX(Partidos!$K$4:$K$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E83=$F83,($E83-$F83)=(INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0)))),IF(AND($H83&lt;&gt;"",$H83=INDEX(Partidos!$K$4:$K$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H83&lt;&gt;"",$H83=INDEX(Partidos!$K$4:$K$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E83=INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0)),$F83=INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E83-$F83)=(INDEX(Partidos!$F$4:$F$107,MATCH($A83,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H83&lt;&gt;"",$H83=INDEX(Partidos!$K$4:$K$107,MATCH($A83,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H83" s="19">
@@ -13427,7 +13472,7 @@
         <v/>
       </c>
       <c r="G84" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A84,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E84)),NOT(ISNUMBER($F84))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A84,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E84=INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0)),$F84=INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E84-$F84)=(INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E84&gt;$F84,INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),AND($E84=$F84,INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),AND($E84&lt;$F84,INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E84=INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0)),$F84=INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E84-$F84)=(INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H84&lt;&gt;"",$H84=INDEX(Partidos!$K$4:$K$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A84,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E84)),NOT(ISNUMBER($F84))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A84,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E84=INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0)),$F84=INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E84-$F84)=(INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E84&gt;$F84,INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),AND($E84=$F84,INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),AND($E84&lt;$F84,INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0)),IF(AND($E84=INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0)),$F84=INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),IF(AND($H84&lt;&gt;"",$H84=INDEX(Partidos!$K$4:$K$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E84=$F84,($E84-$F84)=(INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0)))),IF(AND($H84&lt;&gt;"",$H84=INDEX(Partidos!$K$4:$K$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H84&lt;&gt;"",$H84=INDEX(Partidos!$K$4:$K$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E84=INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0)),$F84=INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E84-$F84)=(INDEX(Partidos!$F$4:$F$107,MATCH($A84,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H84&lt;&gt;"",$H84=INDEX(Partidos!$K$4:$K$107,MATCH($A84,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H84" s="19">
@@ -13469,7 +13514,7 @@
         <v/>
       </c>
       <c r="G85" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A85,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E85)),NOT(ISNUMBER($F85))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A85,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E85=INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0)),$F85=INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E85-$F85)=(INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E85&gt;$F85,INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),AND($E85=$F85,INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),AND($E85&lt;$F85,INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E85=INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0)),$F85=INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E85-$F85)=(INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H85&lt;&gt;"",$H85=INDEX(Partidos!$K$4:$K$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A85,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E85)),NOT(ISNUMBER($F85))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A85,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E85=INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0)),$F85=INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E85-$F85)=(INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E85&gt;$F85,INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),AND($E85=$F85,INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),AND($E85&lt;$F85,INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0)),IF(AND($E85=INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0)),$F85=INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),IF(AND($H85&lt;&gt;"",$H85=INDEX(Partidos!$K$4:$K$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E85=$F85,($E85-$F85)=(INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0)))),IF(AND($H85&lt;&gt;"",$H85=INDEX(Partidos!$K$4:$K$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H85&lt;&gt;"",$H85=INDEX(Partidos!$K$4:$K$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E85=INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0)),$F85=INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E85-$F85)=(INDEX(Partidos!$F$4:$F$107,MATCH($A85,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H85&lt;&gt;"",$H85=INDEX(Partidos!$K$4:$K$107,MATCH($A85,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H85" s="19">
@@ -13511,7 +13556,7 @@
         <v/>
       </c>
       <c r="G86" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A86,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E86)),NOT(ISNUMBER($F86))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A86,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E86=INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0)),$F86=INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E86-$F86)=(INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E86&gt;$F86,INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),AND($E86=$F86,INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),AND($E86&lt;$F86,INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E86=INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0)),$F86=INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E86-$F86)=(INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H86&lt;&gt;"",$H86=INDEX(Partidos!$K$4:$K$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A86,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E86)),NOT(ISNUMBER($F86))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A86,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E86=INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0)),$F86=INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E86-$F86)=(INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E86&gt;$F86,INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),AND($E86=$F86,INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),AND($E86&lt;$F86,INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0)),IF(AND($E86=INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0)),$F86=INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),IF(AND($H86&lt;&gt;"",$H86=INDEX(Partidos!$K$4:$K$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E86=$F86,($E86-$F86)=(INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0)))),IF(AND($H86&lt;&gt;"",$H86=INDEX(Partidos!$K$4:$K$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H86&lt;&gt;"",$H86=INDEX(Partidos!$K$4:$K$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E86=INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0)),$F86=INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E86-$F86)=(INDEX(Partidos!$F$4:$F$107,MATCH($A86,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H86&lt;&gt;"",$H86=INDEX(Partidos!$K$4:$K$107,MATCH($A86,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H86" s="19">
@@ -13553,7 +13598,7 @@
         <v/>
       </c>
       <c r="G87" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A87,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E87)),NOT(ISNUMBER($F87))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A87,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E87=INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0)),$F87=INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E87-$F87)=(INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E87&gt;$F87,INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),AND($E87=$F87,INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),AND($E87&lt;$F87,INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E87=INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0)),$F87=INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E87-$F87)=(INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H87&lt;&gt;"",$H87=INDEX(Partidos!$K$4:$K$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A87,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E87)),NOT(ISNUMBER($F87))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A87,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E87=INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0)),$F87=INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E87-$F87)=(INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E87&gt;$F87,INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),AND($E87=$F87,INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),AND($E87&lt;$F87,INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0)),IF(AND($E87=INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0)),$F87=INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),IF(AND($H87&lt;&gt;"",$H87=INDEX(Partidos!$K$4:$K$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E87=$F87,($E87-$F87)=(INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0)))),IF(AND($H87&lt;&gt;"",$H87=INDEX(Partidos!$K$4:$K$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H87&lt;&gt;"",$H87=INDEX(Partidos!$K$4:$K$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E87=INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0)),$F87=INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E87-$F87)=(INDEX(Partidos!$F$4:$F$107,MATCH($A87,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H87&lt;&gt;"",$H87=INDEX(Partidos!$K$4:$K$107,MATCH($A87,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H87" s="19">
@@ -13595,7 +13640,7 @@
         <v/>
       </c>
       <c r="G88" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A88,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E88)),NOT(ISNUMBER($F88))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A88,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E88=INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0)),$F88=INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E88-$F88)=(INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E88&gt;$F88,INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),AND($E88=$F88,INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),AND($E88&lt;$F88,INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E88=INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0)),$F88=INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E88-$F88)=(INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H88&lt;&gt;"",$H88=INDEX(Partidos!$K$4:$K$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A88,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E88)),NOT(ISNUMBER($F88))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A88,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E88=INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0)),$F88=INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E88-$F88)=(INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E88&gt;$F88,INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),AND($E88=$F88,INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),AND($E88&lt;$F88,INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0)),IF(AND($E88=INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0)),$F88=INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),IF(AND($H88&lt;&gt;"",$H88=INDEX(Partidos!$K$4:$K$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E88=$F88,($E88-$F88)=(INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0)))),IF(AND($H88&lt;&gt;"",$H88=INDEX(Partidos!$K$4:$K$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H88&lt;&gt;"",$H88=INDEX(Partidos!$K$4:$K$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E88=INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0)),$F88=INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E88-$F88)=(INDEX(Partidos!$F$4:$F$107,MATCH($A88,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H88&lt;&gt;"",$H88=INDEX(Partidos!$K$4:$K$107,MATCH($A88,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H88" s="19">
@@ -13637,7 +13682,7 @@
         <v/>
       </c>
       <c r="G89" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A89,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E89)),NOT(ISNUMBER($F89))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A89,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E89=INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0)),$F89=INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E89-$F89)=(INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E89&gt;$F89,INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),AND($E89=$F89,INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),AND($E89&lt;$F89,INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E89=INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0)),$F89=INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E89-$F89)=(INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H89&lt;&gt;"",$H89=INDEX(Partidos!$K$4:$K$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A89,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E89)),NOT(ISNUMBER($F89))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A89,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E89=INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0)),$F89=INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E89-$F89)=(INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E89&gt;$F89,INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),AND($E89=$F89,INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),AND($E89&lt;$F89,INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0)),IF(AND($E89=INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0)),$F89=INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),IF(AND($H89&lt;&gt;"",$H89=INDEX(Partidos!$K$4:$K$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E89=$F89,($E89-$F89)=(INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0)))),IF(AND($H89&lt;&gt;"",$H89=INDEX(Partidos!$K$4:$K$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H89&lt;&gt;"",$H89=INDEX(Partidos!$K$4:$K$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E89=INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0)),$F89=INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E89-$F89)=(INDEX(Partidos!$F$4:$F$107,MATCH($A89,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H89&lt;&gt;"",$H89=INDEX(Partidos!$K$4:$K$107,MATCH($A89,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H89" s="19">
@@ -13679,7 +13724,7 @@
         <v/>
       </c>
       <c r="G90" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A90,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E90)),NOT(ISNUMBER($F90))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A90,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E90=INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0)),$F90=INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E90-$F90)=(INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E90&gt;$F90,INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),AND($E90=$F90,INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),AND($E90&lt;$F90,INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E90=INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0)),$F90=INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E90-$F90)=(INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H90&lt;&gt;"",$H90=INDEX(Partidos!$K$4:$K$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A90,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E90)),NOT(ISNUMBER($F90))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A90,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E90=INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0)),$F90=INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E90-$F90)=(INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E90&gt;$F90,INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),AND($E90=$F90,INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),AND($E90&lt;$F90,INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0)),IF(AND($E90=INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0)),$F90=INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),IF(AND($H90&lt;&gt;"",$H90=INDEX(Partidos!$K$4:$K$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E90=$F90,($E90-$F90)=(INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0)))),IF(AND($H90&lt;&gt;"",$H90=INDEX(Partidos!$K$4:$K$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H90&lt;&gt;"",$H90=INDEX(Partidos!$K$4:$K$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E90=INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0)),$F90=INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E90-$F90)=(INDEX(Partidos!$F$4:$F$107,MATCH($A90,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H90&lt;&gt;"",$H90=INDEX(Partidos!$K$4:$K$107,MATCH($A90,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H90" s="19">
@@ -13721,7 +13766,7 @@
         <v/>
       </c>
       <c r="G91" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A91,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E91)),NOT(ISNUMBER($F91))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A91,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E91=INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0)),$F91=INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E91-$F91)=(INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E91&gt;$F91,INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),AND($E91=$F91,INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),AND($E91&lt;$F91,INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E91=INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0)),$F91=INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E91-$F91)=(INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H91&lt;&gt;"",$H91=INDEX(Partidos!$K$4:$K$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A91,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E91)),NOT(ISNUMBER($F91))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A91,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E91=INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0)),$F91=INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E91-$F91)=(INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E91&gt;$F91,INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),AND($E91=$F91,INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),AND($E91&lt;$F91,INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0)),IF(AND($E91=INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0)),$F91=INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),IF(AND($H91&lt;&gt;"",$H91=INDEX(Partidos!$K$4:$K$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E91=$F91,($E91-$F91)=(INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0)))),IF(AND($H91&lt;&gt;"",$H91=INDEX(Partidos!$K$4:$K$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H91&lt;&gt;"",$H91=INDEX(Partidos!$K$4:$K$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E91=INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0)),$F91=INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E91-$F91)=(INDEX(Partidos!$F$4:$F$107,MATCH($A91,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H91&lt;&gt;"",$H91=INDEX(Partidos!$K$4:$K$107,MATCH($A91,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H91" s="19">
@@ -13763,7 +13808,7 @@
         <v/>
       </c>
       <c r="G92" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A92,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E92)),NOT(ISNUMBER($F92))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A92,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E92=INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0)),$F92=INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E92-$F92)=(INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E92&gt;$F92,INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),AND($E92=$F92,INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),AND($E92&lt;$F92,INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E92=INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0)),$F92=INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E92-$F92)=(INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H92&lt;&gt;"",$H92=INDEX(Partidos!$K$4:$K$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A92,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E92)),NOT(ISNUMBER($F92))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A92,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E92=INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0)),$F92=INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E92-$F92)=(INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E92&gt;$F92,INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),AND($E92=$F92,INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),AND($E92&lt;$F92,INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0)),IF(AND($E92=INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0)),$F92=INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),IF(AND($H92&lt;&gt;"",$H92=INDEX(Partidos!$K$4:$K$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E92=$F92,($E92-$F92)=(INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0)))),IF(AND($H92&lt;&gt;"",$H92=INDEX(Partidos!$K$4:$K$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H92&lt;&gt;"",$H92=INDEX(Partidos!$K$4:$K$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E92=INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0)),$F92=INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E92-$F92)=(INDEX(Partidos!$F$4:$F$107,MATCH($A92,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H92&lt;&gt;"",$H92=INDEX(Partidos!$K$4:$K$107,MATCH($A92,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H92" s="19">
@@ -13805,7 +13850,7 @@
         <v/>
       </c>
       <c r="G93" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A93,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E93)),NOT(ISNUMBER($F93))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A93,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E93=INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0)),$F93=INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E93-$F93)=(INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E93&gt;$F93,INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),AND($E93=$F93,INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),AND($E93&lt;$F93,INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E93=INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0)),$F93=INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E93-$F93)=(INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H93&lt;&gt;"",$H93=INDEX(Partidos!$K$4:$K$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A93,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E93)),NOT(ISNUMBER($F93))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A93,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E93=INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0)),$F93=INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E93-$F93)=(INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E93&gt;$F93,INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),AND($E93=$F93,INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),AND($E93&lt;$F93,INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0)),IF(AND($E93=INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0)),$F93=INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),IF(AND($H93&lt;&gt;"",$H93=INDEX(Partidos!$K$4:$K$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E93=$F93,($E93-$F93)=(INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0)))),IF(AND($H93&lt;&gt;"",$H93=INDEX(Partidos!$K$4:$K$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H93&lt;&gt;"",$H93=INDEX(Partidos!$K$4:$K$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E93=INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0)),$F93=INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E93-$F93)=(INDEX(Partidos!$F$4:$F$107,MATCH($A93,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H93&lt;&gt;"",$H93=INDEX(Partidos!$K$4:$K$107,MATCH($A93,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H93" s="19">
@@ -13847,7 +13892,7 @@
         <v/>
       </c>
       <c r="G94" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A94,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E94)),NOT(ISNUMBER($F94))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A94,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E94=INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0)),$F94=INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E94-$F94)=(INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E94&gt;$F94,INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),AND($E94=$F94,INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),AND($E94&lt;$F94,INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E94=INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0)),$F94=INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E94-$F94)=(INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H94&lt;&gt;"",$H94=INDEX(Partidos!$K$4:$K$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A94,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E94)),NOT(ISNUMBER($F94))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A94,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E94=INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0)),$F94=INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E94-$F94)=(INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E94&gt;$F94,INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),AND($E94=$F94,INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),AND($E94&lt;$F94,INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0)),IF(AND($E94=INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0)),$F94=INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),IF(AND($H94&lt;&gt;"",$H94=INDEX(Partidos!$K$4:$K$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E94=$F94,($E94-$F94)=(INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0)))),IF(AND($H94&lt;&gt;"",$H94=INDEX(Partidos!$K$4:$K$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H94&lt;&gt;"",$H94=INDEX(Partidos!$K$4:$K$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E94=INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0)),$F94=INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E94-$F94)=(INDEX(Partidos!$F$4:$F$107,MATCH($A94,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H94&lt;&gt;"",$H94=INDEX(Partidos!$K$4:$K$107,MATCH($A94,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H94" s="19">
@@ -13889,7 +13934,7 @@
         <v/>
       </c>
       <c r="G95" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A95,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E95)),NOT(ISNUMBER($F95))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A95,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E95=INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0)),$F95=INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E95-$F95)=(INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E95&gt;$F95,INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),AND($E95=$F95,INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),AND($E95&lt;$F95,INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E95=INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0)),$F95=INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E95-$F95)=(INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H95&lt;&gt;"",$H95=INDEX(Partidos!$K$4:$K$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A95,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E95)),NOT(ISNUMBER($F95))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A95,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E95=INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0)),$F95=INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E95-$F95)=(INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E95&gt;$F95,INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),AND($E95=$F95,INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),AND($E95&lt;$F95,INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0)),IF(AND($E95=INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0)),$F95=INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),IF(AND($H95&lt;&gt;"",$H95=INDEX(Partidos!$K$4:$K$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E95=$F95,($E95-$F95)=(INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0)))),IF(AND($H95&lt;&gt;"",$H95=INDEX(Partidos!$K$4:$K$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H95&lt;&gt;"",$H95=INDEX(Partidos!$K$4:$K$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E95=INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0)),$F95=INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E95-$F95)=(INDEX(Partidos!$F$4:$F$107,MATCH($A95,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H95&lt;&gt;"",$H95=INDEX(Partidos!$K$4:$K$107,MATCH($A95,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H95" s="19">
@@ -13931,7 +13976,7 @@
         <v/>
       </c>
       <c r="G96" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A96,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E96)),NOT(ISNUMBER($F96))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A96,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E96=INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0)),$F96=INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E96-$F96)=(INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E96&gt;$F96,INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),AND($E96=$F96,INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),AND($E96&lt;$F96,INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E96=INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0)),$F96=INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E96-$F96)=(INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H96&lt;&gt;"",$H96=INDEX(Partidos!$K$4:$K$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A96,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E96)),NOT(ISNUMBER($F96))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A96,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E96=INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0)),$F96=INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E96-$F96)=(INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E96&gt;$F96,INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),AND($E96=$F96,INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),AND($E96&lt;$F96,INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0)),IF(AND($E96=INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0)),$F96=INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),IF(AND($H96&lt;&gt;"",$H96=INDEX(Partidos!$K$4:$K$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E96=$F96,($E96-$F96)=(INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0)))),IF(AND($H96&lt;&gt;"",$H96=INDEX(Partidos!$K$4:$K$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H96&lt;&gt;"",$H96=INDEX(Partidos!$K$4:$K$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E96=INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0)),$F96=INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E96-$F96)=(INDEX(Partidos!$F$4:$F$107,MATCH($A96,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H96&lt;&gt;"",$H96=INDEX(Partidos!$K$4:$K$107,MATCH($A96,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H96" s="19">
@@ -13973,7 +14018,7 @@
         <v/>
       </c>
       <c r="G97" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A97,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E97)),NOT(ISNUMBER($F97))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A97,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E97=INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0)),$F97=INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E97-$F97)=(INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E97&gt;$F97,INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),AND($E97=$F97,INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),AND($E97&lt;$F97,INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E97=INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0)),$F97=INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E97-$F97)=(INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H97&lt;&gt;"",$H97=INDEX(Partidos!$K$4:$K$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A97,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E97)),NOT(ISNUMBER($F97))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A97,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E97=INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0)),$F97=INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E97-$F97)=(INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E97&gt;$F97,INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),AND($E97=$F97,INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),AND($E97&lt;$F97,INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0)),IF(AND($E97=INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0)),$F97=INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),IF(AND($H97&lt;&gt;"",$H97=INDEX(Partidos!$K$4:$K$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E97=$F97,($E97-$F97)=(INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0)))),IF(AND($H97&lt;&gt;"",$H97=INDEX(Partidos!$K$4:$K$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H97&lt;&gt;"",$H97=INDEX(Partidos!$K$4:$K$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E97=INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0)),$F97=INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E97-$F97)=(INDEX(Partidos!$F$4:$F$107,MATCH($A97,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H97&lt;&gt;"",$H97=INDEX(Partidos!$K$4:$K$107,MATCH($A97,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H97" s="19">
@@ -14015,7 +14060,7 @@
         <v/>
       </c>
       <c r="G98" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A98,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E98)),NOT(ISNUMBER($F98))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A98,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E98=INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0)),$F98=INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E98-$F98)=(INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E98&gt;$F98,INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),AND($E98=$F98,INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),AND($E98&lt;$F98,INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E98=INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0)),$F98=INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E98-$F98)=(INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H98&lt;&gt;"",$H98=INDEX(Partidos!$K$4:$K$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A98,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E98)),NOT(ISNUMBER($F98))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A98,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E98=INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0)),$F98=INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E98-$F98)=(INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E98&gt;$F98,INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),AND($E98=$F98,INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),AND($E98&lt;$F98,INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0)),IF(AND($E98=INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0)),$F98=INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),IF(AND($H98&lt;&gt;"",$H98=INDEX(Partidos!$K$4:$K$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E98=$F98,($E98-$F98)=(INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0)))),IF(AND($H98&lt;&gt;"",$H98=INDEX(Partidos!$K$4:$K$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H98&lt;&gt;"",$H98=INDEX(Partidos!$K$4:$K$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E98=INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0)),$F98=INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E98-$F98)=(INDEX(Partidos!$F$4:$F$107,MATCH($A98,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H98&lt;&gt;"",$H98=INDEX(Partidos!$K$4:$K$107,MATCH($A98,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H98" s="19">
@@ -14057,7 +14102,7 @@
         <v/>
       </c>
       <c r="G99" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A99,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E99)),NOT(ISNUMBER($F99))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A99,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E99=INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0)),$F99=INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E99-$F99)=(INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E99&gt;$F99,INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),AND($E99=$F99,INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),AND($E99&lt;$F99,INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E99=INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0)),$F99=INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E99-$F99)=(INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H99&lt;&gt;"",$H99=INDEX(Partidos!$K$4:$K$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A99,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E99)),NOT(ISNUMBER($F99))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A99,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E99=INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0)),$F99=INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E99-$F99)=(INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E99&gt;$F99,INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),AND($E99=$F99,INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),AND($E99&lt;$F99,INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0)),IF(AND($E99=INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0)),$F99=INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),IF(AND($H99&lt;&gt;"",$H99=INDEX(Partidos!$K$4:$K$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E99=$F99,($E99-$F99)=(INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0)))),IF(AND($H99&lt;&gt;"",$H99=INDEX(Partidos!$K$4:$K$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H99&lt;&gt;"",$H99=INDEX(Partidos!$K$4:$K$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E99=INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0)),$F99=INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E99-$F99)=(INDEX(Partidos!$F$4:$F$107,MATCH($A99,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H99&lt;&gt;"",$H99=INDEX(Partidos!$K$4:$K$107,MATCH($A99,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H99" s="19">
@@ -14099,7 +14144,7 @@
         <v/>
       </c>
       <c r="G100" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A100,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E100)),NOT(ISNUMBER($F100))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A100,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E100=INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0)),$F100=INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E100-$F100)=(INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E100&gt;$F100,INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),AND($E100=$F100,INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),AND($E100&lt;$F100,INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E100=INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0)),$F100=INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E100-$F100)=(INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H100&lt;&gt;"",$H100=INDEX(Partidos!$K$4:$K$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A100,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E100)),NOT(ISNUMBER($F100))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A100,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E100=INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0)),$F100=INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E100-$F100)=(INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E100&gt;$F100,INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),AND($E100=$F100,INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),AND($E100&lt;$F100,INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0)),IF(AND($E100=INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0)),$F100=INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),IF(AND($H100&lt;&gt;"",$H100=INDEX(Partidos!$K$4:$K$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E100=$F100,($E100-$F100)=(INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0)))),IF(AND($H100&lt;&gt;"",$H100=INDEX(Partidos!$K$4:$K$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H100&lt;&gt;"",$H100=INDEX(Partidos!$K$4:$K$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E100=INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0)),$F100=INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E100-$F100)=(INDEX(Partidos!$F$4:$F$107,MATCH($A100,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H100&lt;&gt;"",$H100=INDEX(Partidos!$K$4:$K$107,MATCH($A100,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H100" s="19">
@@ -14141,7 +14186,7 @@
         <v/>
       </c>
       <c r="G101" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A101,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E101)),NOT(ISNUMBER($F101))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A101,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E101=INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0)),$F101=INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E101-$F101)=(INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E101&gt;$F101,INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),AND($E101=$F101,INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),AND($E101&lt;$F101,INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E101=INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0)),$F101=INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E101-$F101)=(INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H101&lt;&gt;"",$H101=INDEX(Partidos!$K$4:$K$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A101,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E101)),NOT(ISNUMBER($F101))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A101,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E101=INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0)),$F101=INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E101-$F101)=(INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E101&gt;$F101,INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),AND($E101=$F101,INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),AND($E101&lt;$F101,INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0)),IF(AND($E101=INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0)),$F101=INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),IF(AND($H101&lt;&gt;"",$H101=INDEX(Partidos!$K$4:$K$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E101=$F101,($E101-$F101)=(INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0)))),IF(AND($H101&lt;&gt;"",$H101=INDEX(Partidos!$K$4:$K$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H101&lt;&gt;"",$H101=INDEX(Partidos!$K$4:$K$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E101=INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0)),$F101=INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E101-$F101)=(INDEX(Partidos!$F$4:$F$107,MATCH($A101,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H101&lt;&gt;"",$H101=INDEX(Partidos!$K$4:$K$107,MATCH($A101,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H101" s="19">
@@ -14183,7 +14228,7 @@
         <v/>
       </c>
       <c r="G102" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A102,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E102)),NOT(ISNUMBER($F102))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A102,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E102=INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0)),$F102=INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E102-$F102)=(INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E102&gt;$F102,INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),AND($E102=$F102,INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),AND($E102&lt;$F102,INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E102=INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0)),$F102=INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E102-$F102)=(INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H102&lt;&gt;"",$H102=INDEX(Partidos!$K$4:$K$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A102,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E102)),NOT(ISNUMBER($F102))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A102,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E102=INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0)),$F102=INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E102-$F102)=(INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E102&gt;$F102,INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),AND($E102=$F102,INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),AND($E102&lt;$F102,INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0)),IF(AND($E102=INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0)),$F102=INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),IF(AND($H102&lt;&gt;"",$H102=INDEX(Partidos!$K$4:$K$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E102=$F102,($E102-$F102)=(INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0)))),IF(AND($H102&lt;&gt;"",$H102=INDEX(Partidos!$K$4:$K$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H102&lt;&gt;"",$H102=INDEX(Partidos!$K$4:$K$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E102=INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0)),$F102=INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E102-$F102)=(INDEX(Partidos!$F$4:$F$107,MATCH($A102,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H102&lt;&gt;"",$H102=INDEX(Partidos!$K$4:$K$107,MATCH($A102,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H102" s="19">
@@ -14225,7 +14270,7 @@
         <v/>
       </c>
       <c r="G103" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A103,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E103)),NOT(ISNUMBER($F103))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A103,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E103=INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0)),$F103=INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E103-$F103)=(INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E103&gt;$F103,INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),AND($E103=$F103,INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),AND($E103&lt;$F103,INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E103=INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0)),$F103=INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E103-$F103)=(INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H103&lt;&gt;"",$H103=INDEX(Partidos!$K$4:$K$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A103,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E103)),NOT(ISNUMBER($F103))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A103,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E103=INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0)),$F103=INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E103-$F103)=(INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E103&gt;$F103,INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),AND($E103=$F103,INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),AND($E103&lt;$F103,INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0)),IF(AND($E103=INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0)),$F103=INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),IF(AND($H103&lt;&gt;"",$H103=INDEX(Partidos!$K$4:$K$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E103=$F103,($E103-$F103)=(INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0)))),IF(AND($H103&lt;&gt;"",$H103=INDEX(Partidos!$K$4:$K$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H103&lt;&gt;"",$H103=INDEX(Partidos!$K$4:$K$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E103=INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0)),$F103=INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E103-$F103)=(INDEX(Partidos!$F$4:$F$107,MATCH($A103,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H103&lt;&gt;"",$H103=INDEX(Partidos!$K$4:$K$107,MATCH($A103,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H103" s="19">
@@ -14267,7 +14312,7 @@
         <v/>
       </c>
       <c r="G104" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A104,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E104)),NOT(ISNUMBER($F104))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A104,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E104=INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0)),$F104=INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E104-$F104)=(INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E104&gt;$F104,INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),AND($E104=$F104,INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),AND($E104&lt;$F104,INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E104=INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0)),$F104=INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E104-$F104)=(INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H104&lt;&gt;"",$H104=INDEX(Partidos!$K$4:$K$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A104,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E104)),NOT(ISNUMBER($F104))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A104,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E104=INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0)),$F104=INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E104-$F104)=(INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E104&gt;$F104,INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),AND($E104=$F104,INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),AND($E104&lt;$F104,INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0)),IF(AND($E104=INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0)),$F104=INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),IF(AND($H104&lt;&gt;"",$H104=INDEX(Partidos!$K$4:$K$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E104=$F104,($E104-$F104)=(INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0)))),IF(AND($H104&lt;&gt;"",$H104=INDEX(Partidos!$K$4:$K$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H104&lt;&gt;"",$H104=INDEX(Partidos!$K$4:$K$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E104=INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0)),$F104=INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E104-$F104)=(INDEX(Partidos!$F$4:$F$107,MATCH($A104,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H104&lt;&gt;"",$H104=INDEX(Partidos!$K$4:$K$107,MATCH($A104,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H104" s="19">
@@ -14309,7 +14354,7 @@
         <v/>
       </c>
       <c r="G105" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A105,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E105)),NOT(ISNUMBER($F105))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A105,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E105=INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0)),$F105=INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E105-$F105)=(INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E105&gt;$F105,INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),AND($E105=$F105,INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),AND($E105&lt;$F105,INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E105=INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0)),$F105=INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E105-$F105)=(INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H105&lt;&gt;"",$H105=INDEX(Partidos!$K$4:$K$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A105,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E105)),NOT(ISNUMBER($F105))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A105,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E105=INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0)),$F105=INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E105-$F105)=(INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E105&gt;$F105,INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),AND($E105=$F105,INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),AND($E105&lt;$F105,INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0)),IF(AND($E105=INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0)),$F105=INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),IF(AND($H105&lt;&gt;"",$H105=INDEX(Partidos!$K$4:$K$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E105=$F105,($E105-$F105)=(INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0)))),IF(AND($H105&lt;&gt;"",$H105=INDEX(Partidos!$K$4:$K$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H105&lt;&gt;"",$H105=INDEX(Partidos!$K$4:$K$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E105=INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0)),$F105=INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E105-$F105)=(INDEX(Partidos!$F$4:$F$107,MATCH($A105,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H105&lt;&gt;"",$H105=INDEX(Partidos!$K$4:$K$107,MATCH($A105,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H105" s="19">
@@ -14351,7 +14396,7 @@
         <v/>
       </c>
       <c r="G106" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A106,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E106)),NOT(ISNUMBER($F106))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A106,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E106=INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0)),$F106=INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E106-$F106)=(INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E106&gt;$F106,INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),AND($E106=$F106,INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),AND($E106&lt;$F106,INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E106=INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0)),$F106=INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E106-$F106)=(INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H106&lt;&gt;"",$H106=INDEX(Partidos!$K$4:$K$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A106,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E106)),NOT(ISNUMBER($F106))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A106,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E106=INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0)),$F106=INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E106-$F106)=(INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E106&gt;$F106,INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),AND($E106=$F106,INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),AND($E106&lt;$F106,INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0)),IF(AND($E106=INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0)),$F106=INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),IF(AND($H106&lt;&gt;"",$H106=INDEX(Partidos!$K$4:$K$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E106=$F106,($E106-$F106)=(INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0)))),IF(AND($H106&lt;&gt;"",$H106=INDEX(Partidos!$K$4:$K$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H106&lt;&gt;"",$H106=INDEX(Partidos!$K$4:$K$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E106=INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0)),$F106=INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E106-$F106)=(INDEX(Partidos!$F$4:$F$107,MATCH($A106,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H106&lt;&gt;"",$H106=INDEX(Partidos!$K$4:$K$107,MATCH($A106,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H106" s="19">
@@ -14393,7 +14438,7 @@
         <v/>
       </c>
       <c r="G107" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A107,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E107)),NOT(ISNUMBER($F107))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A107,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E107=INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0)),$F107=INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E107-$F107)=(INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E107&gt;$F107,INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),AND($E107=$F107,INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),AND($E107&lt;$F107,INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E107=INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0)),$F107=INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E107-$F107)=(INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H107&lt;&gt;"",$H107=INDEX(Partidos!$K$4:$K$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A107,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E107)),NOT(ISNUMBER($F107))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A107,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E107=INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0)),$F107=INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E107-$F107)=(INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E107&gt;$F107,INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),AND($E107=$F107,INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),AND($E107&lt;$F107,INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0)),IF(AND($E107=INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0)),$F107=INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),IF(AND($H107&lt;&gt;"",$H107=INDEX(Partidos!$K$4:$K$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E107=$F107,($E107-$F107)=(INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0)))),IF(AND($H107&lt;&gt;"",$H107=INDEX(Partidos!$K$4:$K$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H107&lt;&gt;"",$H107=INDEX(Partidos!$K$4:$K$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E107=INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0)),$F107=INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E107-$F107)=(INDEX(Partidos!$F$4:$F$107,MATCH($A107,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H107&lt;&gt;"",$H107=INDEX(Partidos!$K$4:$K$107,MATCH($A107,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H107" s="19">
@@ -14435,7 +14480,7 @@
         <v/>
       </c>
       <c r="G108" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A108,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E108)),NOT(ISNUMBER($F108))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A108,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E108=INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0)),$F108=INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E108-$F108)=(INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E108&gt;$F108,INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),AND($E108=$F108,INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),AND($E108&lt;$F108,INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E108=INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0)),$F108=INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E108-$F108)=(INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H108&lt;&gt;"",$H108=INDEX(Partidos!$K$4:$K$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A108,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E108)),NOT(ISNUMBER($F108))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A108,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E108=INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0)),$F108=INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E108-$F108)=(INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E108&gt;$F108,INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),AND($E108=$F108,INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),AND($E108&lt;$F108,INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0)),IF(AND($E108=INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0)),$F108=INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),IF(AND($H108&lt;&gt;"",$H108=INDEX(Partidos!$K$4:$K$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E108=$F108,($E108-$F108)=(INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0)))),IF(AND($H108&lt;&gt;"",$H108=INDEX(Partidos!$K$4:$K$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H108&lt;&gt;"",$H108=INDEX(Partidos!$K$4:$K$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E108=INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0)),$F108=INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E108-$F108)=(INDEX(Partidos!$F$4:$F$107,MATCH($A108,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H108&lt;&gt;"",$H108=INDEX(Partidos!$K$4:$K$107,MATCH($A108,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H108" s="19">
@@ -14477,7 +14522,7 @@
         <v/>
       </c>
       <c r="G109" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A109,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E109)),NOT(ISNUMBER($F109))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A109,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E109=INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0)),$F109=INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E109-$F109)=(INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E109&gt;$F109,INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),AND($E109=$F109,INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),AND($E109&lt;$F109,INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E109=INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0)),$F109=INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E109-$F109)=(INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H109&lt;&gt;"",$H109=INDEX(Partidos!$K$4:$K$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A109,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E109)),NOT(ISNUMBER($F109))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A109,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E109=INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0)),$F109=INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E109-$F109)=(INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E109&gt;$F109,INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),AND($E109=$F109,INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),AND($E109&lt;$F109,INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0)),IF(AND($E109=INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0)),$F109=INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),IF(AND($H109&lt;&gt;"",$H109=INDEX(Partidos!$K$4:$K$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E109=$F109,($E109-$F109)=(INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0)))),IF(AND($H109&lt;&gt;"",$H109=INDEX(Partidos!$K$4:$K$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H109&lt;&gt;"",$H109=INDEX(Partidos!$K$4:$K$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E109=INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0)),$F109=INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E109-$F109)=(INDEX(Partidos!$F$4:$F$107,MATCH($A109,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H109&lt;&gt;"",$H109=INDEX(Partidos!$K$4:$K$107,MATCH($A109,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H109" s="19">
@@ -14519,7 +14564,7 @@
         <v/>
       </c>
       <c r="G110" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A110,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E110)),NOT(ISNUMBER($F110))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A110,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E110=INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0)),$F110=INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E110-$F110)=(INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E110&gt;$F110,INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),AND($E110=$F110,INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),AND($E110&lt;$F110,INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E110=INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0)),$F110=INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E110-$F110)=(INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H110&lt;&gt;"",$H110=INDEX(Partidos!$K$4:$K$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A110,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E110)),NOT(ISNUMBER($F110))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A110,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E110=INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0)),$F110=INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E110-$F110)=(INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E110&gt;$F110,INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),AND($E110=$F110,INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),AND($E110&lt;$F110,INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0)),IF(AND($E110=INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0)),$F110=INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),IF(AND($H110&lt;&gt;"",$H110=INDEX(Partidos!$K$4:$K$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E110=$F110,($E110-$F110)=(INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0)))),IF(AND($H110&lt;&gt;"",$H110=INDEX(Partidos!$K$4:$K$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H110&lt;&gt;"",$H110=INDEX(Partidos!$K$4:$K$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E110=INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0)),$F110=INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E110-$F110)=(INDEX(Partidos!$F$4:$F$107,MATCH($A110,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H110&lt;&gt;"",$H110=INDEX(Partidos!$K$4:$K$107,MATCH($A110,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H110" s="19">
@@ -14561,7 +14606,7 @@
         <v/>
       </c>
       <c r="G111" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A111,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E111)),NOT(ISNUMBER($F111))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A111,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E111=INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0)),$F111=INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E111-$F111)=(INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E111&gt;$F111,INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),AND($E111=$F111,INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),AND($E111&lt;$F111,INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E111=INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0)),$F111=INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E111-$F111)=(INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H111&lt;&gt;"",$H111=INDEX(Partidos!$K$4:$K$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A111,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E111)),NOT(ISNUMBER($F111))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A111,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E111=INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0)),$F111=INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E111-$F111)=(INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E111&gt;$F111,INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),AND($E111=$F111,INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),AND($E111&lt;$F111,INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0)),IF(AND($E111=INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0)),$F111=INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),IF(AND($H111&lt;&gt;"",$H111=INDEX(Partidos!$K$4:$K$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E111=$F111,($E111-$F111)=(INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0)))),IF(AND($H111&lt;&gt;"",$H111=INDEX(Partidos!$K$4:$K$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H111&lt;&gt;"",$H111=INDEX(Partidos!$K$4:$K$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E111=INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0)),$F111=INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E111-$F111)=(INDEX(Partidos!$F$4:$F$107,MATCH($A111,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H111&lt;&gt;"",$H111=INDEX(Partidos!$K$4:$K$107,MATCH($A111,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H111" s="19">
@@ -14603,7 +14648,7 @@
         <v/>
       </c>
       <c r="G112" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A112,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E112)),NOT(ISNUMBER($F112))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A112,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E112=INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0)),$F112=INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E112-$F112)=(INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E112&gt;$F112,INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),AND($E112=$F112,INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),AND($E112&lt;$F112,INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E112=INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0)),$F112=INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E112-$F112)=(INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H112&lt;&gt;"",$H112=INDEX(Partidos!$K$4:$K$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A112,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E112)),NOT(ISNUMBER($F112))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A112,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E112=INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0)),$F112=INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E112-$F112)=(INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E112&gt;$F112,INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),AND($E112=$F112,INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),AND($E112&lt;$F112,INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0)),IF(AND($E112=INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0)),$F112=INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),IF(AND($H112&lt;&gt;"",$H112=INDEX(Partidos!$K$4:$K$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E112=$F112,($E112-$F112)=(INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0)))),IF(AND($H112&lt;&gt;"",$H112=INDEX(Partidos!$K$4:$K$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H112&lt;&gt;"",$H112=INDEX(Partidos!$K$4:$K$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E112=INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0)),$F112=INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E112-$F112)=(INDEX(Partidos!$F$4:$F$107,MATCH($A112,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H112&lt;&gt;"",$H112=INDEX(Partidos!$K$4:$K$107,MATCH($A112,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H112" s="19">
@@ -14645,7 +14690,7 @@
         <v/>
       </c>
       <c r="G113" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A113,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E113)),NOT(ISNUMBER($F113))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A113,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E113=INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0)),$F113=INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E113-$F113)=(INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E113&gt;$F113,INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),AND($E113=$F113,INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),AND($E113&lt;$F113,INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E113=INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0)),$F113=INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E113-$F113)=(INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H113&lt;&gt;"",$H113=INDEX(Partidos!$K$4:$K$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A113,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E113)),NOT(ISNUMBER($F113))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A113,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E113=INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0)),$F113=INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E113-$F113)=(INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E113&gt;$F113,INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),AND($E113=$F113,INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),AND($E113&lt;$F113,INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0)),IF(AND($E113=INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0)),$F113=INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),IF(AND($H113&lt;&gt;"",$H113=INDEX(Partidos!$K$4:$K$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E113=$F113,($E113-$F113)=(INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0)))),IF(AND($H113&lt;&gt;"",$H113=INDEX(Partidos!$K$4:$K$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H113&lt;&gt;"",$H113=INDEX(Partidos!$K$4:$K$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E113=INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0)),$F113=INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E113-$F113)=(INDEX(Partidos!$F$4:$F$107,MATCH($A113,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H113&lt;&gt;"",$H113=INDEX(Partidos!$K$4:$K$107,MATCH($A113,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H113" s="19">
@@ -14687,7 +14732,7 @@
         <v/>
       </c>
       <c r="G114" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A114,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E114)),NOT(ISNUMBER($F114))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A114,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E114=INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0)),$F114=INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E114-$F114)=(INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E114&gt;$F114,INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),AND($E114=$F114,INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),AND($E114&lt;$F114,INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E114=INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0)),$F114=INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E114-$F114)=(INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H114&lt;&gt;"",$H114=INDEX(Partidos!$K$4:$K$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A114,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E114)),NOT(ISNUMBER($F114))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A114,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E114=INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0)),$F114=INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E114-$F114)=(INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E114&gt;$F114,INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),AND($E114=$F114,INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),AND($E114&lt;$F114,INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0)),IF(AND($E114=INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0)),$F114=INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),IF(AND($H114&lt;&gt;"",$H114=INDEX(Partidos!$K$4:$K$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E114=$F114,($E114-$F114)=(INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0)))),IF(AND($H114&lt;&gt;"",$H114=INDEX(Partidos!$K$4:$K$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H114&lt;&gt;"",$H114=INDEX(Partidos!$K$4:$K$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E114=INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0)),$F114=INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E114-$F114)=(INDEX(Partidos!$F$4:$F$107,MATCH($A114,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H114&lt;&gt;"",$H114=INDEX(Partidos!$K$4:$K$107,MATCH($A114,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H114" s="19">
@@ -14729,7 +14774,7 @@
         <v/>
       </c>
       <c r="G115" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A115,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E115)),NOT(ISNUMBER($F115))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A115,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E115=INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0)),$F115=INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E115-$F115)=(INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E115&gt;$F115,INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),AND($E115=$F115,INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),AND($E115&lt;$F115,INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E115=INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0)),$F115=INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E115-$F115)=(INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H115&lt;&gt;"",$H115=INDEX(Partidos!$K$4:$K$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A115,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E115)),NOT(ISNUMBER($F115))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A115,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E115=INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0)),$F115=INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E115-$F115)=(INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E115&gt;$F115,INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),AND($E115=$F115,INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),AND($E115&lt;$F115,INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0)),IF(AND($E115=INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0)),$F115=INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),IF(AND($H115&lt;&gt;"",$H115=INDEX(Partidos!$K$4:$K$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E115=$F115,($E115-$F115)=(INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0)))),IF(AND($H115&lt;&gt;"",$H115=INDEX(Partidos!$K$4:$K$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H115&lt;&gt;"",$H115=INDEX(Partidos!$K$4:$K$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E115=INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0)),$F115=INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E115-$F115)=(INDEX(Partidos!$F$4:$F$107,MATCH($A115,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H115&lt;&gt;"",$H115=INDEX(Partidos!$K$4:$K$107,MATCH($A115,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H115" s="19">
@@ -14771,7 +14816,7 @@
         <v/>
       </c>
       <c r="G116" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A116,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E116)),NOT(ISNUMBER($F116))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A116,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E116=INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0)),$F116=INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E116-$F116)=(INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E116&gt;$F116,INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),AND($E116=$F116,INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),AND($E116&lt;$F116,INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E116=INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0)),$F116=INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E116-$F116)=(INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H116&lt;&gt;"",$H116=INDEX(Partidos!$K$4:$K$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A116,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E116)),NOT(ISNUMBER($F116))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A116,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E116=INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0)),$F116=INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E116-$F116)=(INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E116&gt;$F116,INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),AND($E116=$F116,INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),AND($E116&lt;$F116,INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0)),IF(AND($E116=INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0)),$F116=INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),IF(AND($H116&lt;&gt;"",$H116=INDEX(Partidos!$K$4:$K$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E116=$F116,($E116-$F116)=(INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0)))),IF(AND($H116&lt;&gt;"",$H116=INDEX(Partidos!$K$4:$K$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H116&lt;&gt;"",$H116=INDEX(Partidos!$K$4:$K$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E116=INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0)),$F116=INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E116-$F116)=(INDEX(Partidos!$F$4:$F$107,MATCH($A116,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H116&lt;&gt;"",$H116=INDEX(Partidos!$K$4:$K$107,MATCH($A116,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H116" s="19">
@@ -14813,7 +14858,7 @@
         <v/>
       </c>
       <c r="G117" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A117,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E117)),NOT(ISNUMBER($F117))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A117,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E117=INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0)),$F117=INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E117-$F117)=(INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E117&gt;$F117,INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),AND($E117=$F117,INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),AND($E117&lt;$F117,INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E117=INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0)),$F117=INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E117-$F117)=(INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H117&lt;&gt;"",$H117=INDEX(Partidos!$K$4:$K$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A117,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E117)),NOT(ISNUMBER($F117))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A117,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E117=INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0)),$F117=INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E117-$F117)=(INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E117&gt;$F117,INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),AND($E117=$F117,INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),AND($E117&lt;$F117,INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0)),IF(AND($E117=INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0)),$F117=INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),IF(AND($H117&lt;&gt;"",$H117=INDEX(Partidos!$K$4:$K$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E117=$F117,($E117-$F117)=(INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0)))),IF(AND($H117&lt;&gt;"",$H117=INDEX(Partidos!$K$4:$K$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H117&lt;&gt;"",$H117=INDEX(Partidos!$K$4:$K$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E117=INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0)),$F117=INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E117-$F117)=(INDEX(Partidos!$F$4:$F$107,MATCH($A117,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H117&lt;&gt;"",$H117=INDEX(Partidos!$K$4:$K$107,MATCH($A117,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H117" s="19">
@@ -14855,7 +14900,7 @@
         <v/>
       </c>
       <c r="G118" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A118,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E118)),NOT(ISNUMBER($F118))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A118,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E118=INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0)),$F118=INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E118-$F118)=(INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E118&gt;$F118,INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),AND($E118=$F118,INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),AND($E118&lt;$F118,INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E118=INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0)),$F118=INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E118-$F118)=(INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H118&lt;&gt;"",$H118=INDEX(Partidos!$K$4:$K$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A118,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E118)),NOT(ISNUMBER($F118))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A118,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E118=INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0)),$F118=INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E118-$F118)=(INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E118&gt;$F118,INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),AND($E118=$F118,INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),AND($E118&lt;$F118,INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0)),IF(AND($E118=INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0)),$F118=INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),IF(AND($H118&lt;&gt;"",$H118=INDEX(Partidos!$K$4:$K$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E118=$F118,($E118-$F118)=(INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0)))),IF(AND($H118&lt;&gt;"",$H118=INDEX(Partidos!$K$4:$K$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H118&lt;&gt;"",$H118=INDEX(Partidos!$K$4:$K$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E118=INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0)),$F118=INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E118-$F118)=(INDEX(Partidos!$F$4:$F$107,MATCH($A118,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H118&lt;&gt;"",$H118=INDEX(Partidos!$K$4:$K$107,MATCH($A118,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H118" s="19">
@@ -14897,7 +14942,7 @@
         <v/>
       </c>
       <c r="G119" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A119,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E119)),NOT(ISNUMBER($F119))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A119,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E119=INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0)),$F119=INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E119-$F119)=(INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E119&gt;$F119,INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),AND($E119=$F119,INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),AND($E119&lt;$F119,INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E119=INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0)),$F119=INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E119-$F119)=(INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H119&lt;&gt;"",$H119=INDEX(Partidos!$K$4:$K$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A119,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E119)),NOT(ISNUMBER($F119))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A119,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E119=INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0)),$F119=INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E119-$F119)=(INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E119&gt;$F119,INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),AND($E119=$F119,INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),AND($E119&lt;$F119,INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0)),IF(AND($E119=INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0)),$F119=INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),IF(AND($H119&lt;&gt;"",$H119=INDEX(Partidos!$K$4:$K$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E119=$F119,($E119-$F119)=(INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0)))),IF(AND($H119&lt;&gt;"",$H119=INDEX(Partidos!$K$4:$K$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H119&lt;&gt;"",$H119=INDEX(Partidos!$K$4:$K$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E119=INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0)),$F119=INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E119-$F119)=(INDEX(Partidos!$F$4:$F$107,MATCH($A119,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H119&lt;&gt;"",$H119=INDEX(Partidos!$K$4:$K$107,MATCH($A119,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H119" s="19">
@@ -14939,7 +14984,7 @@
         <v/>
       </c>
       <c r="G120" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A120,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E120)),NOT(ISNUMBER($F120))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A120,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E120=INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0)),$F120=INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E120-$F120)=(INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E120&gt;$F120,INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),AND($E120=$F120,INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),AND($E120&lt;$F120,INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E120=INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0)),$F120=INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E120-$F120)=(INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H120&lt;&gt;"",$H120=INDEX(Partidos!$K$4:$K$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A120,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E120)),NOT(ISNUMBER($F120))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A120,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E120=INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0)),$F120=INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E120-$F120)=(INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E120&gt;$F120,INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),AND($E120=$F120,INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),AND($E120&lt;$F120,INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0)),IF(AND($E120=INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0)),$F120=INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),IF(AND($H120&lt;&gt;"",$H120=INDEX(Partidos!$K$4:$K$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E120=$F120,($E120-$F120)=(INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0)))),IF(AND($H120&lt;&gt;"",$H120=INDEX(Partidos!$K$4:$K$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H120&lt;&gt;"",$H120=INDEX(Partidos!$K$4:$K$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E120=INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0)),$F120=INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E120-$F120)=(INDEX(Partidos!$F$4:$F$107,MATCH($A120,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H120&lt;&gt;"",$H120=INDEX(Partidos!$K$4:$K$107,MATCH($A120,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H120" s="19">
@@ -14981,7 +15026,7 @@
         <v/>
       </c>
       <c r="G121" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A121,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E121)),NOT(ISNUMBER($F121))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A121,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E121=INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0)),$F121=INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E121-$F121)=(INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E121&gt;$F121,INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),AND($E121=$F121,INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),AND($E121&lt;$F121,INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E121=INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0)),$F121=INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E121-$F121)=(INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H121&lt;&gt;"",$H121=INDEX(Partidos!$K$4:$K$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A121,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E121)),NOT(ISNUMBER($F121))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A121,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E121=INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0)),$F121=INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E121-$F121)=(INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E121&gt;$F121,INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),AND($E121=$F121,INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),AND($E121&lt;$F121,INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0)),IF(AND($E121=INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0)),$F121=INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),IF(AND($H121&lt;&gt;"",$H121=INDEX(Partidos!$K$4:$K$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E121=$F121,($E121-$F121)=(INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0)))),IF(AND($H121&lt;&gt;"",$H121=INDEX(Partidos!$K$4:$K$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H121&lt;&gt;"",$H121=INDEX(Partidos!$K$4:$K$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E121=INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0)),$F121=INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E121-$F121)=(INDEX(Partidos!$F$4:$F$107,MATCH($A121,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H121&lt;&gt;"",$H121=INDEX(Partidos!$K$4:$K$107,MATCH($A121,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H121" s="19">
@@ -15023,7 +15068,7 @@
         <v/>
       </c>
       <c r="G122" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A122,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E122)),NOT(ISNUMBER($F122))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A122,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E122=INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0)),$F122=INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E122-$F122)=(INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E122&gt;$F122,INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),AND($E122=$F122,INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),AND($E122&lt;$F122,INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E122=INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0)),$F122=INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E122-$F122)=(INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H122&lt;&gt;"",$H122=INDEX(Partidos!$K$4:$K$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A122,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E122)),NOT(ISNUMBER($F122))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A122,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E122=INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0)),$F122=INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E122-$F122)=(INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E122&gt;$F122,INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),AND($E122=$F122,INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),AND($E122&lt;$F122,INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0)),IF(AND($E122=INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0)),$F122=INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),IF(AND($H122&lt;&gt;"",$H122=INDEX(Partidos!$K$4:$K$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E122=$F122,($E122-$F122)=(INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0)))),IF(AND($H122&lt;&gt;"",$H122=INDEX(Partidos!$K$4:$K$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H122&lt;&gt;"",$H122=INDEX(Partidos!$K$4:$K$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E122=INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0)),$F122=INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E122-$F122)=(INDEX(Partidos!$F$4:$F$107,MATCH($A122,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H122&lt;&gt;"",$H122=INDEX(Partidos!$K$4:$K$107,MATCH($A122,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H122" s="19">
@@ -15065,7 +15110,7 @@
         <v/>
       </c>
       <c r="G123" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A123,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E123)),NOT(ISNUMBER($F123))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A123,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E123=INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0)),$F123=INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E123-$F123)=(INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E123&gt;$F123,INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),AND($E123=$F123,INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),AND($E123&lt;$F123,INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E123=INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0)),$F123=INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E123-$F123)=(INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H123&lt;&gt;"",$H123=INDEX(Partidos!$K$4:$K$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A123,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E123)),NOT(ISNUMBER($F123))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A123,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E123=INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0)),$F123=INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E123-$F123)=(INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E123&gt;$F123,INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),AND($E123=$F123,INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),AND($E123&lt;$F123,INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0)),IF(AND($E123=INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0)),$F123=INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),IF(AND($H123&lt;&gt;"",$H123=INDEX(Partidos!$K$4:$K$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E123=$F123,($E123-$F123)=(INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0)))),IF(AND($H123&lt;&gt;"",$H123=INDEX(Partidos!$K$4:$K$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H123&lt;&gt;"",$H123=INDEX(Partidos!$K$4:$K$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E123=INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0)),$F123=INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E123-$F123)=(INDEX(Partidos!$F$4:$F$107,MATCH($A123,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H123&lt;&gt;"",$H123=INDEX(Partidos!$K$4:$K$107,MATCH($A123,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H123" s="19">
@@ -15107,7 +15152,7 @@
         <v/>
       </c>
       <c r="G124" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A124,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E124)),NOT(ISNUMBER($F124))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A124,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E124=INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0)),$F124=INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E124-$F124)=(INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E124&gt;$F124,INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),AND($E124=$F124,INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),AND($E124&lt;$F124,INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E124=INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0)),$F124=INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E124-$F124)=(INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H124&lt;&gt;"",$H124=INDEX(Partidos!$K$4:$K$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A124,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E124)),NOT(ISNUMBER($F124))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A124,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E124=INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0)),$F124=INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E124-$F124)=(INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E124&gt;$F124,INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),AND($E124=$F124,INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),AND($E124&lt;$F124,INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0)),IF(AND($E124=INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0)),$F124=INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),IF(AND($H124&lt;&gt;"",$H124=INDEX(Partidos!$K$4:$K$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E124=$F124,($E124-$F124)=(INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0)))),IF(AND($H124&lt;&gt;"",$H124=INDEX(Partidos!$K$4:$K$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H124&lt;&gt;"",$H124=INDEX(Partidos!$K$4:$K$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E124=INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0)),$F124=INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E124-$F124)=(INDEX(Partidos!$F$4:$F$107,MATCH($A124,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H124&lt;&gt;"",$H124=INDEX(Partidos!$K$4:$K$107,MATCH($A124,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H124" s="19">
@@ -15149,7 +15194,7 @@
         <v/>
       </c>
       <c r="G125" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A125,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E125)),NOT(ISNUMBER($F125))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A125,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E125=INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0)),$F125=INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E125-$F125)=(INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E125&gt;$F125,INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),AND($E125=$F125,INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),AND($E125&lt;$F125,INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E125=INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0)),$F125=INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E125-$F125)=(INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H125&lt;&gt;"",$H125=INDEX(Partidos!$K$4:$K$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A125,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E125)),NOT(ISNUMBER($F125))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A125,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E125=INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0)),$F125=INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E125-$F125)=(INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E125&gt;$F125,INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),AND($E125=$F125,INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),AND($E125&lt;$F125,INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0)),IF(AND($E125=INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0)),$F125=INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),IF(AND($H125&lt;&gt;"",$H125=INDEX(Partidos!$K$4:$K$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E125=$F125,($E125-$F125)=(INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0)))),IF(AND($H125&lt;&gt;"",$H125=INDEX(Partidos!$K$4:$K$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H125&lt;&gt;"",$H125=INDEX(Partidos!$K$4:$K$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E125=INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0)),$F125=INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E125-$F125)=(INDEX(Partidos!$F$4:$F$107,MATCH($A125,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H125&lt;&gt;"",$H125=INDEX(Partidos!$K$4:$K$107,MATCH($A125,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H125" s="19">
@@ -15191,7 +15236,7 @@
         <v/>
       </c>
       <c r="G126" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A126,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E126)),NOT(ISNUMBER($F126))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A126,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E126=INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0)),$F126=INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E126-$F126)=(INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E126&gt;$F126,INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),AND($E126=$F126,INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),AND($E126&lt;$F126,INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E126=INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0)),$F126=INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E126-$F126)=(INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H126&lt;&gt;"",$H126=INDEX(Partidos!$K$4:$K$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A126,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E126)),NOT(ISNUMBER($F126))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A126,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E126=INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0)),$F126=INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E126-$F126)=(INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E126&gt;$F126,INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),AND($E126=$F126,INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),AND($E126&lt;$F126,INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0)),IF(AND($E126=INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0)),$F126=INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),IF(AND($H126&lt;&gt;"",$H126=INDEX(Partidos!$K$4:$K$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E126=$F126,($E126-$F126)=(INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0)))),IF(AND($H126&lt;&gt;"",$H126=INDEX(Partidos!$K$4:$K$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H126&lt;&gt;"",$H126=INDEX(Partidos!$K$4:$K$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E126=INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0)),$F126=INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E126-$F126)=(INDEX(Partidos!$F$4:$F$107,MATCH($A126,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H126&lt;&gt;"",$H126=INDEX(Partidos!$K$4:$K$107,MATCH($A126,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H126" s="19">
@@ -15233,7 +15278,7 @@
         <v/>
       </c>
       <c r="G127" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A127,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E127)),NOT(ISNUMBER($F127))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A127,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E127=INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0)),$F127=INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E127-$F127)=(INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E127&gt;$F127,INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),AND($E127=$F127,INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),AND($E127&lt;$F127,INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E127=INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0)),$F127=INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E127-$F127)=(INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H127&lt;&gt;"",$H127=INDEX(Partidos!$K$4:$K$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A127,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E127)),NOT(ISNUMBER($F127))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A127,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E127=INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0)),$F127=INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E127-$F127)=(INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E127&gt;$F127,INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),AND($E127=$F127,INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),AND($E127&lt;$F127,INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0)),IF(AND($E127=INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0)),$F127=INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),IF(AND($H127&lt;&gt;"",$H127=INDEX(Partidos!$K$4:$K$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E127=$F127,($E127-$F127)=(INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0)))),IF(AND($H127&lt;&gt;"",$H127=INDEX(Partidos!$K$4:$K$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H127&lt;&gt;"",$H127=INDEX(Partidos!$K$4:$K$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E127=INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0)),$F127=INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E127-$F127)=(INDEX(Partidos!$F$4:$F$107,MATCH($A127,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H127&lt;&gt;"",$H127=INDEX(Partidos!$K$4:$K$107,MATCH($A127,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H127" s="19">
@@ -15275,7 +15320,7 @@
         <v/>
       </c>
       <c r="G128" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A128,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E128)),NOT(ISNUMBER($F128))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A128,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E128=INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0)),$F128=INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E128-$F128)=(INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E128&gt;$F128,INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),AND($E128=$F128,INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),AND($E128&lt;$F128,INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E128=INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0)),$F128=INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E128-$F128)=(INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H128&lt;&gt;"",$H128=INDEX(Partidos!$K$4:$K$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A128,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E128)),NOT(ISNUMBER($F128))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A128,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E128=INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0)),$F128=INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E128-$F128)=(INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E128&gt;$F128,INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),AND($E128=$F128,INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),AND($E128&lt;$F128,INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0)),IF(AND($E128=INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0)),$F128=INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),IF(AND($H128&lt;&gt;"",$H128=INDEX(Partidos!$K$4:$K$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E128=$F128,($E128-$F128)=(INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0)))),IF(AND($H128&lt;&gt;"",$H128=INDEX(Partidos!$K$4:$K$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H128&lt;&gt;"",$H128=INDEX(Partidos!$K$4:$K$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E128=INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0)),$F128=INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E128-$F128)=(INDEX(Partidos!$F$4:$F$107,MATCH($A128,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H128&lt;&gt;"",$H128=INDEX(Partidos!$K$4:$K$107,MATCH($A128,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H128" s="19">
@@ -15317,7 +15362,7 @@
         <v/>
       </c>
       <c r="G129" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A129,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E129)),NOT(ISNUMBER($F129))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A129,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E129=INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0)),$F129=INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E129-$F129)=(INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E129&gt;$F129,INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),AND($E129=$F129,INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),AND($E129&lt;$F129,INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E129=INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0)),$F129=INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E129-$F129)=(INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H129&lt;&gt;"",$H129=INDEX(Partidos!$K$4:$K$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A129,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E129)),NOT(ISNUMBER($F129))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A129,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E129=INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0)),$F129=INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E129-$F129)=(INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E129&gt;$F129,INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),AND($E129=$F129,INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),AND($E129&lt;$F129,INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0)),IF(AND($E129=INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0)),$F129=INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),IF(AND($H129&lt;&gt;"",$H129=INDEX(Partidos!$K$4:$K$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E129=$F129,($E129-$F129)=(INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0)))),IF(AND($H129&lt;&gt;"",$H129=INDEX(Partidos!$K$4:$K$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H129&lt;&gt;"",$H129=INDEX(Partidos!$K$4:$K$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E129=INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0)),$F129=INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E129-$F129)=(INDEX(Partidos!$F$4:$F$107,MATCH($A129,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H129&lt;&gt;"",$H129=INDEX(Partidos!$K$4:$K$107,MATCH($A129,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H129" s="19">
@@ -15359,7 +15404,7 @@
         <v/>
       </c>
       <c r="G130" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A130,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E130)),NOT(ISNUMBER($F130))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A130,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E130=INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0)),$F130=INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E130-$F130)=(INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E130&gt;$F130,INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),AND($E130=$F130,INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),AND($E130&lt;$F130,INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E130=INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0)),$F130=INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E130-$F130)=(INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H130&lt;&gt;"",$H130=INDEX(Partidos!$K$4:$K$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A130,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E130)),NOT(ISNUMBER($F130))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A130,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E130=INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0)),$F130=INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E130-$F130)=(INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E130&gt;$F130,INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),AND($E130=$F130,INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),AND($E130&lt;$F130,INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0)),IF(AND($E130=INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0)),$F130=INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),IF(AND($H130&lt;&gt;"",$H130=INDEX(Partidos!$K$4:$K$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E130=$F130,($E130-$F130)=(INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0)))),IF(AND($H130&lt;&gt;"",$H130=INDEX(Partidos!$K$4:$K$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H130&lt;&gt;"",$H130=INDEX(Partidos!$K$4:$K$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E130=INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0)),$F130=INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E130-$F130)=(INDEX(Partidos!$F$4:$F$107,MATCH($A130,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H130&lt;&gt;"",$H130=INDEX(Partidos!$K$4:$K$107,MATCH($A130,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H130" s="19">
@@ -15401,7 +15446,7 @@
         <v/>
       </c>
       <c r="G131" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A131,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E131)),NOT(ISNUMBER($F131))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A131,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E131=INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0)),$F131=INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E131-$F131)=(INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E131&gt;$F131,INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),AND($E131=$F131,INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),AND($E131&lt;$F131,INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E131=INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0)),$F131=INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E131-$F131)=(INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H131&lt;&gt;"",$H131=INDEX(Partidos!$K$4:$K$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A131,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E131)),NOT(ISNUMBER($F131))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A131,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E131=INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0)),$F131=INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E131-$F131)=(INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E131&gt;$F131,INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),AND($E131=$F131,INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),AND($E131&lt;$F131,INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0)),IF(AND($E131=INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0)),$F131=INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),IF(AND($H131&lt;&gt;"",$H131=INDEX(Partidos!$K$4:$K$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E131=$F131,($E131-$F131)=(INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0)))),IF(AND($H131&lt;&gt;"",$H131=INDEX(Partidos!$K$4:$K$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H131&lt;&gt;"",$H131=INDEX(Partidos!$K$4:$K$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E131=INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0)),$F131=INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E131-$F131)=(INDEX(Partidos!$F$4:$F$107,MATCH($A131,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H131&lt;&gt;"",$H131=INDEX(Partidos!$K$4:$K$107,MATCH($A131,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H131" s="19">
@@ -15443,7 +15488,7 @@
         <v/>
       </c>
       <c r="G132" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A132,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E132)),NOT(ISNUMBER($F132))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A132,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E132=INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0)),$F132=INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E132-$F132)=(INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E132&gt;$F132,INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),AND($E132=$F132,INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),AND($E132&lt;$F132,INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E132=INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0)),$F132=INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E132-$F132)=(INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H132&lt;&gt;"",$H132=INDEX(Partidos!$K$4:$K$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A132,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E132)),NOT(ISNUMBER($F132))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A132,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E132=INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0)),$F132=INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E132-$F132)=(INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E132&gt;$F132,INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),AND($E132=$F132,INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),AND($E132&lt;$F132,INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0)),IF(AND($E132=INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0)),$F132=INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),IF(AND($H132&lt;&gt;"",$H132=INDEX(Partidos!$K$4:$K$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E132=$F132,($E132-$F132)=(INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0)))),IF(AND($H132&lt;&gt;"",$H132=INDEX(Partidos!$K$4:$K$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H132&lt;&gt;"",$H132=INDEX(Partidos!$K$4:$K$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E132=INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0)),$F132=INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E132-$F132)=(INDEX(Partidos!$F$4:$F$107,MATCH($A132,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H132&lt;&gt;"",$H132=INDEX(Partidos!$K$4:$K$107,MATCH($A132,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H132" s="19">
@@ -15485,7 +15530,7 @@
         <v/>
       </c>
       <c r="G133" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A133,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E133)),NOT(ISNUMBER($F133))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A133,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E133=INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0)),$F133=INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E133-$F133)=(INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E133&gt;$F133,INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),AND($E133=$F133,INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),AND($E133&lt;$F133,INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E133=INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0)),$F133=INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E133-$F133)=(INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H133&lt;&gt;"",$H133=INDEX(Partidos!$K$4:$K$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A133,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E133)),NOT(ISNUMBER($F133))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A133,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E133=INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0)),$F133=INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E133-$F133)=(INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E133&gt;$F133,INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),AND($E133=$F133,INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),AND($E133&lt;$F133,INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0)),IF(AND($E133=INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0)),$F133=INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),IF(AND($H133&lt;&gt;"",$H133=INDEX(Partidos!$K$4:$K$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E133=$F133,($E133-$F133)=(INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0)))),IF(AND($H133&lt;&gt;"",$H133=INDEX(Partidos!$K$4:$K$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H133&lt;&gt;"",$H133=INDEX(Partidos!$K$4:$K$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E133=INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0)),$F133=INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E133-$F133)=(INDEX(Partidos!$F$4:$F$107,MATCH($A133,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H133&lt;&gt;"",$H133=INDEX(Partidos!$K$4:$K$107,MATCH($A133,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H133" s="19">
@@ -15527,7 +15572,7 @@
         <v/>
       </c>
       <c r="G134" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A134,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E134)),NOT(ISNUMBER($F134))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A134,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E134=INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0)),$F134=INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E134-$F134)=(INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E134&gt;$F134,INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),AND($E134=$F134,INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),AND($E134&lt;$F134,INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E134=INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0)),$F134=INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E134-$F134)=(INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H134&lt;&gt;"",$H134=INDEX(Partidos!$K$4:$K$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A134,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E134)),NOT(ISNUMBER($F134))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A134,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E134=INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0)),$F134=INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E134-$F134)=(INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E134&gt;$F134,INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),AND($E134=$F134,INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),AND($E134&lt;$F134,INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0)),IF(AND($E134=INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0)),$F134=INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),IF(AND($H134&lt;&gt;"",$H134=INDEX(Partidos!$K$4:$K$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E134=$F134,($E134-$F134)=(INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0)))),IF(AND($H134&lt;&gt;"",$H134=INDEX(Partidos!$K$4:$K$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H134&lt;&gt;"",$H134=INDEX(Partidos!$K$4:$K$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E134=INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0)),$F134=INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E134-$F134)=(INDEX(Partidos!$F$4:$F$107,MATCH($A134,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H134&lt;&gt;"",$H134=INDEX(Partidos!$K$4:$K$107,MATCH($A134,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H134" s="19">
@@ -15569,7 +15614,7 @@
         <v/>
       </c>
       <c r="G135" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A135,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E135)),NOT(ISNUMBER($F135))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A135,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E135=INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0)),$F135=INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E135-$F135)=(INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E135&gt;$F135,INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),AND($E135=$F135,INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),AND($E135&lt;$F135,INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E135=INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0)),$F135=INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E135-$F135)=(INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H135&lt;&gt;"",$H135=INDEX(Partidos!$K$4:$K$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A135,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E135)),NOT(ISNUMBER($F135))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A135,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E135=INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0)),$F135=INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E135-$F135)=(INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E135&gt;$F135,INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),AND($E135=$F135,INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),AND($E135&lt;$F135,INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0)),IF(AND($E135=INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0)),$F135=INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),IF(AND($H135&lt;&gt;"",$H135=INDEX(Partidos!$K$4:$K$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E135=$F135,($E135-$F135)=(INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0)))),IF(AND($H135&lt;&gt;"",$H135=INDEX(Partidos!$K$4:$K$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H135&lt;&gt;"",$H135=INDEX(Partidos!$K$4:$K$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E135=INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0)),$F135=INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E135-$F135)=(INDEX(Partidos!$F$4:$F$107,MATCH($A135,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H135&lt;&gt;"",$H135=INDEX(Partidos!$K$4:$K$107,MATCH($A135,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H135" s="19">
@@ -15611,7 +15656,7 @@
         <v/>
       </c>
       <c r="G136" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A136,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E136)),NOT(ISNUMBER($F136))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A136,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E136=INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0)),$F136=INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E136-$F136)=(INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E136&gt;$F136,INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),AND($E136=$F136,INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),AND($E136&lt;$F136,INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E136=INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0)),$F136=INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E136-$F136)=(INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H136&lt;&gt;"",$H136=INDEX(Partidos!$K$4:$K$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A136,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E136)),NOT(ISNUMBER($F136))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A136,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E136=INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0)),$F136=INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E136-$F136)=(INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E136&gt;$F136,INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),AND($E136=$F136,INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),AND($E136&lt;$F136,INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0)),IF(AND($E136=INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0)),$F136=INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),IF(AND($H136&lt;&gt;"",$H136=INDEX(Partidos!$K$4:$K$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E136=$F136,($E136-$F136)=(INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0)))),IF(AND($H136&lt;&gt;"",$H136=INDEX(Partidos!$K$4:$K$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H136&lt;&gt;"",$H136=INDEX(Partidos!$K$4:$K$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E136=INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0)),$F136=INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E136-$F136)=(INDEX(Partidos!$F$4:$F$107,MATCH($A136,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H136&lt;&gt;"",$H136=INDEX(Partidos!$K$4:$K$107,MATCH($A136,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H136" s="19">
@@ -15653,7 +15698,7 @@
         <v/>
       </c>
       <c r="G137" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A137,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E137)),NOT(ISNUMBER($F137))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A137,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E137=INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0)),$F137=INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E137-$F137)=(INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E137&gt;$F137,INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),AND($E137=$F137,INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),AND($E137&lt;$F137,INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E137=INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0)),$F137=INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E137-$F137)=(INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H137&lt;&gt;"",$H137=INDEX(Partidos!$K$4:$K$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A137,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E137)),NOT(ISNUMBER($F137))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A137,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E137=INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0)),$F137=INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E137-$F137)=(INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E137&gt;$F137,INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),AND($E137=$F137,INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),AND($E137&lt;$F137,INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0)),IF(AND($E137=INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0)),$F137=INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),IF(AND($H137&lt;&gt;"",$H137=INDEX(Partidos!$K$4:$K$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E137=$F137,($E137-$F137)=(INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0)))),IF(AND($H137&lt;&gt;"",$H137=INDEX(Partidos!$K$4:$K$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H137&lt;&gt;"",$H137=INDEX(Partidos!$K$4:$K$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E137=INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0)),$F137=INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E137-$F137)=(INDEX(Partidos!$F$4:$F$107,MATCH($A137,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H137&lt;&gt;"",$H137=INDEX(Partidos!$K$4:$K$107,MATCH($A137,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H137" s="19">
@@ -15695,7 +15740,7 @@
         <v/>
       </c>
       <c r="G138" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A138,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E138)),NOT(ISNUMBER($F138))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A138,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E138=INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0)),$F138=INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E138-$F138)=(INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E138&gt;$F138,INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),AND($E138=$F138,INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),AND($E138&lt;$F138,INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E138=INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0)),$F138=INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E138-$F138)=(INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H138&lt;&gt;"",$H138=INDEX(Partidos!$K$4:$K$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A138,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E138)),NOT(ISNUMBER($F138))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A138,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E138=INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0)),$F138=INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E138-$F138)=(INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E138&gt;$F138,INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),AND($E138=$F138,INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),AND($E138&lt;$F138,INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0)),IF(AND($E138=INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0)),$F138=INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),IF(AND($H138&lt;&gt;"",$H138=INDEX(Partidos!$K$4:$K$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E138=$F138,($E138-$F138)=(INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0)))),IF(AND($H138&lt;&gt;"",$H138=INDEX(Partidos!$K$4:$K$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H138&lt;&gt;"",$H138=INDEX(Partidos!$K$4:$K$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E138=INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0)),$F138=INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E138-$F138)=(INDEX(Partidos!$F$4:$F$107,MATCH($A138,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H138&lt;&gt;"",$H138=INDEX(Partidos!$K$4:$K$107,MATCH($A138,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H138" s="19">
@@ -15737,7 +15782,7 @@
         <v/>
       </c>
       <c r="G139" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A139,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E139)),NOT(ISNUMBER($F139))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A139,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E139=INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0)),$F139=INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E139-$F139)=(INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E139&gt;$F139,INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),AND($E139=$F139,INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),AND($E139&lt;$F139,INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E139=INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0)),$F139=INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E139-$F139)=(INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H139&lt;&gt;"",$H139=INDEX(Partidos!$K$4:$K$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A139,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E139)),NOT(ISNUMBER($F139))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A139,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E139=INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0)),$F139=INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E139-$F139)=(INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E139&gt;$F139,INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),AND($E139=$F139,INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),AND($E139&lt;$F139,INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0)),IF(AND($E139=INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0)),$F139=INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),IF(AND($H139&lt;&gt;"",$H139=INDEX(Partidos!$K$4:$K$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E139=$F139,($E139-$F139)=(INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0)))),IF(AND($H139&lt;&gt;"",$H139=INDEX(Partidos!$K$4:$K$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H139&lt;&gt;"",$H139=INDEX(Partidos!$K$4:$K$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E139=INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0)),$F139=INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E139-$F139)=(INDEX(Partidos!$F$4:$F$107,MATCH($A139,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H139&lt;&gt;"",$H139=INDEX(Partidos!$K$4:$K$107,MATCH($A139,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H139" s="19">
@@ -15779,7 +15824,7 @@
         <v/>
       </c>
       <c r="G140" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A140,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E140)),NOT(ISNUMBER($F140))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A140,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E140=INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0)),$F140=INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E140-$F140)=(INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E140&gt;$F140,INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),AND($E140=$F140,INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),AND($E140&lt;$F140,INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E140=INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0)),$F140=INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E140-$F140)=(INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H140&lt;&gt;"",$H140=INDEX(Partidos!$K$4:$K$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A140,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E140)),NOT(ISNUMBER($F140))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A140,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E140=INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0)),$F140=INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E140-$F140)=(INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E140&gt;$F140,INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),AND($E140=$F140,INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),AND($E140&lt;$F140,INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0)),IF(AND($E140=INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0)),$F140=INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),IF(AND($H140&lt;&gt;"",$H140=INDEX(Partidos!$K$4:$K$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E140=$F140,($E140-$F140)=(INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0)))),IF(AND($H140&lt;&gt;"",$H140=INDEX(Partidos!$K$4:$K$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H140&lt;&gt;"",$H140=INDEX(Partidos!$K$4:$K$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E140=INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0)),$F140=INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E140-$F140)=(INDEX(Partidos!$F$4:$F$107,MATCH($A140,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H140&lt;&gt;"",$H140=INDEX(Partidos!$K$4:$K$107,MATCH($A140,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H140" s="19">
@@ -15821,7 +15866,7 @@
         <v/>
       </c>
       <c r="G141" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A141,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E141)),NOT(ISNUMBER($F141))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A141,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E141=INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0)),$F141=INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E141-$F141)=(INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E141&gt;$F141,INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),AND($E141=$F141,INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),AND($E141&lt;$F141,INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E141=INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0)),$F141=INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E141-$F141)=(INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H141&lt;&gt;"",$H141=INDEX(Partidos!$K$4:$K$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A141,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E141)),NOT(ISNUMBER($F141))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A141,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E141=INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0)),$F141=INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E141-$F141)=(INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E141&gt;$F141,INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),AND($E141=$F141,INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),AND($E141&lt;$F141,INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0)),IF(AND($E141=INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0)),$F141=INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),IF(AND($H141&lt;&gt;"",$H141=INDEX(Partidos!$K$4:$K$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E141=$F141,($E141-$F141)=(INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0)))),IF(AND($H141&lt;&gt;"",$H141=INDEX(Partidos!$K$4:$K$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H141&lt;&gt;"",$H141=INDEX(Partidos!$K$4:$K$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E141=INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0)),$F141=INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E141-$F141)=(INDEX(Partidos!$F$4:$F$107,MATCH($A141,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H141&lt;&gt;"",$H141=INDEX(Partidos!$K$4:$K$107,MATCH($A141,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H141" s="19">
@@ -15863,7 +15908,7 @@
         <v/>
       </c>
       <c r="G142" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A142,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E142)),NOT(ISNUMBER($F142))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A142,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E142=INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0)),$F142=INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E142-$F142)=(INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E142&gt;$F142,INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),AND($E142=$F142,INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),AND($E142&lt;$F142,INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E142=INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0)),$F142=INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E142-$F142)=(INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H142&lt;&gt;"",$H142=INDEX(Partidos!$K$4:$K$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A142,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E142)),NOT(ISNUMBER($F142))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A142,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E142=INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0)),$F142=INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E142-$F142)=(INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E142&gt;$F142,INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),AND($E142=$F142,INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),AND($E142&lt;$F142,INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0)),IF(AND($E142=INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0)),$F142=INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),IF(AND($H142&lt;&gt;"",$H142=INDEX(Partidos!$K$4:$K$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E142=$F142,($E142-$F142)=(INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0)))),IF(AND($H142&lt;&gt;"",$H142=INDEX(Partidos!$K$4:$K$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H142&lt;&gt;"",$H142=INDEX(Partidos!$K$4:$K$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E142=INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0)),$F142=INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E142-$F142)=(INDEX(Partidos!$F$4:$F$107,MATCH($A142,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H142&lt;&gt;"",$H142=INDEX(Partidos!$K$4:$K$107,MATCH($A142,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H142" s="19">
@@ -15905,7 +15950,7 @@
         <v/>
       </c>
       <c r="G143" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A143,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E143)),NOT(ISNUMBER($F143))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A143,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E143=INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0)),$F143=INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E143-$F143)=(INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E143&gt;$F143,INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),AND($E143=$F143,INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),AND($E143&lt;$F143,INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E143=INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0)),$F143=INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E143-$F143)=(INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H143&lt;&gt;"",$H143=INDEX(Partidos!$K$4:$K$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A143,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E143)),NOT(ISNUMBER($F143))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A143,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E143=INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0)),$F143=INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E143-$F143)=(INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E143&gt;$F143,INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),AND($E143=$F143,INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),AND($E143&lt;$F143,INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0)),IF(AND($E143=INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0)),$F143=INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),IF(AND($H143&lt;&gt;"",$H143=INDEX(Partidos!$K$4:$K$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E143=$F143,($E143-$F143)=(INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0)))),IF(AND($H143&lt;&gt;"",$H143=INDEX(Partidos!$K$4:$K$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H143&lt;&gt;"",$H143=INDEX(Partidos!$K$4:$K$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E143=INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0)),$F143=INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E143-$F143)=(INDEX(Partidos!$F$4:$F$107,MATCH($A143,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H143&lt;&gt;"",$H143=INDEX(Partidos!$K$4:$K$107,MATCH($A143,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H143" s="19">
@@ -15947,7 +15992,7 @@
         <v/>
       </c>
       <c r="G144" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A144,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E144)),NOT(ISNUMBER($F144))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A144,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E144=INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0)),$F144=INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E144-$F144)=(INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E144&gt;$F144,INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),AND($E144=$F144,INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),AND($E144&lt;$F144,INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E144=INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0)),$F144=INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E144-$F144)=(INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H144&lt;&gt;"",$H144=INDEX(Partidos!$K$4:$K$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A144,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E144)),NOT(ISNUMBER($F144))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A144,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E144=INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0)),$F144=INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E144-$F144)=(INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E144&gt;$F144,INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),AND($E144=$F144,INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),AND($E144&lt;$F144,INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0)),IF(AND($E144=INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0)),$F144=INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),IF(AND($H144&lt;&gt;"",$H144=INDEX(Partidos!$K$4:$K$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E144=$F144,($E144-$F144)=(INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0)))),IF(AND($H144&lt;&gt;"",$H144=INDEX(Partidos!$K$4:$K$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H144&lt;&gt;"",$H144=INDEX(Partidos!$K$4:$K$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E144=INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0)),$F144=INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E144-$F144)=(INDEX(Partidos!$F$4:$F$107,MATCH($A144,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H144&lt;&gt;"",$H144=INDEX(Partidos!$K$4:$K$107,MATCH($A144,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H144" s="19">
@@ -15989,7 +16034,7 @@
         <v/>
       </c>
       <c r="G145" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A145,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E145)),NOT(ISNUMBER($F145))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A145,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E145=INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0)),$F145=INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E145-$F145)=(INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E145&gt;$F145,INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),AND($E145=$F145,INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),AND($E145&lt;$F145,INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E145=INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0)),$F145=INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E145-$F145)=(INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H145&lt;&gt;"",$H145=INDEX(Partidos!$K$4:$K$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A145,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E145)),NOT(ISNUMBER($F145))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A145,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E145=INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0)),$F145=INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E145-$F145)=(INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E145&gt;$F145,INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),AND($E145=$F145,INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),AND($E145&lt;$F145,INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0)),IF(AND($E145=INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0)),$F145=INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),IF(AND($H145&lt;&gt;"",$H145=INDEX(Partidos!$K$4:$K$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E145=$F145,($E145-$F145)=(INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0)))),IF(AND($H145&lt;&gt;"",$H145=INDEX(Partidos!$K$4:$K$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H145&lt;&gt;"",$H145=INDEX(Partidos!$K$4:$K$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E145=INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0)),$F145=INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E145-$F145)=(INDEX(Partidos!$F$4:$F$107,MATCH($A145,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H145&lt;&gt;"",$H145=INDEX(Partidos!$K$4:$K$107,MATCH($A145,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H145" s="19">
@@ -16031,7 +16076,7 @@
         <v/>
       </c>
       <c r="G146" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A146,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E146)),NOT(ISNUMBER($F146))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A146,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E146=INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0)),$F146=INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E146-$F146)=(INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E146&gt;$F146,INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),AND($E146=$F146,INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),AND($E146&lt;$F146,INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E146=INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0)),$F146=INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E146-$F146)=(INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H146&lt;&gt;"",$H146=INDEX(Partidos!$K$4:$K$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A146,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E146)),NOT(ISNUMBER($F146))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A146,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E146=INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0)),$F146=INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E146-$F146)=(INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E146&gt;$F146,INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),AND($E146=$F146,INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),AND($E146&lt;$F146,INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0)),IF(AND($E146=INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0)),$F146=INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),IF(AND($H146&lt;&gt;"",$H146=INDEX(Partidos!$K$4:$K$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E146=$F146,($E146-$F146)=(INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0)))),IF(AND($H146&lt;&gt;"",$H146=INDEX(Partidos!$K$4:$K$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H146&lt;&gt;"",$H146=INDEX(Partidos!$K$4:$K$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E146=INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0)),$F146=INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E146-$F146)=(INDEX(Partidos!$F$4:$F$107,MATCH($A146,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H146&lt;&gt;"",$H146=INDEX(Partidos!$K$4:$K$107,MATCH($A146,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H146" s="19">
@@ -16073,7 +16118,7 @@
         <v/>
       </c>
       <c r="G147" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A147,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E147)),NOT(ISNUMBER($F147))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A147,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E147=INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0)),$F147=INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E147-$F147)=(INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E147&gt;$F147,INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),AND($E147=$F147,INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),AND($E147&lt;$F147,INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E147=INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0)),$F147=INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E147-$F147)=(INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H147&lt;&gt;"",$H147=INDEX(Partidos!$K$4:$K$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A147,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E147)),NOT(ISNUMBER($F147))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A147,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E147=INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0)),$F147=INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E147-$F147)=(INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E147&gt;$F147,INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),AND($E147=$F147,INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),AND($E147&lt;$F147,INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0)),IF(AND($E147=INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0)),$F147=INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),IF(AND($H147&lt;&gt;"",$H147=INDEX(Partidos!$K$4:$K$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E147=$F147,($E147-$F147)=(INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0)))),IF(AND($H147&lt;&gt;"",$H147=INDEX(Partidos!$K$4:$K$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H147&lt;&gt;"",$H147=INDEX(Partidos!$K$4:$K$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E147=INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0)),$F147=INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E147-$F147)=(INDEX(Partidos!$F$4:$F$107,MATCH($A147,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H147&lt;&gt;"",$H147=INDEX(Partidos!$K$4:$K$107,MATCH($A147,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H147" s="19">
@@ -16115,7 +16160,7 @@
         <v/>
       </c>
       <c r="G148" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A148,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E148)),NOT(ISNUMBER($F148))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A148,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E148=INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0)),$F148=INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E148-$F148)=(INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E148&gt;$F148,INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),AND($E148=$F148,INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),AND($E148&lt;$F148,INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E148=INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0)),$F148=INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E148-$F148)=(INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H148&lt;&gt;"",$H148=INDEX(Partidos!$K$4:$K$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A148,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E148)),NOT(ISNUMBER($F148))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A148,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E148=INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0)),$F148=INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E148-$F148)=(INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E148&gt;$F148,INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),AND($E148=$F148,INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),AND($E148&lt;$F148,INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0)),IF(AND($E148=INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0)),$F148=INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),IF(AND($H148&lt;&gt;"",$H148=INDEX(Partidos!$K$4:$K$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E148=$F148,($E148-$F148)=(INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0)))),IF(AND($H148&lt;&gt;"",$H148=INDEX(Partidos!$K$4:$K$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H148&lt;&gt;"",$H148=INDEX(Partidos!$K$4:$K$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E148=INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0)),$F148=INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E148-$F148)=(INDEX(Partidos!$F$4:$F$107,MATCH($A148,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H148&lt;&gt;"",$H148=INDEX(Partidos!$K$4:$K$107,MATCH($A148,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H148" s="19">
@@ -16157,7 +16202,7 @@
         <v/>
       </c>
       <c r="G149" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A149,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E149)),NOT(ISNUMBER($F149))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A149,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E149=INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0)),$F149=INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E149-$F149)=(INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E149&gt;$F149,INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),AND($E149=$F149,INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),AND($E149&lt;$F149,INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E149=INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0)),$F149=INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E149-$F149)=(INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H149&lt;&gt;"",$H149=INDEX(Partidos!$K$4:$K$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A149,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E149)),NOT(ISNUMBER($F149))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A149,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E149=INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0)),$F149=INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E149-$F149)=(INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E149&gt;$F149,INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),AND($E149=$F149,INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),AND($E149&lt;$F149,INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0)),IF(AND($E149=INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0)),$F149=INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),IF(AND($H149&lt;&gt;"",$H149=INDEX(Partidos!$K$4:$K$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E149=$F149,($E149-$F149)=(INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0)))),IF(AND($H149&lt;&gt;"",$H149=INDEX(Partidos!$K$4:$K$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H149&lt;&gt;"",$H149=INDEX(Partidos!$K$4:$K$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E149=INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0)),$F149=INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E149-$F149)=(INDEX(Partidos!$F$4:$F$107,MATCH($A149,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H149&lt;&gt;"",$H149=INDEX(Partidos!$K$4:$K$107,MATCH($A149,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H149" s="19">
@@ -16199,7 +16244,7 @@
         <v/>
       </c>
       <c r="G150" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A150,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E150)),NOT(ISNUMBER($F150))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A150,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E150=INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0)),$F150=INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E150-$F150)=(INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E150&gt;$F150,INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),AND($E150=$F150,INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),AND($E150&lt;$F150,INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E150=INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0)),$F150=INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E150-$F150)=(INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H150&lt;&gt;"",$H150=INDEX(Partidos!$K$4:$K$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A150,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E150)),NOT(ISNUMBER($F150))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A150,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E150=INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0)),$F150=INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E150-$F150)=(INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E150&gt;$F150,INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),AND($E150=$F150,INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),AND($E150&lt;$F150,INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0)),IF(AND($E150=INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0)),$F150=INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),IF(AND($H150&lt;&gt;"",$H150=INDEX(Partidos!$K$4:$K$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E150=$F150,($E150-$F150)=(INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0)))),IF(AND($H150&lt;&gt;"",$H150=INDEX(Partidos!$K$4:$K$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H150&lt;&gt;"",$H150=INDEX(Partidos!$K$4:$K$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E150=INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0)),$F150=INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E150-$F150)=(INDEX(Partidos!$F$4:$F$107,MATCH($A150,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H150&lt;&gt;"",$H150=INDEX(Partidos!$K$4:$K$107,MATCH($A150,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H150" s="19">
@@ -16241,7 +16286,7 @@
         <v/>
       </c>
       <c r="G151" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A151,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E151)),NOT(ISNUMBER($F151))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A151,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E151=INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0)),$F151=INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E151-$F151)=(INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E151&gt;$F151,INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),AND($E151=$F151,INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),AND($E151&lt;$F151,INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E151=INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0)),$F151=INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E151-$F151)=(INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H151&lt;&gt;"",$H151=INDEX(Partidos!$K$4:$K$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A151,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E151)),NOT(ISNUMBER($F151))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A151,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E151=INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0)),$F151=INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E151-$F151)=(INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E151&gt;$F151,INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),AND($E151=$F151,INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),AND($E151&lt;$F151,INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0)),IF(AND($E151=INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0)),$F151=INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),IF(AND($H151&lt;&gt;"",$H151=INDEX(Partidos!$K$4:$K$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E151=$F151,($E151-$F151)=(INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0)))),IF(AND($H151&lt;&gt;"",$H151=INDEX(Partidos!$K$4:$K$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H151&lt;&gt;"",$H151=INDEX(Partidos!$K$4:$K$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E151=INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0)),$F151=INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E151-$F151)=(INDEX(Partidos!$F$4:$F$107,MATCH($A151,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H151&lt;&gt;"",$H151=INDEX(Partidos!$K$4:$K$107,MATCH($A151,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H151" s="19">
@@ -16283,7 +16328,7 @@
         <v/>
       </c>
       <c r="G152" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A152,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E152)),NOT(ISNUMBER($F152))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A152,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E152=INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0)),$F152=INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E152-$F152)=(INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E152&gt;$F152,INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),AND($E152=$F152,INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),AND($E152&lt;$F152,INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E152=INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0)),$F152=INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E152-$F152)=(INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H152&lt;&gt;"",$H152=INDEX(Partidos!$K$4:$K$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A152,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E152)),NOT(ISNUMBER($F152))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A152,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E152=INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0)),$F152=INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E152-$F152)=(INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E152&gt;$F152,INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),AND($E152=$F152,INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),AND($E152&lt;$F152,INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0)),IF(AND($E152=INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0)),$F152=INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),IF(AND($H152&lt;&gt;"",$H152=INDEX(Partidos!$K$4:$K$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E152=$F152,($E152-$F152)=(INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0)))),IF(AND($H152&lt;&gt;"",$H152=INDEX(Partidos!$K$4:$K$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H152&lt;&gt;"",$H152=INDEX(Partidos!$K$4:$K$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E152=INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0)),$F152=INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E152-$F152)=(INDEX(Partidos!$F$4:$F$107,MATCH($A152,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H152&lt;&gt;"",$H152=INDEX(Partidos!$K$4:$K$107,MATCH($A152,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H152" s="19">
@@ -16325,7 +16370,7 @@
         <v/>
       </c>
       <c r="G153" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A153,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E153)),NOT(ISNUMBER($F153))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A153,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E153=INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0)),$F153=INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E153-$F153)=(INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E153&gt;$F153,INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),AND($E153=$F153,INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),AND($E153&lt;$F153,INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E153=INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0)),$F153=INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E153-$F153)=(INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H153&lt;&gt;"",$H153=INDEX(Partidos!$K$4:$K$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A153,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E153)),NOT(ISNUMBER($F153))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A153,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E153=INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0)),$F153=INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E153-$F153)=(INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E153&gt;$F153,INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),AND($E153=$F153,INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),AND($E153&lt;$F153,INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0)),IF(AND($E153=INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0)),$F153=INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),IF(AND($H153&lt;&gt;"",$H153=INDEX(Partidos!$K$4:$K$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E153=$F153,($E153-$F153)=(INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0)))),IF(AND($H153&lt;&gt;"",$H153=INDEX(Partidos!$K$4:$K$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H153&lt;&gt;"",$H153=INDEX(Partidos!$K$4:$K$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E153=INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0)),$F153=INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E153-$F153)=(INDEX(Partidos!$F$4:$F$107,MATCH($A153,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H153&lt;&gt;"",$H153=INDEX(Partidos!$K$4:$K$107,MATCH($A153,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H153" s="19">
@@ -16367,7 +16412,7 @@
         <v/>
       </c>
       <c r="G154" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A154,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E154)),NOT(ISNUMBER($F154))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A154,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E154=INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0)),$F154=INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E154-$F154)=(INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E154&gt;$F154,INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),AND($E154=$F154,INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),AND($E154&lt;$F154,INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E154=INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0)),$F154=INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E154-$F154)=(INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H154&lt;&gt;"",$H154=INDEX(Partidos!$K$4:$K$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A154,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E154)),NOT(ISNUMBER($F154))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A154,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E154=INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0)),$F154=INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E154-$F154)=(INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E154&gt;$F154,INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),AND($E154=$F154,INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),AND($E154&lt;$F154,INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0)),IF(AND($E154=INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0)),$F154=INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),IF(AND($H154&lt;&gt;"",$H154=INDEX(Partidos!$K$4:$K$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E154=$F154,($E154-$F154)=(INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0)))),IF(AND($H154&lt;&gt;"",$H154=INDEX(Partidos!$K$4:$K$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H154&lt;&gt;"",$H154=INDEX(Partidos!$K$4:$K$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E154=INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0)),$F154=INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E154-$F154)=(INDEX(Partidos!$F$4:$F$107,MATCH($A154,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H154&lt;&gt;"",$H154=INDEX(Partidos!$K$4:$K$107,MATCH($A154,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H154" s="19">
@@ -16409,7 +16454,7 @@
         <v/>
       </c>
       <c r="G155" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A155,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E155)),NOT(ISNUMBER($F155))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A155,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E155=INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0)),$F155=INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E155-$F155)=(INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E155&gt;$F155,INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),AND($E155=$F155,INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),AND($E155&lt;$F155,INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E155=INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0)),$F155=INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E155-$F155)=(INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H155&lt;&gt;"",$H155=INDEX(Partidos!$K$4:$K$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A155,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E155)),NOT(ISNUMBER($F155))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A155,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E155=INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0)),$F155=INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E155-$F155)=(INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E155&gt;$F155,INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),AND($E155=$F155,INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),AND($E155&lt;$F155,INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0)),IF(AND($E155=INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0)),$F155=INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),IF(AND($H155&lt;&gt;"",$H155=INDEX(Partidos!$K$4:$K$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E155=$F155,($E155-$F155)=(INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0)))),IF(AND($H155&lt;&gt;"",$H155=INDEX(Partidos!$K$4:$K$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H155&lt;&gt;"",$H155=INDEX(Partidos!$K$4:$K$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E155=INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0)),$F155=INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E155-$F155)=(INDEX(Partidos!$F$4:$F$107,MATCH($A155,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H155&lt;&gt;"",$H155=INDEX(Partidos!$K$4:$K$107,MATCH($A155,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H155" s="19">
@@ -16451,7 +16496,7 @@
         <v/>
       </c>
       <c r="G156" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A156,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E156)),NOT(ISNUMBER($F156))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A156,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E156=INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0)),$F156=INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E156-$F156)=(INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E156&gt;$F156,INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),AND($E156=$F156,INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),AND($E156&lt;$F156,INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E156=INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0)),$F156=INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E156-$F156)=(INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H156&lt;&gt;"",$H156=INDEX(Partidos!$K$4:$K$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A156,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E156)),NOT(ISNUMBER($F156))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A156,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E156=INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0)),$F156=INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E156-$F156)=(INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E156&gt;$F156,INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),AND($E156=$F156,INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),AND($E156&lt;$F156,INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0)),IF(AND($E156=INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0)),$F156=INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),IF(AND($H156&lt;&gt;"",$H156=INDEX(Partidos!$K$4:$K$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E156=$F156,($E156-$F156)=(INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0)))),IF(AND($H156&lt;&gt;"",$H156=INDEX(Partidos!$K$4:$K$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H156&lt;&gt;"",$H156=INDEX(Partidos!$K$4:$K$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E156=INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0)),$F156=INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E156-$F156)=(INDEX(Partidos!$F$4:$F$107,MATCH($A156,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H156&lt;&gt;"",$H156=INDEX(Partidos!$K$4:$K$107,MATCH($A156,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H156" s="19">
@@ -16493,7 +16538,7 @@
         <v/>
       </c>
       <c r="G157" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A157,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E157)),NOT(ISNUMBER($F157))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A157,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E157=INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0)),$F157=INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E157-$F157)=(INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E157&gt;$F157,INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),AND($E157=$F157,INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),AND($E157&lt;$F157,INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E157=INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0)),$F157=INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E157-$F157)=(INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H157&lt;&gt;"",$H157=INDEX(Partidos!$K$4:$K$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A157,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E157)),NOT(ISNUMBER($F157))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A157,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E157=INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0)),$F157=INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E157-$F157)=(INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E157&gt;$F157,INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),AND($E157=$F157,INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),AND($E157&lt;$F157,INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0)),IF(AND($E157=INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0)),$F157=INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),IF(AND($H157&lt;&gt;"",$H157=INDEX(Partidos!$K$4:$K$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E157=$F157,($E157-$F157)=(INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0)))),IF(AND($H157&lt;&gt;"",$H157=INDEX(Partidos!$K$4:$K$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H157&lt;&gt;"",$H157=INDEX(Partidos!$K$4:$K$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E157=INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0)),$F157=INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E157-$F157)=(INDEX(Partidos!$F$4:$F$107,MATCH($A157,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H157&lt;&gt;"",$H157=INDEX(Partidos!$K$4:$K$107,MATCH($A157,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H157" s="19">
@@ -16535,7 +16580,7 @@
         <v/>
       </c>
       <c r="G158" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A158,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E158)),NOT(ISNUMBER($F158))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A158,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E158=INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0)),$F158=INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E158-$F158)=(INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E158&gt;$F158,INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),AND($E158=$F158,INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),AND($E158&lt;$F158,INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E158=INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0)),$F158=INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E158-$F158)=(INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H158&lt;&gt;"",$H158=INDEX(Partidos!$K$4:$K$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A158,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E158)),NOT(ISNUMBER($F158))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A158,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E158=INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0)),$F158=INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E158-$F158)=(INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E158&gt;$F158,INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),AND($E158=$F158,INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),AND($E158&lt;$F158,INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0)),IF(AND($E158=INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0)),$F158=INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),IF(AND($H158&lt;&gt;"",$H158=INDEX(Partidos!$K$4:$K$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E158=$F158,($E158-$F158)=(INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0)))),IF(AND($H158&lt;&gt;"",$H158=INDEX(Partidos!$K$4:$K$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H158&lt;&gt;"",$H158=INDEX(Partidos!$K$4:$K$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E158=INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0)),$F158=INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E158-$F158)=(INDEX(Partidos!$F$4:$F$107,MATCH($A158,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H158&lt;&gt;"",$H158=INDEX(Partidos!$K$4:$K$107,MATCH($A158,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H158" s="19">
@@ -16577,7 +16622,7 @@
         <v/>
       </c>
       <c r="G159" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A159,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E159)),NOT(ISNUMBER($F159))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A159,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E159=INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0)),$F159=INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E159-$F159)=(INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E159&gt;$F159,INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),AND($E159=$F159,INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),AND($E159&lt;$F159,INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E159=INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0)),$F159=INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E159-$F159)=(INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H159&lt;&gt;"",$H159=INDEX(Partidos!$K$4:$K$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A159,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E159)),NOT(ISNUMBER($F159))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A159,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E159=INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0)),$F159=INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E159-$F159)=(INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E159&gt;$F159,INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),AND($E159=$F159,INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),AND($E159&lt;$F159,INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0)),IF(AND($E159=INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0)),$F159=INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),IF(AND($H159&lt;&gt;"",$H159=INDEX(Partidos!$K$4:$K$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E159=$F159,($E159-$F159)=(INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0)))),IF(AND($H159&lt;&gt;"",$H159=INDEX(Partidos!$K$4:$K$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H159&lt;&gt;"",$H159=INDEX(Partidos!$K$4:$K$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E159=INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0)),$F159=INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E159-$F159)=(INDEX(Partidos!$F$4:$F$107,MATCH($A159,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H159&lt;&gt;"",$H159=INDEX(Partidos!$K$4:$K$107,MATCH($A159,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H159" s="19">
@@ -16619,7 +16664,7 @@
         <v/>
       </c>
       <c r="G160" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A160,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E160)),NOT(ISNUMBER($F160))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A160,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E160=INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0)),$F160=INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E160-$F160)=(INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E160&gt;$F160,INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),AND($E160=$F160,INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),AND($E160&lt;$F160,INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E160=INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0)),$F160=INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E160-$F160)=(INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H160&lt;&gt;"",$H160=INDEX(Partidos!$K$4:$K$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A160,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E160)),NOT(ISNUMBER($F160))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A160,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E160=INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0)),$F160=INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E160-$F160)=(INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E160&gt;$F160,INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),AND($E160=$F160,INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),AND($E160&lt;$F160,INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0)),IF(AND($E160=INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0)),$F160=INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),IF(AND($H160&lt;&gt;"",$H160=INDEX(Partidos!$K$4:$K$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E160=$F160,($E160-$F160)=(INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0)))),IF(AND($H160&lt;&gt;"",$H160=INDEX(Partidos!$K$4:$K$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H160&lt;&gt;"",$H160=INDEX(Partidos!$K$4:$K$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E160=INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0)),$F160=INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E160-$F160)=(INDEX(Partidos!$F$4:$F$107,MATCH($A160,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H160&lt;&gt;"",$H160=INDEX(Partidos!$K$4:$K$107,MATCH($A160,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H160" s="19">
@@ -16661,7 +16706,7 @@
         <v/>
       </c>
       <c r="G161" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A161,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E161)),NOT(ISNUMBER($F161))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A161,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E161=INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0)),$F161=INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E161-$F161)=(INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E161&gt;$F161,INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),AND($E161=$F161,INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),AND($E161&lt;$F161,INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E161=INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0)),$F161=INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E161-$F161)=(INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H161&lt;&gt;"",$H161=INDEX(Partidos!$K$4:$K$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A161,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E161)),NOT(ISNUMBER($F161))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A161,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E161=INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0)),$F161=INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E161-$F161)=(INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E161&gt;$F161,INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),AND($E161=$F161,INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),AND($E161&lt;$F161,INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0)),IF(AND($E161=INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0)),$F161=INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),IF(AND($H161&lt;&gt;"",$H161=INDEX(Partidos!$K$4:$K$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E161=$F161,($E161-$F161)=(INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0)))),IF(AND($H161&lt;&gt;"",$H161=INDEX(Partidos!$K$4:$K$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H161&lt;&gt;"",$H161=INDEX(Partidos!$K$4:$K$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E161=INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0)),$F161=INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E161-$F161)=(INDEX(Partidos!$F$4:$F$107,MATCH($A161,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H161&lt;&gt;"",$H161=INDEX(Partidos!$K$4:$K$107,MATCH($A161,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H161" s="19">
@@ -16703,7 +16748,7 @@
         <v/>
       </c>
       <c r="G162" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A162,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E162)),NOT(ISNUMBER($F162))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A162,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E162=INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0)),$F162=INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E162-$F162)=(INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E162&gt;$F162,INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),AND($E162=$F162,INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),AND($E162&lt;$F162,INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E162=INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0)),$F162=INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E162-$F162)=(INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H162&lt;&gt;"",$H162=INDEX(Partidos!$K$4:$K$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A162,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E162)),NOT(ISNUMBER($F162))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A162,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E162=INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0)),$F162=INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E162-$F162)=(INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E162&gt;$F162,INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),AND($E162=$F162,INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),AND($E162&lt;$F162,INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0)),IF(AND($E162=INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0)),$F162=INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),IF(AND($H162&lt;&gt;"",$H162=INDEX(Partidos!$K$4:$K$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E162=$F162,($E162-$F162)=(INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0)))),IF(AND($H162&lt;&gt;"",$H162=INDEX(Partidos!$K$4:$K$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H162&lt;&gt;"",$H162=INDEX(Partidos!$K$4:$K$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E162=INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0)),$F162=INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E162-$F162)=(INDEX(Partidos!$F$4:$F$107,MATCH($A162,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H162&lt;&gt;"",$H162=INDEX(Partidos!$K$4:$K$107,MATCH($A162,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H162" s="19">
@@ -16745,7 +16790,7 @@
         <v/>
       </c>
       <c r="G163" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A163,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E163)),NOT(ISNUMBER($F163))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A163,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E163=INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0)),$F163=INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E163-$F163)=(INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E163&gt;$F163,INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),AND($E163=$F163,INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),AND($E163&lt;$F163,INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E163=INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0)),$F163=INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E163-$F163)=(INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H163&lt;&gt;"",$H163=INDEX(Partidos!$K$4:$K$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A163,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E163)),NOT(ISNUMBER($F163))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A163,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E163=INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0)),$F163=INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E163-$F163)=(INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E163&gt;$F163,INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),AND($E163=$F163,INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),AND($E163&lt;$F163,INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0)),IF(AND($E163=INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0)),$F163=INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),IF(AND($H163&lt;&gt;"",$H163=INDEX(Partidos!$K$4:$K$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E163=$F163,($E163-$F163)=(INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0)))),IF(AND($H163&lt;&gt;"",$H163=INDEX(Partidos!$K$4:$K$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H163&lt;&gt;"",$H163=INDEX(Partidos!$K$4:$K$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E163=INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0)),$F163=INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E163-$F163)=(INDEX(Partidos!$F$4:$F$107,MATCH($A163,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H163&lt;&gt;"",$H163=INDEX(Partidos!$K$4:$K$107,MATCH($A163,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H163" s="19">
@@ -16787,7 +16832,7 @@
         <v/>
       </c>
       <c r="G164" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A164,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E164)),NOT(ISNUMBER($F164))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A164,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E164=INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0)),$F164=INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E164-$F164)=(INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E164&gt;$F164,INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),AND($E164=$F164,INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),AND($E164&lt;$F164,INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E164=INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0)),$F164=INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E164-$F164)=(INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H164&lt;&gt;"",$H164=INDEX(Partidos!$K$4:$K$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A164,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E164)),NOT(ISNUMBER($F164))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A164,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E164=INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0)),$F164=INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E164-$F164)=(INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E164&gt;$F164,INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),AND($E164=$F164,INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),AND($E164&lt;$F164,INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0)),IF(AND($E164=INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0)),$F164=INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),IF(AND($H164&lt;&gt;"",$H164=INDEX(Partidos!$K$4:$K$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E164=$F164,($E164-$F164)=(INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0)))),IF(AND($H164&lt;&gt;"",$H164=INDEX(Partidos!$K$4:$K$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H164&lt;&gt;"",$H164=INDEX(Partidos!$K$4:$K$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E164=INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0)),$F164=INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E164-$F164)=(INDEX(Partidos!$F$4:$F$107,MATCH($A164,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H164&lt;&gt;"",$H164=INDEX(Partidos!$K$4:$K$107,MATCH($A164,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H164" s="19">
@@ -16829,7 +16874,7 @@
         <v/>
       </c>
       <c r="G165" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A165,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E165)),NOT(ISNUMBER($F165))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A165,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E165=INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0)),$F165=INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E165-$F165)=(INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E165&gt;$F165,INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),AND($E165=$F165,INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),AND($E165&lt;$F165,INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E165=INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0)),$F165=INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E165-$F165)=(INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H165&lt;&gt;"",$H165=INDEX(Partidos!$K$4:$K$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A165,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E165)),NOT(ISNUMBER($F165))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A165,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E165=INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0)),$F165=INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E165-$F165)=(INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E165&gt;$F165,INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),AND($E165=$F165,INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),AND($E165&lt;$F165,INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0)),IF(AND($E165=INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0)),$F165=INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),IF(AND($H165&lt;&gt;"",$H165=INDEX(Partidos!$K$4:$K$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E165=$F165,($E165-$F165)=(INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0)))),IF(AND($H165&lt;&gt;"",$H165=INDEX(Partidos!$K$4:$K$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H165&lt;&gt;"",$H165=INDEX(Partidos!$K$4:$K$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E165=INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0)),$F165=INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E165-$F165)=(INDEX(Partidos!$F$4:$F$107,MATCH($A165,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H165&lt;&gt;"",$H165=INDEX(Partidos!$K$4:$K$107,MATCH($A165,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H165" s="19">
@@ -16871,7 +16916,7 @@
         <v/>
       </c>
       <c r="G166" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A166,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E166)),NOT(ISNUMBER($F166))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A166,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E166=INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0)),$F166=INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E166-$F166)=(INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E166&gt;$F166,INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),AND($E166=$F166,INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),AND($E166&lt;$F166,INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E166=INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0)),$F166=INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E166-$F166)=(INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H166&lt;&gt;"",$H166=INDEX(Partidos!$K$4:$K$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A166,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E166)),NOT(ISNUMBER($F166))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A166,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E166=INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0)),$F166=INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E166-$F166)=(INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E166&gt;$F166,INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),AND($E166=$F166,INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),AND($E166&lt;$F166,INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0)),IF(AND($E166=INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0)),$F166=INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),IF(AND($H166&lt;&gt;"",$H166=INDEX(Partidos!$K$4:$K$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E166=$F166,($E166-$F166)=(INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0)))),IF(AND($H166&lt;&gt;"",$H166=INDEX(Partidos!$K$4:$K$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H166&lt;&gt;"",$H166=INDEX(Partidos!$K$4:$K$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E166=INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0)),$F166=INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E166-$F166)=(INDEX(Partidos!$F$4:$F$107,MATCH($A166,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H166&lt;&gt;"",$H166=INDEX(Partidos!$K$4:$K$107,MATCH($A166,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H166" s="19">
@@ -16913,7 +16958,7 @@
         <v/>
       </c>
       <c r="G167" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A167,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E167)),NOT(ISNUMBER($F167))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A167,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E167=INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0)),$F167=INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E167-$F167)=(INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E167&gt;$F167,INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),AND($E167=$F167,INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),AND($E167&lt;$F167,INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E167=INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0)),$F167=INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E167-$F167)=(INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H167&lt;&gt;"",$H167=INDEX(Partidos!$K$4:$K$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A167,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E167)),NOT(ISNUMBER($F167))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A167,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E167=INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0)),$F167=INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E167-$F167)=(INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E167&gt;$F167,INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),AND($E167=$F167,INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),AND($E167&lt;$F167,INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0)),IF(AND($E167=INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0)),$F167=INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),IF(AND($H167&lt;&gt;"",$H167=INDEX(Partidos!$K$4:$K$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E167=$F167,($E167-$F167)=(INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0)))),IF(AND($H167&lt;&gt;"",$H167=INDEX(Partidos!$K$4:$K$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H167&lt;&gt;"",$H167=INDEX(Partidos!$K$4:$K$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E167=INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0)),$F167=INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E167-$F167)=(INDEX(Partidos!$F$4:$F$107,MATCH($A167,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H167&lt;&gt;"",$H167=INDEX(Partidos!$K$4:$K$107,MATCH($A167,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H167" s="19">
@@ -16955,7 +17000,7 @@
         <v/>
       </c>
       <c r="G168" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A168,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E168)),NOT(ISNUMBER($F168))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A168,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E168=INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0)),$F168=INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E168-$F168)=(INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E168&gt;$F168,INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),AND($E168=$F168,INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),AND($E168&lt;$F168,INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E168=INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0)),$F168=INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E168-$F168)=(INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H168&lt;&gt;"",$H168=INDEX(Partidos!$K$4:$K$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A168,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E168)),NOT(ISNUMBER($F168))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A168,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E168=INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0)),$F168=INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E168-$F168)=(INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E168&gt;$F168,INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),AND($E168=$F168,INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),AND($E168&lt;$F168,INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0)),IF(AND($E168=INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0)),$F168=INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),IF(AND($H168&lt;&gt;"",$H168=INDEX(Partidos!$K$4:$K$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E168=$F168,($E168-$F168)=(INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0)))),IF(AND($H168&lt;&gt;"",$H168=INDEX(Partidos!$K$4:$K$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H168&lt;&gt;"",$H168=INDEX(Partidos!$K$4:$K$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E168=INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0)),$F168=INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E168-$F168)=(INDEX(Partidos!$F$4:$F$107,MATCH($A168,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H168&lt;&gt;"",$H168=INDEX(Partidos!$K$4:$K$107,MATCH($A168,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H168" s="19">
@@ -16997,7 +17042,7 @@
         <v/>
       </c>
       <c r="G169" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A169,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E169)),NOT(ISNUMBER($F169))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A169,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E169=INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0)),$F169=INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E169-$F169)=(INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E169&gt;$F169,INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),AND($E169=$F169,INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),AND($E169&lt;$F169,INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E169=INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0)),$F169=INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E169-$F169)=(INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H169&lt;&gt;"",$H169=INDEX(Partidos!$K$4:$K$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A169,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E169)),NOT(ISNUMBER($F169))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A169,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E169=INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0)),$F169=INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E169-$F169)=(INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E169&gt;$F169,INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),AND($E169=$F169,INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),AND($E169&lt;$F169,INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0)),IF(AND($E169=INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0)),$F169=INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),IF(AND($H169&lt;&gt;"",$H169=INDEX(Partidos!$K$4:$K$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E169=$F169,($E169-$F169)=(INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0)))),IF(AND($H169&lt;&gt;"",$H169=INDEX(Partidos!$K$4:$K$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H169&lt;&gt;"",$H169=INDEX(Partidos!$K$4:$K$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E169=INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0)),$F169=INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E169-$F169)=(INDEX(Partidos!$F$4:$F$107,MATCH($A169,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H169&lt;&gt;"",$H169=INDEX(Partidos!$K$4:$K$107,MATCH($A169,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H169" s="19">
@@ -17039,7 +17084,7 @@
         <v/>
       </c>
       <c r="G170" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A170,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E170)),NOT(ISNUMBER($F170))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A170,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E170=INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0)),$F170=INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E170-$F170)=(INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E170&gt;$F170,INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),AND($E170=$F170,INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),AND($E170&lt;$F170,INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E170=INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0)),$F170=INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E170-$F170)=(INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H170&lt;&gt;"",$H170=INDEX(Partidos!$K$4:$K$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A170,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E170)),NOT(ISNUMBER($F170))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A170,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E170=INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0)),$F170=INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E170-$F170)=(INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E170&gt;$F170,INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),AND($E170=$F170,INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),AND($E170&lt;$F170,INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0)),IF(AND($E170=INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0)),$F170=INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),IF(AND($H170&lt;&gt;"",$H170=INDEX(Partidos!$K$4:$K$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E170=$F170,($E170-$F170)=(INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0)))),IF(AND($H170&lt;&gt;"",$H170=INDEX(Partidos!$K$4:$K$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H170&lt;&gt;"",$H170=INDEX(Partidos!$K$4:$K$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E170=INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0)),$F170=INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E170-$F170)=(INDEX(Partidos!$F$4:$F$107,MATCH($A170,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H170&lt;&gt;"",$H170=INDEX(Partidos!$K$4:$K$107,MATCH($A170,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H170" s="19">
@@ -17081,7 +17126,7 @@
         <v/>
       </c>
       <c r="G171" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A171,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E171)),NOT(ISNUMBER($F171))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A171,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E171=INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0)),$F171=INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E171-$F171)=(INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E171&gt;$F171,INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),AND($E171=$F171,INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),AND($E171&lt;$F171,INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E171=INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0)),$F171=INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E171-$F171)=(INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H171&lt;&gt;"",$H171=INDEX(Partidos!$K$4:$K$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A171,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E171)),NOT(ISNUMBER($F171))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A171,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E171=INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0)),$F171=INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E171-$F171)=(INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E171&gt;$F171,INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),AND($E171=$F171,INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),AND($E171&lt;$F171,INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0)),IF(AND($E171=INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0)),$F171=INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),IF(AND($H171&lt;&gt;"",$H171=INDEX(Partidos!$K$4:$K$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E171=$F171,($E171-$F171)=(INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0)))),IF(AND($H171&lt;&gt;"",$H171=INDEX(Partidos!$K$4:$K$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H171&lt;&gt;"",$H171=INDEX(Partidos!$K$4:$K$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E171=INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0)),$F171=INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E171-$F171)=(INDEX(Partidos!$F$4:$F$107,MATCH($A171,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H171&lt;&gt;"",$H171=INDEX(Partidos!$K$4:$K$107,MATCH($A171,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H171" s="19">
@@ -17123,7 +17168,7 @@
         <v/>
       </c>
       <c r="G172" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A172,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E172)),NOT(ISNUMBER($F172))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A172,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E172=INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0)),$F172=INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E172-$F172)=(INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E172&gt;$F172,INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),AND($E172=$F172,INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),AND($E172&lt;$F172,INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E172=INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0)),$F172=INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E172-$F172)=(INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H172&lt;&gt;"",$H172=INDEX(Partidos!$K$4:$K$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A172,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E172)),NOT(ISNUMBER($F172))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A172,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E172=INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0)),$F172=INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E172-$F172)=(INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E172&gt;$F172,INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),AND($E172=$F172,INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),AND($E172&lt;$F172,INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0)),IF(AND($E172=INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0)),$F172=INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),IF(AND($H172&lt;&gt;"",$H172=INDEX(Partidos!$K$4:$K$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E172=$F172,($E172-$F172)=(INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0)))),IF(AND($H172&lt;&gt;"",$H172=INDEX(Partidos!$K$4:$K$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H172&lt;&gt;"",$H172=INDEX(Partidos!$K$4:$K$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E172=INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0)),$F172=INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E172-$F172)=(INDEX(Partidos!$F$4:$F$107,MATCH($A172,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H172&lt;&gt;"",$H172=INDEX(Partidos!$K$4:$K$107,MATCH($A172,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H172" s="19">
@@ -17165,7 +17210,7 @@
         <v/>
       </c>
       <c r="G173" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A173,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E173)),NOT(ISNUMBER($F173))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A173,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E173=INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0)),$F173=INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E173-$F173)=(INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E173&gt;$F173,INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),AND($E173=$F173,INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),AND($E173&lt;$F173,INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E173=INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0)),$F173=INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E173-$F173)=(INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H173&lt;&gt;"",$H173=INDEX(Partidos!$K$4:$K$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A173,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E173)),NOT(ISNUMBER($F173))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A173,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E173=INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0)),$F173=INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E173-$F173)=(INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E173&gt;$F173,INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),AND($E173=$F173,INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),AND($E173&lt;$F173,INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0)),IF(AND($E173=INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0)),$F173=INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),IF(AND($H173&lt;&gt;"",$H173=INDEX(Partidos!$K$4:$K$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E173=$F173,($E173-$F173)=(INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0)))),IF(AND($H173&lt;&gt;"",$H173=INDEX(Partidos!$K$4:$K$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H173&lt;&gt;"",$H173=INDEX(Partidos!$K$4:$K$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E173=INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0)),$F173=INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E173-$F173)=(INDEX(Partidos!$F$4:$F$107,MATCH($A173,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H173&lt;&gt;"",$H173=INDEX(Partidos!$K$4:$K$107,MATCH($A173,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H173" s="19">
@@ -17207,7 +17252,7 @@
         <v/>
       </c>
       <c r="G174" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A174,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E174)),NOT(ISNUMBER($F174))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A174,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E174=INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0)),$F174=INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E174-$F174)=(INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E174&gt;$F174,INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),AND($E174=$F174,INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),AND($E174&lt;$F174,INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E174=INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0)),$F174=INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E174-$F174)=(INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H174&lt;&gt;"",$H174=INDEX(Partidos!$K$4:$K$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A174,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E174)),NOT(ISNUMBER($F174))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A174,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E174=INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0)),$F174=INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E174-$F174)=(INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E174&gt;$F174,INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),AND($E174=$F174,INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),AND($E174&lt;$F174,INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0)),IF(AND($E174=INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0)),$F174=INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),IF(AND($H174&lt;&gt;"",$H174=INDEX(Partidos!$K$4:$K$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E174=$F174,($E174-$F174)=(INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0)))),IF(AND($H174&lt;&gt;"",$H174=INDEX(Partidos!$K$4:$K$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H174&lt;&gt;"",$H174=INDEX(Partidos!$K$4:$K$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E174=INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0)),$F174=INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E174-$F174)=(INDEX(Partidos!$F$4:$F$107,MATCH($A174,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H174&lt;&gt;"",$H174=INDEX(Partidos!$K$4:$K$107,MATCH($A174,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H174" s="19">
@@ -17249,7 +17294,7 @@
         <v/>
       </c>
       <c r="G175" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A175,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E175)),NOT(ISNUMBER($F175))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A175,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E175=INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0)),$F175=INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E175-$F175)=(INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E175&gt;$F175,INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),AND($E175=$F175,INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),AND($E175&lt;$F175,INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E175=INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0)),$F175=INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E175-$F175)=(INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H175&lt;&gt;"",$H175=INDEX(Partidos!$K$4:$K$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A175,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E175)),NOT(ISNUMBER($F175))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A175,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E175=INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0)),$F175=INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E175-$F175)=(INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E175&gt;$F175,INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),AND($E175=$F175,INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),AND($E175&lt;$F175,INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0)),IF(AND($E175=INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0)),$F175=INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),IF(AND($H175&lt;&gt;"",$H175=INDEX(Partidos!$K$4:$K$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E175=$F175,($E175-$F175)=(INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0)))),IF(AND($H175&lt;&gt;"",$H175=INDEX(Partidos!$K$4:$K$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H175&lt;&gt;"",$H175=INDEX(Partidos!$K$4:$K$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E175=INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0)),$F175=INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E175-$F175)=(INDEX(Partidos!$F$4:$F$107,MATCH($A175,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H175&lt;&gt;"",$H175=INDEX(Partidos!$K$4:$K$107,MATCH($A175,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H175" s="19">
@@ -17291,7 +17336,7 @@
         <v/>
       </c>
       <c r="G176" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A176,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E176)),NOT(ISNUMBER($F176))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A176,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E176=INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0)),$F176=INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E176-$F176)=(INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E176&gt;$F176,INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),AND($E176=$F176,INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),AND($E176&lt;$F176,INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E176=INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0)),$F176=INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E176-$F176)=(INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H176&lt;&gt;"",$H176=INDEX(Partidos!$K$4:$K$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A176,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E176)),NOT(ISNUMBER($F176))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A176,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E176=INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0)),$F176=INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E176-$F176)=(INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E176&gt;$F176,INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),AND($E176=$F176,INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),AND($E176&lt;$F176,INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0)),IF(AND($E176=INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0)),$F176=INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),IF(AND($H176&lt;&gt;"",$H176=INDEX(Partidos!$K$4:$K$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E176=$F176,($E176-$F176)=(INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0)))),IF(AND($H176&lt;&gt;"",$H176=INDEX(Partidos!$K$4:$K$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H176&lt;&gt;"",$H176=INDEX(Partidos!$K$4:$K$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E176=INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0)),$F176=INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E176-$F176)=(INDEX(Partidos!$F$4:$F$107,MATCH($A176,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H176&lt;&gt;"",$H176=INDEX(Partidos!$K$4:$K$107,MATCH($A176,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H176" s="19">
@@ -17333,7 +17378,7 @@
         <v/>
       </c>
       <c r="G177" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A177,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E177)),NOT(ISNUMBER($F177))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A177,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E177=INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0)),$F177=INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E177-$F177)=(INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E177&gt;$F177,INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),AND($E177=$F177,INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),AND($E177&lt;$F177,INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E177=INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0)),$F177=INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E177-$F177)=(INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H177&lt;&gt;"",$H177=INDEX(Partidos!$K$4:$K$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A177,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E177)),NOT(ISNUMBER($F177))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A177,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E177=INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0)),$F177=INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E177-$F177)=(INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E177&gt;$F177,INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),AND($E177=$F177,INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),AND($E177&lt;$F177,INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0)),IF(AND($E177=INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0)),$F177=INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),IF(AND($H177&lt;&gt;"",$H177=INDEX(Partidos!$K$4:$K$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E177=$F177,($E177-$F177)=(INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0)))),IF(AND($H177&lt;&gt;"",$H177=INDEX(Partidos!$K$4:$K$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H177&lt;&gt;"",$H177=INDEX(Partidos!$K$4:$K$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E177=INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0)),$F177=INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E177-$F177)=(INDEX(Partidos!$F$4:$F$107,MATCH($A177,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H177&lt;&gt;"",$H177=INDEX(Partidos!$K$4:$K$107,MATCH($A177,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H177" s="19">
@@ -17375,7 +17420,7 @@
         <v/>
       </c>
       <c r="G178" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A178,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E178)),NOT(ISNUMBER($F178))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A178,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E178=INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0)),$F178=INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E178-$F178)=(INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E178&gt;$F178,INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),AND($E178=$F178,INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),AND($E178&lt;$F178,INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E178=INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0)),$F178=INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E178-$F178)=(INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H178&lt;&gt;"",$H178=INDEX(Partidos!$K$4:$K$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A178,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E178)),NOT(ISNUMBER($F178))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A178,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E178=INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0)),$F178=INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E178-$F178)=(INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E178&gt;$F178,INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),AND($E178=$F178,INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),AND($E178&lt;$F178,INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0)),IF(AND($E178=INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0)),$F178=INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),IF(AND($H178&lt;&gt;"",$H178=INDEX(Partidos!$K$4:$K$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E178=$F178,($E178-$F178)=(INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0)))),IF(AND($H178&lt;&gt;"",$H178=INDEX(Partidos!$K$4:$K$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H178&lt;&gt;"",$H178=INDEX(Partidos!$K$4:$K$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E178=INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0)),$F178=INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E178-$F178)=(INDEX(Partidos!$F$4:$F$107,MATCH($A178,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H178&lt;&gt;"",$H178=INDEX(Partidos!$K$4:$K$107,MATCH($A178,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H178" s="19">
@@ -17417,7 +17462,7 @@
         <v/>
       </c>
       <c r="G179" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A179,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E179)),NOT(ISNUMBER($F179))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A179,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E179=INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0)),$F179=INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E179-$F179)=(INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E179&gt;$F179,INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),AND($E179=$F179,INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),AND($E179&lt;$F179,INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E179=INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0)),$F179=INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E179-$F179)=(INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H179&lt;&gt;"",$H179=INDEX(Partidos!$K$4:$K$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A179,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E179)),NOT(ISNUMBER($F179))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A179,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E179=INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0)),$F179=INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E179-$F179)=(INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E179&gt;$F179,INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),AND($E179=$F179,INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),AND($E179&lt;$F179,INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0)),IF(AND($E179=INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0)),$F179=INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),IF(AND($H179&lt;&gt;"",$H179=INDEX(Partidos!$K$4:$K$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E179=$F179,($E179-$F179)=(INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0)))),IF(AND($H179&lt;&gt;"",$H179=INDEX(Partidos!$K$4:$K$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H179&lt;&gt;"",$H179=INDEX(Partidos!$K$4:$K$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E179=INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0)),$F179=INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E179-$F179)=(INDEX(Partidos!$F$4:$F$107,MATCH($A179,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H179&lt;&gt;"",$H179=INDEX(Partidos!$K$4:$K$107,MATCH($A179,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H179" s="19">
@@ -17459,7 +17504,7 @@
         <v/>
       </c>
       <c r="G180" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A180,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E180)),NOT(ISNUMBER($F180))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A180,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E180=INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0)),$F180=INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E180-$F180)=(INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E180&gt;$F180,INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),AND($E180=$F180,INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),AND($E180&lt;$F180,INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E180=INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0)),$F180=INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E180-$F180)=(INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H180&lt;&gt;"",$H180=INDEX(Partidos!$K$4:$K$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A180,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E180)),NOT(ISNUMBER($F180))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A180,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E180=INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0)),$F180=INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E180-$F180)=(INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E180&gt;$F180,INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),AND($E180=$F180,INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),AND($E180&lt;$F180,INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0)),IF(AND($E180=INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0)),$F180=INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),IF(AND($H180&lt;&gt;"",$H180=INDEX(Partidos!$K$4:$K$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E180=$F180,($E180-$F180)=(INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0)))),IF(AND($H180&lt;&gt;"",$H180=INDEX(Partidos!$K$4:$K$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H180&lt;&gt;"",$H180=INDEX(Partidos!$K$4:$K$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E180=INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0)),$F180=INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E180-$F180)=(INDEX(Partidos!$F$4:$F$107,MATCH($A180,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H180&lt;&gt;"",$H180=INDEX(Partidos!$K$4:$K$107,MATCH($A180,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H180" s="19">
@@ -17501,7 +17546,7 @@
         <v/>
       </c>
       <c r="G181" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A181,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E181)),NOT(ISNUMBER($F181))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A181,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E181=INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0)),$F181=INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E181-$F181)=(INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E181&gt;$F181,INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),AND($E181=$F181,INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),AND($E181&lt;$F181,INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E181=INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0)),$F181=INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E181-$F181)=(INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H181&lt;&gt;"",$H181=INDEX(Partidos!$K$4:$K$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A181,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E181)),NOT(ISNUMBER($F181))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A181,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E181=INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0)),$F181=INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E181-$F181)=(INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E181&gt;$F181,INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),AND($E181=$F181,INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),AND($E181&lt;$F181,INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0)),IF(AND($E181=INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0)),$F181=INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),IF(AND($H181&lt;&gt;"",$H181=INDEX(Partidos!$K$4:$K$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E181=$F181,($E181-$F181)=(INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0)))),IF(AND($H181&lt;&gt;"",$H181=INDEX(Partidos!$K$4:$K$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H181&lt;&gt;"",$H181=INDEX(Partidos!$K$4:$K$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E181=INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0)),$F181=INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E181-$F181)=(INDEX(Partidos!$F$4:$F$107,MATCH($A181,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H181&lt;&gt;"",$H181=INDEX(Partidos!$K$4:$K$107,MATCH($A181,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H181" s="19">
@@ -17543,7 +17588,7 @@
         <v/>
       </c>
       <c r="G182" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A182,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E182)),NOT(ISNUMBER($F182))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A182,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E182=INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0)),$F182=INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E182-$F182)=(INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E182&gt;$F182,INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),AND($E182=$F182,INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),AND($E182&lt;$F182,INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E182=INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0)),$F182=INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E182-$F182)=(INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H182&lt;&gt;"",$H182=INDEX(Partidos!$K$4:$K$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A182,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E182)),NOT(ISNUMBER($F182))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A182,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E182=INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0)),$F182=INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E182-$F182)=(INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E182&gt;$F182,INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),AND($E182=$F182,INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),AND($E182&lt;$F182,INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0)),IF(AND($E182=INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0)),$F182=INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),IF(AND($H182&lt;&gt;"",$H182=INDEX(Partidos!$K$4:$K$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E182=$F182,($E182-$F182)=(INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0)))),IF(AND($H182&lt;&gt;"",$H182=INDEX(Partidos!$K$4:$K$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H182&lt;&gt;"",$H182=INDEX(Partidos!$K$4:$K$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E182=INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0)),$F182=INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E182-$F182)=(INDEX(Partidos!$F$4:$F$107,MATCH($A182,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H182&lt;&gt;"",$H182=INDEX(Partidos!$K$4:$K$107,MATCH($A182,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H182" s="19">
@@ -17585,7 +17630,7 @@
         <v/>
       </c>
       <c r="G183" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A183,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E183)),NOT(ISNUMBER($F183))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A183,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E183=INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0)),$F183=INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E183-$F183)=(INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E183&gt;$F183,INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),AND($E183=$F183,INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),AND($E183&lt;$F183,INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E183=INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0)),$F183=INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E183-$F183)=(INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H183&lt;&gt;"",$H183=INDEX(Partidos!$K$4:$K$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A183,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E183)),NOT(ISNUMBER($F183))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A183,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E183=INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0)),$F183=INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E183-$F183)=(INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E183&gt;$F183,INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),AND($E183=$F183,INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),AND($E183&lt;$F183,INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0)),IF(AND($E183=INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0)),$F183=INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),IF(AND($H183&lt;&gt;"",$H183=INDEX(Partidos!$K$4:$K$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E183=$F183,($E183-$F183)=(INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0)))),IF(AND($H183&lt;&gt;"",$H183=INDEX(Partidos!$K$4:$K$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H183&lt;&gt;"",$H183=INDEX(Partidos!$K$4:$K$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E183=INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0)),$F183=INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E183-$F183)=(INDEX(Partidos!$F$4:$F$107,MATCH($A183,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H183&lt;&gt;"",$H183=INDEX(Partidos!$K$4:$K$107,MATCH($A183,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H183" s="19">
@@ -17627,7 +17672,7 @@
         <v/>
       </c>
       <c r="G184" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A184,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E184)),NOT(ISNUMBER($F184))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A184,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E184=INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0)),$F184=INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E184-$F184)=(INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E184&gt;$F184,INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),AND($E184=$F184,INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),AND($E184&lt;$F184,INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E184=INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0)),$F184=INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E184-$F184)=(INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H184&lt;&gt;"",$H184=INDEX(Partidos!$K$4:$K$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A184,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E184)),NOT(ISNUMBER($F184))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A184,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E184=INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0)),$F184=INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E184-$F184)=(INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E184&gt;$F184,INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),AND($E184=$F184,INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),AND($E184&lt;$F184,INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0)),IF(AND($E184=INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0)),$F184=INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),IF(AND($H184&lt;&gt;"",$H184=INDEX(Partidos!$K$4:$K$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E184=$F184,($E184-$F184)=(INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0)))),IF(AND($H184&lt;&gt;"",$H184=INDEX(Partidos!$K$4:$K$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H184&lt;&gt;"",$H184=INDEX(Partidos!$K$4:$K$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E184=INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0)),$F184=INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E184-$F184)=(INDEX(Partidos!$F$4:$F$107,MATCH($A184,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H184&lt;&gt;"",$H184=INDEX(Partidos!$K$4:$K$107,MATCH($A184,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H184" s="19">
@@ -17669,7 +17714,7 @@
         <v/>
       </c>
       <c r="G185" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A185,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E185)),NOT(ISNUMBER($F185))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A185,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E185=INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0)),$F185=INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E185-$F185)=(INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E185&gt;$F185,INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),AND($E185=$F185,INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),AND($E185&lt;$F185,INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E185=INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0)),$F185=INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E185-$F185)=(INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H185&lt;&gt;"",$H185=INDEX(Partidos!$K$4:$K$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A185,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E185)),NOT(ISNUMBER($F185))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A185,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E185=INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0)),$F185=INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E185-$F185)=(INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E185&gt;$F185,INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),AND($E185=$F185,INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),AND($E185&lt;$F185,INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0)),IF(AND($E185=INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0)),$F185=INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),IF(AND($H185&lt;&gt;"",$H185=INDEX(Partidos!$K$4:$K$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E185=$F185,($E185-$F185)=(INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0)))),IF(AND($H185&lt;&gt;"",$H185=INDEX(Partidos!$K$4:$K$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H185&lt;&gt;"",$H185=INDEX(Partidos!$K$4:$K$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E185=INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0)),$F185=INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E185-$F185)=(INDEX(Partidos!$F$4:$F$107,MATCH($A185,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H185&lt;&gt;"",$H185=INDEX(Partidos!$K$4:$K$107,MATCH($A185,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H185" s="19">
@@ -17711,7 +17756,7 @@
         <v/>
       </c>
       <c r="G186" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A186,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E186)),NOT(ISNUMBER($F186))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A186,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E186=INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0)),$F186=INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E186-$F186)=(INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E186&gt;$F186,INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),AND($E186=$F186,INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),AND($E186&lt;$F186,INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E186=INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0)),$F186=INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E186-$F186)=(INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H186&lt;&gt;"",$H186=INDEX(Partidos!$K$4:$K$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A186,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E186)),NOT(ISNUMBER($F186))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A186,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E186=INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0)),$F186=INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E186-$F186)=(INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E186&gt;$F186,INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),AND($E186=$F186,INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),AND($E186&lt;$F186,INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0)),IF(AND($E186=INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0)),$F186=INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),IF(AND($H186&lt;&gt;"",$H186=INDEX(Partidos!$K$4:$K$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E186=$F186,($E186-$F186)=(INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0)))),IF(AND($H186&lt;&gt;"",$H186=INDEX(Partidos!$K$4:$K$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H186&lt;&gt;"",$H186=INDEX(Partidos!$K$4:$K$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E186=INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0)),$F186=INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E186-$F186)=(INDEX(Partidos!$F$4:$F$107,MATCH($A186,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H186&lt;&gt;"",$H186=INDEX(Partidos!$K$4:$K$107,MATCH($A186,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H186" s="19">
@@ -17753,7 +17798,7 @@
         <v/>
       </c>
       <c r="G187" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A187,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E187)),NOT(ISNUMBER($F187))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A187,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E187=INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0)),$F187=INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E187-$F187)=(INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E187&gt;$F187,INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),AND($E187=$F187,INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),AND($E187&lt;$F187,INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E187=INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0)),$F187=INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E187-$F187)=(INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H187&lt;&gt;"",$H187=INDEX(Partidos!$K$4:$K$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A187,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E187)),NOT(ISNUMBER($F187))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A187,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E187=INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0)),$F187=INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E187-$F187)=(INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E187&gt;$F187,INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),AND($E187=$F187,INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),AND($E187&lt;$F187,INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0)),IF(AND($E187=INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0)),$F187=INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),IF(AND($H187&lt;&gt;"",$H187=INDEX(Partidos!$K$4:$K$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E187=$F187,($E187-$F187)=(INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0)))),IF(AND($H187&lt;&gt;"",$H187=INDEX(Partidos!$K$4:$K$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H187&lt;&gt;"",$H187=INDEX(Partidos!$K$4:$K$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E187=INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0)),$F187=INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E187-$F187)=(INDEX(Partidos!$F$4:$F$107,MATCH($A187,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H187&lt;&gt;"",$H187=INDEX(Partidos!$K$4:$K$107,MATCH($A187,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H187" s="19">
@@ -17795,7 +17840,7 @@
         <v/>
       </c>
       <c r="G188" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A188,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E188)),NOT(ISNUMBER($F188))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A188,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E188=INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0)),$F188=INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E188-$F188)=(INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E188&gt;$F188,INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),AND($E188=$F188,INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),AND($E188&lt;$F188,INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E188=INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0)),$F188=INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E188-$F188)=(INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H188&lt;&gt;"",$H188=INDEX(Partidos!$K$4:$K$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A188,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E188)),NOT(ISNUMBER($F188))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A188,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E188=INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0)),$F188=INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E188-$F188)=(INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E188&gt;$F188,INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),AND($E188=$F188,INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),AND($E188&lt;$F188,INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0)),IF(AND($E188=INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0)),$F188=INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),IF(AND($H188&lt;&gt;"",$H188=INDEX(Partidos!$K$4:$K$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E188=$F188,($E188-$F188)=(INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0)))),IF(AND($H188&lt;&gt;"",$H188=INDEX(Partidos!$K$4:$K$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H188&lt;&gt;"",$H188=INDEX(Partidos!$K$4:$K$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E188=INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0)),$F188=INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E188-$F188)=(INDEX(Partidos!$F$4:$F$107,MATCH($A188,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H188&lt;&gt;"",$H188=INDEX(Partidos!$K$4:$K$107,MATCH($A188,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H188" s="19">
@@ -17837,7 +17882,7 @@
         <v/>
       </c>
       <c r="G189" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A189,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E189)),NOT(ISNUMBER($F189))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A189,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E189=INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0)),$F189=INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E189-$F189)=(INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E189&gt;$F189,INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),AND($E189=$F189,INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),AND($E189&lt;$F189,INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E189=INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0)),$F189=INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E189-$F189)=(INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H189&lt;&gt;"",$H189=INDEX(Partidos!$K$4:$K$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A189,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E189)),NOT(ISNUMBER($F189))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A189,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E189=INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0)),$F189=INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E189-$F189)=(INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E189&gt;$F189,INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),AND($E189=$F189,INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),AND($E189&lt;$F189,INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0)),IF(AND($E189=INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0)),$F189=INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),IF(AND($H189&lt;&gt;"",$H189=INDEX(Partidos!$K$4:$K$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E189=$F189,($E189-$F189)=(INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0)))),IF(AND($H189&lt;&gt;"",$H189=INDEX(Partidos!$K$4:$K$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H189&lt;&gt;"",$H189=INDEX(Partidos!$K$4:$K$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E189=INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0)),$F189=INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E189-$F189)=(INDEX(Partidos!$F$4:$F$107,MATCH($A189,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H189&lt;&gt;"",$H189=INDEX(Partidos!$K$4:$K$107,MATCH($A189,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H189" s="19">
@@ -17879,7 +17924,7 @@
         <v/>
       </c>
       <c r="G190" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A190,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E190)),NOT(ISNUMBER($F190))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A190,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E190=INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0)),$F190=INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E190-$F190)=(INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E190&gt;$F190,INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),AND($E190=$F190,INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),AND($E190&lt;$F190,INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E190=INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0)),$F190=INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E190-$F190)=(INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H190&lt;&gt;"",$H190=INDEX(Partidos!$K$4:$K$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A190,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E190)),NOT(ISNUMBER($F190))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A190,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E190=INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0)),$F190=INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E190-$F190)=(INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E190&gt;$F190,INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),AND($E190=$F190,INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),AND($E190&lt;$F190,INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0)),IF(AND($E190=INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0)),$F190=INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),IF(AND($H190&lt;&gt;"",$H190=INDEX(Partidos!$K$4:$K$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E190=$F190,($E190-$F190)=(INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0)))),IF(AND($H190&lt;&gt;"",$H190=INDEX(Partidos!$K$4:$K$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H190&lt;&gt;"",$H190=INDEX(Partidos!$K$4:$K$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E190=INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0)),$F190=INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E190-$F190)=(INDEX(Partidos!$F$4:$F$107,MATCH($A190,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H190&lt;&gt;"",$H190=INDEX(Partidos!$K$4:$K$107,MATCH($A190,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H190" s="19">
@@ -17921,7 +17966,7 @@
         <v/>
       </c>
       <c r="G191" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A191,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E191)),NOT(ISNUMBER($F191))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A191,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E191=INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0)),$F191=INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E191-$F191)=(INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E191&gt;$F191,INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),AND($E191=$F191,INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),AND($E191&lt;$F191,INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E191=INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0)),$F191=INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E191-$F191)=(INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H191&lt;&gt;"",$H191=INDEX(Partidos!$K$4:$K$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A191,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E191)),NOT(ISNUMBER($F191))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A191,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E191=INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0)),$F191=INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E191-$F191)=(INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E191&gt;$F191,INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),AND($E191=$F191,INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),AND($E191&lt;$F191,INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0)),IF(AND($E191=INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0)),$F191=INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),IF(AND($H191&lt;&gt;"",$H191=INDEX(Partidos!$K$4:$K$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E191=$F191,($E191-$F191)=(INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0)))),IF(AND($H191&lt;&gt;"",$H191=INDEX(Partidos!$K$4:$K$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H191&lt;&gt;"",$H191=INDEX(Partidos!$K$4:$K$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E191=INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0)),$F191=INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E191-$F191)=(INDEX(Partidos!$F$4:$F$107,MATCH($A191,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H191&lt;&gt;"",$H191=INDEX(Partidos!$K$4:$K$107,MATCH($A191,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H191" s="19">
@@ -17963,7 +18008,7 @@
         <v/>
       </c>
       <c r="G192" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A192,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E192)),NOT(ISNUMBER($F192))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A192,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E192=INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0)),$F192=INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E192-$F192)=(INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E192&gt;$F192,INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),AND($E192=$F192,INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),AND($E192&lt;$F192,INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E192=INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0)),$F192=INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E192-$F192)=(INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H192&lt;&gt;"",$H192=INDEX(Partidos!$K$4:$K$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A192,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E192)),NOT(ISNUMBER($F192))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A192,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E192=INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0)),$F192=INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E192-$F192)=(INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E192&gt;$F192,INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),AND($E192=$F192,INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),AND($E192&lt;$F192,INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0)),IF(AND($E192=INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0)),$F192=INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),IF(AND($H192&lt;&gt;"",$H192=INDEX(Partidos!$K$4:$K$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E192=$F192,($E192-$F192)=(INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0)))),IF(AND($H192&lt;&gt;"",$H192=INDEX(Partidos!$K$4:$K$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H192&lt;&gt;"",$H192=INDEX(Partidos!$K$4:$K$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E192=INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0)),$F192=INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E192-$F192)=(INDEX(Partidos!$F$4:$F$107,MATCH($A192,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H192&lt;&gt;"",$H192=INDEX(Partidos!$K$4:$K$107,MATCH($A192,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H192" s="19">
@@ -18005,7 +18050,7 @@
         <v/>
       </c>
       <c r="G193" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A193,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E193)),NOT(ISNUMBER($F193))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A193,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E193=INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0)),$F193=INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E193-$F193)=(INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E193&gt;$F193,INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),AND($E193=$F193,INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),AND($E193&lt;$F193,INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E193=INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0)),$F193=INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E193-$F193)=(INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H193&lt;&gt;"",$H193=INDEX(Partidos!$K$4:$K$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A193,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E193)),NOT(ISNUMBER($F193))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A193,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E193=INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0)),$F193=INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E193-$F193)=(INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E193&gt;$F193,INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),AND($E193=$F193,INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),AND($E193&lt;$F193,INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0)),IF(AND($E193=INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0)),$F193=INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),IF(AND($H193&lt;&gt;"",$H193=INDEX(Partidos!$K$4:$K$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E193=$F193,($E193-$F193)=(INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0)))),IF(AND($H193&lt;&gt;"",$H193=INDEX(Partidos!$K$4:$K$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H193&lt;&gt;"",$H193=INDEX(Partidos!$K$4:$K$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E193=INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0)),$F193=INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E193-$F193)=(INDEX(Partidos!$F$4:$F$107,MATCH($A193,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H193&lt;&gt;"",$H193=INDEX(Partidos!$K$4:$K$107,MATCH($A193,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H193" s="19">
@@ -18047,7 +18092,7 @@
         <v/>
       </c>
       <c r="G194" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A194,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E194)),NOT(ISNUMBER($F194))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A194,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E194=INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0)),$F194=INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E194-$F194)=(INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E194&gt;$F194,INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),AND($E194=$F194,INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),AND($E194&lt;$F194,INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E194=INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0)),$F194=INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E194-$F194)=(INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H194&lt;&gt;"",$H194=INDEX(Partidos!$K$4:$K$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A194,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E194)),NOT(ISNUMBER($F194))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A194,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E194=INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0)),$F194=INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E194-$F194)=(INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E194&gt;$F194,INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),AND($E194=$F194,INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),AND($E194&lt;$F194,INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0)),IF(AND($E194=INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0)),$F194=INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),IF(AND($H194&lt;&gt;"",$H194=INDEX(Partidos!$K$4:$K$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E194=$F194,($E194-$F194)=(INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0)))),IF(AND($H194&lt;&gt;"",$H194=INDEX(Partidos!$K$4:$K$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H194&lt;&gt;"",$H194=INDEX(Partidos!$K$4:$K$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E194=INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0)),$F194=INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E194-$F194)=(INDEX(Partidos!$F$4:$F$107,MATCH($A194,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H194&lt;&gt;"",$H194=INDEX(Partidos!$K$4:$K$107,MATCH($A194,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H194" s="19">
@@ -18089,7 +18134,7 @@
         <v/>
       </c>
       <c r="G195" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A195,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E195)),NOT(ISNUMBER($F195))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A195,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E195=INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0)),$F195=INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E195-$F195)=(INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E195&gt;$F195,INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),AND($E195=$F195,INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),AND($E195&lt;$F195,INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E195=INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0)),$F195=INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E195-$F195)=(INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H195&lt;&gt;"",$H195=INDEX(Partidos!$K$4:$K$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A195,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E195)),NOT(ISNUMBER($F195))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A195,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E195=INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0)),$F195=INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E195-$F195)=(INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E195&gt;$F195,INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),AND($E195=$F195,INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),AND($E195&lt;$F195,INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0)),IF(AND($E195=INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0)),$F195=INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),IF(AND($H195&lt;&gt;"",$H195=INDEX(Partidos!$K$4:$K$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E195=$F195,($E195-$F195)=(INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0)))),IF(AND($H195&lt;&gt;"",$H195=INDEX(Partidos!$K$4:$K$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H195&lt;&gt;"",$H195=INDEX(Partidos!$K$4:$K$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E195=INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0)),$F195=INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E195-$F195)=(INDEX(Partidos!$F$4:$F$107,MATCH($A195,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H195&lt;&gt;"",$H195=INDEX(Partidos!$K$4:$K$107,MATCH($A195,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H195" s="19">
@@ -18131,7 +18176,7 @@
         <v/>
       </c>
       <c r="G196" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A196,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E196)),NOT(ISNUMBER($F196))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A196,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E196=INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0)),$F196=INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E196-$F196)=(INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E196&gt;$F196,INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),AND($E196=$F196,INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),AND($E196&lt;$F196,INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E196=INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0)),$F196=INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E196-$F196)=(INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H196&lt;&gt;"",$H196=INDEX(Partidos!$K$4:$K$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A196,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E196)),NOT(ISNUMBER($F196))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A196,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E196=INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0)),$F196=INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E196-$F196)=(INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E196&gt;$F196,INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),AND($E196=$F196,INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),AND($E196&lt;$F196,INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0)),IF(AND($E196=INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0)),$F196=INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),IF(AND($H196&lt;&gt;"",$H196=INDEX(Partidos!$K$4:$K$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E196=$F196,($E196-$F196)=(INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0)))),IF(AND($H196&lt;&gt;"",$H196=INDEX(Partidos!$K$4:$K$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H196&lt;&gt;"",$H196=INDEX(Partidos!$K$4:$K$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E196=INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0)),$F196=INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E196-$F196)=(INDEX(Partidos!$F$4:$F$107,MATCH($A196,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H196&lt;&gt;"",$H196=INDEX(Partidos!$K$4:$K$107,MATCH($A196,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H196" s="19">
@@ -18173,7 +18218,7 @@
         <v/>
       </c>
       <c r="G197" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A197,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E197)),NOT(ISNUMBER($F197))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A197,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E197=INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0)),$F197=INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E197-$F197)=(INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E197&gt;$F197,INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),AND($E197=$F197,INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),AND($E197&lt;$F197,INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E197=INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0)),$F197=INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E197-$F197)=(INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H197&lt;&gt;"",$H197=INDEX(Partidos!$K$4:$K$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A197,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E197)),NOT(ISNUMBER($F197))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A197,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E197=INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0)),$F197=INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E197-$F197)=(INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E197&gt;$F197,INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),AND($E197=$F197,INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),AND($E197&lt;$F197,INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0)),IF(AND($E197=INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0)),$F197=INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),IF(AND($H197&lt;&gt;"",$H197=INDEX(Partidos!$K$4:$K$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E197=$F197,($E197-$F197)=(INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0)))),IF(AND($H197&lt;&gt;"",$H197=INDEX(Partidos!$K$4:$K$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H197&lt;&gt;"",$H197=INDEX(Partidos!$K$4:$K$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E197=INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0)),$F197=INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E197-$F197)=(INDEX(Partidos!$F$4:$F$107,MATCH($A197,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H197&lt;&gt;"",$H197=INDEX(Partidos!$K$4:$K$107,MATCH($A197,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H197" s="19">
@@ -18215,7 +18260,7 @@
         <v/>
       </c>
       <c r="G198" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A198,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E198)),NOT(ISNUMBER($F198))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A198,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E198=INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0)),$F198=INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E198-$F198)=(INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E198&gt;$F198,INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),AND($E198=$F198,INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),AND($E198&lt;$F198,INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E198=INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0)),$F198=INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E198-$F198)=(INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H198&lt;&gt;"",$H198=INDEX(Partidos!$K$4:$K$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A198,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E198)),NOT(ISNUMBER($F198))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A198,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E198=INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0)),$F198=INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E198-$F198)=(INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E198&gt;$F198,INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),AND($E198=$F198,INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),AND($E198&lt;$F198,INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0)),IF(AND($E198=INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0)),$F198=INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),IF(AND($H198&lt;&gt;"",$H198=INDEX(Partidos!$K$4:$K$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E198=$F198,($E198-$F198)=(INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0)))),IF(AND($H198&lt;&gt;"",$H198=INDEX(Partidos!$K$4:$K$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H198&lt;&gt;"",$H198=INDEX(Partidos!$K$4:$K$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E198=INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0)),$F198=INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E198-$F198)=(INDEX(Partidos!$F$4:$F$107,MATCH($A198,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H198&lt;&gt;"",$H198=INDEX(Partidos!$K$4:$K$107,MATCH($A198,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H198" s="19">
@@ -18257,7 +18302,7 @@
         <v/>
       </c>
       <c r="G199" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A199,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E199)),NOT(ISNUMBER($F199))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A199,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E199=INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0)),$F199=INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E199-$F199)=(INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E199&gt;$F199,INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),AND($E199=$F199,INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),AND($E199&lt;$F199,INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E199=INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0)),$F199=INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E199-$F199)=(INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H199&lt;&gt;"",$H199=INDEX(Partidos!$K$4:$K$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A199,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E199)),NOT(ISNUMBER($F199))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A199,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E199=INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0)),$F199=INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E199-$F199)=(INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E199&gt;$F199,INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),AND($E199=$F199,INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),AND($E199&lt;$F199,INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0)),IF(AND($E199=INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0)),$F199=INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),IF(AND($H199&lt;&gt;"",$H199=INDEX(Partidos!$K$4:$K$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E199=$F199,($E199-$F199)=(INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0)))),IF(AND($H199&lt;&gt;"",$H199=INDEX(Partidos!$K$4:$K$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H199&lt;&gt;"",$H199=INDEX(Partidos!$K$4:$K$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E199=INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0)),$F199=INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E199-$F199)=(INDEX(Partidos!$F$4:$F$107,MATCH($A199,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H199&lt;&gt;"",$H199=INDEX(Partidos!$K$4:$K$107,MATCH($A199,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H199" s="19">
@@ -18299,7 +18344,7 @@
         <v/>
       </c>
       <c r="G200" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A200,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E200)),NOT(ISNUMBER($F200))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A200,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E200=INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0)),$F200=INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E200-$F200)=(INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E200&gt;$F200,INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),AND($E200=$F200,INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),AND($E200&lt;$F200,INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E200=INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0)),$F200=INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E200-$F200)=(INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H200&lt;&gt;"",$H200=INDEX(Partidos!$K$4:$K$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A200,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E200)),NOT(ISNUMBER($F200))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A200,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E200=INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0)),$F200=INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E200-$F200)=(INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E200&gt;$F200,INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),AND($E200=$F200,INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),AND($E200&lt;$F200,INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0)),IF(AND($E200=INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0)),$F200=INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),IF(AND($H200&lt;&gt;"",$H200=INDEX(Partidos!$K$4:$K$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E200=$F200,($E200-$F200)=(INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0)))),IF(AND($H200&lt;&gt;"",$H200=INDEX(Partidos!$K$4:$K$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H200&lt;&gt;"",$H200=INDEX(Partidos!$K$4:$K$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E200=INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0)),$F200=INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E200-$F200)=(INDEX(Partidos!$F$4:$F$107,MATCH($A200,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H200&lt;&gt;"",$H200=INDEX(Partidos!$K$4:$K$107,MATCH($A200,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H200" s="19">
@@ -18341,7 +18386,7 @@
         <v/>
       </c>
       <c r="G201" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A201,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E201)),NOT(ISNUMBER($F201))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A201,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E201=INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0)),$F201=INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E201-$F201)=(INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E201&gt;$F201,INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),AND($E201=$F201,INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),AND($E201&lt;$F201,INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E201=INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0)),$F201=INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E201-$F201)=(INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H201&lt;&gt;"",$H201=INDEX(Partidos!$K$4:$K$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A201,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E201)),NOT(ISNUMBER($F201))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A201,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E201=INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0)),$F201=INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E201-$F201)=(INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E201&gt;$F201,INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),AND($E201=$F201,INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),AND($E201&lt;$F201,INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0)),IF(AND($E201=INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0)),$F201=INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),IF(AND($H201&lt;&gt;"",$H201=INDEX(Partidos!$K$4:$K$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E201=$F201,($E201-$F201)=(INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0)))),IF(AND($H201&lt;&gt;"",$H201=INDEX(Partidos!$K$4:$K$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H201&lt;&gt;"",$H201=INDEX(Partidos!$K$4:$K$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E201=INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0)),$F201=INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E201-$F201)=(INDEX(Partidos!$F$4:$F$107,MATCH($A201,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H201&lt;&gt;"",$H201=INDEX(Partidos!$K$4:$K$107,MATCH($A201,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H201" s="19">
@@ -18383,7 +18428,7 @@
         <v/>
       </c>
       <c r="G202" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A202,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E202)),NOT(ISNUMBER($F202))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A202,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E202=INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0)),$F202=INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E202-$F202)=(INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E202&gt;$F202,INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),AND($E202=$F202,INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),AND($E202&lt;$F202,INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E202=INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0)),$F202=INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E202-$F202)=(INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H202&lt;&gt;"",$H202=INDEX(Partidos!$K$4:$K$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A202,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E202)),NOT(ISNUMBER($F202))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A202,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E202=INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0)),$F202=INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E202-$F202)=(INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E202&gt;$F202,INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),AND($E202=$F202,INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),AND($E202&lt;$F202,INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0)),IF(AND($E202=INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0)),$F202=INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),IF(AND($H202&lt;&gt;"",$H202=INDEX(Partidos!$K$4:$K$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E202=$F202,($E202-$F202)=(INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0)))),IF(AND($H202&lt;&gt;"",$H202=INDEX(Partidos!$K$4:$K$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H202&lt;&gt;"",$H202=INDEX(Partidos!$K$4:$K$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E202=INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0)),$F202=INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E202-$F202)=(INDEX(Partidos!$F$4:$F$107,MATCH($A202,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H202&lt;&gt;"",$H202=INDEX(Partidos!$K$4:$K$107,MATCH($A202,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H202" s="19">
@@ -18425,7 +18470,7 @@
         <v/>
       </c>
       <c r="G203" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A203,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E203)),NOT(ISNUMBER($F203))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A203,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E203=INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0)),$F203=INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E203-$F203)=(INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E203&gt;$F203,INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),AND($E203=$F203,INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),AND($E203&lt;$F203,INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E203=INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0)),$F203=INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E203-$F203)=(INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H203&lt;&gt;"",$H203=INDEX(Partidos!$K$4:$K$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A203,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E203)),NOT(ISNUMBER($F203))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A203,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E203=INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0)),$F203=INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E203-$F203)=(INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E203&gt;$F203,INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),AND($E203=$F203,INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),AND($E203&lt;$F203,INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0)),IF(AND($E203=INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0)),$F203=INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),IF(AND($H203&lt;&gt;"",$H203=INDEX(Partidos!$K$4:$K$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E203=$F203,($E203-$F203)=(INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0)))),IF(AND($H203&lt;&gt;"",$H203=INDEX(Partidos!$K$4:$K$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H203&lt;&gt;"",$H203=INDEX(Partidos!$K$4:$K$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E203=INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0)),$F203=INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E203-$F203)=(INDEX(Partidos!$F$4:$F$107,MATCH($A203,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H203&lt;&gt;"",$H203=INDEX(Partidos!$K$4:$K$107,MATCH($A203,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H203" s="19">
@@ -18467,7 +18512,7 @@
         <v/>
       </c>
       <c r="G204" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A204,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E204)),NOT(ISNUMBER($F204))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A204,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E204=INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0)),$F204=INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E204-$F204)=(INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E204&gt;$F204,INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),AND($E204=$F204,INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),AND($E204&lt;$F204,INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E204=INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0)),$F204=INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E204-$F204)=(INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H204&lt;&gt;"",$H204=INDEX(Partidos!$K$4:$K$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A204,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E204)),NOT(ISNUMBER($F204))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A204,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E204=INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0)),$F204=INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E204-$F204)=(INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E204&gt;$F204,INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),AND($E204=$F204,INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),AND($E204&lt;$F204,INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0)),IF(AND($E204=INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0)),$F204=INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),IF(AND($H204&lt;&gt;"",$H204=INDEX(Partidos!$K$4:$K$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E204=$F204,($E204-$F204)=(INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0)))),IF(AND($H204&lt;&gt;"",$H204=INDEX(Partidos!$K$4:$K$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H204&lt;&gt;"",$H204=INDEX(Partidos!$K$4:$K$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E204=INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0)),$F204=INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E204-$F204)=(INDEX(Partidos!$F$4:$F$107,MATCH($A204,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H204&lt;&gt;"",$H204=INDEX(Partidos!$K$4:$K$107,MATCH($A204,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H204" s="19">
@@ -18509,7 +18554,7 @@
         <v/>
       </c>
       <c r="G205" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A205,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E205)),NOT(ISNUMBER($F205))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A205,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E205=INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0)),$F205=INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E205-$F205)=(INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E205&gt;$F205,INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),AND($E205=$F205,INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),AND($E205&lt;$F205,INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E205=INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0)),$F205=INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E205-$F205)=(INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H205&lt;&gt;"",$H205=INDEX(Partidos!$K$4:$K$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A205,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E205)),NOT(ISNUMBER($F205))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A205,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E205=INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0)),$F205=INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E205-$F205)=(INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E205&gt;$F205,INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),AND($E205=$F205,INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),AND($E205&lt;$F205,INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0)),IF(AND($E205=INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0)),$F205=INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),IF(AND($H205&lt;&gt;"",$H205=INDEX(Partidos!$K$4:$K$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E205=$F205,($E205-$F205)=(INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0)))),IF(AND($H205&lt;&gt;"",$H205=INDEX(Partidos!$K$4:$K$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H205&lt;&gt;"",$H205=INDEX(Partidos!$K$4:$K$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E205=INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0)),$F205=INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E205-$F205)=(INDEX(Partidos!$F$4:$F$107,MATCH($A205,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H205&lt;&gt;"",$H205=INDEX(Partidos!$K$4:$K$107,MATCH($A205,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H205" s="19">
@@ -18551,7 +18596,7 @@
         <v/>
       </c>
       <c r="G206" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A206,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E206)),NOT(ISNUMBER($F206))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A206,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E206=INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0)),$F206=INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E206-$F206)=(INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E206&gt;$F206,INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),AND($E206=$F206,INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),AND($E206&lt;$F206,INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E206=INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0)),$F206=INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E206-$F206)=(INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H206&lt;&gt;"",$H206=INDEX(Partidos!$K$4:$K$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A206,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E206)),NOT(ISNUMBER($F206))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A206,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E206=INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0)),$F206=INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E206-$F206)=(INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E206&gt;$F206,INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),AND($E206=$F206,INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),AND($E206&lt;$F206,INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0)),IF(AND($E206=INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0)),$F206=INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),IF(AND($H206&lt;&gt;"",$H206=INDEX(Partidos!$K$4:$K$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E206=$F206,($E206-$F206)=(INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0)))),IF(AND($H206&lt;&gt;"",$H206=INDEX(Partidos!$K$4:$K$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H206&lt;&gt;"",$H206=INDEX(Partidos!$K$4:$K$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E206=INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0)),$F206=INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E206-$F206)=(INDEX(Partidos!$F$4:$F$107,MATCH($A206,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H206&lt;&gt;"",$H206=INDEX(Partidos!$K$4:$K$107,MATCH($A206,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H206" s="19">
@@ -18593,7 +18638,7 @@
         <v/>
       </c>
       <c r="G207" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A207,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E207)),NOT(ISNUMBER($F207))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A207,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E207=INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0)),$F207=INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E207-$F207)=(INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E207&gt;$F207,INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),AND($E207=$F207,INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),AND($E207&lt;$F207,INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E207=INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0)),$F207=INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E207-$F207)=(INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H207&lt;&gt;"",$H207=INDEX(Partidos!$K$4:$K$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A207,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E207)),NOT(ISNUMBER($F207))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A207,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E207=INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0)),$F207=INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E207-$F207)=(INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E207&gt;$F207,INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),AND($E207=$F207,INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),AND($E207&lt;$F207,INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0)),IF(AND($E207=INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0)),$F207=INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),IF(AND($H207&lt;&gt;"",$H207=INDEX(Partidos!$K$4:$K$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E207=$F207,($E207-$F207)=(INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0)))),IF(AND($H207&lt;&gt;"",$H207=INDEX(Partidos!$K$4:$K$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H207&lt;&gt;"",$H207=INDEX(Partidos!$K$4:$K$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E207=INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0)),$F207=INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E207-$F207)=(INDEX(Partidos!$F$4:$F$107,MATCH($A207,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H207&lt;&gt;"",$H207=INDEX(Partidos!$K$4:$K$107,MATCH($A207,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H207" s="19">
@@ -18635,7 +18680,7 @@
         <v/>
       </c>
       <c r="G208" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A208,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E208)),NOT(ISNUMBER($F208))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A208,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E208=INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0)),$F208=INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E208-$F208)=(INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E208&gt;$F208,INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),AND($E208=$F208,INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),AND($E208&lt;$F208,INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E208=INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0)),$F208=INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E208-$F208)=(INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H208&lt;&gt;"",$H208=INDEX(Partidos!$K$4:$K$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A208,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E208)),NOT(ISNUMBER($F208))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A208,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E208=INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0)),$F208=INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E208-$F208)=(INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E208&gt;$F208,INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),AND($E208=$F208,INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),AND($E208&lt;$F208,INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0)),IF(AND($E208=INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0)),$F208=INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),IF(AND($H208&lt;&gt;"",$H208=INDEX(Partidos!$K$4:$K$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E208=$F208,($E208-$F208)=(INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0)))),IF(AND($H208&lt;&gt;"",$H208=INDEX(Partidos!$K$4:$K$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H208&lt;&gt;"",$H208=INDEX(Partidos!$K$4:$K$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E208=INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0)),$F208=INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E208-$F208)=(INDEX(Partidos!$F$4:$F$107,MATCH($A208,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H208&lt;&gt;"",$H208=INDEX(Partidos!$K$4:$K$107,MATCH($A208,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H208" s="19">
@@ -18677,7 +18722,7 @@
         <v/>
       </c>
       <c r="G209" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A209,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E209)),NOT(ISNUMBER($F209))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A209,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E209=INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0)),$F209=INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E209-$F209)=(INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E209&gt;$F209,INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),AND($E209=$F209,INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),AND($E209&lt;$F209,INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E209=INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0)),$F209=INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E209-$F209)=(INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H209&lt;&gt;"",$H209=INDEX(Partidos!$K$4:$K$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A209,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E209)),NOT(ISNUMBER($F209))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A209,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E209=INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0)),$F209=INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E209-$F209)=(INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E209&gt;$F209,INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),AND($E209=$F209,INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),AND($E209&lt;$F209,INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0)),IF(AND($E209=INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0)),$F209=INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),IF(AND($H209&lt;&gt;"",$H209=INDEX(Partidos!$K$4:$K$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E209=$F209,($E209-$F209)=(INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0)))),IF(AND($H209&lt;&gt;"",$H209=INDEX(Partidos!$K$4:$K$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H209&lt;&gt;"",$H209=INDEX(Partidos!$K$4:$K$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E209=INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0)),$F209=INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E209-$F209)=(INDEX(Partidos!$F$4:$F$107,MATCH($A209,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H209&lt;&gt;"",$H209=INDEX(Partidos!$K$4:$K$107,MATCH($A209,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H209" s="19">
@@ -18719,7 +18764,7 @@
         <v/>
       </c>
       <c r="G210" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A210,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E210)),NOT(ISNUMBER($F210))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A210,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E210=INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0)),$F210=INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E210-$F210)=(INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E210&gt;$F210,INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),AND($E210=$F210,INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),AND($E210&lt;$F210,INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E210=INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0)),$F210=INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E210-$F210)=(INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H210&lt;&gt;"",$H210=INDEX(Partidos!$K$4:$K$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A210,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E210)),NOT(ISNUMBER($F210))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A210,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E210=INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0)),$F210=INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E210-$F210)=(INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E210&gt;$F210,INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),AND($E210=$F210,INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),AND($E210&lt;$F210,INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0)),IF(AND($E210=INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0)),$F210=INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),IF(AND($H210&lt;&gt;"",$H210=INDEX(Partidos!$K$4:$K$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E210=$F210,($E210-$F210)=(INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0)))),IF(AND($H210&lt;&gt;"",$H210=INDEX(Partidos!$K$4:$K$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H210&lt;&gt;"",$H210=INDEX(Partidos!$K$4:$K$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E210=INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0)),$F210=INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E210-$F210)=(INDEX(Partidos!$F$4:$F$107,MATCH($A210,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H210&lt;&gt;"",$H210=INDEX(Partidos!$K$4:$K$107,MATCH($A210,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H210" s="19">
@@ -18761,7 +18806,7 @@
         <v/>
       </c>
       <c r="G211" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A211,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E211)),NOT(ISNUMBER($F211))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A211,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E211=INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0)),$F211=INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E211-$F211)=(INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E211&gt;$F211,INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),AND($E211=$F211,INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),AND($E211&lt;$F211,INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E211=INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0)),$F211=INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E211-$F211)=(INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H211&lt;&gt;"",$H211=INDEX(Partidos!$K$4:$K$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A211,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E211)),NOT(ISNUMBER($F211))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A211,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E211=INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0)),$F211=INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E211-$F211)=(INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E211&gt;$F211,INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),AND($E211=$F211,INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),AND($E211&lt;$F211,INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0)),IF(AND($E211=INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0)),$F211=INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),IF(AND($H211&lt;&gt;"",$H211=INDEX(Partidos!$K$4:$K$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E211=$F211,($E211-$F211)=(INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0)))),IF(AND($H211&lt;&gt;"",$H211=INDEX(Partidos!$K$4:$K$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H211&lt;&gt;"",$H211=INDEX(Partidos!$K$4:$K$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E211=INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0)),$F211=INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E211-$F211)=(INDEX(Partidos!$F$4:$F$107,MATCH($A211,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H211&lt;&gt;"",$H211=INDEX(Partidos!$K$4:$K$107,MATCH($A211,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H211" s="19">
@@ -18803,7 +18848,7 @@
         <v/>
       </c>
       <c r="G212" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A212,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E212)),NOT(ISNUMBER($F212))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A212,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E212=INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0)),$F212=INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E212-$F212)=(INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E212&gt;$F212,INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),AND($E212=$F212,INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),AND($E212&lt;$F212,INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E212=INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0)),$F212=INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E212-$F212)=(INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H212&lt;&gt;"",$H212=INDEX(Partidos!$K$4:$K$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A212,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E212)),NOT(ISNUMBER($F212))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A212,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E212=INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0)),$F212=INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E212-$F212)=(INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E212&gt;$F212,INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),AND($E212=$F212,INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),AND($E212&lt;$F212,INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0)),IF(AND($E212=INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0)),$F212=INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),IF(AND($H212&lt;&gt;"",$H212=INDEX(Partidos!$K$4:$K$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E212=$F212,($E212-$F212)=(INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0)))),IF(AND($H212&lt;&gt;"",$H212=INDEX(Partidos!$K$4:$K$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H212&lt;&gt;"",$H212=INDEX(Partidos!$K$4:$K$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E212=INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0)),$F212=INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E212-$F212)=(INDEX(Partidos!$F$4:$F$107,MATCH($A212,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H212&lt;&gt;"",$H212=INDEX(Partidos!$K$4:$K$107,MATCH($A212,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H212" s="19">
@@ -18845,7 +18890,7 @@
         <v/>
       </c>
       <c r="G213" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A213,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E213)),NOT(ISNUMBER($F213))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A213,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E213=INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0)),$F213=INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E213-$F213)=(INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E213&gt;$F213,INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),AND($E213=$F213,INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),AND($E213&lt;$F213,INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E213=INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0)),$F213=INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E213-$F213)=(INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H213&lt;&gt;"",$H213=INDEX(Partidos!$K$4:$K$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A213,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E213)),NOT(ISNUMBER($F213))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A213,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E213=INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0)),$F213=INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E213-$F213)=(INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E213&gt;$F213,INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),AND($E213=$F213,INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),AND($E213&lt;$F213,INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0)),IF(AND($E213=INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0)),$F213=INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),IF(AND($H213&lt;&gt;"",$H213=INDEX(Partidos!$K$4:$K$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E213=$F213,($E213-$F213)=(INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0)))),IF(AND($H213&lt;&gt;"",$H213=INDEX(Partidos!$K$4:$K$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H213&lt;&gt;"",$H213=INDEX(Partidos!$K$4:$K$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E213=INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0)),$F213=INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E213-$F213)=(INDEX(Partidos!$F$4:$F$107,MATCH($A213,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H213&lt;&gt;"",$H213=INDEX(Partidos!$K$4:$K$107,MATCH($A213,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H213" s="19">
@@ -18887,7 +18932,7 @@
         <v/>
       </c>
       <c r="G214" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A214,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E214)),NOT(ISNUMBER($F214))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A214,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E214=INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0)),$F214=INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E214-$F214)=(INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E214&gt;$F214,INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),AND($E214=$F214,INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),AND($E214&lt;$F214,INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E214=INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0)),$F214=INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E214-$F214)=(INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H214&lt;&gt;"",$H214=INDEX(Partidos!$K$4:$K$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A214,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E214)),NOT(ISNUMBER($F214))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A214,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E214=INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0)),$F214=INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E214-$F214)=(INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E214&gt;$F214,INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),AND($E214=$F214,INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),AND($E214&lt;$F214,INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0)),IF(AND($E214=INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0)),$F214=INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),IF(AND($H214&lt;&gt;"",$H214=INDEX(Partidos!$K$4:$K$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E214=$F214,($E214-$F214)=(INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0)))),IF(AND($H214&lt;&gt;"",$H214=INDEX(Partidos!$K$4:$K$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H214&lt;&gt;"",$H214=INDEX(Partidos!$K$4:$K$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E214=INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0)),$F214=INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E214-$F214)=(INDEX(Partidos!$F$4:$F$107,MATCH($A214,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H214&lt;&gt;"",$H214=INDEX(Partidos!$K$4:$K$107,MATCH($A214,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H214" s="19">
@@ -18929,7 +18974,7 @@
         <v/>
       </c>
       <c r="G215" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A215,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E215)),NOT(ISNUMBER($F215))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A215,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E215=INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0)),$F215=INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E215-$F215)=(INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E215&gt;$F215,INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),AND($E215=$F215,INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),AND($E215&lt;$F215,INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E215=INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0)),$F215=INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E215-$F215)=(INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H215&lt;&gt;"",$H215=INDEX(Partidos!$K$4:$K$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A215,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E215)),NOT(ISNUMBER($F215))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A215,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E215=INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0)),$F215=INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E215-$F215)=(INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E215&gt;$F215,INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),AND($E215=$F215,INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),AND($E215&lt;$F215,INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0)),IF(AND($E215=INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0)),$F215=INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),IF(AND($H215&lt;&gt;"",$H215=INDEX(Partidos!$K$4:$K$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E215=$F215,($E215-$F215)=(INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0)))),IF(AND($H215&lt;&gt;"",$H215=INDEX(Partidos!$K$4:$K$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H215&lt;&gt;"",$H215=INDEX(Partidos!$K$4:$K$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E215=INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0)),$F215=INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E215-$F215)=(INDEX(Partidos!$F$4:$F$107,MATCH($A215,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H215&lt;&gt;"",$H215=INDEX(Partidos!$K$4:$K$107,MATCH($A215,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H215" s="19">
@@ -18971,7 +19016,7 @@
         <v/>
       </c>
       <c r="G216" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A216,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E216)),NOT(ISNUMBER($F216))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A216,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E216=INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0)),$F216=INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E216-$F216)=(INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E216&gt;$F216,INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),AND($E216=$F216,INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),AND($E216&lt;$F216,INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E216=INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0)),$F216=INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E216-$F216)=(INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H216&lt;&gt;"",$H216=INDEX(Partidos!$K$4:$K$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A216,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E216)),NOT(ISNUMBER($F216))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A216,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E216=INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0)),$F216=INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E216-$F216)=(INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E216&gt;$F216,INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),AND($E216=$F216,INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),AND($E216&lt;$F216,INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0)),IF(AND($E216=INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0)),$F216=INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),IF(AND($H216&lt;&gt;"",$H216=INDEX(Partidos!$K$4:$K$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E216=$F216,($E216-$F216)=(INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0)))),IF(AND($H216&lt;&gt;"",$H216=INDEX(Partidos!$K$4:$K$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H216&lt;&gt;"",$H216=INDEX(Partidos!$K$4:$K$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E216=INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0)),$F216=INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E216-$F216)=(INDEX(Partidos!$F$4:$F$107,MATCH($A216,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H216&lt;&gt;"",$H216=INDEX(Partidos!$K$4:$K$107,MATCH($A216,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H216" s="19">
@@ -19013,7 +19058,7 @@
         <v/>
       </c>
       <c r="G217" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A217,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E217)),NOT(ISNUMBER($F217))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A217,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E217=INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0)),$F217=INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E217-$F217)=(INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E217&gt;$F217,INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),AND($E217=$F217,INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),AND($E217&lt;$F217,INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E217=INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0)),$F217=INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E217-$F217)=(INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H217&lt;&gt;"",$H217=INDEX(Partidos!$K$4:$K$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A217,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E217)),NOT(ISNUMBER($F217))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A217,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E217=INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0)),$F217=INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E217-$F217)=(INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E217&gt;$F217,INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),AND($E217=$F217,INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),AND($E217&lt;$F217,INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0)),IF(AND($E217=INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0)),$F217=INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),IF(AND($H217&lt;&gt;"",$H217=INDEX(Partidos!$K$4:$K$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E217=$F217,($E217-$F217)=(INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0)))),IF(AND($H217&lt;&gt;"",$H217=INDEX(Partidos!$K$4:$K$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H217&lt;&gt;"",$H217=INDEX(Partidos!$K$4:$K$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E217=INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0)),$F217=INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E217-$F217)=(INDEX(Partidos!$F$4:$F$107,MATCH($A217,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H217&lt;&gt;"",$H217=INDEX(Partidos!$K$4:$K$107,MATCH($A217,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H217" s="19">
@@ -19055,7 +19100,7 @@
         <v/>
       </c>
       <c r="G218" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A218,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E218)),NOT(ISNUMBER($F218))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A218,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E218=INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0)),$F218=INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E218-$F218)=(INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E218&gt;$F218,INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),AND($E218=$F218,INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),AND($E218&lt;$F218,INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E218=INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0)),$F218=INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E218-$F218)=(INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H218&lt;&gt;"",$H218=INDEX(Partidos!$K$4:$K$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A218,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E218)),NOT(ISNUMBER($F218))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A218,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E218=INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0)),$F218=INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E218-$F218)=(INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E218&gt;$F218,INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),AND($E218=$F218,INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),AND($E218&lt;$F218,INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0)),IF(AND($E218=INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0)),$F218=INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),IF(AND($H218&lt;&gt;"",$H218=INDEX(Partidos!$K$4:$K$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E218=$F218,($E218-$F218)=(INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0)))),IF(AND($H218&lt;&gt;"",$H218=INDEX(Partidos!$K$4:$K$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H218&lt;&gt;"",$H218=INDEX(Partidos!$K$4:$K$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E218=INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0)),$F218=INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E218-$F218)=(INDEX(Partidos!$F$4:$F$107,MATCH($A218,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H218&lt;&gt;"",$H218=INDEX(Partidos!$K$4:$K$107,MATCH($A218,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H218" s="19">
@@ -19097,7 +19142,7 @@
         <v/>
       </c>
       <c r="G219" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A219,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E219)),NOT(ISNUMBER($F219))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A219,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E219=INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0)),$F219=INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E219-$F219)=(INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E219&gt;$F219,INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),AND($E219=$F219,INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),AND($E219&lt;$F219,INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E219=INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0)),$F219=INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E219-$F219)=(INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H219&lt;&gt;"",$H219=INDEX(Partidos!$K$4:$K$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A219,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E219)),NOT(ISNUMBER($F219))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A219,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E219=INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0)),$F219=INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E219-$F219)=(INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E219&gt;$F219,INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),AND($E219=$F219,INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),AND($E219&lt;$F219,INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0)),IF(AND($E219=INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0)),$F219=INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),IF(AND($H219&lt;&gt;"",$H219=INDEX(Partidos!$K$4:$K$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E219=$F219,($E219-$F219)=(INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0)))),IF(AND($H219&lt;&gt;"",$H219=INDEX(Partidos!$K$4:$K$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H219&lt;&gt;"",$H219=INDEX(Partidos!$K$4:$K$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E219=INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0)),$F219=INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E219-$F219)=(INDEX(Partidos!$F$4:$F$107,MATCH($A219,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H219&lt;&gt;"",$H219=INDEX(Partidos!$K$4:$K$107,MATCH($A219,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H219" s="19">
@@ -19139,7 +19184,7 @@
         <v/>
       </c>
       <c r="G220" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A220,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E220)),NOT(ISNUMBER($F220))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A220,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E220=INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0)),$F220=INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E220-$F220)=(INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E220&gt;$F220,INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),AND($E220=$F220,INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),AND($E220&lt;$F220,INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E220=INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0)),$F220=INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E220-$F220)=(INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H220&lt;&gt;"",$H220=INDEX(Partidos!$K$4:$K$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A220,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E220)),NOT(ISNUMBER($F220))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A220,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E220=INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0)),$F220=INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E220-$F220)=(INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E220&gt;$F220,INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),AND($E220=$F220,INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),AND($E220&lt;$F220,INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0)),IF(AND($E220=INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0)),$F220=INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),IF(AND($H220&lt;&gt;"",$H220=INDEX(Partidos!$K$4:$K$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E220=$F220,($E220-$F220)=(INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0)))),IF(AND($H220&lt;&gt;"",$H220=INDEX(Partidos!$K$4:$K$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H220&lt;&gt;"",$H220=INDEX(Partidos!$K$4:$K$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E220=INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0)),$F220=INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E220-$F220)=(INDEX(Partidos!$F$4:$F$107,MATCH($A220,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H220&lt;&gt;"",$H220=INDEX(Partidos!$K$4:$K$107,MATCH($A220,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H220" s="19">
@@ -19181,7 +19226,7 @@
         <v/>
       </c>
       <c r="G221" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A221,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E221)),NOT(ISNUMBER($F221))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A221,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E221=INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0)),$F221=INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E221-$F221)=(INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E221&gt;$F221,INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),AND($E221=$F221,INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),AND($E221&lt;$F221,INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E221=INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0)),$F221=INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E221-$F221)=(INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H221&lt;&gt;"",$H221=INDEX(Partidos!$K$4:$K$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A221,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E221)),NOT(ISNUMBER($F221))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A221,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E221=INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0)),$F221=INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E221-$F221)=(INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E221&gt;$F221,INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),AND($E221=$F221,INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),AND($E221&lt;$F221,INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0)),IF(AND($E221=INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0)),$F221=INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),IF(AND($H221&lt;&gt;"",$H221=INDEX(Partidos!$K$4:$K$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E221=$F221,($E221-$F221)=(INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0)))),IF(AND($H221&lt;&gt;"",$H221=INDEX(Partidos!$K$4:$K$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H221&lt;&gt;"",$H221=INDEX(Partidos!$K$4:$K$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E221=INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0)),$F221=INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E221-$F221)=(INDEX(Partidos!$F$4:$F$107,MATCH($A221,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H221&lt;&gt;"",$H221=INDEX(Partidos!$K$4:$K$107,MATCH($A221,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H221" s="19">
@@ -19223,7 +19268,7 @@
         <v/>
       </c>
       <c r="G222" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A222,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E222)),NOT(ISNUMBER($F222))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A222,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E222=INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0)),$F222=INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E222-$F222)=(INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E222&gt;$F222,INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),AND($E222=$F222,INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),AND($E222&lt;$F222,INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E222=INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0)),$F222=INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E222-$F222)=(INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H222&lt;&gt;"",$H222=INDEX(Partidos!$K$4:$K$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A222,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E222)),NOT(ISNUMBER($F222))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A222,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E222=INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0)),$F222=INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E222-$F222)=(INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E222&gt;$F222,INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),AND($E222=$F222,INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),AND($E222&lt;$F222,INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0)),IF(AND($E222=INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0)),$F222=INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),IF(AND($H222&lt;&gt;"",$H222=INDEX(Partidos!$K$4:$K$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E222=$F222,($E222-$F222)=(INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0)))),IF(AND($H222&lt;&gt;"",$H222=INDEX(Partidos!$K$4:$K$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H222&lt;&gt;"",$H222=INDEX(Partidos!$K$4:$K$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E222=INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0)),$F222=INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E222-$F222)=(INDEX(Partidos!$F$4:$F$107,MATCH($A222,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H222&lt;&gt;"",$H222=INDEX(Partidos!$K$4:$K$107,MATCH($A222,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H222" s="19">
@@ -19265,7 +19310,7 @@
         <v/>
       </c>
       <c r="G223" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A223,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E223)),NOT(ISNUMBER($F223))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A223,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E223=INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0)),$F223=INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E223-$F223)=(INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E223&gt;$F223,INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),AND($E223=$F223,INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),AND($E223&lt;$F223,INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E223=INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0)),$F223=INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E223-$F223)=(INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H223&lt;&gt;"",$H223=INDEX(Partidos!$K$4:$K$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A223,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E223)),NOT(ISNUMBER($F223))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A223,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E223=INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0)),$F223=INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E223-$F223)=(INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E223&gt;$F223,INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),AND($E223=$F223,INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),AND($E223&lt;$F223,INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0)),IF(AND($E223=INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0)),$F223=INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),IF(AND($H223&lt;&gt;"",$H223=INDEX(Partidos!$K$4:$K$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E223=$F223,($E223-$F223)=(INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0)))),IF(AND($H223&lt;&gt;"",$H223=INDEX(Partidos!$K$4:$K$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H223&lt;&gt;"",$H223=INDEX(Partidos!$K$4:$K$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E223=INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0)),$F223=INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E223-$F223)=(INDEX(Partidos!$F$4:$F$107,MATCH($A223,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H223&lt;&gt;"",$H223=INDEX(Partidos!$K$4:$K$107,MATCH($A223,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H223" s="19">
@@ -19307,7 +19352,7 @@
         <v/>
       </c>
       <c r="G224" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A224,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E224)),NOT(ISNUMBER($F224))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A224,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E224=INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0)),$F224=INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E224-$F224)=(INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E224&gt;$F224,INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),AND($E224=$F224,INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),AND($E224&lt;$F224,INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E224=INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0)),$F224=INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E224-$F224)=(INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H224&lt;&gt;"",$H224=INDEX(Partidos!$K$4:$K$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A224,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E224)),NOT(ISNUMBER($F224))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A224,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E224=INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0)),$F224=INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E224-$F224)=(INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E224&gt;$F224,INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),AND($E224=$F224,INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),AND($E224&lt;$F224,INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0)),IF(AND($E224=INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0)),$F224=INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),IF(AND($H224&lt;&gt;"",$H224=INDEX(Partidos!$K$4:$K$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E224=$F224,($E224-$F224)=(INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0)))),IF(AND($H224&lt;&gt;"",$H224=INDEX(Partidos!$K$4:$K$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H224&lt;&gt;"",$H224=INDEX(Partidos!$K$4:$K$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E224=INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0)),$F224=INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E224-$F224)=(INDEX(Partidos!$F$4:$F$107,MATCH($A224,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H224&lt;&gt;"",$H224=INDEX(Partidos!$K$4:$K$107,MATCH($A224,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H224" s="19">
@@ -19349,7 +19394,7 @@
         <v/>
       </c>
       <c r="G225" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A225,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E225)),NOT(ISNUMBER($F225))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A225,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E225=INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0)),$F225=INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E225-$F225)=(INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E225&gt;$F225,INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),AND($E225=$F225,INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),AND($E225&lt;$F225,INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E225=INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0)),$F225=INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E225-$F225)=(INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H225&lt;&gt;"",$H225=INDEX(Partidos!$K$4:$K$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A225,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E225)),NOT(ISNUMBER($F225))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A225,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E225=INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0)),$F225=INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E225-$F225)=(INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E225&gt;$F225,INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),AND($E225=$F225,INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),AND($E225&lt;$F225,INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0)),IF(AND($E225=INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0)),$F225=INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),IF(AND($H225&lt;&gt;"",$H225=INDEX(Partidos!$K$4:$K$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E225=$F225,($E225-$F225)=(INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0)))),IF(AND($H225&lt;&gt;"",$H225=INDEX(Partidos!$K$4:$K$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H225&lt;&gt;"",$H225=INDEX(Partidos!$K$4:$K$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E225=INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0)),$F225=INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E225-$F225)=(INDEX(Partidos!$F$4:$F$107,MATCH($A225,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H225&lt;&gt;"",$H225=INDEX(Partidos!$K$4:$K$107,MATCH($A225,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H225" s="19">
@@ -19391,7 +19436,7 @@
         <v/>
       </c>
       <c r="G226" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A226,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E226)),NOT(ISNUMBER($F226))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A226,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E226=INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0)),$F226=INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E226-$F226)=(INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E226&gt;$F226,INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),AND($E226=$F226,INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),AND($E226&lt;$F226,INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E226=INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0)),$F226=INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E226-$F226)=(INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H226&lt;&gt;"",$H226=INDEX(Partidos!$K$4:$K$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A226,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E226)),NOT(ISNUMBER($F226))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A226,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E226=INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0)),$F226=INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E226-$F226)=(INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E226&gt;$F226,INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),AND($E226=$F226,INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),AND($E226&lt;$F226,INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0)),IF(AND($E226=INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0)),$F226=INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),IF(AND($H226&lt;&gt;"",$H226=INDEX(Partidos!$K$4:$K$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E226=$F226,($E226-$F226)=(INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0)))),IF(AND($H226&lt;&gt;"",$H226=INDEX(Partidos!$K$4:$K$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H226&lt;&gt;"",$H226=INDEX(Partidos!$K$4:$K$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E226=INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0)),$F226=INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E226-$F226)=(INDEX(Partidos!$F$4:$F$107,MATCH($A226,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H226&lt;&gt;"",$H226=INDEX(Partidos!$K$4:$K$107,MATCH($A226,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H226" s="19">
@@ -19433,7 +19478,7 @@
         <v/>
       </c>
       <c r="G227" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A227,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E227)),NOT(ISNUMBER($F227))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A227,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E227=INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0)),$F227=INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E227-$F227)=(INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E227&gt;$F227,INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),AND($E227=$F227,INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),AND($E227&lt;$F227,INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E227=INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0)),$F227=INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E227-$F227)=(INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H227&lt;&gt;"",$H227=INDEX(Partidos!$K$4:$K$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A227,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E227)),NOT(ISNUMBER($F227))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A227,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E227=INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0)),$F227=INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E227-$F227)=(INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E227&gt;$F227,INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),AND($E227=$F227,INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),AND($E227&lt;$F227,INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0)),IF(AND($E227=INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0)),$F227=INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),IF(AND($H227&lt;&gt;"",$H227=INDEX(Partidos!$K$4:$K$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E227=$F227,($E227-$F227)=(INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0)))),IF(AND($H227&lt;&gt;"",$H227=INDEX(Partidos!$K$4:$K$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H227&lt;&gt;"",$H227=INDEX(Partidos!$K$4:$K$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E227=INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0)),$F227=INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E227-$F227)=(INDEX(Partidos!$F$4:$F$107,MATCH($A227,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H227&lt;&gt;"",$H227=INDEX(Partidos!$K$4:$K$107,MATCH($A227,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H227" s="19">
@@ -19475,7 +19520,7 @@
         <v/>
       </c>
       <c r="G228" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A228,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E228)),NOT(ISNUMBER($F228))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A228,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E228=INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0)),$F228=INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E228-$F228)=(INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E228&gt;$F228,INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),AND($E228=$F228,INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),AND($E228&lt;$F228,INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E228=INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0)),$F228=INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E228-$F228)=(INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H228&lt;&gt;"",$H228=INDEX(Partidos!$K$4:$K$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A228,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E228)),NOT(ISNUMBER($F228))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A228,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E228=INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0)),$F228=INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E228-$F228)=(INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E228&gt;$F228,INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),AND($E228=$F228,INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),AND($E228&lt;$F228,INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0)),IF(AND($E228=INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0)),$F228=INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),IF(AND($H228&lt;&gt;"",$H228=INDEX(Partidos!$K$4:$K$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E228=$F228,($E228-$F228)=(INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0)))),IF(AND($H228&lt;&gt;"",$H228=INDEX(Partidos!$K$4:$K$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H228&lt;&gt;"",$H228=INDEX(Partidos!$K$4:$K$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E228=INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0)),$F228=INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E228-$F228)=(INDEX(Partidos!$F$4:$F$107,MATCH($A228,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H228&lt;&gt;"",$H228=INDEX(Partidos!$K$4:$K$107,MATCH($A228,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H228" s="19">
@@ -19517,7 +19562,7 @@
         <v/>
       </c>
       <c r="G229" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A229,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E229)),NOT(ISNUMBER($F229))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A229,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E229=INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0)),$F229=INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E229-$F229)=(INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E229&gt;$F229,INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),AND($E229=$F229,INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),AND($E229&lt;$F229,INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E229=INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0)),$F229=INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E229-$F229)=(INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H229&lt;&gt;"",$H229=INDEX(Partidos!$K$4:$K$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A229,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E229)),NOT(ISNUMBER($F229))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A229,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E229=INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0)),$F229=INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E229-$F229)=(INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E229&gt;$F229,INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),AND($E229=$F229,INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),AND($E229&lt;$F229,INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0)),IF(AND($E229=INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0)),$F229=INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),IF(AND($H229&lt;&gt;"",$H229=INDEX(Partidos!$K$4:$K$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E229=$F229,($E229-$F229)=(INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0)))),IF(AND($H229&lt;&gt;"",$H229=INDEX(Partidos!$K$4:$K$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H229&lt;&gt;"",$H229=INDEX(Partidos!$K$4:$K$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E229=INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0)),$F229=INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E229-$F229)=(INDEX(Partidos!$F$4:$F$107,MATCH($A229,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H229&lt;&gt;"",$H229=INDEX(Partidos!$K$4:$K$107,MATCH($A229,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H229" s="19">
@@ -19559,7 +19604,7 @@
         <v/>
       </c>
       <c r="G230" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A230,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E230)),NOT(ISNUMBER($F230))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A230,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E230=INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0)),$F230=INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E230-$F230)=(INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E230&gt;$F230,INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),AND($E230=$F230,INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),AND($E230&lt;$F230,INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E230=INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0)),$F230=INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E230-$F230)=(INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H230&lt;&gt;"",$H230=INDEX(Partidos!$K$4:$K$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A230,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E230)),NOT(ISNUMBER($F230))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A230,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E230=INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0)),$F230=INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E230-$F230)=(INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E230&gt;$F230,INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),AND($E230=$F230,INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),AND($E230&lt;$F230,INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0)),IF(AND($E230=INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0)),$F230=INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),IF(AND($H230&lt;&gt;"",$H230=INDEX(Partidos!$K$4:$K$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E230=$F230,($E230-$F230)=(INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0)))),IF(AND($H230&lt;&gt;"",$H230=INDEX(Partidos!$K$4:$K$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H230&lt;&gt;"",$H230=INDEX(Partidos!$K$4:$K$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E230=INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0)),$F230=INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E230-$F230)=(INDEX(Partidos!$F$4:$F$107,MATCH($A230,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H230&lt;&gt;"",$H230=INDEX(Partidos!$K$4:$K$107,MATCH($A230,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H230" s="19">
@@ -19601,7 +19646,7 @@
         <v/>
       </c>
       <c r="G231" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A231,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E231)),NOT(ISNUMBER($F231))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A231,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E231=INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0)),$F231=INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E231-$F231)=(INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E231&gt;$F231,INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),AND($E231=$F231,INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),AND($E231&lt;$F231,INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E231=INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0)),$F231=INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E231-$F231)=(INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H231&lt;&gt;"",$H231=INDEX(Partidos!$K$4:$K$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A231,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E231)),NOT(ISNUMBER($F231))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A231,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E231=INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0)),$F231=INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E231-$F231)=(INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E231&gt;$F231,INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),AND($E231=$F231,INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),AND($E231&lt;$F231,INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0)),IF(AND($E231=INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0)),$F231=INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),IF(AND($H231&lt;&gt;"",$H231=INDEX(Partidos!$K$4:$K$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E231=$F231,($E231-$F231)=(INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0)))),IF(AND($H231&lt;&gt;"",$H231=INDEX(Partidos!$K$4:$K$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H231&lt;&gt;"",$H231=INDEX(Partidos!$K$4:$K$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E231=INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0)),$F231=INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E231-$F231)=(INDEX(Partidos!$F$4:$F$107,MATCH($A231,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H231&lt;&gt;"",$H231=INDEX(Partidos!$K$4:$K$107,MATCH($A231,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H231" s="19">
@@ -19643,7 +19688,7 @@
         <v/>
       </c>
       <c r="G232" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A232,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E232)),NOT(ISNUMBER($F232))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A232,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E232=INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0)),$F232=INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E232-$F232)=(INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E232&gt;$F232,INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),AND($E232=$F232,INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),AND($E232&lt;$F232,INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E232=INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0)),$F232=INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E232-$F232)=(INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H232&lt;&gt;"",$H232=INDEX(Partidos!$K$4:$K$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A232,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E232)),NOT(ISNUMBER($F232))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A232,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E232=INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0)),$F232=INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E232-$F232)=(INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E232&gt;$F232,INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),AND($E232=$F232,INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),AND($E232&lt;$F232,INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0)),IF(AND($E232=INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0)),$F232=INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),IF(AND($H232&lt;&gt;"",$H232=INDEX(Partidos!$K$4:$K$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E232=$F232,($E232-$F232)=(INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0)))),IF(AND($H232&lt;&gt;"",$H232=INDEX(Partidos!$K$4:$K$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H232&lt;&gt;"",$H232=INDEX(Partidos!$K$4:$K$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E232=INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0)),$F232=INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E232-$F232)=(INDEX(Partidos!$F$4:$F$107,MATCH($A232,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H232&lt;&gt;"",$H232=INDEX(Partidos!$K$4:$K$107,MATCH($A232,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H232" s="19">
@@ -19685,7 +19730,7 @@
         <v/>
       </c>
       <c r="G233" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A233,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E233)),NOT(ISNUMBER($F233))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A233,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E233=INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0)),$F233=INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E233-$F233)=(INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E233&gt;$F233,INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),AND($E233=$F233,INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),AND($E233&lt;$F233,INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E233=INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0)),$F233=INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E233-$F233)=(INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H233&lt;&gt;"",$H233=INDEX(Partidos!$K$4:$K$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A233,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E233)),NOT(ISNUMBER($F233))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A233,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E233=INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0)),$F233=INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E233-$F233)=(INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E233&gt;$F233,INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),AND($E233=$F233,INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),AND($E233&lt;$F233,INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0)),IF(AND($E233=INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0)),$F233=INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),IF(AND($H233&lt;&gt;"",$H233=INDEX(Partidos!$K$4:$K$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E233=$F233,($E233-$F233)=(INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0)))),IF(AND($H233&lt;&gt;"",$H233=INDEX(Partidos!$K$4:$K$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H233&lt;&gt;"",$H233=INDEX(Partidos!$K$4:$K$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E233=INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0)),$F233=INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E233-$F233)=(INDEX(Partidos!$F$4:$F$107,MATCH($A233,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H233&lt;&gt;"",$H233=INDEX(Partidos!$K$4:$K$107,MATCH($A233,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H233" s="19">
@@ -19727,7 +19772,7 @@
         <v/>
       </c>
       <c r="G234" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A234,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E234)),NOT(ISNUMBER($F234))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A234,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E234=INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0)),$F234=INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E234-$F234)=(INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E234&gt;$F234,INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),AND($E234=$F234,INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),AND($E234&lt;$F234,INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E234=INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0)),$F234=INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E234-$F234)=(INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H234&lt;&gt;"",$H234=INDEX(Partidos!$K$4:$K$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A234,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E234)),NOT(ISNUMBER($F234))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A234,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E234=INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0)),$F234=INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E234-$F234)=(INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E234&gt;$F234,INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),AND($E234=$F234,INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),AND($E234&lt;$F234,INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0)),IF(AND($E234=INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0)),$F234=INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),IF(AND($H234&lt;&gt;"",$H234=INDEX(Partidos!$K$4:$K$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E234=$F234,($E234-$F234)=(INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0)))),IF(AND($H234&lt;&gt;"",$H234=INDEX(Partidos!$K$4:$K$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H234&lt;&gt;"",$H234=INDEX(Partidos!$K$4:$K$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E234=INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0)),$F234=INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E234-$F234)=(INDEX(Partidos!$F$4:$F$107,MATCH($A234,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H234&lt;&gt;"",$H234=INDEX(Partidos!$K$4:$K$107,MATCH($A234,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H234" s="19">
@@ -19769,7 +19814,7 @@
         <v/>
       </c>
       <c r="G235" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A235,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E235)),NOT(ISNUMBER($F235))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A235,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E235=INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0)),$F235=INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E235-$F235)=(INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E235&gt;$F235,INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),AND($E235=$F235,INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),AND($E235&lt;$F235,INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E235=INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0)),$F235=INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E235-$F235)=(INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H235&lt;&gt;"",$H235=INDEX(Partidos!$K$4:$K$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A235,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E235)),NOT(ISNUMBER($F235))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A235,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E235=INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0)),$F235=INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E235-$F235)=(INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E235&gt;$F235,INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),AND($E235=$F235,INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),AND($E235&lt;$F235,INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0)),IF(AND($E235=INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0)),$F235=INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),IF(AND($H235&lt;&gt;"",$H235=INDEX(Partidos!$K$4:$K$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E235=$F235,($E235-$F235)=(INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0)))),IF(AND($H235&lt;&gt;"",$H235=INDEX(Partidos!$K$4:$K$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H235&lt;&gt;"",$H235=INDEX(Partidos!$K$4:$K$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E235=INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0)),$F235=INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E235-$F235)=(INDEX(Partidos!$F$4:$F$107,MATCH($A235,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H235&lt;&gt;"",$H235=INDEX(Partidos!$K$4:$K$107,MATCH($A235,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H235" s="19">
@@ -19811,7 +19856,7 @@
         <v/>
       </c>
       <c r="G236" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A236,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E236)),NOT(ISNUMBER($F236))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A236,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E236=INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0)),$F236=INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E236-$F236)=(INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E236&gt;$F236,INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),AND($E236=$F236,INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),AND($E236&lt;$F236,INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E236=INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0)),$F236=INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E236-$F236)=(INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H236&lt;&gt;"",$H236=INDEX(Partidos!$K$4:$K$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A236,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E236)),NOT(ISNUMBER($F236))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A236,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E236=INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0)),$F236=INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E236-$F236)=(INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E236&gt;$F236,INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),AND($E236=$F236,INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),AND($E236&lt;$F236,INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0)),IF(AND($E236=INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0)),$F236=INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),IF(AND($H236&lt;&gt;"",$H236=INDEX(Partidos!$K$4:$K$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E236=$F236,($E236-$F236)=(INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0)))),IF(AND($H236&lt;&gt;"",$H236=INDEX(Partidos!$K$4:$K$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H236&lt;&gt;"",$H236=INDEX(Partidos!$K$4:$K$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E236=INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0)),$F236=INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E236-$F236)=(INDEX(Partidos!$F$4:$F$107,MATCH($A236,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H236&lt;&gt;"",$H236=INDEX(Partidos!$K$4:$K$107,MATCH($A236,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H236" s="19">
@@ -19853,7 +19898,7 @@
         <v/>
       </c>
       <c r="G237" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A237,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E237)),NOT(ISNUMBER($F237))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A237,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E237=INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0)),$F237=INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E237-$F237)=(INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E237&gt;$F237,INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),AND($E237=$F237,INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),AND($E237&lt;$F237,INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E237=INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0)),$F237=INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E237-$F237)=(INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H237&lt;&gt;"",$H237=INDEX(Partidos!$K$4:$K$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A237,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E237)),NOT(ISNUMBER($F237))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A237,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E237=INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0)),$F237=INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E237-$F237)=(INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E237&gt;$F237,INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),AND($E237=$F237,INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),AND($E237&lt;$F237,INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0)),IF(AND($E237=INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0)),$F237=INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),IF(AND($H237&lt;&gt;"",$H237=INDEX(Partidos!$K$4:$K$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E237=$F237,($E237-$F237)=(INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0)))),IF(AND($H237&lt;&gt;"",$H237=INDEX(Partidos!$K$4:$K$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H237&lt;&gt;"",$H237=INDEX(Partidos!$K$4:$K$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E237=INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0)),$F237=INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E237-$F237)=(INDEX(Partidos!$F$4:$F$107,MATCH($A237,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H237&lt;&gt;"",$H237=INDEX(Partidos!$K$4:$K$107,MATCH($A237,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H237" s="19">
@@ -19895,7 +19940,7 @@
         <v/>
       </c>
       <c r="G238" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A238,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E238)),NOT(ISNUMBER($F238))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A238,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E238=INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0)),$F238=INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E238-$F238)=(INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E238&gt;$F238,INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),AND($E238=$F238,INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),AND($E238&lt;$F238,INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E238=INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0)),$F238=INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E238-$F238)=(INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H238&lt;&gt;"",$H238=INDEX(Partidos!$K$4:$K$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A238,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E238)),NOT(ISNUMBER($F238))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A238,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E238=INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0)),$F238=INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E238-$F238)=(INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E238&gt;$F238,INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),AND($E238=$F238,INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),AND($E238&lt;$F238,INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0)),IF(AND($E238=INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0)),$F238=INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),IF(AND($H238&lt;&gt;"",$H238=INDEX(Partidos!$K$4:$K$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E238=$F238,($E238-$F238)=(INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0)))),IF(AND($H238&lt;&gt;"",$H238=INDEX(Partidos!$K$4:$K$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H238&lt;&gt;"",$H238=INDEX(Partidos!$K$4:$K$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E238=INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0)),$F238=INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E238-$F238)=(INDEX(Partidos!$F$4:$F$107,MATCH($A238,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H238&lt;&gt;"",$H238=INDEX(Partidos!$K$4:$K$107,MATCH($A238,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H238" s="19">
@@ -19937,7 +19982,7 @@
         <v/>
       </c>
       <c r="G239" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A239,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E239)),NOT(ISNUMBER($F239))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A239,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E239=INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0)),$F239=INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E239-$F239)=(INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E239&gt;$F239,INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),AND($E239=$F239,INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),AND($E239&lt;$F239,INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E239=INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0)),$F239=INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E239-$F239)=(INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H239&lt;&gt;"",$H239=INDEX(Partidos!$K$4:$K$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A239,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E239)),NOT(ISNUMBER($F239))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A239,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E239=INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0)),$F239=INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E239-$F239)=(INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E239&gt;$F239,INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),AND($E239=$F239,INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),AND($E239&lt;$F239,INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0)),IF(AND($E239=INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0)),$F239=INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),IF(AND($H239&lt;&gt;"",$H239=INDEX(Partidos!$K$4:$K$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E239=$F239,($E239-$F239)=(INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0)))),IF(AND($H239&lt;&gt;"",$H239=INDEX(Partidos!$K$4:$K$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H239&lt;&gt;"",$H239=INDEX(Partidos!$K$4:$K$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E239=INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0)),$F239=INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E239-$F239)=(INDEX(Partidos!$F$4:$F$107,MATCH($A239,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H239&lt;&gt;"",$H239=INDEX(Partidos!$K$4:$K$107,MATCH($A239,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H239" s="19">
@@ -19979,7 +20024,7 @@
         <v/>
       </c>
       <c r="G240" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A240,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E240)),NOT(ISNUMBER($F240))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A240,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E240=INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0)),$F240=INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E240-$F240)=(INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E240&gt;$F240,INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),AND($E240=$F240,INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),AND($E240&lt;$F240,INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E240=INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0)),$F240=INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E240-$F240)=(INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H240&lt;&gt;"",$H240=INDEX(Partidos!$K$4:$K$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A240,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E240)),NOT(ISNUMBER($F240))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A240,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E240=INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0)),$F240=INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E240-$F240)=(INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E240&gt;$F240,INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),AND($E240=$F240,INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),AND($E240&lt;$F240,INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0)),IF(AND($E240=INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0)),$F240=INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),IF(AND($H240&lt;&gt;"",$H240=INDEX(Partidos!$K$4:$K$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E240=$F240,($E240-$F240)=(INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0)))),IF(AND($H240&lt;&gt;"",$H240=INDEX(Partidos!$K$4:$K$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H240&lt;&gt;"",$H240=INDEX(Partidos!$K$4:$K$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E240=INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0)),$F240=INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E240-$F240)=(INDEX(Partidos!$F$4:$F$107,MATCH($A240,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H240&lt;&gt;"",$H240=INDEX(Partidos!$K$4:$K$107,MATCH($A240,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H240" s="19">
@@ -20021,7 +20066,7 @@
         <v/>
       </c>
       <c r="G241" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A241,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E241)),NOT(ISNUMBER($F241))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A241,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E241=INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0)),$F241=INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E241-$F241)=(INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E241&gt;$F241,INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),AND($E241=$F241,INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),AND($E241&lt;$F241,INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E241=INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0)),$F241=INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E241-$F241)=(INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H241&lt;&gt;"",$H241=INDEX(Partidos!$K$4:$K$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A241,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E241)),NOT(ISNUMBER($F241))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A241,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E241=INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0)),$F241=INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E241-$F241)=(INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E241&gt;$F241,INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),AND($E241=$F241,INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),AND($E241&lt;$F241,INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0)),IF(AND($E241=INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0)),$F241=INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),IF(AND($H241&lt;&gt;"",$H241=INDEX(Partidos!$K$4:$K$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E241=$F241,($E241-$F241)=(INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0)))),IF(AND($H241&lt;&gt;"",$H241=INDEX(Partidos!$K$4:$K$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H241&lt;&gt;"",$H241=INDEX(Partidos!$K$4:$K$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E241=INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0)),$F241=INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E241-$F241)=(INDEX(Partidos!$F$4:$F$107,MATCH($A241,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H241&lt;&gt;"",$H241=INDEX(Partidos!$K$4:$K$107,MATCH($A241,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H241" s="19">
@@ -20063,7 +20108,7 @@
         <v/>
       </c>
       <c r="G242" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A242,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E242)),NOT(ISNUMBER($F242))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A242,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E242=INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0)),$F242=INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E242-$F242)=(INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E242&gt;$F242,INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),AND($E242=$F242,INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),AND($E242&lt;$F242,INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E242=INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0)),$F242=INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E242-$F242)=(INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H242&lt;&gt;"",$H242=INDEX(Partidos!$K$4:$K$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A242,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E242)),NOT(ISNUMBER($F242))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A242,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E242=INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0)),$F242=INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E242-$F242)=(INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E242&gt;$F242,INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),AND($E242=$F242,INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),AND($E242&lt;$F242,INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0)),IF(AND($E242=INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0)),$F242=INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),IF(AND($H242&lt;&gt;"",$H242=INDEX(Partidos!$K$4:$K$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E242=$F242,($E242-$F242)=(INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0)))),IF(AND($H242&lt;&gt;"",$H242=INDEX(Partidos!$K$4:$K$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H242&lt;&gt;"",$H242=INDEX(Partidos!$K$4:$K$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E242=INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0)),$F242=INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E242-$F242)=(INDEX(Partidos!$F$4:$F$107,MATCH($A242,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H242&lt;&gt;"",$H242=INDEX(Partidos!$K$4:$K$107,MATCH($A242,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H242" s="19">
@@ -20105,7 +20150,7 @@
         <v/>
       </c>
       <c r="G243" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A243,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E243)),NOT(ISNUMBER($F243))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A243,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E243=INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0)),$F243=INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E243-$F243)=(INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E243&gt;$F243,INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),AND($E243=$F243,INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),AND($E243&lt;$F243,INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E243=INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0)),$F243=INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E243-$F243)=(INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H243&lt;&gt;"",$H243=INDEX(Partidos!$K$4:$K$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A243,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E243)),NOT(ISNUMBER($F243))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A243,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E243=INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0)),$F243=INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E243-$F243)=(INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E243&gt;$F243,INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),AND($E243=$F243,INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),AND($E243&lt;$F243,INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0)),IF(AND($E243=INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0)),$F243=INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),IF(AND($H243&lt;&gt;"",$H243=INDEX(Partidos!$K$4:$K$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E243=$F243,($E243-$F243)=(INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0)))),IF(AND($H243&lt;&gt;"",$H243=INDEX(Partidos!$K$4:$K$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H243&lt;&gt;"",$H243=INDEX(Partidos!$K$4:$K$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E243=INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0)),$F243=INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E243-$F243)=(INDEX(Partidos!$F$4:$F$107,MATCH($A243,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H243&lt;&gt;"",$H243=INDEX(Partidos!$K$4:$K$107,MATCH($A243,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H243" s="19">
@@ -20147,7 +20192,7 @@
         <v/>
       </c>
       <c r="G244" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A244,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E244)),NOT(ISNUMBER($F244))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A244,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E244=INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0)),$F244=INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E244-$F244)=(INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E244&gt;$F244,INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),AND($E244=$F244,INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),AND($E244&lt;$F244,INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E244=INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0)),$F244=INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E244-$F244)=(INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H244&lt;&gt;"",$H244=INDEX(Partidos!$K$4:$K$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A244,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E244)),NOT(ISNUMBER($F244))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A244,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E244=INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0)),$F244=INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E244-$F244)=(INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E244&gt;$F244,INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),AND($E244=$F244,INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),AND($E244&lt;$F244,INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0)),IF(AND($E244=INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0)),$F244=INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),IF(AND($H244&lt;&gt;"",$H244=INDEX(Partidos!$K$4:$K$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E244=$F244,($E244-$F244)=(INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0)))),IF(AND($H244&lt;&gt;"",$H244=INDEX(Partidos!$K$4:$K$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H244&lt;&gt;"",$H244=INDEX(Partidos!$K$4:$K$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E244=INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0)),$F244=INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E244-$F244)=(INDEX(Partidos!$F$4:$F$107,MATCH($A244,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H244&lt;&gt;"",$H244=INDEX(Partidos!$K$4:$K$107,MATCH($A244,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H244" s="19">
@@ -20189,7 +20234,7 @@
         <v/>
       </c>
       <c r="G245" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A245,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E245)),NOT(ISNUMBER($F245))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A245,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E245=INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0)),$F245=INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E245-$F245)=(INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E245&gt;$F245,INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),AND($E245=$F245,INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),AND($E245&lt;$F245,INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E245=INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0)),$F245=INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E245-$F245)=(INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H245&lt;&gt;"",$H245=INDEX(Partidos!$K$4:$K$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A245,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E245)),NOT(ISNUMBER($F245))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A245,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E245=INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0)),$F245=INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E245-$F245)=(INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E245&gt;$F245,INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),AND($E245=$F245,INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),AND($E245&lt;$F245,INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0)),IF(AND($E245=INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0)),$F245=INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),IF(AND($H245&lt;&gt;"",$H245=INDEX(Partidos!$K$4:$K$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E245=$F245,($E245-$F245)=(INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0)))),IF(AND($H245&lt;&gt;"",$H245=INDEX(Partidos!$K$4:$K$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H245&lt;&gt;"",$H245=INDEX(Partidos!$K$4:$K$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E245=INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0)),$F245=INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E245-$F245)=(INDEX(Partidos!$F$4:$F$107,MATCH($A245,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H245&lt;&gt;"",$H245=INDEX(Partidos!$K$4:$K$107,MATCH($A245,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H245" s="19">
@@ -20231,7 +20276,7 @@
         <v/>
       </c>
       <c r="G246" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A246,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E246)),NOT(ISNUMBER($F246))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A246,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E246=INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0)),$F246=INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E246-$F246)=(INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E246&gt;$F246,INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),AND($E246=$F246,INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),AND($E246&lt;$F246,INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E246=INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0)),$F246=INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E246-$F246)=(INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H246&lt;&gt;"",$H246=INDEX(Partidos!$K$4:$K$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A246,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E246)),NOT(ISNUMBER($F246))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A246,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E246=INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0)),$F246=INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E246-$F246)=(INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E246&gt;$F246,INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),AND($E246=$F246,INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),AND($E246&lt;$F246,INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0)),IF(AND($E246=INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0)),$F246=INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),IF(AND($H246&lt;&gt;"",$H246=INDEX(Partidos!$K$4:$K$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E246=$F246,($E246-$F246)=(INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0)))),IF(AND($H246&lt;&gt;"",$H246=INDEX(Partidos!$K$4:$K$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H246&lt;&gt;"",$H246=INDEX(Partidos!$K$4:$K$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E246=INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0)),$F246=INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E246-$F246)=(INDEX(Partidos!$F$4:$F$107,MATCH($A246,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H246&lt;&gt;"",$H246=INDEX(Partidos!$K$4:$K$107,MATCH($A246,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H246" s="19">
@@ -20273,7 +20318,7 @@
         <v/>
       </c>
       <c r="G247" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A247,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E247)),NOT(ISNUMBER($F247))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A247,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E247=INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0)),$F247=INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E247-$F247)=(INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E247&gt;$F247,INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),AND($E247=$F247,INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),AND($E247&lt;$F247,INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E247=INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0)),$F247=INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E247-$F247)=(INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H247&lt;&gt;"",$H247=INDEX(Partidos!$K$4:$K$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A247,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E247)),NOT(ISNUMBER($F247))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A247,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E247=INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0)),$F247=INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E247-$F247)=(INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E247&gt;$F247,INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),AND($E247=$F247,INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),AND($E247&lt;$F247,INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0)),IF(AND($E247=INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0)),$F247=INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),IF(AND($H247&lt;&gt;"",$H247=INDEX(Partidos!$K$4:$K$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E247=$F247,($E247-$F247)=(INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0)))),IF(AND($H247&lt;&gt;"",$H247=INDEX(Partidos!$K$4:$K$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H247&lt;&gt;"",$H247=INDEX(Partidos!$K$4:$K$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E247=INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0)),$F247=INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E247-$F247)=(INDEX(Partidos!$F$4:$F$107,MATCH($A247,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H247&lt;&gt;"",$H247=INDEX(Partidos!$K$4:$K$107,MATCH($A247,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H247" s="19">
@@ -20315,7 +20360,7 @@
         <v/>
       </c>
       <c r="G248" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A248,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E248)),NOT(ISNUMBER($F248))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A248,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E248=INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0)),$F248=INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E248-$F248)=(INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E248&gt;$F248,INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),AND($E248=$F248,INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),AND($E248&lt;$F248,INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E248=INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0)),$F248=INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E248-$F248)=(INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H248&lt;&gt;"",$H248=INDEX(Partidos!$K$4:$K$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A248,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E248)),NOT(ISNUMBER($F248))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A248,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E248=INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0)),$F248=INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E248-$F248)=(INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E248&gt;$F248,INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),AND($E248=$F248,INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),AND($E248&lt;$F248,INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0)),IF(AND($E248=INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0)),$F248=INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),IF(AND($H248&lt;&gt;"",$H248=INDEX(Partidos!$K$4:$K$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E248=$F248,($E248-$F248)=(INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0)))),IF(AND($H248&lt;&gt;"",$H248=INDEX(Partidos!$K$4:$K$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H248&lt;&gt;"",$H248=INDEX(Partidos!$K$4:$K$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E248=INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0)),$F248=INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E248-$F248)=(INDEX(Partidos!$F$4:$F$107,MATCH($A248,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H248&lt;&gt;"",$H248=INDEX(Partidos!$K$4:$K$107,MATCH($A248,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H248" s="19">
@@ -20357,7 +20402,7 @@
         <v/>
       </c>
       <c r="G249" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A249,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E249)),NOT(ISNUMBER($F249))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A249,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E249=INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0)),$F249=INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E249-$F249)=(INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E249&gt;$F249,INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),AND($E249=$F249,INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),AND($E249&lt;$F249,INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E249=INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0)),$F249=INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E249-$F249)=(INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H249&lt;&gt;"",$H249=INDEX(Partidos!$K$4:$K$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A249,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E249)),NOT(ISNUMBER($F249))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A249,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E249=INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0)),$F249=INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E249-$F249)=(INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E249&gt;$F249,INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),AND($E249=$F249,INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),AND($E249&lt;$F249,INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0)),IF(AND($E249=INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0)),$F249=INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),IF(AND($H249&lt;&gt;"",$H249=INDEX(Partidos!$K$4:$K$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E249=$F249,($E249-$F249)=(INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0)))),IF(AND($H249&lt;&gt;"",$H249=INDEX(Partidos!$K$4:$K$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H249&lt;&gt;"",$H249=INDEX(Partidos!$K$4:$K$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E249=INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0)),$F249=INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E249-$F249)=(INDEX(Partidos!$F$4:$F$107,MATCH($A249,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H249&lt;&gt;"",$H249=INDEX(Partidos!$K$4:$K$107,MATCH($A249,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H249" s="19">
@@ -20399,7 +20444,7 @@
         <v/>
       </c>
       <c r="G250" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A250,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E250)),NOT(ISNUMBER($F250))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A250,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E250=INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0)),$F250=INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E250-$F250)=(INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E250&gt;$F250,INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),AND($E250=$F250,INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),AND($E250&lt;$F250,INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E250=INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0)),$F250=INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E250-$F250)=(INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H250&lt;&gt;"",$H250=INDEX(Partidos!$K$4:$K$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A250,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E250)),NOT(ISNUMBER($F250))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A250,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E250=INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0)),$F250=INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E250-$F250)=(INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E250&gt;$F250,INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),AND($E250=$F250,INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),AND($E250&lt;$F250,INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0)),IF(AND($E250=INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0)),$F250=INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),IF(AND($H250&lt;&gt;"",$H250=INDEX(Partidos!$K$4:$K$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E250=$F250,($E250-$F250)=(INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0)))),IF(AND($H250&lt;&gt;"",$H250=INDEX(Partidos!$K$4:$K$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H250&lt;&gt;"",$H250=INDEX(Partidos!$K$4:$K$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E250=INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0)),$F250=INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E250-$F250)=(INDEX(Partidos!$F$4:$F$107,MATCH($A250,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H250&lt;&gt;"",$H250=INDEX(Partidos!$K$4:$K$107,MATCH($A250,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H250" s="19">
@@ -20441,7 +20486,7 @@
         <v/>
       </c>
       <c r="G251" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A251,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E251)),NOT(ISNUMBER($F251))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A251,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E251=INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0)),$F251=INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E251-$F251)=(INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E251&gt;$F251,INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),AND($E251=$F251,INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),AND($E251&lt;$F251,INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E251=INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0)),$F251=INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E251-$F251)=(INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H251&lt;&gt;"",$H251=INDEX(Partidos!$K$4:$K$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A251,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E251)),NOT(ISNUMBER($F251))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A251,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E251=INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0)),$F251=INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E251-$F251)=(INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E251&gt;$F251,INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),AND($E251=$F251,INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),AND($E251&lt;$F251,INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0)),IF(AND($E251=INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0)),$F251=INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),IF(AND($H251&lt;&gt;"",$H251=INDEX(Partidos!$K$4:$K$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E251=$F251,($E251-$F251)=(INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0)))),IF(AND($H251&lt;&gt;"",$H251=INDEX(Partidos!$K$4:$K$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H251&lt;&gt;"",$H251=INDEX(Partidos!$K$4:$K$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E251=INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0)),$F251=INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E251-$F251)=(INDEX(Partidos!$F$4:$F$107,MATCH($A251,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H251&lt;&gt;"",$H251=INDEX(Partidos!$K$4:$K$107,MATCH($A251,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H251" s="19">
@@ -20483,7 +20528,7 @@
         <v/>
       </c>
       <c r="G252" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A252,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E252)),NOT(ISNUMBER($F252))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A252,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E252=INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0)),$F252=INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E252-$F252)=(INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E252&gt;$F252,INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),AND($E252=$F252,INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),AND($E252&lt;$F252,INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E252=INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0)),$F252=INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E252-$F252)=(INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H252&lt;&gt;"",$H252=INDEX(Partidos!$K$4:$K$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A252,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E252)),NOT(ISNUMBER($F252))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A252,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E252=INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0)),$F252=INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E252-$F252)=(INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E252&gt;$F252,INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),AND($E252=$F252,INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),AND($E252&lt;$F252,INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0)),IF(AND($E252=INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0)),$F252=INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),IF(AND($H252&lt;&gt;"",$H252=INDEX(Partidos!$K$4:$K$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E252=$F252,($E252-$F252)=(INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0)))),IF(AND($H252&lt;&gt;"",$H252=INDEX(Partidos!$K$4:$K$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H252&lt;&gt;"",$H252=INDEX(Partidos!$K$4:$K$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E252=INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0)),$F252=INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E252-$F252)=(INDEX(Partidos!$F$4:$F$107,MATCH($A252,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H252&lt;&gt;"",$H252=INDEX(Partidos!$K$4:$K$107,MATCH($A252,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H252" s="19">
@@ -20525,7 +20570,7 @@
         <v/>
       </c>
       <c r="G253" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A253,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E253)),NOT(ISNUMBER($F253))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A253,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E253=INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0)),$F253=INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E253-$F253)=(INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E253&gt;$F253,INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),AND($E253=$F253,INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),AND($E253&lt;$F253,INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E253=INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0)),$F253=INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E253-$F253)=(INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H253&lt;&gt;"",$H253=INDEX(Partidos!$K$4:$K$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A253,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E253)),NOT(ISNUMBER($F253))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A253,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E253=INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0)),$F253=INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E253-$F253)=(INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E253&gt;$F253,INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),AND($E253=$F253,INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),AND($E253&lt;$F253,INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0)),IF(AND($E253=INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0)),$F253=INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),IF(AND($H253&lt;&gt;"",$H253=INDEX(Partidos!$K$4:$K$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E253=$F253,($E253-$F253)=(INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0)))),IF(AND($H253&lt;&gt;"",$H253=INDEX(Partidos!$K$4:$K$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H253&lt;&gt;"",$H253=INDEX(Partidos!$K$4:$K$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E253=INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0)),$F253=INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E253-$F253)=(INDEX(Partidos!$F$4:$F$107,MATCH($A253,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H253&lt;&gt;"",$H253=INDEX(Partidos!$K$4:$K$107,MATCH($A253,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H253" s="19">
@@ -20567,7 +20612,7 @@
         <v/>
       </c>
       <c r="G254" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A254,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E254)),NOT(ISNUMBER($F254))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A254,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E254=INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0)),$F254=INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E254-$F254)=(INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E254&gt;$F254,INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),AND($E254=$F254,INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),AND($E254&lt;$F254,INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E254=INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0)),$F254=INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E254-$F254)=(INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H254&lt;&gt;"",$H254=INDEX(Partidos!$K$4:$K$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A254,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E254)),NOT(ISNUMBER($F254))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A254,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E254=INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0)),$F254=INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E254-$F254)=(INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E254&gt;$F254,INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),AND($E254=$F254,INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),AND($E254&lt;$F254,INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0)),IF(AND($E254=INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0)),$F254=INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),IF(AND($H254&lt;&gt;"",$H254=INDEX(Partidos!$K$4:$K$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E254=$F254,($E254-$F254)=(INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0)))),IF(AND($H254&lt;&gt;"",$H254=INDEX(Partidos!$K$4:$K$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H254&lt;&gt;"",$H254=INDEX(Partidos!$K$4:$K$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E254=INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0)),$F254=INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E254-$F254)=(INDEX(Partidos!$F$4:$F$107,MATCH($A254,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H254&lt;&gt;"",$H254=INDEX(Partidos!$K$4:$K$107,MATCH($A254,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H254" s="19">
@@ -20609,7 +20654,7 @@
         <v/>
       </c>
       <c r="G255" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A255,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E255)),NOT(ISNUMBER($F255))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A255,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E255=INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0)),$F255=INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E255-$F255)=(INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E255&gt;$F255,INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),AND($E255=$F255,INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),AND($E255&lt;$F255,INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E255=INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0)),$F255=INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E255-$F255)=(INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H255&lt;&gt;"",$H255=INDEX(Partidos!$K$4:$K$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A255,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E255)),NOT(ISNUMBER($F255))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A255,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E255=INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0)),$F255=INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E255-$F255)=(INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E255&gt;$F255,INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),AND($E255=$F255,INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),AND($E255&lt;$F255,INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0)),IF(AND($E255=INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0)),$F255=INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),IF(AND($H255&lt;&gt;"",$H255=INDEX(Partidos!$K$4:$K$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E255=$F255,($E255-$F255)=(INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0)))),IF(AND($H255&lt;&gt;"",$H255=INDEX(Partidos!$K$4:$K$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H255&lt;&gt;"",$H255=INDEX(Partidos!$K$4:$K$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E255=INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0)),$F255=INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E255-$F255)=(INDEX(Partidos!$F$4:$F$107,MATCH($A255,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H255&lt;&gt;"",$H255=INDEX(Partidos!$K$4:$K$107,MATCH($A255,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H255" s="19">
@@ -20651,7 +20696,7 @@
         <v/>
       </c>
       <c r="G256" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A256,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E256)),NOT(ISNUMBER($F256))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A256,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E256=INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0)),$F256=INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E256-$F256)=(INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E256&gt;$F256,INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),AND($E256=$F256,INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),AND($E256&lt;$F256,INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E256=INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0)),$F256=INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E256-$F256)=(INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H256&lt;&gt;"",$H256=INDEX(Partidos!$K$4:$K$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A256,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E256)),NOT(ISNUMBER($F256))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A256,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E256=INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0)),$F256=INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E256-$F256)=(INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E256&gt;$F256,INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),AND($E256=$F256,INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),AND($E256&lt;$F256,INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0)),IF(AND($E256=INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0)),$F256=INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),IF(AND($H256&lt;&gt;"",$H256=INDEX(Partidos!$K$4:$K$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E256=$F256,($E256-$F256)=(INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0)))),IF(AND($H256&lt;&gt;"",$H256=INDEX(Partidos!$K$4:$K$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H256&lt;&gt;"",$H256=INDEX(Partidos!$K$4:$K$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E256=INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0)),$F256=INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E256-$F256)=(INDEX(Partidos!$F$4:$F$107,MATCH($A256,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H256&lt;&gt;"",$H256=INDEX(Partidos!$K$4:$K$107,MATCH($A256,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H256" s="19">
@@ -20693,7 +20738,7 @@
         <v/>
       </c>
       <c r="G257" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A257,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E257)),NOT(ISNUMBER($F257))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A257,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E257=INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0)),$F257=INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E257-$F257)=(INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E257&gt;$F257,INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),AND($E257=$F257,INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),AND($E257&lt;$F257,INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E257=INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0)),$F257=INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E257-$F257)=(INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H257&lt;&gt;"",$H257=INDEX(Partidos!$K$4:$K$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A257,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E257)),NOT(ISNUMBER($F257))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A257,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E257=INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0)),$F257=INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E257-$F257)=(INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E257&gt;$F257,INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),AND($E257=$F257,INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),AND($E257&lt;$F257,INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0)),IF(AND($E257=INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0)),$F257=INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),IF(AND($H257&lt;&gt;"",$H257=INDEX(Partidos!$K$4:$K$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E257=$F257,($E257-$F257)=(INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0)))),IF(AND($H257&lt;&gt;"",$H257=INDEX(Partidos!$K$4:$K$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H257&lt;&gt;"",$H257=INDEX(Partidos!$K$4:$K$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E257=INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0)),$F257=INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E257-$F257)=(INDEX(Partidos!$F$4:$F$107,MATCH($A257,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H257&lt;&gt;"",$H257=INDEX(Partidos!$K$4:$K$107,MATCH($A257,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H257" s="19">
@@ -20735,7 +20780,7 @@
         <v/>
       </c>
       <c r="G258" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A258,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E258)),NOT(ISNUMBER($F258))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A258,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E258=INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0)),$F258=INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E258-$F258)=(INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E258&gt;$F258,INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),AND($E258=$F258,INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),AND($E258&lt;$F258,INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E258=INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0)),$F258=INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E258-$F258)=(INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H258&lt;&gt;"",$H258=INDEX(Partidos!$K$4:$K$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A258,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E258)),NOT(ISNUMBER($F258))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A258,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E258=INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0)),$F258=INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E258-$F258)=(INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E258&gt;$F258,INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),AND($E258=$F258,INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),AND($E258&lt;$F258,INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0)),IF(AND($E258=INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0)),$F258=INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),IF(AND($H258&lt;&gt;"",$H258=INDEX(Partidos!$K$4:$K$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E258=$F258,($E258-$F258)=(INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0)))),IF(AND($H258&lt;&gt;"",$H258=INDEX(Partidos!$K$4:$K$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H258&lt;&gt;"",$H258=INDEX(Partidos!$K$4:$K$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E258=INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0)),$F258=INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E258-$F258)=(INDEX(Partidos!$F$4:$F$107,MATCH($A258,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H258&lt;&gt;"",$H258=INDEX(Partidos!$K$4:$K$107,MATCH($A258,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H258" s="19">
@@ -20777,7 +20822,7 @@
         <v/>
       </c>
       <c r="G259" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A259,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E259)),NOT(ISNUMBER($F259))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A259,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E259=INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0)),$F259=INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E259-$F259)=(INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E259&gt;$F259,INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),AND($E259=$F259,INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),AND($E259&lt;$F259,INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E259=INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0)),$F259=INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E259-$F259)=(INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H259&lt;&gt;"",$H259=INDEX(Partidos!$K$4:$K$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A259,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E259)),NOT(ISNUMBER($F259))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A259,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E259=INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0)),$F259=INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E259-$F259)=(INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E259&gt;$F259,INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),AND($E259=$F259,INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),AND($E259&lt;$F259,INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0)),IF(AND($E259=INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0)),$F259=INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),IF(AND($H259&lt;&gt;"",$H259=INDEX(Partidos!$K$4:$K$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E259=$F259,($E259-$F259)=(INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0)))),IF(AND($H259&lt;&gt;"",$H259=INDEX(Partidos!$K$4:$K$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H259&lt;&gt;"",$H259=INDEX(Partidos!$K$4:$K$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E259=INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0)),$F259=INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E259-$F259)=(INDEX(Partidos!$F$4:$F$107,MATCH($A259,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H259&lt;&gt;"",$H259=INDEX(Partidos!$K$4:$K$107,MATCH($A259,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H259" s="19">
@@ -20819,7 +20864,7 @@
         <v/>
       </c>
       <c r="G260" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A260,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E260)),NOT(ISNUMBER($F260))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A260,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E260=INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0)),$F260=INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E260-$F260)=(INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E260&gt;$F260,INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),AND($E260=$F260,INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),AND($E260&lt;$F260,INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E260=INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0)),$F260=INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E260-$F260)=(INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H260&lt;&gt;"",$H260=INDEX(Partidos!$K$4:$K$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A260,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E260)),NOT(ISNUMBER($F260))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A260,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E260=INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0)),$F260=INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E260-$F260)=(INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E260&gt;$F260,INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),AND($E260=$F260,INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),AND($E260&lt;$F260,INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0)),IF(AND($E260=INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0)),$F260=INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),IF(AND($H260&lt;&gt;"",$H260=INDEX(Partidos!$K$4:$K$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E260=$F260,($E260-$F260)=(INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0)))),IF(AND($H260&lt;&gt;"",$H260=INDEX(Partidos!$K$4:$K$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H260&lt;&gt;"",$H260=INDEX(Partidos!$K$4:$K$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E260=INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0)),$F260=INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E260-$F260)=(INDEX(Partidos!$F$4:$F$107,MATCH($A260,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H260&lt;&gt;"",$H260=INDEX(Partidos!$K$4:$K$107,MATCH($A260,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H260" s="19">
@@ -20861,7 +20906,7 @@
         <v/>
       </c>
       <c r="G261" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A261,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E261)),NOT(ISNUMBER($F261))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A261,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E261=INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0)),$F261=INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E261-$F261)=(INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E261&gt;$F261,INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),AND($E261=$F261,INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),AND($E261&lt;$F261,INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E261=INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0)),$F261=INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E261-$F261)=(INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H261&lt;&gt;"",$H261=INDEX(Partidos!$K$4:$K$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A261,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E261)),NOT(ISNUMBER($F261))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A261,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E261=INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0)),$F261=INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E261-$F261)=(INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E261&gt;$F261,INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),AND($E261=$F261,INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),AND($E261&lt;$F261,INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0)),IF(AND($E261=INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0)),$F261=INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),IF(AND($H261&lt;&gt;"",$H261=INDEX(Partidos!$K$4:$K$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E261=$F261,($E261-$F261)=(INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0)))),IF(AND($H261&lt;&gt;"",$H261=INDEX(Partidos!$K$4:$K$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H261&lt;&gt;"",$H261=INDEX(Partidos!$K$4:$K$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E261=INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0)),$F261=INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E261-$F261)=(INDEX(Partidos!$F$4:$F$107,MATCH($A261,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H261&lt;&gt;"",$H261=INDEX(Partidos!$K$4:$K$107,MATCH($A261,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H261" s="19">
@@ -20903,7 +20948,7 @@
         <v/>
       </c>
       <c r="G262" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A262,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E262)),NOT(ISNUMBER($F262))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A262,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E262=INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0)),$F262=INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E262-$F262)=(INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E262&gt;$F262,INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),AND($E262=$F262,INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),AND($E262&lt;$F262,INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E262=INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0)),$F262=INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E262-$F262)=(INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H262&lt;&gt;"",$H262=INDEX(Partidos!$K$4:$K$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A262,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E262)),NOT(ISNUMBER($F262))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A262,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E262=INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0)),$F262=INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E262-$F262)=(INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E262&gt;$F262,INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),AND($E262=$F262,INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),AND($E262&lt;$F262,INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0)),IF(AND($E262=INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0)),$F262=INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),IF(AND($H262&lt;&gt;"",$H262=INDEX(Partidos!$K$4:$K$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E262=$F262,($E262-$F262)=(INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0)))),IF(AND($H262&lt;&gt;"",$H262=INDEX(Partidos!$K$4:$K$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H262&lt;&gt;"",$H262=INDEX(Partidos!$K$4:$K$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E262=INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0)),$F262=INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E262-$F262)=(INDEX(Partidos!$F$4:$F$107,MATCH($A262,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H262&lt;&gt;"",$H262=INDEX(Partidos!$K$4:$K$107,MATCH($A262,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H262" s="19">
@@ -20945,7 +20990,7 @@
         <v/>
       </c>
       <c r="G263" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A263,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E263)),NOT(ISNUMBER($F263))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A263,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E263=INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0)),$F263=INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E263-$F263)=(INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E263&gt;$F263,INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),AND($E263=$F263,INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),AND($E263&lt;$F263,INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E263=INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0)),$F263=INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E263-$F263)=(INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H263&lt;&gt;"",$H263=INDEX(Partidos!$K$4:$K$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A263,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E263)),NOT(ISNUMBER($F263))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A263,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E263=INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0)),$F263=INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E263-$F263)=(INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E263&gt;$F263,INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),AND($E263=$F263,INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),AND($E263&lt;$F263,INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0)),IF(AND($E263=INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0)),$F263=INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),IF(AND($H263&lt;&gt;"",$H263=INDEX(Partidos!$K$4:$K$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E263=$F263,($E263-$F263)=(INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0)))),IF(AND($H263&lt;&gt;"",$H263=INDEX(Partidos!$K$4:$K$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H263&lt;&gt;"",$H263=INDEX(Partidos!$K$4:$K$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E263=INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0)),$F263=INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E263-$F263)=(INDEX(Partidos!$F$4:$F$107,MATCH($A263,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H263&lt;&gt;"",$H263=INDEX(Partidos!$K$4:$K$107,MATCH($A263,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H263" s="19">
@@ -20987,7 +21032,7 @@
         <v/>
       </c>
       <c r="G264" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A264,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E264)),NOT(ISNUMBER($F264))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A264,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E264=INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0)),$F264=INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E264-$F264)=(INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E264&gt;$F264,INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),AND($E264=$F264,INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),AND($E264&lt;$F264,INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E264=INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0)),$F264=INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E264-$F264)=(INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H264&lt;&gt;"",$H264=INDEX(Partidos!$K$4:$K$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A264,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E264)),NOT(ISNUMBER($F264))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A264,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E264=INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0)),$F264=INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E264-$F264)=(INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E264&gt;$F264,INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),AND($E264=$F264,INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),AND($E264&lt;$F264,INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0)),IF(AND($E264=INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0)),$F264=INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),IF(AND($H264&lt;&gt;"",$H264=INDEX(Partidos!$K$4:$K$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E264=$F264,($E264-$F264)=(INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0)))),IF(AND($H264&lt;&gt;"",$H264=INDEX(Partidos!$K$4:$K$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H264&lt;&gt;"",$H264=INDEX(Partidos!$K$4:$K$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E264=INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0)),$F264=INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E264-$F264)=(INDEX(Partidos!$F$4:$F$107,MATCH($A264,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H264&lt;&gt;"",$H264=INDEX(Partidos!$K$4:$K$107,MATCH($A264,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H264" s="19">
@@ -21029,7 +21074,7 @@
         <v/>
       </c>
       <c r="G265" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A265,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E265)),NOT(ISNUMBER($F265))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A265,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E265=INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0)),$F265=INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E265-$F265)=(INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E265&gt;$F265,INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),AND($E265=$F265,INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),AND($E265&lt;$F265,INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E265=INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0)),$F265=INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E265-$F265)=(INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H265&lt;&gt;"",$H265=INDEX(Partidos!$K$4:$K$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A265,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E265)),NOT(ISNUMBER($F265))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A265,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E265=INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0)),$F265=INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E265-$F265)=(INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E265&gt;$F265,INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),AND($E265=$F265,INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),AND($E265&lt;$F265,INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0)),IF(AND($E265=INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0)),$F265=INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),IF(AND($H265&lt;&gt;"",$H265=INDEX(Partidos!$K$4:$K$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E265=$F265,($E265-$F265)=(INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0)))),IF(AND($H265&lt;&gt;"",$H265=INDEX(Partidos!$K$4:$K$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H265&lt;&gt;"",$H265=INDEX(Partidos!$K$4:$K$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E265=INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0)),$F265=INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E265-$F265)=(INDEX(Partidos!$F$4:$F$107,MATCH($A265,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H265&lt;&gt;"",$H265=INDEX(Partidos!$K$4:$K$107,MATCH($A265,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H265" s="19">
@@ -21071,7 +21116,7 @@
         <v/>
       </c>
       <c r="G266" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A266,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E266)),NOT(ISNUMBER($F266))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A266,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E266=INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0)),$F266=INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E266-$F266)=(INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E266&gt;$F266,INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),AND($E266=$F266,INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),AND($E266&lt;$F266,INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E266=INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0)),$F266=INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E266-$F266)=(INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H266&lt;&gt;"",$H266=INDEX(Partidos!$K$4:$K$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A266,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E266)),NOT(ISNUMBER($F266))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A266,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E266=INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0)),$F266=INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E266-$F266)=(INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E266&gt;$F266,INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),AND($E266=$F266,INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),AND($E266&lt;$F266,INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0)),IF(AND($E266=INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0)),$F266=INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),IF(AND($H266&lt;&gt;"",$H266=INDEX(Partidos!$K$4:$K$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E266=$F266,($E266-$F266)=(INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0)))),IF(AND($H266&lt;&gt;"",$H266=INDEX(Partidos!$K$4:$K$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H266&lt;&gt;"",$H266=INDEX(Partidos!$K$4:$K$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E266=INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0)),$F266=INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E266-$F266)=(INDEX(Partidos!$F$4:$F$107,MATCH($A266,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H266&lt;&gt;"",$H266=INDEX(Partidos!$K$4:$K$107,MATCH($A266,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H266" s="19">
@@ -21113,7 +21158,7 @@
         <v/>
       </c>
       <c r="G267" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A267,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E267)),NOT(ISNUMBER($F267))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A267,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E267=INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0)),$F267=INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E267-$F267)=(INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E267&gt;$F267,INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),AND($E267=$F267,INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),AND($E267&lt;$F267,INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E267=INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0)),$F267=INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E267-$F267)=(INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H267&lt;&gt;"",$H267=INDEX(Partidos!$K$4:$K$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A267,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E267)),NOT(ISNUMBER($F267))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A267,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E267=INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0)),$F267=INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E267-$F267)=(INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E267&gt;$F267,INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),AND($E267=$F267,INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),AND($E267&lt;$F267,INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0)),IF(AND($E267=INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0)),$F267=INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),IF(AND($H267&lt;&gt;"",$H267=INDEX(Partidos!$K$4:$K$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E267=$F267,($E267-$F267)=(INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0)))),IF(AND($H267&lt;&gt;"",$H267=INDEX(Partidos!$K$4:$K$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H267&lt;&gt;"",$H267=INDEX(Partidos!$K$4:$K$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E267=INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0)),$F267=INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E267-$F267)=(INDEX(Partidos!$F$4:$F$107,MATCH($A267,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H267&lt;&gt;"",$H267=INDEX(Partidos!$K$4:$K$107,MATCH($A267,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H267" s="19">
@@ -21155,7 +21200,7 @@
         <v/>
       </c>
       <c r="G268" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A268,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E268)),NOT(ISNUMBER($F268))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A268,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E268=INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0)),$F268=INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E268-$F268)=(INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E268&gt;$F268,INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),AND($E268=$F268,INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),AND($E268&lt;$F268,INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E268=INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0)),$F268=INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E268-$F268)=(INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H268&lt;&gt;"",$H268=INDEX(Partidos!$K$4:$K$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A268,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E268)),NOT(ISNUMBER($F268))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A268,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E268=INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0)),$F268=INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E268-$F268)=(INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E268&gt;$F268,INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),AND($E268=$F268,INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),AND($E268&lt;$F268,INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0)),IF(AND($E268=INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0)),$F268=INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),IF(AND($H268&lt;&gt;"",$H268=INDEX(Partidos!$K$4:$K$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E268=$F268,($E268-$F268)=(INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0)))),IF(AND($H268&lt;&gt;"",$H268=INDEX(Partidos!$K$4:$K$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H268&lt;&gt;"",$H268=INDEX(Partidos!$K$4:$K$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E268=INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0)),$F268=INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E268-$F268)=(INDEX(Partidos!$F$4:$F$107,MATCH($A268,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H268&lt;&gt;"",$H268=INDEX(Partidos!$K$4:$K$107,MATCH($A268,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H268" s="19">
@@ -21197,7 +21242,7 @@
         <v/>
       </c>
       <c r="G269" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A269,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E269)),NOT(ISNUMBER($F269))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A269,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E269=INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0)),$F269=INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E269-$F269)=(INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E269&gt;$F269,INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),AND($E269=$F269,INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),AND($E269&lt;$F269,INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E269=INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0)),$F269=INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E269-$F269)=(INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H269&lt;&gt;"",$H269=INDEX(Partidos!$K$4:$K$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A269,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E269)),NOT(ISNUMBER($F269))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A269,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E269=INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0)),$F269=INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E269-$F269)=(INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E269&gt;$F269,INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),AND($E269=$F269,INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),AND($E269&lt;$F269,INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0)),IF(AND($E269=INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0)),$F269=INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),IF(AND($H269&lt;&gt;"",$H269=INDEX(Partidos!$K$4:$K$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E269=$F269,($E269-$F269)=(INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0)))),IF(AND($H269&lt;&gt;"",$H269=INDEX(Partidos!$K$4:$K$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H269&lt;&gt;"",$H269=INDEX(Partidos!$K$4:$K$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E269=INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0)),$F269=INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E269-$F269)=(INDEX(Partidos!$F$4:$F$107,MATCH($A269,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H269&lt;&gt;"",$H269=INDEX(Partidos!$K$4:$K$107,MATCH($A269,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H269" s="19">
@@ -21239,7 +21284,7 @@
         <v/>
       </c>
       <c r="G270" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A270,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E270)),NOT(ISNUMBER($F270))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A270,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E270=INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0)),$F270=INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E270-$F270)=(INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E270&gt;$F270,INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),AND($E270=$F270,INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),AND($E270&lt;$F270,INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E270=INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0)),$F270=INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E270-$F270)=(INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H270&lt;&gt;"",$H270=INDEX(Partidos!$K$4:$K$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A270,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E270)),NOT(ISNUMBER($F270))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A270,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E270=INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0)),$F270=INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E270-$F270)=(INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E270&gt;$F270,INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),AND($E270=$F270,INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),AND($E270&lt;$F270,INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0)),IF(AND($E270=INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0)),$F270=INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),IF(AND($H270&lt;&gt;"",$H270=INDEX(Partidos!$K$4:$K$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E270=$F270,($E270-$F270)=(INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0)))),IF(AND($H270&lt;&gt;"",$H270=INDEX(Partidos!$K$4:$K$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H270&lt;&gt;"",$H270=INDEX(Partidos!$K$4:$K$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E270=INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0)),$F270=INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E270-$F270)=(INDEX(Partidos!$F$4:$F$107,MATCH($A270,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H270&lt;&gt;"",$H270=INDEX(Partidos!$K$4:$K$107,MATCH($A270,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H270" s="19">
@@ -21281,7 +21326,7 @@
         <v/>
       </c>
       <c r="G271" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A271,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E271)),NOT(ISNUMBER($F271))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A271,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E271=INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0)),$F271=INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E271-$F271)=(INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E271&gt;$F271,INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),AND($E271=$F271,INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),AND($E271&lt;$F271,INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E271=INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0)),$F271=INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E271-$F271)=(INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H271&lt;&gt;"",$H271=INDEX(Partidos!$K$4:$K$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A271,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E271)),NOT(ISNUMBER($F271))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A271,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E271=INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0)),$F271=INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E271-$F271)=(INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E271&gt;$F271,INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),AND($E271=$F271,INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),AND($E271&lt;$F271,INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0)),IF(AND($E271=INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0)),$F271=INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),IF(AND($H271&lt;&gt;"",$H271=INDEX(Partidos!$K$4:$K$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E271=$F271,($E271-$F271)=(INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0)))),IF(AND($H271&lt;&gt;"",$H271=INDEX(Partidos!$K$4:$K$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H271&lt;&gt;"",$H271=INDEX(Partidos!$K$4:$K$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E271=INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0)),$F271=INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E271-$F271)=(INDEX(Partidos!$F$4:$F$107,MATCH($A271,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H271&lt;&gt;"",$H271=INDEX(Partidos!$K$4:$K$107,MATCH($A271,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H271" s="19">
@@ -21323,7 +21368,7 @@
         <v/>
       </c>
       <c r="G272" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A272,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E272)),NOT(ISNUMBER($F272))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A272,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E272=INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0)),$F272=INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E272-$F272)=(INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E272&gt;$F272,INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),AND($E272=$F272,INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),AND($E272&lt;$F272,INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E272=INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0)),$F272=INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E272-$F272)=(INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H272&lt;&gt;"",$H272=INDEX(Partidos!$K$4:$K$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A272,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E272)),NOT(ISNUMBER($F272))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A272,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E272=INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0)),$F272=INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E272-$F272)=(INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E272&gt;$F272,INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),AND($E272=$F272,INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),AND($E272&lt;$F272,INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0)),IF(AND($E272=INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0)),$F272=INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),IF(AND($H272&lt;&gt;"",$H272=INDEX(Partidos!$K$4:$K$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E272=$F272,($E272-$F272)=(INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0)))),IF(AND($H272&lt;&gt;"",$H272=INDEX(Partidos!$K$4:$K$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H272&lt;&gt;"",$H272=INDEX(Partidos!$K$4:$K$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E272=INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0)),$F272=INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E272-$F272)=(INDEX(Partidos!$F$4:$F$107,MATCH($A272,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H272&lt;&gt;"",$H272=INDEX(Partidos!$K$4:$K$107,MATCH($A272,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H272" s="19">
@@ -21365,7 +21410,7 @@
         <v/>
       </c>
       <c r="G273" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A273,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E273)),NOT(ISNUMBER($F273))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A273,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E273=INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0)),$F273=INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E273-$F273)=(INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E273&gt;$F273,INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),AND($E273=$F273,INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),AND($E273&lt;$F273,INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E273=INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0)),$F273=INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E273-$F273)=(INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H273&lt;&gt;"",$H273=INDEX(Partidos!$K$4:$K$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A273,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E273)),NOT(ISNUMBER($F273))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A273,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E273=INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0)),$F273=INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E273-$F273)=(INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E273&gt;$F273,INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),AND($E273=$F273,INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),AND($E273&lt;$F273,INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0)),IF(AND($E273=INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0)),$F273=INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),IF(AND($H273&lt;&gt;"",$H273=INDEX(Partidos!$K$4:$K$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E273=$F273,($E273-$F273)=(INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0)))),IF(AND($H273&lt;&gt;"",$H273=INDEX(Partidos!$K$4:$K$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H273&lt;&gt;"",$H273=INDEX(Partidos!$K$4:$K$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E273=INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0)),$F273=INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E273-$F273)=(INDEX(Partidos!$F$4:$F$107,MATCH($A273,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H273&lt;&gt;"",$H273=INDEX(Partidos!$K$4:$K$107,MATCH($A273,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H273" s="19">
@@ -21407,7 +21452,7 @@
         <v/>
       </c>
       <c r="G274" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A274,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E274)),NOT(ISNUMBER($F274))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A274,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E274=INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0)),$F274=INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E274-$F274)=(INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E274&gt;$F274,INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),AND($E274=$F274,INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),AND($E274&lt;$F274,INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E274=INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0)),$F274=INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E274-$F274)=(INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H274&lt;&gt;"",$H274=INDEX(Partidos!$K$4:$K$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A274,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E274)),NOT(ISNUMBER($F274))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A274,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E274=INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0)),$F274=INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E274-$F274)=(INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E274&gt;$F274,INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),AND($E274=$F274,INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),AND($E274&lt;$F274,INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0)),IF(AND($E274=INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0)),$F274=INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),IF(AND($H274&lt;&gt;"",$H274=INDEX(Partidos!$K$4:$K$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E274=$F274,($E274-$F274)=(INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0)))),IF(AND($H274&lt;&gt;"",$H274=INDEX(Partidos!$K$4:$K$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H274&lt;&gt;"",$H274=INDEX(Partidos!$K$4:$K$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E274=INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0)),$F274=INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E274-$F274)=(INDEX(Partidos!$F$4:$F$107,MATCH($A274,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H274&lt;&gt;"",$H274=INDEX(Partidos!$K$4:$K$107,MATCH($A274,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H274" s="19">
@@ -21449,7 +21494,7 @@
         <v/>
       </c>
       <c r="G275" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A275,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E275)),NOT(ISNUMBER($F275))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A275,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E275=INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0)),$F275=INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E275-$F275)=(INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E275&gt;$F275,INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),AND($E275=$F275,INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),AND($E275&lt;$F275,INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E275=INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0)),$F275=INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E275-$F275)=(INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H275&lt;&gt;"",$H275=INDEX(Partidos!$K$4:$K$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A275,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E275)),NOT(ISNUMBER($F275))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A275,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E275=INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0)),$F275=INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E275-$F275)=(INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E275&gt;$F275,INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),AND($E275=$F275,INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),AND($E275&lt;$F275,INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0)),IF(AND($E275=INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0)),$F275=INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),IF(AND($H275&lt;&gt;"",$H275=INDEX(Partidos!$K$4:$K$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E275=$F275,($E275-$F275)=(INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0)))),IF(AND($H275&lt;&gt;"",$H275=INDEX(Partidos!$K$4:$K$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H275&lt;&gt;"",$H275=INDEX(Partidos!$K$4:$K$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E275=INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0)),$F275=INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E275-$F275)=(INDEX(Partidos!$F$4:$F$107,MATCH($A275,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H275&lt;&gt;"",$H275=INDEX(Partidos!$K$4:$K$107,MATCH($A275,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H275" s="19">
@@ -21491,7 +21536,7 @@
         <v/>
       </c>
       <c r="G276" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A276,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E276)),NOT(ISNUMBER($F276))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A276,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E276=INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0)),$F276=INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E276-$F276)=(INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E276&gt;$F276,INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),AND($E276=$F276,INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),AND($E276&lt;$F276,INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E276=INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0)),$F276=INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E276-$F276)=(INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H276&lt;&gt;"",$H276=INDEX(Partidos!$K$4:$K$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A276,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E276)),NOT(ISNUMBER($F276))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A276,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E276=INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0)),$F276=INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E276-$F276)=(INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E276&gt;$F276,INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),AND($E276=$F276,INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),AND($E276&lt;$F276,INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0)),IF(AND($E276=INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0)),$F276=INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),IF(AND($H276&lt;&gt;"",$H276=INDEX(Partidos!$K$4:$K$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E276=$F276,($E276-$F276)=(INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0)))),IF(AND($H276&lt;&gt;"",$H276=INDEX(Partidos!$K$4:$K$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H276&lt;&gt;"",$H276=INDEX(Partidos!$K$4:$K$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E276=INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0)),$F276=INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E276-$F276)=(INDEX(Partidos!$F$4:$F$107,MATCH($A276,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H276&lt;&gt;"",$H276=INDEX(Partidos!$K$4:$K$107,MATCH($A276,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H276" s="19">
@@ -21533,7 +21578,7 @@
         <v/>
       </c>
       <c r="G277" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A277,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E277)),NOT(ISNUMBER($F277))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A277,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E277=INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0)),$F277=INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E277-$F277)=(INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E277&gt;$F277,INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),AND($E277=$F277,INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),AND($E277&lt;$F277,INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E277=INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0)),$F277=INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E277-$F277)=(INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H277&lt;&gt;"",$H277=INDEX(Partidos!$K$4:$K$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A277,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E277)),NOT(ISNUMBER($F277))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A277,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E277=INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0)),$F277=INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E277-$F277)=(INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E277&gt;$F277,INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),AND($E277=$F277,INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),AND($E277&lt;$F277,INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0)),IF(AND($E277=INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0)),$F277=INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),IF(AND($H277&lt;&gt;"",$H277=INDEX(Partidos!$K$4:$K$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E277=$F277,($E277-$F277)=(INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0)))),IF(AND($H277&lt;&gt;"",$H277=INDEX(Partidos!$K$4:$K$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H277&lt;&gt;"",$H277=INDEX(Partidos!$K$4:$K$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E277=INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0)),$F277=INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E277-$F277)=(INDEX(Partidos!$F$4:$F$107,MATCH($A277,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H277&lt;&gt;"",$H277=INDEX(Partidos!$K$4:$K$107,MATCH($A277,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H277" s="19">
@@ -21575,7 +21620,7 @@
         <v/>
       </c>
       <c r="G278" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A278,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E278)),NOT(ISNUMBER($F278))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A278,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E278=INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0)),$F278=INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E278-$F278)=(INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E278&gt;$F278,INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),AND($E278=$F278,INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),AND($E278&lt;$F278,INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E278=INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0)),$F278=INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E278-$F278)=(INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H278&lt;&gt;"",$H278=INDEX(Partidos!$K$4:$K$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A278,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E278)),NOT(ISNUMBER($F278))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A278,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E278=INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0)),$F278=INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E278-$F278)=(INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E278&gt;$F278,INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),AND($E278=$F278,INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),AND($E278&lt;$F278,INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0)),IF(AND($E278=INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0)),$F278=INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),IF(AND($H278&lt;&gt;"",$H278=INDEX(Partidos!$K$4:$K$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E278=$F278,($E278-$F278)=(INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0)))),IF(AND($H278&lt;&gt;"",$H278=INDEX(Partidos!$K$4:$K$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H278&lt;&gt;"",$H278=INDEX(Partidos!$K$4:$K$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E278=INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0)),$F278=INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E278-$F278)=(INDEX(Partidos!$F$4:$F$107,MATCH($A278,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H278&lt;&gt;"",$H278=INDEX(Partidos!$K$4:$K$107,MATCH($A278,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H278" s="19">
@@ -21617,7 +21662,7 @@
         <v/>
       </c>
       <c r="G279" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A279,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E279)),NOT(ISNUMBER($F279))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A279,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E279=INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0)),$F279=INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E279-$F279)=(INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E279&gt;$F279,INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),AND($E279=$F279,INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),AND($E279&lt;$F279,INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E279=INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0)),$F279=INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E279-$F279)=(INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H279&lt;&gt;"",$H279=INDEX(Partidos!$K$4:$K$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A279,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E279)),NOT(ISNUMBER($F279))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A279,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E279=INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0)),$F279=INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E279-$F279)=(INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E279&gt;$F279,INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),AND($E279=$F279,INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),AND($E279&lt;$F279,INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0)),IF(AND($E279=INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0)),$F279=INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),IF(AND($H279&lt;&gt;"",$H279=INDEX(Partidos!$K$4:$K$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E279=$F279,($E279-$F279)=(INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0)))),IF(AND($H279&lt;&gt;"",$H279=INDEX(Partidos!$K$4:$K$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H279&lt;&gt;"",$H279=INDEX(Partidos!$K$4:$K$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E279=INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0)),$F279=INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E279-$F279)=(INDEX(Partidos!$F$4:$F$107,MATCH($A279,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H279&lt;&gt;"",$H279=INDEX(Partidos!$K$4:$K$107,MATCH($A279,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H279" s="19">
@@ -21659,7 +21704,7 @@
         <v/>
       </c>
       <c r="G280" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A280,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E280)),NOT(ISNUMBER($F280))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A280,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E280=INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0)),$F280=INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E280-$F280)=(INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E280&gt;$F280,INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),AND($E280=$F280,INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),AND($E280&lt;$F280,INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E280=INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0)),$F280=INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E280-$F280)=(INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H280&lt;&gt;"",$H280=INDEX(Partidos!$K$4:$K$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A280,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E280)),NOT(ISNUMBER($F280))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A280,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E280=INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0)),$F280=INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E280-$F280)=(INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E280&gt;$F280,INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),AND($E280=$F280,INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),AND($E280&lt;$F280,INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0)),IF(AND($E280=INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0)),$F280=INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),IF(AND($H280&lt;&gt;"",$H280=INDEX(Partidos!$K$4:$K$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E280=$F280,($E280-$F280)=(INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0)))),IF(AND($H280&lt;&gt;"",$H280=INDEX(Partidos!$K$4:$K$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H280&lt;&gt;"",$H280=INDEX(Partidos!$K$4:$K$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E280=INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0)),$F280=INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E280-$F280)=(INDEX(Partidos!$F$4:$F$107,MATCH($A280,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H280&lt;&gt;"",$H280=INDEX(Partidos!$K$4:$K$107,MATCH($A280,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H280" s="19">
@@ -21701,7 +21746,7 @@
         <v/>
       </c>
       <c r="G281" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A281,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E281)),NOT(ISNUMBER($F281))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A281,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E281=INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0)),$F281=INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E281-$F281)=(INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E281&gt;$F281,INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),AND($E281=$F281,INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),AND($E281&lt;$F281,INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E281=INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0)),$F281=INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E281-$F281)=(INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H281&lt;&gt;"",$H281=INDEX(Partidos!$K$4:$K$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A281,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E281)),NOT(ISNUMBER($F281))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A281,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E281=INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0)),$F281=INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E281-$F281)=(INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E281&gt;$F281,INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),AND($E281=$F281,INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),AND($E281&lt;$F281,INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0)),IF(AND($E281=INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0)),$F281=INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),IF(AND($H281&lt;&gt;"",$H281=INDEX(Partidos!$K$4:$K$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E281=$F281,($E281-$F281)=(INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0)))),IF(AND($H281&lt;&gt;"",$H281=INDEX(Partidos!$K$4:$K$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H281&lt;&gt;"",$H281=INDEX(Partidos!$K$4:$K$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E281=INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0)),$F281=INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E281-$F281)=(INDEX(Partidos!$F$4:$F$107,MATCH($A281,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H281&lt;&gt;"",$H281=INDEX(Partidos!$K$4:$K$107,MATCH($A281,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H281" s="19">
@@ -21743,7 +21788,7 @@
         <v/>
       </c>
       <c r="G282" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A282,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E282)),NOT(ISNUMBER($F282))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A282,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E282=INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0)),$F282=INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E282-$F282)=(INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E282&gt;$F282,INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),AND($E282=$F282,INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),AND($E282&lt;$F282,INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E282=INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0)),$F282=INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E282-$F282)=(INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H282&lt;&gt;"",$H282=INDEX(Partidos!$K$4:$K$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A282,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E282)),NOT(ISNUMBER($F282))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A282,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E282=INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0)),$F282=INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E282-$F282)=(INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E282&gt;$F282,INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),AND($E282=$F282,INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),AND($E282&lt;$F282,INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0)),IF(AND($E282=INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0)),$F282=INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),IF(AND($H282&lt;&gt;"",$H282=INDEX(Partidos!$K$4:$K$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E282=$F282,($E282-$F282)=(INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0)))),IF(AND($H282&lt;&gt;"",$H282=INDEX(Partidos!$K$4:$K$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H282&lt;&gt;"",$H282=INDEX(Partidos!$K$4:$K$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E282=INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0)),$F282=INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E282-$F282)=(INDEX(Partidos!$F$4:$F$107,MATCH($A282,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H282&lt;&gt;"",$H282=INDEX(Partidos!$K$4:$K$107,MATCH($A282,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H282" s="19">
@@ -21785,7 +21830,7 @@
         <v/>
       </c>
       <c r="G283" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A283,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E283)),NOT(ISNUMBER($F283))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A283,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E283=INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0)),$F283=INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E283-$F283)=(INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E283&gt;$F283,INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),AND($E283=$F283,INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),AND($E283&lt;$F283,INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E283=INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0)),$F283=INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E283-$F283)=(INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H283&lt;&gt;"",$H283=INDEX(Partidos!$K$4:$K$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A283,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E283)),NOT(ISNUMBER($F283))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A283,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E283=INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0)),$F283=INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E283-$F283)=(INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E283&gt;$F283,INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),AND($E283=$F283,INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),AND($E283&lt;$F283,INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0)),IF(AND($E283=INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0)),$F283=INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),IF(AND($H283&lt;&gt;"",$H283=INDEX(Partidos!$K$4:$K$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E283=$F283,($E283-$F283)=(INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0)))),IF(AND($H283&lt;&gt;"",$H283=INDEX(Partidos!$K$4:$K$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H283&lt;&gt;"",$H283=INDEX(Partidos!$K$4:$K$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E283=INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0)),$F283=INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E283-$F283)=(INDEX(Partidos!$F$4:$F$107,MATCH($A283,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H283&lt;&gt;"",$H283=INDEX(Partidos!$K$4:$K$107,MATCH($A283,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H283" s="19">
@@ -21827,7 +21872,7 @@
         <v/>
       </c>
       <c r="G284" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A284,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E284)),NOT(ISNUMBER($F284))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A284,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E284=INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0)),$F284=INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E284-$F284)=(INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E284&gt;$F284,INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),AND($E284=$F284,INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),AND($E284&lt;$F284,INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E284=INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0)),$F284=INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E284-$F284)=(INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H284&lt;&gt;"",$H284=INDEX(Partidos!$K$4:$K$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A284,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E284)),NOT(ISNUMBER($F284))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A284,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E284=INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0)),$F284=INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E284-$F284)=(INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E284&gt;$F284,INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),AND($E284=$F284,INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),AND($E284&lt;$F284,INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0)),IF(AND($E284=INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0)),$F284=INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),IF(AND($H284&lt;&gt;"",$H284=INDEX(Partidos!$K$4:$K$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E284=$F284,($E284-$F284)=(INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0)))),IF(AND($H284&lt;&gt;"",$H284=INDEX(Partidos!$K$4:$K$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H284&lt;&gt;"",$H284=INDEX(Partidos!$K$4:$K$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E284=INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0)),$F284=INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E284-$F284)=(INDEX(Partidos!$F$4:$F$107,MATCH($A284,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H284&lt;&gt;"",$H284=INDEX(Partidos!$K$4:$K$107,MATCH($A284,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H284" s="19">
@@ -21869,7 +21914,7 @@
         <v/>
       </c>
       <c r="G285" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A285,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E285)),NOT(ISNUMBER($F285))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A285,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E285=INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0)),$F285=INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E285-$F285)=(INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E285&gt;$F285,INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),AND($E285=$F285,INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),AND($E285&lt;$F285,INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E285=INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0)),$F285=INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E285-$F285)=(INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H285&lt;&gt;"",$H285=INDEX(Partidos!$K$4:$K$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A285,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E285)),NOT(ISNUMBER($F285))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A285,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E285=INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0)),$F285=INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E285-$F285)=(INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E285&gt;$F285,INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),AND($E285=$F285,INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),AND($E285&lt;$F285,INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0)),IF(AND($E285=INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0)),$F285=INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),IF(AND($H285&lt;&gt;"",$H285=INDEX(Partidos!$K$4:$K$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E285=$F285,($E285-$F285)=(INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0)))),IF(AND($H285&lt;&gt;"",$H285=INDEX(Partidos!$K$4:$K$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H285&lt;&gt;"",$H285=INDEX(Partidos!$K$4:$K$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E285=INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0)),$F285=INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E285-$F285)=(INDEX(Partidos!$F$4:$F$107,MATCH($A285,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H285&lt;&gt;"",$H285=INDEX(Partidos!$K$4:$K$107,MATCH($A285,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H285" s="19">
@@ -21911,7 +21956,7 @@
         <v/>
       </c>
       <c r="G286" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A286,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E286)),NOT(ISNUMBER($F286))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A286,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E286=INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0)),$F286=INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E286-$F286)=(INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E286&gt;$F286,INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),AND($E286=$F286,INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),AND($E286&lt;$F286,INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E286=INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0)),$F286=INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E286-$F286)=(INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H286&lt;&gt;"",$H286=INDEX(Partidos!$K$4:$K$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A286,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E286)),NOT(ISNUMBER($F286))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A286,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E286=INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0)),$F286=INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E286-$F286)=(INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E286&gt;$F286,INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),AND($E286=$F286,INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),AND($E286&lt;$F286,INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0)),IF(AND($E286=INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0)),$F286=INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),IF(AND($H286&lt;&gt;"",$H286=INDEX(Partidos!$K$4:$K$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E286=$F286,($E286-$F286)=(INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0)))),IF(AND($H286&lt;&gt;"",$H286=INDEX(Partidos!$K$4:$K$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H286&lt;&gt;"",$H286=INDEX(Partidos!$K$4:$K$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E286=INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0)),$F286=INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E286-$F286)=(INDEX(Partidos!$F$4:$F$107,MATCH($A286,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H286&lt;&gt;"",$H286=INDEX(Partidos!$K$4:$K$107,MATCH($A286,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H286" s="19">
@@ -21953,7 +21998,7 @@
         <v/>
       </c>
       <c r="G287" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A287,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E287)),NOT(ISNUMBER($F287))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A287,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E287=INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0)),$F287=INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E287-$F287)=(INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E287&gt;$F287,INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),AND($E287=$F287,INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),AND($E287&lt;$F287,INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E287=INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0)),$F287=INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E287-$F287)=(INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H287&lt;&gt;"",$H287=INDEX(Partidos!$K$4:$K$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A287,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E287)),NOT(ISNUMBER($F287))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A287,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E287=INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0)),$F287=INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E287-$F287)=(INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E287&gt;$F287,INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),AND($E287=$F287,INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),AND($E287&lt;$F287,INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0)),IF(AND($E287=INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0)),$F287=INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),IF(AND($H287&lt;&gt;"",$H287=INDEX(Partidos!$K$4:$K$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E287=$F287,($E287-$F287)=(INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0)))),IF(AND($H287&lt;&gt;"",$H287=INDEX(Partidos!$K$4:$K$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H287&lt;&gt;"",$H287=INDEX(Partidos!$K$4:$K$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E287=INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0)),$F287=INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E287-$F287)=(INDEX(Partidos!$F$4:$F$107,MATCH($A287,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H287&lt;&gt;"",$H287=INDEX(Partidos!$K$4:$K$107,MATCH($A287,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H287" s="19">
@@ -21995,7 +22040,7 @@
         <v/>
       </c>
       <c r="G288" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A288,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E288)),NOT(ISNUMBER($F288))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A288,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E288=INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0)),$F288=INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E288-$F288)=(INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E288&gt;$F288,INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),AND($E288=$F288,INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),AND($E288&lt;$F288,INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E288=INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0)),$F288=INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E288-$F288)=(INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H288&lt;&gt;"",$H288=INDEX(Partidos!$K$4:$K$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A288,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E288)),NOT(ISNUMBER($F288))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A288,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E288=INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0)),$F288=INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E288-$F288)=(INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E288&gt;$F288,INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),AND($E288=$F288,INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),AND($E288&lt;$F288,INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0)),IF(AND($E288=INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0)),$F288=INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),IF(AND($H288&lt;&gt;"",$H288=INDEX(Partidos!$K$4:$K$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E288=$F288,($E288-$F288)=(INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0)))),IF(AND($H288&lt;&gt;"",$H288=INDEX(Partidos!$K$4:$K$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H288&lt;&gt;"",$H288=INDEX(Partidos!$K$4:$K$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E288=INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0)),$F288=INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E288-$F288)=(INDEX(Partidos!$F$4:$F$107,MATCH($A288,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H288&lt;&gt;"",$H288=INDEX(Partidos!$K$4:$K$107,MATCH($A288,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H288" s="19">
@@ -22037,7 +22082,7 @@
         <v/>
       </c>
       <c r="G289" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A289,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E289)),NOT(ISNUMBER($F289))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A289,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E289=INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0)),$F289=INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E289-$F289)=(INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E289&gt;$F289,INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),AND($E289=$F289,INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),AND($E289&lt;$F289,INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E289=INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0)),$F289=INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E289-$F289)=(INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H289&lt;&gt;"",$H289=INDEX(Partidos!$K$4:$K$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A289,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E289)),NOT(ISNUMBER($F289))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A289,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E289=INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0)),$F289=INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E289-$F289)=(INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E289&gt;$F289,INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),AND($E289=$F289,INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),AND($E289&lt;$F289,INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0)),IF(AND($E289=INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0)),$F289=INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),IF(AND($H289&lt;&gt;"",$H289=INDEX(Partidos!$K$4:$K$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E289=$F289,($E289-$F289)=(INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0)))),IF(AND($H289&lt;&gt;"",$H289=INDEX(Partidos!$K$4:$K$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H289&lt;&gt;"",$H289=INDEX(Partidos!$K$4:$K$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E289=INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0)),$F289=INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E289-$F289)=(INDEX(Partidos!$F$4:$F$107,MATCH($A289,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H289&lt;&gt;"",$H289=INDEX(Partidos!$K$4:$K$107,MATCH($A289,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H289" s="19">
@@ -22079,7 +22124,7 @@
         <v/>
       </c>
       <c r="G290" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A290,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E290)),NOT(ISNUMBER($F290))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A290,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E290=INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0)),$F290=INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E290-$F290)=(INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E290&gt;$F290,INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),AND($E290=$F290,INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),AND($E290&lt;$F290,INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E290=INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0)),$F290=INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E290-$F290)=(INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H290&lt;&gt;"",$H290=INDEX(Partidos!$K$4:$K$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A290,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E290)),NOT(ISNUMBER($F290))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A290,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E290=INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0)),$F290=INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E290-$F290)=(INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E290&gt;$F290,INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),AND($E290=$F290,INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),AND($E290&lt;$F290,INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0)),IF(AND($E290=INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0)),$F290=INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),IF(AND($H290&lt;&gt;"",$H290=INDEX(Partidos!$K$4:$K$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E290=$F290,($E290-$F290)=(INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0)))),IF(AND($H290&lt;&gt;"",$H290=INDEX(Partidos!$K$4:$K$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H290&lt;&gt;"",$H290=INDEX(Partidos!$K$4:$K$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E290=INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0)),$F290=INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E290-$F290)=(INDEX(Partidos!$F$4:$F$107,MATCH($A290,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H290&lt;&gt;"",$H290=INDEX(Partidos!$K$4:$K$107,MATCH($A290,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H290" s="19">
@@ -22121,7 +22166,7 @@
         <v/>
       </c>
       <c r="G291" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A291,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E291)),NOT(ISNUMBER($F291))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A291,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E291=INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0)),$F291=INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E291-$F291)=(INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E291&gt;$F291,INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),AND($E291=$F291,INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),AND($E291&lt;$F291,INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E291=INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0)),$F291=INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E291-$F291)=(INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H291&lt;&gt;"",$H291=INDEX(Partidos!$K$4:$K$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A291,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E291)),NOT(ISNUMBER($F291))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A291,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E291=INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0)),$F291=INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E291-$F291)=(INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E291&gt;$F291,INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),AND($E291=$F291,INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),AND($E291&lt;$F291,INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0)),IF(AND($E291=INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0)),$F291=INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),IF(AND($H291&lt;&gt;"",$H291=INDEX(Partidos!$K$4:$K$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E291=$F291,($E291-$F291)=(INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0)))),IF(AND($H291&lt;&gt;"",$H291=INDEX(Partidos!$K$4:$K$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H291&lt;&gt;"",$H291=INDEX(Partidos!$K$4:$K$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E291=INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0)),$F291=INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E291-$F291)=(INDEX(Partidos!$F$4:$F$107,MATCH($A291,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H291&lt;&gt;"",$H291=INDEX(Partidos!$K$4:$K$107,MATCH($A291,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H291" s="19">
@@ -22163,7 +22208,7 @@
         <v/>
       </c>
       <c r="G292" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A292,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E292)),NOT(ISNUMBER($F292))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A292,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E292=INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0)),$F292=INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E292-$F292)=(INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E292&gt;$F292,INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),AND($E292=$F292,INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),AND($E292&lt;$F292,INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E292=INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0)),$F292=INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E292-$F292)=(INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H292&lt;&gt;"",$H292=INDEX(Partidos!$K$4:$K$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A292,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E292)),NOT(ISNUMBER($F292))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A292,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E292=INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0)),$F292=INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E292-$F292)=(INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E292&gt;$F292,INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),AND($E292=$F292,INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),AND($E292&lt;$F292,INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0)),IF(AND($E292=INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0)),$F292=INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),IF(AND($H292&lt;&gt;"",$H292=INDEX(Partidos!$K$4:$K$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E292=$F292,($E292-$F292)=(INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0)))),IF(AND($H292&lt;&gt;"",$H292=INDEX(Partidos!$K$4:$K$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H292&lt;&gt;"",$H292=INDEX(Partidos!$K$4:$K$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E292=INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0)),$F292=INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E292-$F292)=(INDEX(Partidos!$F$4:$F$107,MATCH($A292,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H292&lt;&gt;"",$H292=INDEX(Partidos!$K$4:$K$107,MATCH($A292,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H292" s="19">
@@ -22205,7 +22250,7 @@
         <v/>
       </c>
       <c r="G293" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A293,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E293)),NOT(ISNUMBER($F293))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A293,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E293=INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0)),$F293=INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E293-$F293)=(INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E293&gt;$F293,INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),AND($E293=$F293,INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),AND($E293&lt;$F293,INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E293=INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0)),$F293=INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E293-$F293)=(INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H293&lt;&gt;"",$H293=INDEX(Partidos!$K$4:$K$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A293,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E293)),NOT(ISNUMBER($F293))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A293,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E293=INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0)),$F293=INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E293-$F293)=(INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E293&gt;$F293,INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),AND($E293=$F293,INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),AND($E293&lt;$F293,INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0)),IF(AND($E293=INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0)),$F293=INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),IF(AND($H293&lt;&gt;"",$H293=INDEX(Partidos!$K$4:$K$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E293=$F293,($E293-$F293)=(INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0)))),IF(AND($H293&lt;&gt;"",$H293=INDEX(Partidos!$K$4:$K$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H293&lt;&gt;"",$H293=INDEX(Partidos!$K$4:$K$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E293=INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0)),$F293=INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E293-$F293)=(INDEX(Partidos!$F$4:$F$107,MATCH($A293,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H293&lt;&gt;"",$H293=INDEX(Partidos!$K$4:$K$107,MATCH($A293,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H293" s="19">
@@ -22247,7 +22292,7 @@
         <v/>
       </c>
       <c r="G294" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A294,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E294)),NOT(ISNUMBER($F294))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A294,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E294=INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0)),$F294=INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E294-$F294)=(INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E294&gt;$F294,INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),AND($E294=$F294,INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),AND($E294&lt;$F294,INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E294=INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0)),$F294=INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E294-$F294)=(INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H294&lt;&gt;"",$H294=INDEX(Partidos!$K$4:$K$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A294,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E294)),NOT(ISNUMBER($F294))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A294,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E294=INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0)),$F294=INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E294-$F294)=(INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E294&gt;$F294,INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),AND($E294=$F294,INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),AND($E294&lt;$F294,INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0)),IF(AND($E294=INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0)),$F294=INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),IF(AND($H294&lt;&gt;"",$H294=INDEX(Partidos!$K$4:$K$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E294=$F294,($E294-$F294)=(INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0)))),IF(AND($H294&lt;&gt;"",$H294=INDEX(Partidos!$K$4:$K$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H294&lt;&gt;"",$H294=INDEX(Partidos!$K$4:$K$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E294=INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0)),$F294=INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E294-$F294)=(INDEX(Partidos!$F$4:$F$107,MATCH($A294,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H294&lt;&gt;"",$H294=INDEX(Partidos!$K$4:$K$107,MATCH($A294,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H294" s="19">
@@ -22289,7 +22334,7 @@
         <v/>
       </c>
       <c r="G295" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A295,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E295)),NOT(ISNUMBER($F295))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A295,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E295=INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0)),$F295=INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E295-$F295)=(INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E295&gt;$F295,INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),AND($E295=$F295,INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),AND($E295&lt;$F295,INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E295=INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0)),$F295=INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E295-$F295)=(INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H295&lt;&gt;"",$H295=INDEX(Partidos!$K$4:$K$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A295,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E295)),NOT(ISNUMBER($F295))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A295,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E295=INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0)),$F295=INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E295-$F295)=(INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E295&gt;$F295,INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),AND($E295=$F295,INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),AND($E295&lt;$F295,INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0)),IF(AND($E295=INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0)),$F295=INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),IF(AND($H295&lt;&gt;"",$H295=INDEX(Partidos!$K$4:$K$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E295=$F295,($E295-$F295)=(INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0)))),IF(AND($H295&lt;&gt;"",$H295=INDEX(Partidos!$K$4:$K$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H295&lt;&gt;"",$H295=INDEX(Partidos!$K$4:$K$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E295=INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0)),$F295=INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E295-$F295)=(INDEX(Partidos!$F$4:$F$107,MATCH($A295,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H295&lt;&gt;"",$H295=INDEX(Partidos!$K$4:$K$107,MATCH($A295,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H295" s="19">
@@ -22331,7 +22376,7 @@
         <v/>
       </c>
       <c r="G296" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A296,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E296)),NOT(ISNUMBER($F296))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A296,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E296=INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0)),$F296=INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E296-$F296)=(INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E296&gt;$F296,INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),AND($E296=$F296,INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),AND($E296&lt;$F296,INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E296=INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0)),$F296=INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E296-$F296)=(INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H296&lt;&gt;"",$H296=INDEX(Partidos!$K$4:$K$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A296,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E296)),NOT(ISNUMBER($F296))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A296,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E296=INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0)),$F296=INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E296-$F296)=(INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E296&gt;$F296,INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),AND($E296=$F296,INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),AND($E296&lt;$F296,INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0)),IF(AND($E296=INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0)),$F296=INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),IF(AND($H296&lt;&gt;"",$H296=INDEX(Partidos!$K$4:$K$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E296=$F296,($E296-$F296)=(INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0)))),IF(AND($H296&lt;&gt;"",$H296=INDEX(Partidos!$K$4:$K$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H296&lt;&gt;"",$H296=INDEX(Partidos!$K$4:$K$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E296=INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0)),$F296=INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E296-$F296)=(INDEX(Partidos!$F$4:$F$107,MATCH($A296,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H296&lt;&gt;"",$H296=INDEX(Partidos!$K$4:$K$107,MATCH($A296,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H296" s="19">
@@ -22373,7 +22418,7 @@
         <v/>
       </c>
       <c r="G297" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A297,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E297)),NOT(ISNUMBER($F297))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A297,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E297=INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0)),$F297=INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E297-$F297)=(INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E297&gt;$F297,INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),AND($E297=$F297,INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),AND($E297&lt;$F297,INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E297=INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0)),$F297=INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E297-$F297)=(INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H297&lt;&gt;"",$H297=INDEX(Partidos!$K$4:$K$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A297,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E297)),NOT(ISNUMBER($F297))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A297,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E297=INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0)),$F297=INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E297-$F297)=(INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E297&gt;$F297,INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),AND($E297=$F297,INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),AND($E297&lt;$F297,INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0)),IF(AND($E297=INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0)),$F297=INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),IF(AND($H297&lt;&gt;"",$H297=INDEX(Partidos!$K$4:$K$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E297=$F297,($E297-$F297)=(INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0)))),IF(AND($H297&lt;&gt;"",$H297=INDEX(Partidos!$K$4:$K$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H297&lt;&gt;"",$H297=INDEX(Partidos!$K$4:$K$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E297=INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0)),$F297=INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E297-$F297)=(INDEX(Partidos!$F$4:$F$107,MATCH($A297,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H297&lt;&gt;"",$H297=INDEX(Partidos!$K$4:$K$107,MATCH($A297,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H297" s="19">
@@ -22415,7 +22460,7 @@
         <v/>
       </c>
       <c r="G298" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A298,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E298)),NOT(ISNUMBER($F298))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A298,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E298=INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0)),$F298=INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E298-$F298)=(INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E298&gt;$F298,INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),AND($E298=$F298,INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),AND($E298&lt;$F298,INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E298=INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0)),$F298=INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E298-$F298)=(INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H298&lt;&gt;"",$H298=INDEX(Partidos!$K$4:$K$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A298,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E298)),NOT(ISNUMBER($F298))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A298,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E298=INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0)),$F298=INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E298-$F298)=(INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E298&gt;$F298,INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),AND($E298=$F298,INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),AND($E298&lt;$F298,INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0)),IF(AND($E298=INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0)),$F298=INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),IF(AND($H298&lt;&gt;"",$H298=INDEX(Partidos!$K$4:$K$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E298=$F298,($E298-$F298)=(INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0)))),IF(AND($H298&lt;&gt;"",$H298=INDEX(Partidos!$K$4:$K$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H298&lt;&gt;"",$H298=INDEX(Partidos!$K$4:$K$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E298=INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0)),$F298=INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E298-$F298)=(INDEX(Partidos!$F$4:$F$107,MATCH($A298,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H298&lt;&gt;"",$H298=INDEX(Partidos!$K$4:$K$107,MATCH($A298,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H298" s="19">
@@ -22457,7 +22502,7 @@
         <v/>
       </c>
       <c r="G299" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A299,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E299)),NOT(ISNUMBER($F299))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A299,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E299=INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0)),$F299=INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E299-$F299)=(INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E299&gt;$F299,INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),AND($E299=$F299,INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),AND($E299&lt;$F299,INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E299=INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0)),$F299=INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E299-$F299)=(INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H299&lt;&gt;"",$H299=INDEX(Partidos!$K$4:$K$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A299,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E299)),NOT(ISNUMBER($F299))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A299,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E299=INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0)),$F299=INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E299-$F299)=(INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E299&gt;$F299,INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),AND($E299=$F299,INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),AND($E299&lt;$F299,INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0)),IF(AND($E299=INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0)),$F299=INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),IF(AND($H299&lt;&gt;"",$H299=INDEX(Partidos!$K$4:$K$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E299=$F299,($E299-$F299)=(INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0)))),IF(AND($H299&lt;&gt;"",$H299=INDEX(Partidos!$K$4:$K$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H299&lt;&gt;"",$H299=INDEX(Partidos!$K$4:$K$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E299=INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0)),$F299=INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E299-$F299)=(INDEX(Partidos!$F$4:$F$107,MATCH($A299,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H299&lt;&gt;"",$H299=INDEX(Partidos!$K$4:$K$107,MATCH($A299,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H299" s="19">
@@ -22499,7 +22544,7 @@
         <v/>
       </c>
       <c r="G300" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A300,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E300)),NOT(ISNUMBER($F300))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A300,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E300=INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0)),$F300=INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E300-$F300)=(INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E300&gt;$F300,INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),AND($E300=$F300,INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),AND($E300&lt;$F300,INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E300=INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0)),$F300=INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E300-$F300)=(INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H300&lt;&gt;"",$H300=INDEX(Partidos!$K$4:$K$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A300,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E300)),NOT(ISNUMBER($F300))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A300,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E300=INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0)),$F300=INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E300-$F300)=(INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E300&gt;$F300,INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),AND($E300=$F300,INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),AND($E300&lt;$F300,INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0)),IF(AND($E300=INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0)),$F300=INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),IF(AND($H300&lt;&gt;"",$H300=INDEX(Partidos!$K$4:$K$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E300=$F300,($E300-$F300)=(INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0)))),IF(AND($H300&lt;&gt;"",$H300=INDEX(Partidos!$K$4:$K$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H300&lt;&gt;"",$H300=INDEX(Partidos!$K$4:$K$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E300=INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0)),$F300=INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E300-$F300)=(INDEX(Partidos!$F$4:$F$107,MATCH($A300,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H300&lt;&gt;"",$H300=INDEX(Partidos!$K$4:$K$107,MATCH($A300,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H300" s="19">
@@ -22541,7 +22586,7 @@
         <v/>
       </c>
       <c r="G301" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A301,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E301)),NOT(ISNUMBER($F301))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A301,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E301=INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0)),$F301=INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E301-$F301)=(INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E301&gt;$F301,INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),AND($E301=$F301,INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),AND($E301&lt;$F301,INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E301=INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0)),$F301=INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E301-$F301)=(INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H301&lt;&gt;"",$H301=INDEX(Partidos!$K$4:$K$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A301,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E301)),NOT(ISNUMBER($F301))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A301,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E301=INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0)),$F301=INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E301-$F301)=(INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E301&gt;$F301,INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),AND($E301=$F301,INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),AND($E301&lt;$F301,INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0)),IF(AND($E301=INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0)),$F301=INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),IF(AND($H301&lt;&gt;"",$H301=INDEX(Partidos!$K$4:$K$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E301=$F301,($E301-$F301)=(INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0)))),IF(AND($H301&lt;&gt;"",$H301=INDEX(Partidos!$K$4:$K$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H301&lt;&gt;"",$H301=INDEX(Partidos!$K$4:$K$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E301=INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0)),$F301=INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E301-$F301)=(INDEX(Partidos!$F$4:$F$107,MATCH($A301,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H301&lt;&gt;"",$H301=INDEX(Partidos!$K$4:$K$107,MATCH($A301,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H301" s="19">
@@ -22583,7 +22628,7 @@
         <v/>
       </c>
       <c r="G302" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A302,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E302)),NOT(ISNUMBER($F302))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A302,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E302=INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0)),$F302=INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E302-$F302)=(INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E302&gt;$F302,INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),AND($E302=$F302,INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),AND($E302&lt;$F302,INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E302=INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0)),$F302=INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E302-$F302)=(INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H302&lt;&gt;"",$H302=INDEX(Partidos!$K$4:$K$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A302,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E302)),NOT(ISNUMBER($F302))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A302,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E302=INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0)),$F302=INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E302-$F302)=(INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E302&gt;$F302,INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),AND($E302=$F302,INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),AND($E302&lt;$F302,INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0)),IF(AND($E302=INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0)),$F302=INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),IF(AND($H302&lt;&gt;"",$H302=INDEX(Partidos!$K$4:$K$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E302=$F302,($E302-$F302)=(INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0)))),IF(AND($H302&lt;&gt;"",$H302=INDEX(Partidos!$K$4:$K$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H302&lt;&gt;"",$H302=INDEX(Partidos!$K$4:$K$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E302=INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0)),$F302=INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E302-$F302)=(INDEX(Partidos!$F$4:$F$107,MATCH($A302,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H302&lt;&gt;"",$H302=INDEX(Partidos!$K$4:$K$107,MATCH($A302,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H302" s="19">
@@ -22625,7 +22670,7 @@
         <v/>
       </c>
       <c r="G303" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A303,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E303)),NOT(ISNUMBER($F303))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A303,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E303=INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0)),$F303=INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E303-$F303)=(INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E303&gt;$F303,INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),AND($E303=$F303,INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),AND($E303&lt;$F303,INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E303=INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0)),$F303=INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E303-$F303)=(INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H303&lt;&gt;"",$H303=INDEX(Partidos!$K$4:$K$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A303,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E303)),NOT(ISNUMBER($F303))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A303,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E303=INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0)),$F303=INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E303-$F303)=(INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E303&gt;$F303,INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),AND($E303=$F303,INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),AND($E303&lt;$F303,INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0)),IF(AND($E303=INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0)),$F303=INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),IF(AND($H303&lt;&gt;"",$H303=INDEX(Partidos!$K$4:$K$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E303=$F303,($E303-$F303)=(INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0)))),IF(AND($H303&lt;&gt;"",$H303=INDEX(Partidos!$K$4:$K$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H303&lt;&gt;"",$H303=INDEX(Partidos!$K$4:$K$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E303=INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0)),$F303=INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E303-$F303)=(INDEX(Partidos!$F$4:$F$107,MATCH($A303,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H303&lt;&gt;"",$H303=INDEX(Partidos!$K$4:$K$107,MATCH($A303,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H303" s="19">
@@ -22667,7 +22712,7 @@
         <v/>
       </c>
       <c r="G304" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A304,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E304)),NOT(ISNUMBER($F304))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A304,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E304=INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0)),$F304=INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E304-$F304)=(INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E304&gt;$F304,INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),AND($E304=$F304,INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),AND($E304&lt;$F304,INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E304=INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0)),$F304=INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E304-$F304)=(INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H304&lt;&gt;"",$H304=INDEX(Partidos!$K$4:$K$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A304,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E304)),NOT(ISNUMBER($F304))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A304,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E304=INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0)),$F304=INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E304-$F304)=(INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E304&gt;$F304,INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),AND($E304=$F304,INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),AND($E304&lt;$F304,INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0)),IF(AND($E304=INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0)),$F304=INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),IF(AND($H304&lt;&gt;"",$H304=INDEX(Partidos!$K$4:$K$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E304=$F304,($E304-$F304)=(INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0)))),IF(AND($H304&lt;&gt;"",$H304=INDEX(Partidos!$K$4:$K$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H304&lt;&gt;"",$H304=INDEX(Partidos!$K$4:$K$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E304=INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0)),$F304=INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E304-$F304)=(INDEX(Partidos!$F$4:$F$107,MATCH($A304,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H304&lt;&gt;"",$H304=INDEX(Partidos!$K$4:$K$107,MATCH($A304,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H304" s="19">
@@ -22709,7 +22754,7 @@
         <v/>
       </c>
       <c r="G305" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A305,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E305)),NOT(ISNUMBER($F305))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A305,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E305=INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0)),$F305=INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E305-$F305)=(INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E305&gt;$F305,INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),AND($E305=$F305,INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),AND($E305&lt;$F305,INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E305=INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0)),$F305=INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E305-$F305)=(INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H305&lt;&gt;"",$H305=INDEX(Partidos!$K$4:$K$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A305,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E305)),NOT(ISNUMBER($F305))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A305,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E305=INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0)),$F305=INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E305-$F305)=(INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E305&gt;$F305,INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),AND($E305=$F305,INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),AND($E305&lt;$F305,INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0)),IF(AND($E305=INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0)),$F305=INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),IF(AND($H305&lt;&gt;"",$H305=INDEX(Partidos!$K$4:$K$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E305=$F305,($E305-$F305)=(INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0)))),IF(AND($H305&lt;&gt;"",$H305=INDEX(Partidos!$K$4:$K$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H305&lt;&gt;"",$H305=INDEX(Partidos!$K$4:$K$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E305=INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0)),$F305=INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E305-$F305)=(INDEX(Partidos!$F$4:$F$107,MATCH($A305,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H305&lt;&gt;"",$H305=INDEX(Partidos!$K$4:$K$107,MATCH($A305,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H305" s="19">
@@ -22751,7 +22796,7 @@
         <v/>
       </c>
       <c r="G306" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A306,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E306)),NOT(ISNUMBER($F306))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A306,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E306=INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0)),$F306=INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E306-$F306)=(INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E306&gt;$F306,INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),AND($E306=$F306,INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),AND($E306&lt;$F306,INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E306=INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0)),$F306=INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E306-$F306)=(INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H306&lt;&gt;"",$H306=INDEX(Partidos!$K$4:$K$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A306,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E306)),NOT(ISNUMBER($F306))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A306,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E306=INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0)),$F306=INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E306-$F306)=(INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E306&gt;$F306,INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),AND($E306=$F306,INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),AND($E306&lt;$F306,INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0)),IF(AND($E306=INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0)),$F306=INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),IF(AND($H306&lt;&gt;"",$H306=INDEX(Partidos!$K$4:$K$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E306=$F306,($E306-$F306)=(INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0)))),IF(AND($H306&lt;&gt;"",$H306=INDEX(Partidos!$K$4:$K$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H306&lt;&gt;"",$H306=INDEX(Partidos!$K$4:$K$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E306=INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0)),$F306=INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E306-$F306)=(INDEX(Partidos!$F$4:$F$107,MATCH($A306,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H306&lt;&gt;"",$H306=INDEX(Partidos!$K$4:$K$107,MATCH($A306,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H306" s="19">
@@ -22793,7 +22838,7 @@
         <v/>
       </c>
       <c r="G307" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A307,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E307)),NOT(ISNUMBER($F307))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A307,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E307=INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0)),$F307=INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E307-$F307)=(INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E307&gt;$F307,INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),AND($E307=$F307,INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),AND($E307&lt;$F307,INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E307=INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0)),$F307=INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E307-$F307)=(INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H307&lt;&gt;"",$H307=INDEX(Partidos!$K$4:$K$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A307,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E307)),NOT(ISNUMBER($F307))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A307,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E307=INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0)),$F307=INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E307-$F307)=(INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E307&gt;$F307,INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),AND($E307=$F307,INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),AND($E307&lt;$F307,INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0)),IF(AND($E307=INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0)),$F307=INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),IF(AND($H307&lt;&gt;"",$H307=INDEX(Partidos!$K$4:$K$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E307=$F307,($E307-$F307)=(INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0)))),IF(AND($H307&lt;&gt;"",$H307=INDEX(Partidos!$K$4:$K$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H307&lt;&gt;"",$H307=INDEX(Partidos!$K$4:$K$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E307=INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0)),$F307=INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E307-$F307)=(INDEX(Partidos!$F$4:$F$107,MATCH($A307,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H307&lt;&gt;"",$H307=INDEX(Partidos!$K$4:$K$107,MATCH($A307,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H307" s="19">
@@ -22835,7 +22880,7 @@
         <v/>
       </c>
       <c r="G308" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A308,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E308)),NOT(ISNUMBER($F308))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A308,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E308=INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0)),$F308=INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E308-$F308)=(INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E308&gt;$F308,INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),AND($E308=$F308,INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),AND($E308&lt;$F308,INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E308=INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0)),$F308=INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E308-$F308)=(INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H308&lt;&gt;"",$H308=INDEX(Partidos!$K$4:$K$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A308,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E308)),NOT(ISNUMBER($F308))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A308,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E308=INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0)),$F308=INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E308-$F308)=(INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E308&gt;$F308,INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),AND($E308=$F308,INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),AND($E308&lt;$F308,INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0)),IF(AND($E308=INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0)),$F308=INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),IF(AND($H308&lt;&gt;"",$H308=INDEX(Partidos!$K$4:$K$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E308=$F308,($E308-$F308)=(INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0)))),IF(AND($H308&lt;&gt;"",$H308=INDEX(Partidos!$K$4:$K$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H308&lt;&gt;"",$H308=INDEX(Partidos!$K$4:$K$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E308=INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0)),$F308=INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E308-$F308)=(INDEX(Partidos!$F$4:$F$107,MATCH($A308,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H308&lt;&gt;"",$H308=INDEX(Partidos!$K$4:$K$107,MATCH($A308,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H308" s="19">
@@ -22877,7 +22922,7 @@
         <v/>
       </c>
       <c r="G309" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A309,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E309)),NOT(ISNUMBER($F309))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A309,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E309=INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0)),$F309=INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E309-$F309)=(INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E309&gt;$F309,INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),AND($E309=$F309,INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),AND($E309&lt;$F309,INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E309=INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0)),$F309=INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E309-$F309)=(INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H309&lt;&gt;"",$H309=INDEX(Partidos!$K$4:$K$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A309,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E309)),NOT(ISNUMBER($F309))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A309,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E309=INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0)),$F309=INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E309-$F309)=(INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E309&gt;$F309,INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),AND($E309=$F309,INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),AND($E309&lt;$F309,INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0)),IF(AND($E309=INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0)),$F309=INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),IF(AND($H309&lt;&gt;"",$H309=INDEX(Partidos!$K$4:$K$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E309=$F309,($E309-$F309)=(INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0)))),IF(AND($H309&lt;&gt;"",$H309=INDEX(Partidos!$K$4:$K$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H309&lt;&gt;"",$H309=INDEX(Partidos!$K$4:$K$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E309=INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0)),$F309=INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E309-$F309)=(INDEX(Partidos!$F$4:$F$107,MATCH($A309,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H309&lt;&gt;"",$H309=INDEX(Partidos!$K$4:$K$107,MATCH($A309,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H309" s="19">
@@ -22919,7 +22964,7 @@
         <v/>
       </c>
       <c r="G310" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A310,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E310)),NOT(ISNUMBER($F310))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A310,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E310=INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0)),$F310=INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E310-$F310)=(INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E310&gt;$F310,INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),AND($E310=$F310,INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),AND($E310&lt;$F310,INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E310=INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0)),$F310=INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E310-$F310)=(INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H310&lt;&gt;"",$H310=INDEX(Partidos!$K$4:$K$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A310,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E310)),NOT(ISNUMBER($F310))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A310,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E310=INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0)),$F310=INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E310-$F310)=(INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E310&gt;$F310,INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),AND($E310=$F310,INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),AND($E310&lt;$F310,INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0)),IF(AND($E310=INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0)),$F310=INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),IF(AND($H310&lt;&gt;"",$H310=INDEX(Partidos!$K$4:$K$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E310=$F310,($E310-$F310)=(INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0)))),IF(AND($H310&lt;&gt;"",$H310=INDEX(Partidos!$K$4:$K$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H310&lt;&gt;"",$H310=INDEX(Partidos!$K$4:$K$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E310=INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0)),$F310=INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E310-$F310)=(INDEX(Partidos!$F$4:$F$107,MATCH($A310,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H310&lt;&gt;"",$H310=INDEX(Partidos!$K$4:$K$107,MATCH($A310,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H310" s="19">
@@ -22961,7 +23006,7 @@
         <v/>
       </c>
       <c r="G311" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A311,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E311)),NOT(ISNUMBER($F311))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A311,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E311=INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0)),$F311=INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E311-$F311)=(INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E311&gt;$F311,INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),AND($E311=$F311,INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),AND($E311&lt;$F311,INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E311=INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0)),$F311=INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E311-$F311)=(INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H311&lt;&gt;"",$H311=INDEX(Partidos!$K$4:$K$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A311,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E311)),NOT(ISNUMBER($F311))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A311,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E311=INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0)),$F311=INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E311-$F311)=(INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E311&gt;$F311,INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),AND($E311=$F311,INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),AND($E311&lt;$F311,INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0)),IF(AND($E311=INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0)),$F311=INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),IF(AND($H311&lt;&gt;"",$H311=INDEX(Partidos!$K$4:$K$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E311=$F311,($E311-$F311)=(INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0)))),IF(AND($H311&lt;&gt;"",$H311=INDEX(Partidos!$K$4:$K$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H311&lt;&gt;"",$H311=INDEX(Partidos!$K$4:$K$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E311=INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0)),$F311=INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E311-$F311)=(INDEX(Partidos!$F$4:$F$107,MATCH($A311,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H311&lt;&gt;"",$H311=INDEX(Partidos!$K$4:$K$107,MATCH($A311,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H311" s="19">
@@ -23003,7 +23048,7 @@
         <v/>
       </c>
       <c r="G312" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A312,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E312)),NOT(ISNUMBER($F312))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A312,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E312=INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0)),$F312=INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E312-$F312)=(INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E312&gt;$F312,INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),AND($E312=$F312,INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),AND($E312&lt;$F312,INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E312=INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0)),$F312=INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E312-$F312)=(INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H312&lt;&gt;"",$H312=INDEX(Partidos!$K$4:$K$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A312,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E312)),NOT(ISNUMBER($F312))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A312,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E312=INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0)),$F312=INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E312-$F312)=(INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E312&gt;$F312,INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),AND($E312=$F312,INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),AND($E312&lt;$F312,INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0)),IF(AND($E312=INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0)),$F312=INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),IF(AND($H312&lt;&gt;"",$H312=INDEX(Partidos!$K$4:$K$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E312=$F312,($E312-$F312)=(INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0)))),IF(AND($H312&lt;&gt;"",$H312=INDEX(Partidos!$K$4:$K$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H312&lt;&gt;"",$H312=INDEX(Partidos!$K$4:$K$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E312=INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0)),$F312=INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E312-$F312)=(INDEX(Partidos!$F$4:$F$107,MATCH($A312,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H312&lt;&gt;"",$H312=INDEX(Partidos!$K$4:$K$107,MATCH($A312,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H312" s="19">
@@ -23045,7 +23090,7 @@
         <v/>
       </c>
       <c r="G313" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A313,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E313)),NOT(ISNUMBER($F313))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A313,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E313=INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0)),$F313=INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E313-$F313)=(INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E313&gt;$F313,INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),AND($E313=$F313,INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),AND($E313&lt;$F313,INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E313=INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0)),$F313=INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E313-$F313)=(INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H313&lt;&gt;"",$H313=INDEX(Partidos!$K$4:$K$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A313,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E313)),NOT(ISNUMBER($F313))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A313,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E313=INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0)),$F313=INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E313-$F313)=(INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E313&gt;$F313,INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),AND($E313=$F313,INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),AND($E313&lt;$F313,INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0)),IF(AND($E313=INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0)),$F313=INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),IF(AND($H313&lt;&gt;"",$H313=INDEX(Partidos!$K$4:$K$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E313=$F313,($E313-$F313)=(INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0)))),IF(AND($H313&lt;&gt;"",$H313=INDEX(Partidos!$K$4:$K$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H313&lt;&gt;"",$H313=INDEX(Partidos!$K$4:$K$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E313=INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0)),$F313=INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E313-$F313)=(INDEX(Partidos!$F$4:$F$107,MATCH($A313,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H313&lt;&gt;"",$H313=INDEX(Partidos!$K$4:$K$107,MATCH($A313,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H313" s="19">
@@ -23087,7 +23132,7 @@
         <v/>
       </c>
       <c r="G314" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A314,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E314)),NOT(ISNUMBER($F314))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A314,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E314=INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0)),$F314=INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E314-$F314)=(INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E314&gt;$F314,INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),AND($E314=$F314,INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),AND($E314&lt;$F314,INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E314=INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0)),$F314=INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E314-$F314)=(INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H314&lt;&gt;"",$H314=INDEX(Partidos!$K$4:$K$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A314,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E314)),NOT(ISNUMBER($F314))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A314,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E314=INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0)),$F314=INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E314-$F314)=(INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E314&gt;$F314,INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),AND($E314=$F314,INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),AND($E314&lt;$F314,INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0)),IF(AND($E314=INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0)),$F314=INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),IF(AND($H314&lt;&gt;"",$H314=INDEX(Partidos!$K$4:$K$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E314=$F314,($E314-$F314)=(INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0)))),IF(AND($H314&lt;&gt;"",$H314=INDEX(Partidos!$K$4:$K$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H314&lt;&gt;"",$H314=INDEX(Partidos!$K$4:$K$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E314=INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0)),$F314=INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E314-$F314)=(INDEX(Partidos!$F$4:$F$107,MATCH($A314,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H314&lt;&gt;"",$H314=INDEX(Partidos!$K$4:$K$107,MATCH($A314,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H314" s="19">
@@ -23129,7 +23174,7 @@
         <v/>
       </c>
       <c r="G315" s="16">
-        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A315,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E315)),NOT(ISNUMBER($F315))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A315,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E315=INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0)),$F315=INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E315-$F315)=(INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E315&gt;$F315,INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),AND($E315=$F315,INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),AND($E315&lt;$F315,INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(AND($E315=INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0)),$F315=INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E315-$F315)=(INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H315&lt;&gt;"",$H315=INDEX(Partidos!$K$4:$K$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0)))))),"")</f>
+        <f>IFERROR(IF(INDEX(Partidos!$H$4:$H$107,MATCH($A315,Partidos!$A$4:$A$107,0))&lt;&gt;"Finalizado","",IF(OR(NOT(ISNUMBER($E315)),NOT(ISNUMBER($F315))),"",IF(INDEX(Partidos!$J$4:$J$107,MATCH($A315,Partidos!$A$4:$A$107,0))="Grupos",IF(AND($E315=INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0)),$F315=INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$4,IF(($E315-$F315)=(INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$5,IF(OR(AND($E315&gt;$F315,INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0))&gt;INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),AND($E315=$F315,INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),AND($E315&lt;$F315,INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0))&lt;INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0)))),Puntuacion!$B$6,0))),IF(INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0))=INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0)),IF(AND($E315=INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0)),$F315=INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),IF(AND($H315&lt;&gt;"",$H315=INDEX(Partidos!$K$4:$K$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,Puntuacion!$B$12),IF(AND($E315=$F315,($E315-$F315)=(INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0)))),IF(AND($H315&lt;&gt;"",$H315=INDEX(Partidos!$K$4:$K$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$13,Puntuacion!$B$14),IF(AND($H315&lt;&gt;"",$H315=INDEX(Partidos!$K$4:$K$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))),IF(AND($E315=INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0)),$F315=INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$9,IF(($E315-$F315)=(INDEX(Partidos!$F$4:$F$107,MATCH($A315,Partidos!$A$4:$A$107,0))-INDEX(Partidos!$G$4:$G$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$10,IF(AND($H315&lt;&gt;"",$H315=INDEX(Partidos!$K$4:$K$107,MATCH($A315,Partidos!$A$4:$A$107,0))),Puntuacion!$B$11,0))))))),"")</f>
         <v/>
       </c>
       <c r="H315" s="19">

</xml_diff>

<commit_message>
Ajustar ponderacion eliminatorias a 8/4/3.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -2458,7 +2458,6 @@
       <c r="C1" s="1" t="n"/>
       <c r="D1" s="1" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="21" t="inlineStr">
         <is>
@@ -2511,7 +2510,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
@@ -2526,7 +2524,7 @@
         </is>
       </c>
       <c r="B9" s="32" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -2541,7 +2539,7 @@
         </is>
       </c>
       <c r="B10" s="32" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -2556,7 +2554,7 @@
         </is>
       </c>
       <c r="B11" s="32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -2571,7 +2569,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -2586,7 +2584,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -2661,7 +2659,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="21" t="inlineStr">
         <is>
@@ -2922,7 +2919,6 @@
         <v/>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
@@ -3033,7 +3029,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -3311,7 +3306,6 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
@@ -3626,7 +3620,6 @@
         <v/>
       </c>
     </row>
-    <row r="32"/>
     <row r="33" ht="28.8" customHeight="1">
       <c r="A33" s="14" t="inlineStr">
         <is>
@@ -3800,7 +3793,6 @@
         <v/>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
         <is>
@@ -3894,7 +3886,6 @@
         <v/>
       </c>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
@@ -4169,7 +4160,6 @@
         <v/>
       </c>
     </row>
-    <row r="68"/>
     <row r="69">
       <c r="U69">
         <f>IF(1&lt;=COUNTIF(Partidos!$H$4:$H$107,"Finalizado"),INDEX(Partidos!$D$4:$D$107,COUNTIF(Partidos!$H$4:$H$107,"Finalizado")-0),"")</f>
@@ -4348,7 +4338,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -4368,7 +4357,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
@@ -4388,7 +4376,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -4408,7 +4395,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
@@ -4428,7 +4414,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
@@ -4448,8 +4433,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21"/>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -4926,12 +4909,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21" ht="7.95" customHeight="1"/>
     <row r="22" ht="15.6" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -5280,9 +5257,6 @@
         <v/>
       </c>
     </row>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
     <row r="45" ht="7.95" customHeight="1"/>
     <row r="46" ht="15.6" customHeight="1">
       <c r="A46" s="8" t="inlineStr">
@@ -26811,7 +26785,6 @@
       <c r="G107" s="27" t="n"/>
       <c r="H107" s="27" t="n"/>
     </row>
-    <row r="108"/>
     <row r="109" ht="15.6" customHeight="1">
       <c r="A109" s="8" t="inlineStr">
         <is>
@@ -30340,7 +30313,6 @@
       <c r="G107" s="27" t="n"/>
       <c r="H107" s="27" t="n"/>
     </row>
-    <row r="108"/>
     <row r="109" ht="15.6" customHeight="1">
       <c r="A109" s="8" t="inlineStr">
         <is>
@@ -33869,7 +33841,6 @@
       <c r="G107" s="27" t="n"/>
       <c r="H107" s="27" t="n"/>
     </row>
-    <row r="108"/>
     <row r="109" ht="15.6" customHeight="1">
       <c r="A109" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Reorder R32 chronologically, import all predictions, refresh dashboard data.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="1" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="1" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
@@ -573,13 +573,13 @@
               <strCache>
                 <ptCount val="3"/>
                 <pt idx="0">
-                  <v>Diego</v>
+                  <v>Papá</v>
                 </pt>
                 <pt idx="1">
                   <v>Álvaro</v>
                 </pt>
                 <pt idx="2">
-                  <v>Álvaro</v>
+                  <v>Diego</v>
                 </pt>
               </strCache>
             </strRef>
@@ -591,13 +591,13 @@
                 <formatCode>General</formatCode>
                 <ptCount val="3"/>
                 <pt idx="0">
-                  <v>12</v>
+                  <v>130</v>
                 </pt>
                 <pt idx="1">
-                  <v>11</v>
+                  <v>130</v>
                 </pt>
                 <pt idx="2">
-                  <v>11</v>
+                  <v>82</v>
                 </pt>
               </numCache>
             </numRef>
@@ -733,13 +733,13 @@
                 <formatCode>General</formatCode>
                 <ptCount val="3"/>
                 <pt idx="0">
-                  <v>11</v>
+                  <v>130</v>
                 </pt>
                 <pt idx="1">
-                  <v>11</v>
+                  <v>130</v>
                 </pt>
                 <pt idx="2">
-                  <v>12</v>
+                  <v>82</v>
                 </pt>
               </numCache>
             </numRef>
@@ -943,7 +943,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v>Diego</v>
+                  <v>Papá</v>
                 </pt>
               </strCache>
             </strRef>
@@ -971,49 +971,49 @@
                 <formatCode>General</formatCode>
                 <ptCount val="15"/>
                 <pt idx="0">
-                  <v>5</v>
+                  <v>2</v>
                 </pt>
                 <pt idx="1">
-                  <v>5</v>
+                  <v>7</v>
                 </pt>
                 <pt idx="2">
-                  <v>5</v>
+                  <v>7</v>
                 </pt>
                 <pt idx="3">
-                  <v>5</v>
+                  <v>7</v>
                 </pt>
                 <pt idx="4">
-                  <v>5</v>
+                  <v>7</v>
                 </pt>
                 <pt idx="5">
-                  <v>8</v>
+                  <v>7</v>
                 </pt>
                 <pt idx="6">
-                  <v>10</v>
+                  <v>9</v>
                 </pt>
                 <pt idx="7">
-                  <v>10</v>
+                  <v>9</v>
                 </pt>
                 <pt idx="8">
-                  <v>12</v>
+                  <v>11</v>
                 </pt>
                 <pt idx="9">
-                  <v>12</v>
+                  <v>11</v>
                 </pt>
                 <pt idx="10">
-                  <v>12</v>
+                  <v>16</v>
                 </pt>
                 <pt idx="11">
-                  <v>12</v>
+                  <v>16</v>
                 </pt>
                 <pt idx="12">
-                  <v>12</v>
+                  <v>16</v>
                 </pt>
                 <pt idx="13">
-                  <v>12</v>
+                  <v>21</v>
                 </pt>
                 <pt idx="14">
-                  <v>12</v>
+                  <v>21</v>
                 </pt>
               </numCache>
             </numRef>
@@ -1084,22 +1084,22 @@
                   <v>11</v>
                 </pt>
                 <pt idx="9">
-                  <v>11</v>
+                  <v>14</v>
                 </pt>
                 <pt idx="10">
-                  <v>11</v>
+                  <v>14</v>
                 </pt>
                 <pt idx="11">
-                  <v>11</v>
+                  <v>14</v>
                 </pt>
                 <pt idx="12">
-                  <v>11</v>
+                  <v>14</v>
                 </pt>
                 <pt idx="13">
-                  <v>11</v>
+                  <v>14</v>
                 </pt>
                 <pt idx="14">
-                  <v>11</v>
+                  <v>14</v>
                 </pt>
               </numCache>
             </numRef>
@@ -1115,7 +1115,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v>Álvaro</v>
+                  <v>Diego</v>
                 </pt>
               </strCache>
             </strRef>
@@ -1143,49 +1143,49 @@
                 <formatCode>General</formatCode>
                 <ptCount val="15"/>
                 <pt idx="0">
-                  <v>2</v>
+                  <v>5</v>
                 </pt>
                 <pt idx="1">
-                  <v>2</v>
+                  <v>5</v>
                 </pt>
                 <pt idx="2">
-                  <v>2</v>
+                  <v>5</v>
                 </pt>
                 <pt idx="3">
-                  <v>2</v>
+                  <v>5</v>
                 </pt>
                 <pt idx="4">
-                  <v>2</v>
+                  <v>5</v>
                 </pt>
                 <pt idx="5">
-                  <v>7</v>
+                  <v>8</v>
                 </pt>
                 <pt idx="6">
-                  <v>9</v>
+                  <v>10</v>
                 </pt>
                 <pt idx="7">
-                  <v>9</v>
+                  <v>10</v>
                 </pt>
                 <pt idx="8">
-                  <v>11</v>
+                  <v>12</v>
                 </pt>
                 <pt idx="9">
-                  <v>11</v>
+                  <v>12</v>
                 </pt>
                 <pt idx="10">
-                  <v>11</v>
+                  <v>14</v>
                 </pt>
                 <pt idx="11">
-                  <v>11</v>
+                  <v>14</v>
                 </pt>
                 <pt idx="12">
-                  <v>11</v>
+                  <v>14</v>
                 </pt>
                 <pt idx="13">
-                  <v>11</v>
+                  <v>14</v>
                 </pt>
                 <pt idx="14">
-                  <v>11</v>
+                  <v>14</v>
                 </pt>
               </numCache>
             </numRef>
@@ -1332,13 +1332,13 @@
                 <formatCode>General</formatCode>
                 <ptCount val="3"/>
                 <pt idx="0">
-                  <v>1</v>
+                  <v>12</v>
                 </pt>
                 <pt idx="1">
-                  <v>1</v>
+                  <v>9</v>
                 </pt>
                 <pt idx="2">
-                  <v>1</v>
+                  <v>3</v>
                 </pt>
               </numCache>
             </numRef>
@@ -1369,13 +1369,13 @@
                 <formatCode>General</formatCode>
                 <ptCount val="3"/>
                 <pt idx="0">
-                  <v>3</v>
+                  <v>37</v>
                 </pt>
                 <pt idx="1">
-                  <v>3</v>
+                  <v>47</v>
                 </pt>
                 <pt idx="2">
-                  <v>3</v>
+                  <v>35</v>
                 </pt>
               </numCache>
             </numRef>
@@ -1406,13 +1406,13 @@
                 <formatCode>General</formatCode>
                 <ptCount val="3"/>
                 <pt idx="0">
-                  <v>5</v>
+                  <v>31</v>
                 </pt>
                 <pt idx="1">
-                  <v>5</v>
+                  <v>29</v>
                 </pt>
                 <pt idx="2">
-                  <v>5</v>
+                  <v>38</v>
                 </pt>
               </numCache>
             </numRef>
@@ -8923,17 +8923,17 @@
       </c>
       <c r="C77" s="24" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D77" s="19" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E77" s="19" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F77" s="27" t="n"/>
@@ -8963,17 +8963,17 @@
       </c>
       <c r="C78" s="26" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="D78" s="19" t="inlineStr">
         <is>
-          <t>Países Bajos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="E78" s="19" t="inlineStr">
         <is>
-          <t>Marruecos</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="F78" s="27" t="n"/>
@@ -9003,17 +9003,17 @@
       </c>
       <c r="C79" s="24" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D79" s="19" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Países Bajos</t>
         </is>
       </c>
       <c r="E79" s="19" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Marruecos</t>
         </is>
       </c>
       <c r="F79" s="27" t="n"/>
@@ -9043,17 +9043,17 @@
       </c>
       <c r="C80" s="26" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D80" s="19" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Costa de Marfil</t>
         </is>
       </c>
       <c r="E80" s="19" t="inlineStr">
         <is>
-          <t>Suecia</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F80" s="27" t="n"/>
@@ -9083,17 +9083,17 @@
       </c>
       <c r="C81" s="24" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D81" s="19" t="inlineStr">
         <is>
-          <t>Costa de Marfil</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="E81" s="19" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>Suecia</t>
         </is>
       </c>
       <c r="F81" s="27" t="n"/>
@@ -9203,17 +9203,17 @@
       </c>
       <c r="C84" s="26" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D84" s="19" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Bélgica</t>
         </is>
       </c>
       <c r="E84" s="19" t="inlineStr">
         <is>
-          <t>Bosnia y Herzegovina</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="F84" s="27" t="n"/>
@@ -9243,17 +9243,17 @@
       </c>
       <c r="C85" s="24" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D85" s="19" t="inlineStr">
         <is>
-          <t>Bélgica</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E85" s="19" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Bosnia y Herzegovina</t>
         </is>
       </c>
       <c r="F85" s="27" t="n"/>
@@ -9283,17 +9283,17 @@
       </c>
       <c r="C86" s="26" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D86" s="19" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E86" s="19" t="inlineStr">
         <is>
-          <t>Croacia</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="F86" s="27" t="n"/>
@@ -9323,17 +9323,17 @@
       </c>
       <c r="C87" s="24" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D87" s="19" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E87" s="19" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Croacia</t>
         </is>
       </c>
       <c r="F87" s="27" t="n"/>
@@ -9403,17 +9403,17 @@
       </c>
       <c r="C89" s="24" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D89" s="19" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="E89" s="19" t="inlineStr">
         <is>
-          <t>Cabo Verde</t>
+          <t>Egipto</t>
         </is>
       </c>
       <c r="F89" s="27" t="n"/>
@@ -9443,17 +9443,17 @@
       </c>
       <c r="C90" s="26" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D90" s="19" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E90" s="19" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Cabo Verde</t>
         </is>
       </c>
       <c r="F90" s="27" t="n"/>
@@ -9483,17 +9483,17 @@
       </c>
       <c r="C91" s="24" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="D91" s="19" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E91" s="19" t="inlineStr">
         <is>
-          <t>Egipto</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="F91" s="27" t="n"/>
@@ -25983,9 +25983,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A76,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F76" s="27" t="n"/>
-      <c r="G76" s="27" t="n"/>
-      <c r="H76" s="27" t="n"/>
+      <c r="F76" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="24" t="n">
@@ -26009,9 +26017,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A77,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F77" s="27" t="n"/>
-      <c r="G77" s="27" t="n"/>
-      <c r="H77" s="27" t="n"/>
+      <c r="F77" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="26" t="n">
@@ -26035,9 +26051,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A78,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F78" s="27" t="n"/>
-      <c r="G78" s="27" t="n"/>
-      <c r="H78" s="27" t="n"/>
+      <c r="F78" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G78" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="24" t="n">
@@ -26061,9 +26085,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A79,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F79" s="27" t="n"/>
-      <c r="G79" s="27" t="n"/>
-      <c r="H79" s="27" t="n"/>
+      <c r="F79" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H79" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="26" t="n">
@@ -26087,9 +26119,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A80,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F80" s="27" t="n"/>
-      <c r="G80" s="27" t="n"/>
-      <c r="H80" s="27" t="n"/>
+      <c r="F80" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="24" t="n">
@@ -26113,9 +26153,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A81,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F81" s="27" t="n"/>
-      <c r="G81" s="27" t="n"/>
-      <c r="H81" s="27" t="n"/>
+      <c r="F81" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G81" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="26" t="n">
@@ -26139,9 +26187,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A82,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F82" s="27" t="n"/>
-      <c r="G82" s="27" t="n"/>
-      <c r="H82" s="27" t="n"/>
+      <c r="F82" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="24" t="n">
@@ -26165,9 +26221,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A83,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F83" s="27" t="n"/>
-      <c r="G83" s="27" t="n"/>
-      <c r="H83" s="27" t="n"/>
+      <c r="F83" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G83" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="26" t="n">
@@ -26191,9 +26255,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A84,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F84" s="27" t="n"/>
-      <c r="G84" s="27" t="n"/>
-      <c r="H84" s="27" t="n"/>
+      <c r="F84" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H84" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="24" t="n">
@@ -26217,9 +26289,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A85,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F85" s="27" t="n"/>
-      <c r="G85" s="27" t="n"/>
-      <c r="H85" s="27" t="n"/>
+      <c r="F85" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G85" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="26" t="n">
@@ -26243,9 +26323,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A86,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F86" s="27" t="n"/>
-      <c r="G86" s="27" t="n"/>
-      <c r="H86" s="27" t="n"/>
+      <c r="F86" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G86" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="24" t="n">
@@ -26269,9 +26357,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A87,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F87" s="27" t="n"/>
-      <c r="G87" s="27" t="n"/>
-      <c r="H87" s="27" t="n"/>
+      <c r="F87" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H87" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="26" t="n">
@@ -26295,9 +26391,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A88,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F88" s="27" t="n"/>
-      <c r="G88" s="27" t="n"/>
-      <c r="H88" s="27" t="n"/>
+      <c r="F88" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H88" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="24" t="n">
@@ -26321,9 +26425,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A89,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F89" s="27" t="n"/>
-      <c r="G89" s="27" t="n"/>
-      <c r="H89" s="27" t="n"/>
+      <c r="F89" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G89" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H89" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="26" t="n">
@@ -26347,9 +26459,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A90,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F90" s="27" t="n"/>
-      <c r="G90" s="27" t="n"/>
-      <c r="H90" s="27" t="n"/>
+      <c r="F90" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G90" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="24" t="n">
@@ -26373,9 +26493,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A91,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F91" s="27" t="n"/>
-      <c r="G91" s="27" t="n"/>
-      <c r="H91" s="27" t="n"/>
+      <c r="F91" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="26" t="n">
@@ -29511,9 +29639,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A76,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F76" s="27" t="n"/>
-      <c r="G76" s="27" t="n"/>
-      <c r="H76" s="27" t="n"/>
+      <c r="F76" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="24" t="n">
@@ -29537,9 +29673,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A77,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F77" s="27" t="n"/>
-      <c r="G77" s="27" t="n"/>
-      <c r="H77" s="27" t="n"/>
+      <c r="F77" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G77" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="26" t="n">
@@ -29563,9 +29707,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A78,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F78" s="27" t="n"/>
-      <c r="G78" s="27" t="n"/>
-      <c r="H78" s="27" t="n"/>
+      <c r="F78" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G78" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="24" t="n">
@@ -29589,9 +29741,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A79,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F79" s="27" t="n"/>
-      <c r="G79" s="27" t="n"/>
-      <c r="H79" s="27" t="n"/>
+      <c r="F79" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G79" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="H79" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="26" t="n">
@@ -29615,9 +29775,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A80,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F80" s="27" t="n"/>
-      <c r="G80" s="27" t="n"/>
-      <c r="H80" s="27" t="n"/>
+      <c r="F80" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H80" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="24" t="n">
@@ -29641,9 +29809,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A81,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F81" s="27" t="n"/>
-      <c r="G81" s="27" t="n"/>
-      <c r="H81" s="27" t="n"/>
+      <c r="F81" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G81" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H81" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="26" t="n">
@@ -29667,9 +29843,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A82,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F82" s="27" t="n"/>
-      <c r="G82" s="27" t="n"/>
-      <c r="H82" s="27" t="n"/>
+      <c r="F82" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G82" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="24" t="n">
@@ -29693,9 +29877,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A83,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F83" s="27" t="n"/>
-      <c r="G83" s="27" t="n"/>
-      <c r="H83" s="27" t="n"/>
+      <c r="F83" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="26" t="n">
@@ -29719,9 +29911,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A84,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F84" s="27" t="n"/>
-      <c r="G84" s="27" t="n"/>
-      <c r="H84" s="27" t="n"/>
+      <c r="F84" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="24" t="n">
@@ -29745,9 +29945,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A85,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F85" s="27" t="n"/>
-      <c r="G85" s="27" t="n"/>
-      <c r="H85" s="27" t="n"/>
+      <c r="F85" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="26" t="n">
@@ -29771,9 +29979,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A86,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F86" s="27" t="n"/>
-      <c r="G86" s="27" t="n"/>
-      <c r="H86" s="27" t="n"/>
+      <c r="F86" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G86" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="24" t="n">
@@ -29797,9 +30013,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A87,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F87" s="27" t="n"/>
-      <c r="G87" s="27" t="n"/>
-      <c r="H87" s="27" t="n"/>
+      <c r="F87" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H87" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="26" t="n">
@@ -29823,9 +30047,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A88,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F88" s="27" t="n"/>
-      <c r="G88" s="27" t="n"/>
-      <c r="H88" s="27" t="n"/>
+      <c r="F88" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G88" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="24" t="n">
@@ -29849,9 +30081,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A89,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F89" s="27" t="n"/>
-      <c r="G89" s="27" t="n"/>
-      <c r="H89" s="27" t="n"/>
+      <c r="F89" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H89" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="26" t="n">
@@ -29875,9 +30115,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A90,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F90" s="27" t="n"/>
-      <c r="G90" s="27" t="n"/>
-      <c r="H90" s="27" t="n"/>
+      <c r="F90" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G90" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="24" t="n">
@@ -29901,9 +30149,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A91,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F91" s="27" t="n"/>
-      <c r="G91" s="27" t="n"/>
-      <c r="H91" s="27" t="n"/>
+      <c r="F91" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G91" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H91" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="26" t="n">
@@ -33039,9 +33295,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A76,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F76" s="27" t="n"/>
-      <c r="G76" s="27" t="n"/>
-      <c r="H76" s="27" t="n"/>
+      <c r="F76" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H76" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="24" t="n">
@@ -33065,9 +33329,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A77,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F77" s="27" t="n"/>
-      <c r="G77" s="27" t="n"/>
-      <c r="H77" s="27" t="n"/>
+      <c r="F77" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="26" t="n">
@@ -33091,9 +33363,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A78,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F78" s="27" t="n"/>
-      <c r="G78" s="27" t="n"/>
-      <c r="H78" s="27" t="n"/>
+      <c r="F78" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="G78" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H78" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="24" t="n">
@@ -33117,9 +33397,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A79,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F79" s="27" t="n"/>
-      <c r="G79" s="27" t="n"/>
-      <c r="H79" s="27" t="n"/>
+      <c r="F79" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H79" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="26" t="n">
@@ -33143,9 +33431,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A80,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F80" s="27" t="n"/>
-      <c r="G80" s="27" t="n"/>
-      <c r="H80" s="27" t="n"/>
+      <c r="F80" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G80" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="24" t="n">
@@ -33169,9 +33465,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A81,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F81" s="27" t="n"/>
-      <c r="G81" s="27" t="n"/>
-      <c r="H81" s="27" t="n"/>
+      <c r="F81" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G81" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H81" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="26" t="n">
@@ -33195,9 +33499,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A82,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F82" s="27" t="n"/>
-      <c r="G82" s="27" t="n"/>
-      <c r="H82" s="27" t="n"/>
+      <c r="F82" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G82" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H82" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="24" t="n">
@@ -33221,9 +33533,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A83,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F83" s="27" t="n"/>
-      <c r="G83" s="27" t="n"/>
-      <c r="H83" s="27" t="n"/>
+      <c r="F83" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G83" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="26" t="n">
@@ -33247,9 +33567,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A84,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F84" s="27" t="n"/>
-      <c r="G84" s="27" t="n"/>
-      <c r="H84" s="27" t="n"/>
+      <c r="F84" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H84" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="24" t="n">
@@ -33273,9 +33601,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A85,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F85" s="27" t="n"/>
-      <c r="G85" s="27" t="n"/>
-      <c r="H85" s="27" t="n"/>
+      <c r="F85" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G85" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="26" t="n">
@@ -33299,9 +33635,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A86,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F86" s="27" t="n"/>
-      <c r="G86" s="27" t="n"/>
-      <c r="H86" s="27" t="n"/>
+      <c r="F86" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H86" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="24" t="n">
@@ -33325,9 +33669,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A87,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F87" s="27" t="n"/>
-      <c r="G87" s="27" t="n"/>
-      <c r="H87" s="27" t="n"/>
+      <c r="F87" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G87" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H87" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="26" t="n">
@@ -33351,9 +33703,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A88,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F88" s="27" t="n"/>
-      <c r="G88" s="27" t="n"/>
-      <c r="H88" s="27" t="n"/>
+      <c r="F88" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G88" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H88" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="24" t="n">
@@ -33377,9 +33737,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A89,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F89" s="27" t="n"/>
-      <c r="G89" s="27" t="n"/>
-      <c r="H89" s="27" t="n"/>
+      <c r="F89" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G89" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H89" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="26" t="n">
@@ -33403,9 +33771,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A90,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F90" s="27" t="n"/>
-      <c r="G90" s="27" t="n"/>
-      <c r="H90" s="27" t="n"/>
+      <c r="F90" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G90" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="24" t="n">
@@ -33429,9 +33805,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A91,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F91" s="27" t="n"/>
-      <c r="G91" s="27" t="n"/>
-      <c r="H91" s="27" t="n"/>
+      <c r="F91" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="26" t="n">

</xml_diff>

<commit_message>
Fix R32 result sync: match by teams, 90min scores, penalty clasificado
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -8936,8 +8936,12 @@
           <t>Japón</t>
         </is>
       </c>
-      <c r="F77" s="27" t="n"/>
-      <c r="G77" s="27" t="n"/>
+      <c r="F77" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G77" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H77" s="16">
         <f>IF(AND(ISNUMBER(F77),ISNUMBER(G77)),"Finalizado","Pendiente")</f>
         <v/>
@@ -8950,7 +8954,11 @@
           <t>Dieciseisavos</t>
         </is>
       </c>
-      <c r="K77" s="27" t="n"/>
+      <c r="K77" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="26" t="n">
@@ -8976,8 +8984,12 @@
           <t>Paraguay</t>
         </is>
       </c>
-      <c r="F78" s="27" t="n"/>
-      <c r="G78" s="27" t="n"/>
+      <c r="F78" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H78" s="16">
         <f>IF(AND(ISNUMBER(F78),ISNUMBER(G78)),"Finalizado","Pendiente")</f>
         <v/>
@@ -8990,7 +9002,11 @@
           <t>Dieciseisavos</t>
         </is>
       </c>
-      <c r="K78" s="27" t="n"/>
+      <c r="K78" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="24" t="n">
@@ -9016,8 +9032,12 @@
           <t>Marruecos</t>
         </is>
       </c>
-      <c r="F79" s="27" t="n"/>
-      <c r="G79" s="27" t="n"/>
+      <c r="F79" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H79" s="16">
         <f>IF(AND(ISNUMBER(F79),ISNUMBER(G79)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9030,7 +9050,11 @@
           <t>Dieciseisavos</t>
         </is>
       </c>
-      <c r="K79" s="27" t="n"/>
+      <c r="K79" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="26" t="n">

</xml_diff>

<commit_message>
Corregir clasificado en empates resueltos en prórroga (Bélgica-Senegal)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -9080,8 +9080,12 @@
           <t>Noruega</t>
         </is>
       </c>
-      <c r="F80" s="27" t="n"/>
-      <c r="G80" s="27" t="n"/>
+      <c r="F80" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="27" t="n">
+        <v>2</v>
+      </c>
       <c r="H80" s="16">
         <f>IF(AND(ISNUMBER(F80),ISNUMBER(G80)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9094,7 +9098,11 @@
           <t>Dieciseisavos</t>
         </is>
       </c>
-      <c r="K80" s="27" t="n"/>
+      <c r="K80" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="24" t="n">
@@ -9120,8 +9128,12 @@
           <t>Suecia</t>
         </is>
       </c>
-      <c r="F81" s="27" t="n"/>
-      <c r="G81" s="27" t="n"/>
+      <c r="F81" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G81" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="H81" s="16">
         <f>IF(AND(ISNUMBER(F81),ISNUMBER(G81)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9134,7 +9146,11 @@
           <t>Dieciseisavos</t>
         </is>
       </c>
-      <c r="K81" s="27" t="n"/>
+      <c r="K81" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="26" t="n">
@@ -9160,8 +9176,12 @@
           <t>Ecuador</t>
         </is>
       </c>
-      <c r="F82" s="27" t="n"/>
-      <c r="G82" s="27" t="n"/>
+      <c r="F82" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G82" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="H82" s="16">
         <f>IF(AND(ISNUMBER(F82),ISNUMBER(G82)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9174,7 +9194,11 @@
           <t>Dieciseisavos</t>
         </is>
       </c>
-      <c r="K82" s="27" t="n"/>
+      <c r="K82" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="24" t="n">
@@ -9200,8 +9224,12 @@
           <t>RD Congo</t>
         </is>
       </c>
-      <c r="F83" s="27" t="n"/>
-      <c r="G83" s="27" t="n"/>
+      <c r="F83" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G83" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H83" s="16">
         <f>IF(AND(ISNUMBER(F83),ISNUMBER(G83)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9214,7 +9242,11 @@
           <t>Dieciseisavos</t>
         </is>
       </c>
-      <c r="K83" s="27" t="n"/>
+      <c r="K83" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="26" t="n">
@@ -9240,8 +9272,12 @@
           <t>Senegal</t>
         </is>
       </c>
-      <c r="F84" s="27" t="n"/>
-      <c r="G84" s="27" t="n"/>
+      <c r="F84" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G84" s="27" t="n">
+        <v>2</v>
+      </c>
       <c r="H84" s="16">
         <f>IF(AND(ISNUMBER(F84),ISNUMBER(G84)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9254,7 +9290,11 @@
           <t>Dieciseisavos</t>
         </is>
       </c>
-      <c r="K84" s="27" t="n"/>
+      <c r="K84" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="24" t="n">
@@ -9280,8 +9320,12 @@
           <t>Bosnia y Herzegovina</t>
         </is>
       </c>
-      <c r="F85" s="27" t="n"/>
-      <c r="G85" s="27" t="n"/>
+      <c r="F85" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G85" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="H85" s="16">
         <f>IF(AND(ISNUMBER(F85),ISNUMBER(G85)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9294,7 +9338,11 @@
           <t>Dieciseisavos</t>
         </is>
       </c>
-      <c r="K85" s="27" t="n"/>
+      <c r="K85" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="26" t="n">

</xml_diff>

<commit_message>
Anadir octavos con equipos reales y propagacion automatica del cuadro
Propaga ganadores R32 a octavos en cada sync, actualiza matches_2026.json y Excel, e importa pronosticos parciales de amigos.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="1" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Partidos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Pronosticos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Helpers &gt;&gt;" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Álvaro" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Papá" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Diego" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Puntuacion" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="_Helpers" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="_Lists" sheetId="12" state="hidden" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partidos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pronosticos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Helpers &gt;&gt;" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Álvaro" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papá" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diego" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puntuacion" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Helpers" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="12" state="hidden" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Partidos'!$A$3:$K$107</definedName>
@@ -507,14 +507,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -540,10 +540,10 @@
             <v>Puntos</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="051C2C"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="051C2C"/>
               </a:solidFill>
@@ -553,8 +553,8 @@
           <invertIfNegative val="1"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -625,9 +625,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -674,14 +674,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -715,10 +715,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="0066CC"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="0066CC"/>
               </a:solidFill>
@@ -760,10 +760,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="C5A028"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="C5A028"/>
               </a:solidFill>
@@ -805,10 +805,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="051C2C"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="051C2C"/>
               </a:solidFill>
@@ -858,9 +858,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -910,14 +910,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -949,7 +949,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="C5A028"/>
               </a:solidFill>
@@ -959,7 +959,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1035,7 +1035,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="0066CC"/>
               </a:solidFill>
@@ -1045,7 +1045,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1121,7 +1121,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="2E7D32"/>
               </a:solidFill>
@@ -1131,7 +1131,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1214,9 +1214,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1248,9 +1248,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1282,14 +1282,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1314,10 +1314,10 @@
             <v>Exactos</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2E7D32"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="2E7D32"/>
               </a:solidFill>
@@ -1351,10 +1351,10 @@
             <v>Parciales</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="C5A028"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="C5A028"/>
               </a:solidFill>
@@ -1388,10 +1388,10 @@
             <v>Fallos</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="B71C1C"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="B71C1C"/>
               </a:solidFill>
@@ -1441,9 +1441,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1492,7 +1492,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -1510,24 +1510,24 @@
       <nvPicPr>
         <cNvPr id="4" name="Picture 3"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="0" y="0"/>
           <a:ext cx="11469077" cy="4395889"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -1538,7 +1538,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -1553,9 +1553,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1575,9 +1575,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1597,9 +1597,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1619,9 +1619,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -9648,12 +9648,12 @@
       </c>
       <c r="D92" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 1</t>
+          <t>Canadá</t>
         </is>
       </c>
       <c r="E92" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 2</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="F92" s="27" t="n"/>
@@ -9688,12 +9688,12 @@
       </c>
       <c r="D93" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 3</t>
+          <t>Marruecos</t>
         </is>
       </c>
       <c r="E93" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 4</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="F93" s="27" t="n"/>
@@ -9728,12 +9728,12 @@
       </c>
       <c r="D94" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 5</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="E94" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 6</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F94" s="27" t="n"/>
@@ -9768,12 +9768,12 @@
       </c>
       <c r="D95" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 7</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E95" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 8</t>
+          <t>Inglaterra</t>
         </is>
       </c>
       <c r="F95" s="27" t="n"/>
@@ -9808,12 +9808,12 @@
       </c>
       <c r="D96" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 9</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E96" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 10</t>
+          <t>Bélgica</t>
         </is>
       </c>
       <c r="F96" s="27" t="n"/>
@@ -9848,12 +9848,12 @@
       </c>
       <c r="D97" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 11</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E97" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 12</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F97" s="27" t="n"/>
@@ -9888,12 +9888,12 @@
       </c>
       <c r="D98" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 13</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="E98" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 14</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F98" s="27" t="n"/>
@@ -9928,12 +9928,12 @@
       </c>
       <c r="D99" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 15</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E99" s="19" t="inlineStr">
         <is>
-          <t>Ganador Octavos 16</t>
+          <t>Egipto</t>
         </is>
       </c>
       <c r="F99" s="27" t="n"/>
@@ -30381,9 +30381,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A95,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F95" s="27" t="n"/>
-      <c r="G95" s="27" t="n"/>
-      <c r="H95" s="27" t="n"/>
+      <c r="F95" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H95" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="26" t="n">
@@ -30407,9 +30415,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A96,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F96" s="27" t="n"/>
-      <c r="G96" s="27" t="n"/>
-      <c r="H96" s="27" t="n"/>
+      <c r="F96" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G96" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H96" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="24" t="n">
@@ -30433,9 +30449,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A97,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F97" s="27" t="n"/>
-      <c r="G97" s="27" t="n"/>
-      <c r="H97" s="27" t="n"/>
+      <c r="F97" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H97" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="26" t="n">
@@ -34037,9 +34061,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A95,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F95" s="27" t="n"/>
-      <c r="G95" s="27" t="n"/>
-      <c r="H95" s="27" t="n"/>
+      <c r="F95" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H95" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="26" t="n">
@@ -34063,9 +34095,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A96,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F96" s="27" t="n"/>
-      <c r="G96" s="27" t="n"/>
-      <c r="H96" s="27" t="n"/>
+      <c r="F96" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G96" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="24" t="n">
@@ -34089,9 +34129,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A97,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F97" s="27" t="n"/>
-      <c r="G97" s="27" t="n"/>
-      <c r="H97" s="27" t="n"/>
+      <c r="F97" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G97" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H97" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="26" t="n">

</xml_diff>

<commit_message>
Corregir octavos, cuartos y pronosticos con equipos canonicos openfootball
Fija parejas 89-96, mapeo plantilla 89-90, cuartos #97 Francia-Marruecos, importacion amigos, preds Broshu y sync por fecha+hora.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -9648,16 +9648,20 @@
       </c>
       <c r="D92" s="19" t="inlineStr">
         <is>
-          <t>Canadá</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="E92" s="19" t="inlineStr">
         <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-      <c r="F92" s="27" t="n"/>
-      <c r="G92" s="27" t="n"/>
+          <t>Francia</t>
+        </is>
+      </c>
+      <c r="F92" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H92" s="16">
         <f>IF(AND(ISNUMBER(F92),ISNUMBER(G92)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9670,7 +9674,11 @@
           <t>Octavos</t>
         </is>
       </c>
-      <c r="K92" s="27" t="n"/>
+      <c r="K92" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="24" t="n">
@@ -9688,16 +9696,20 @@
       </c>
       <c r="D93" s="19" t="inlineStr">
         <is>
+          <t>Canadá</t>
+        </is>
+      </c>
+      <c r="E93" s="19" t="inlineStr">
+        <is>
           <t>Marruecos</t>
         </is>
       </c>
-      <c r="E93" s="19" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F93" s="27" t="n"/>
-      <c r="G93" s="27" t="n"/>
+      <c r="F93" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" s="27" t="n">
+        <v>3</v>
+      </c>
       <c r="H93" s="16">
         <f>IF(AND(ISNUMBER(F93),ISNUMBER(G93)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9710,7 +9722,11 @@
           <t>Octavos</t>
         </is>
       </c>
-      <c r="K93" s="27" t="n"/>
+      <c r="K93" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="26" t="n">
@@ -9728,7 +9744,7 @@
       </c>
       <c r="D94" s="19" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E94" s="19" t="inlineStr">
@@ -9808,12 +9824,12 @@
       </c>
       <c r="D96" s="19" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E96" s="19" t="inlineStr">
         <is>
-          <t>Bélgica</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F96" s="27" t="n"/>
@@ -9848,12 +9864,12 @@
       </c>
       <c r="D97" s="19" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E97" s="19" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Bélgica</t>
         </is>
       </c>
       <c r="F97" s="27" t="n"/>
@@ -9888,12 +9904,12 @@
       </c>
       <c r="D98" s="19" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E98" s="19" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Egipto</t>
         </is>
       </c>
       <c r="F98" s="27" t="n"/>
@@ -9928,12 +9944,12 @@
       </c>
       <c r="D99" s="19" t="inlineStr">
         <is>
+          <t>Suiza</t>
+        </is>
+      </c>
+      <c r="E99" s="19" t="inlineStr">
+        <is>
           <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E99" s="19" t="inlineStr">
-        <is>
-          <t>Egipto</t>
         </is>
       </c>
       <c r="F99" s="27" t="n"/>
@@ -9968,12 +9984,12 @@
       </c>
       <c r="D100" s="19" t="inlineStr">
         <is>
-          <t>Ganador Cuartos 1</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="E100" s="19" t="inlineStr">
         <is>
-          <t>Ganador Cuartos 2</t>
+          <t>Marruecos</t>
         </is>
       </c>
       <c r="F100" s="27" t="n"/>
@@ -30303,9 +30319,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A92,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F92" s="27" t="n"/>
-      <c r="G92" s="27" t="n"/>
-      <c r="H92" s="27" t="n"/>
+      <c r="F92" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="H92" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="24" t="n">
@@ -30329,9 +30353,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A93,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F93" s="27" t="n"/>
-      <c r="G93" s="27" t="n"/>
-      <c r="H93" s="27" t="n"/>
+      <c r="F93" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H93" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="26" t="n">
@@ -30355,9 +30387,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A94,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F94" s="27" t="n"/>
-      <c r="G94" s="27" t="n"/>
-      <c r="H94" s="27" t="n"/>
+      <c r="F94" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G94" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H94" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="24" t="n">
@@ -30416,14 +30456,14 @@
         <v/>
       </c>
       <c r="F96" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="G96" s="27" t="n">
-        <v>1</v>
-      </c>
       <c r="H96" s="27" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Visitante</t>
         </is>
       </c>
     </row>
@@ -30450,14 +30490,14 @@
         <v/>
       </c>
       <c r="F97" s="27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G97" s="27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H97" s="27" t="inlineStr">
         <is>
-          <t>Visitante</t>
+          <t>Local</t>
         </is>
       </c>
     </row>
@@ -30483,9 +30523,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A98,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F98" s="27" t="n"/>
-      <c r="G98" s="27" t="n"/>
-      <c r="H98" s="27" t="n"/>
+      <c r="F98" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G98" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="24" t="n">
@@ -30509,9 +30557,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A99,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F99" s="27" t="n"/>
-      <c r="G99" s="27" t="n"/>
-      <c r="H99" s="27" t="n"/>
+      <c r="F99" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G99" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H99" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="26" t="n">
@@ -33983,9 +34039,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A92,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F92" s="27" t="n"/>
-      <c r="G92" s="27" t="n"/>
-      <c r="H92" s="27" t="n"/>
+      <c r="F92" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="H92" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="24" t="n">
@@ -34009,9 +34073,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A93,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F93" s="27" t="n"/>
-      <c r="G93" s="27" t="n"/>
-      <c r="H93" s="27" t="n"/>
+      <c r="F93" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H93" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="26" t="n">
@@ -34035,9 +34107,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A94,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F94" s="27" t="n"/>
-      <c r="G94" s="27" t="n"/>
-      <c r="H94" s="27" t="n"/>
+      <c r="F94" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G94" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H94" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="24" t="n">
@@ -34096,14 +34176,14 @@
         <v/>
       </c>
       <c r="F96" s="27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G96" s="27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H96" s="27" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Visitante</t>
         </is>
       </c>
     </row>
@@ -34130,14 +34210,14 @@
         <v/>
       </c>
       <c r="F97" s="27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G97" s="27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H97" s="27" t="inlineStr">
         <is>
-          <t>Visitante</t>
+          <t>Local</t>
         </is>
       </c>
     </row>
@@ -34163,9 +34243,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A98,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F98" s="27" t="n"/>
-      <c r="G98" s="27" t="n"/>
-      <c r="H98" s="27" t="n"/>
+      <c r="F98" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G98" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H98" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="24" t="n">
@@ -34189,9 +34277,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A99,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F99" s="27" t="n"/>
-      <c r="G99" s="27" t="n"/>
-      <c r="H99" s="27" t="n"/>
+      <c r="F99" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G99" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H99" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="26" t="n">

</xml_diff>

<commit_message>
Anadir octavos de Simon y Alvaro en Papinenes
Pronosticos 8/8 octavos para Simon (Broshu) y Alvaro (Papinenes); dashboards regenerados.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -26663,9 +26663,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A92,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F92" s="27" t="n"/>
-      <c r="G92" s="27" t="n"/>
-      <c r="H92" s="27" t="n"/>
+      <c r="F92" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H92" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="24" t="n">
@@ -26689,9 +26697,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A93,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F93" s="27" t="n"/>
-      <c r="G93" s="27" t="n"/>
-      <c r="H93" s="27" t="n"/>
+      <c r="F93" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H93" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="26" t="n">
@@ -26715,9 +26731,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A94,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F94" s="27" t="n"/>
-      <c r="G94" s="27" t="n"/>
-      <c r="H94" s="27" t="n"/>
+      <c r="F94" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G94" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H94" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="24" t="n">
@@ -26741,9 +26765,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A95,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F95" s="27" t="n"/>
-      <c r="G95" s="27" t="n"/>
-      <c r="H95" s="27" t="n"/>
+      <c r="F95" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H95" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="26" t="n">
@@ -26767,9 +26799,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A96,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F96" s="27" t="n"/>
-      <c r="G96" s="27" t="n"/>
-      <c r="H96" s="27" t="n"/>
+      <c r="F96" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G96" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H96" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="24" t="n">
@@ -26793,9 +26833,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A97,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F97" s="27" t="n"/>
-      <c r="G97" s="27" t="n"/>
-      <c r="H97" s="27" t="n"/>
+      <c r="F97" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G97" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H97" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="26" t="n">
@@ -26819,9 +26867,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A98,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F98" s="27" t="n"/>
-      <c r="G98" s="27" t="n"/>
-      <c r="H98" s="27" t="n"/>
+      <c r="F98" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G98" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="24" t="n">
@@ -26845,9 +26901,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A99,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F99" s="27" t="n"/>
-      <c r="G99" s="27" t="n"/>
-      <c r="H99" s="27" t="n"/>
+      <c r="F99" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G99" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H99" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="26" t="n">

</xml_diff>

<commit_message>
Orden cronologico de octavos en dashboard y proteccion del sync
Los partidos se muestran por fecha+hora (90 antes de 89); el sync ya no sobrescribe equipos 89-96. Incluye resultado Brasil-Noruega 1-2.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -9752,8 +9752,12 @@
           <t>Noruega</t>
         </is>
       </c>
-      <c r="F94" s="27" t="n"/>
-      <c r="G94" s="27" t="n"/>
+      <c r="F94" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G94" s="27" t="n">
+        <v>2</v>
+      </c>
       <c r="H94" s="16">
         <f>IF(AND(ISNUMBER(F94),ISNUMBER(G94)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9766,7 +9770,11 @@
           <t>Octavos</t>
         </is>
       </c>
-      <c r="K94" s="27" t="n"/>
+      <c r="K94" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="24" t="n">

</xml_diff>

<commit_message>
Add cuartos predictions and sync latest results
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -9800,8 +9800,12 @@
           <t>Inglaterra</t>
         </is>
       </c>
-      <c r="F95" s="27" t="n"/>
-      <c r="G95" s="27" t="n"/>
+      <c r="F95" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G95" s="27" t="n">
+        <v>3</v>
+      </c>
       <c r="H95" s="16">
         <f>IF(AND(ISNUMBER(F95),ISNUMBER(G95)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9814,7 +9818,11 @@
           <t>Octavos</t>
         </is>
       </c>
-      <c r="K95" s="27" t="n"/>
+      <c r="K95" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="26" t="n">
@@ -9840,8 +9848,12 @@
           <t>España</t>
         </is>
       </c>
-      <c r="F96" s="27" t="n"/>
-      <c r="G96" s="27" t="n"/>
+      <c r="F96" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H96" s="16">
         <f>IF(AND(ISNUMBER(F96),ISNUMBER(G96)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9854,7 +9866,11 @@
           <t>Octavos</t>
         </is>
       </c>
-      <c r="K96" s="27" t="n"/>
+      <c r="K96" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="24" t="n">
@@ -9880,8 +9896,12 @@
           <t>Bélgica</t>
         </is>
       </c>
-      <c r="F97" s="27" t="n"/>
-      <c r="G97" s="27" t="n"/>
+      <c r="F97" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G97" s="27" t="n">
+        <v>4</v>
+      </c>
       <c r="H97" s="16">
         <f>IF(AND(ISNUMBER(F97),ISNUMBER(G97)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9894,7 +9914,11 @@
           <t>Octavos</t>
         </is>
       </c>
-      <c r="K97" s="27" t="n"/>
+      <c r="K97" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="26" t="n">
@@ -9920,8 +9944,12 @@
           <t>Egipto</t>
         </is>
       </c>
-      <c r="F98" s="27" t="n"/>
-      <c r="G98" s="27" t="n"/>
+      <c r="F98" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G98" s="27" t="n">
+        <v>2</v>
+      </c>
       <c r="H98" s="16">
         <f>IF(AND(ISNUMBER(F98),ISNUMBER(G98)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9934,7 +9962,11 @@
           <t>Octavos</t>
         </is>
       </c>
-      <c r="K98" s="27" t="n"/>
+      <c r="K98" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="24" t="n">
@@ -9960,8 +9992,12 @@
           <t>Colombia</t>
         </is>
       </c>
-      <c r="F99" s="27" t="n"/>
-      <c r="G99" s="27" t="n"/>
+      <c r="F99" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="H99" s="16">
         <f>IF(AND(ISNUMBER(F99),ISNUMBER(G99)),"Finalizado","Pendiente")</f>
         <v/>
@@ -9974,7 +10010,11 @@
           <t>Octavos</t>
         </is>
       </c>
-      <c r="K99" s="27" t="n"/>
+      <c r="K99" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="26" t="n">
@@ -10000,8 +10040,12 @@
           <t>Marruecos</t>
         </is>
       </c>
-      <c r="F100" s="27" t="n"/>
-      <c r="G100" s="27" t="n"/>
+      <c r="F100" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G100" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="H100" s="16">
         <f>IF(AND(ISNUMBER(F100),ISNUMBER(G100)),"Finalizado","Pendiente")</f>
         <v/>
@@ -10014,7 +10058,11 @@
           <t>Cuartos</t>
         </is>
       </c>
-      <c r="K100" s="27" t="n"/>
+      <c r="K100" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="24" t="n">
@@ -10032,12 +10080,12 @@
       </c>
       <c r="D101" s="19" t="inlineStr">
         <is>
-          <t>Ganador Cuartos 3</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="E101" s="19" t="inlineStr">
         <is>
-          <t>Ganador Cuartos 4</t>
+          <t>Inglaterra</t>
         </is>
       </c>
       <c r="F101" s="27" t="n"/>
@@ -10072,12 +10120,12 @@
       </c>
       <c r="D102" s="19" t="inlineStr">
         <is>
-          <t>Ganador Cuartos 5</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E102" s="19" t="inlineStr">
         <is>
-          <t>Ganador Cuartos 6</t>
+          <t>Bélgica</t>
         </is>
       </c>
       <c r="F102" s="27" t="n"/>
@@ -10112,12 +10160,12 @@
       </c>
       <c r="D103" s="19" t="inlineStr">
         <is>
-          <t>Ganador Cuartos 7</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E103" s="19" t="inlineStr">
         <is>
-          <t>Ganador Cuartos 8</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="F103" s="27" t="n"/>
@@ -26943,9 +26991,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A100,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F100" s="27" t="n"/>
-      <c r="G100" s="27" t="n"/>
-      <c r="H100" s="27" t="n"/>
+      <c r="F100" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G100" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="24" t="n">
@@ -26969,9 +27025,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A101,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F101" s="27" t="n"/>
-      <c r="G101" s="27" t="n"/>
-      <c r="H101" s="27" t="n"/>
+      <c r="F101" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G101" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H101" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="26" t="n">
@@ -26995,9 +27059,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A102,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F102" s="27" t="n"/>
-      <c r="G102" s="27" t="n"/>
-      <c r="H102" s="27" t="n"/>
+      <c r="F102" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G102" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="24" t="n">
@@ -27021,9 +27093,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A103,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F103" s="27" t="n"/>
-      <c r="G103" s="27" t="n"/>
-      <c r="H103" s="27" t="n"/>
+      <c r="F103" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G103" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="26" t="n">
@@ -30663,9 +30743,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A100,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F100" s="27" t="n"/>
-      <c r="G100" s="27" t="n"/>
-      <c r="H100" s="27" t="n"/>
+      <c r="F100" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G100" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H100" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="24" t="n">
@@ -30689,9 +30777,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A101,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F101" s="27" t="n"/>
-      <c r="G101" s="27" t="n"/>
-      <c r="H101" s="27" t="n"/>
+      <c r="F101" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G101" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H101" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="26" t="n">
@@ -30715,9 +30811,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A102,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F102" s="27" t="n"/>
-      <c r="G102" s="27" t="n"/>
-      <c r="H102" s="27" t="n"/>
+      <c r="F102" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G102" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="24" t="n">
@@ -30741,9 +30845,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A103,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F103" s="27" t="n"/>
-      <c r="G103" s="27" t="n"/>
-      <c r="H103" s="27" t="n"/>
+      <c r="F103" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G103" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H103" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="26" t="n">
@@ -34383,9 +34495,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A100,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F100" s="27" t="n"/>
-      <c r="G100" s="27" t="n"/>
-      <c r="H100" s="27" t="n"/>
+      <c r="F100" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G100" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H100" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="24" t="n">
@@ -34409,9 +34529,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A101,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F101" s="27" t="n"/>
-      <c r="G101" s="27" t="n"/>
-      <c r="H101" s="27" t="n"/>
+      <c r="F101" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G101" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="26" t="n">
@@ -34435,9 +34563,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A102,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F102" s="27" t="n"/>
-      <c r="G102" s="27" t="n"/>
-      <c r="H102" s="27" t="n"/>
+      <c r="F102" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G102" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H102" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="24" t="n">
@@ -34461,9 +34597,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A103,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F103" s="27" t="n"/>
-      <c r="G103" s="27" t="n"/>
-      <c r="H103" s="27" t="n"/>
+      <c r="F103" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G103" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H103" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="26" t="n">

</xml_diff>

<commit_message>
Fix cuartos 98/99 bracket swap and realign predictions
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -10080,16 +10080,20 @@
       </c>
       <c r="D101" s="19" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E101" s="19" t="inlineStr">
         <is>
-          <t>Inglaterra</t>
-        </is>
-      </c>
-      <c r="F101" s="27" t="n"/>
-      <c r="G101" s="27" t="n"/>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="F101" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G101" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H101" s="16">
         <f>IF(AND(ISNUMBER(F101),ISNUMBER(G101)),"Finalizado","Pendiente")</f>
         <v/>
@@ -10102,7 +10106,11 @@
           <t>Cuartos</t>
         </is>
       </c>
-      <c r="K101" s="27" t="n"/>
+      <c r="K101" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="26" t="n">
@@ -10120,16 +10128,20 @@
       </c>
       <c r="D102" s="19" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="E102" s="19" t="inlineStr">
         <is>
-          <t>Bélgica</t>
-        </is>
-      </c>
-      <c r="F102" s="27" t="n"/>
-      <c r="G102" s="27" t="n"/>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="F102" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G102" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H102" s="16">
         <f>IF(AND(ISNUMBER(F102),ISNUMBER(G102)),"Finalizado","Pendiente")</f>
         <v/>
@@ -10142,7 +10154,11 @@
           <t>Cuartos</t>
         </is>
       </c>
-      <c r="K102" s="27" t="n"/>
+      <c r="K102" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="24" t="n">
@@ -10168,8 +10184,12 @@
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F103" s="27" t="n"/>
-      <c r="G103" s="27" t="n"/>
+      <c r="F103" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G103" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="H103" s="16">
         <f>IF(AND(ISNUMBER(F103),ISNUMBER(G103)),"Finalizado","Pendiente")</f>
         <v/>
@@ -10182,7 +10202,11 @@
           <t>Cuartos</t>
         </is>
       </c>
-      <c r="K103" s="27" t="n"/>
+      <c r="K103" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="26" t="n">
@@ -10200,12 +10224,12 @@
       </c>
       <c r="D104" s="19" t="inlineStr">
         <is>
-          <t>Ganador Semifinal 1</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="E104" s="19" t="inlineStr">
         <is>
-          <t>Ganador Semifinal 2</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F104" s="27" t="n"/>
@@ -10240,12 +10264,12 @@
       </c>
       <c r="D105" s="19" t="inlineStr">
         <is>
-          <t>Ganador Semifinal 3</t>
+          <t>Inglaterra</t>
         </is>
       </c>
       <c r="E105" s="19" t="inlineStr">
         <is>
-          <t>Ganador Semifinal 4</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F105" s="27" t="n"/>
@@ -27029,11 +27053,11 @@
         <v>1</v>
       </c>
       <c r="G101" s="27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H101" s="27" t="inlineStr">
         <is>
-          <t>Visitante</t>
+          <t>Local</t>
         </is>
       </c>
     </row>
@@ -27063,11 +27087,11 @@
         <v>1</v>
       </c>
       <c r="G102" s="27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H102" s="27" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Visitante</t>
         </is>
       </c>
     </row>
@@ -30778,14 +30802,14 @@
         <v/>
       </c>
       <c r="F101" s="27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G101" s="27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H101" s="27" t="inlineStr">
         <is>
-          <t>Visitante</t>
+          <t>Local</t>
         </is>
       </c>
     </row>
@@ -30812,14 +30836,14 @@
         <v/>
       </c>
       <c r="F102" s="27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G102" s="27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H102" s="27" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Visitante</t>
         </is>
       </c>
     </row>
@@ -34530,10 +34554,10 @@
         <v/>
       </c>
       <c r="F101" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G101" s="27" t="n">
         <v>1</v>
-      </c>
-      <c r="G101" s="27" t="n">
-        <v>0</v>
       </c>
       <c r="H101" s="27" t="inlineStr">
         <is>
@@ -34564,10 +34588,10 @@
         <v/>
       </c>
       <c r="F102" s="27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G102" s="27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H102" s="27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add semifinal and final predictions, sync latest results
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -10232,8 +10232,12 @@
           <t>España</t>
         </is>
       </c>
-      <c r="F104" s="27" t="n"/>
-      <c r="G104" s="27" t="n"/>
+      <c r="F104" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104" s="27" t="n">
+        <v>2</v>
+      </c>
       <c r="H104" s="16">
         <f>IF(AND(ISNUMBER(F104),ISNUMBER(G104)),"Finalizado","Pendiente")</f>
         <v/>
@@ -10246,7 +10250,11 @@
           <t>Semifinal</t>
         </is>
       </c>
-      <c r="K104" s="27" t="n"/>
+      <c r="K104" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="24" t="n">
@@ -10272,8 +10280,12 @@
           <t>Argentina</t>
         </is>
       </c>
-      <c r="F105" s="27" t="n"/>
-      <c r="G105" s="27" t="n"/>
+      <c r="F105" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G105" s="27" t="n">
+        <v>2</v>
+      </c>
       <c r="H105" s="16">
         <f>IF(AND(ISNUMBER(F105),ISNUMBER(G105)),"Finalizado","Pendiente")</f>
         <v/>
@@ -10286,7 +10298,11 @@
           <t>Semifinal</t>
         </is>
       </c>
-      <c r="K105" s="27" t="n"/>
+      <c r="K105" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="26" t="n">
@@ -10304,12 +10320,12 @@
       </c>
       <c r="D106" s="19" t="inlineStr">
         <is>
-          <t>Perdedor Semifinal 1</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="E106" s="19" t="inlineStr">
         <is>
-          <t>Perdedor Semifinal 2</t>
+          <t>Inglaterra</t>
         </is>
       </c>
       <c r="F106" s="27" t="n"/>
@@ -10344,12 +10360,12 @@
       </c>
       <c r="D107" s="19" t="inlineStr">
         <is>
-          <t>Ganador Semifinal 1</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E107" s="19" t="inlineStr">
         <is>
-          <t>Ganador Semifinal 2</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F107" s="27" t="n"/>
@@ -27151,9 +27167,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A104,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F104" s="27" t="n"/>
-      <c r="G104" s="27" t="n"/>
-      <c r="H104" s="27" t="n"/>
+      <c r="F104" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G104" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H104" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="24" t="n">
@@ -27177,9 +27201,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A105,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F105" s="27" t="n"/>
-      <c r="G105" s="27" t="n"/>
-      <c r="H105" s="27" t="n"/>
+      <c r="F105" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G105" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H105" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="26" t="n">
@@ -30903,9 +30935,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A104,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F104" s="27" t="n"/>
-      <c r="G104" s="27" t="n"/>
-      <c r="H104" s="27" t="n"/>
+      <c r="F104" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G104" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H104" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="24" t="n">
@@ -30929,9 +30969,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A105,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F105" s="27" t="n"/>
-      <c r="G105" s="27" t="n"/>
-      <c r="H105" s="27" t="n"/>
+      <c r="F105" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G105" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H105" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="26" t="n">
@@ -34655,9 +34703,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A104,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F104" s="27" t="n"/>
-      <c r="G104" s="27" t="n"/>
-      <c r="H104" s="27" t="n"/>
+      <c r="F104" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G104" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H104" s="27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="24" t="n">
@@ -34681,9 +34737,17 @@
         <f>IFERROR(INDEX(Partidos!$E$4:$E$107,MATCH($A105,Partidos!$A$4:$A$107,0)),"")</f>
         <v/>
       </c>
-      <c r="F105" s="27" t="n"/>
-      <c r="G105" s="27" t="n"/>
-      <c r="H105" s="27" t="n"/>
+      <c r="F105" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G105" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H105" s="27" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="26" t="n">

</xml_diff>

<commit_message>
Fix Inglaterra-Argentina semifinal predictions (swap scores for local/away)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Porra_Mundial_2026_Papinenes.xlsx
+++ b/output/Porra_Mundial_2026_Papinenes.xlsx
@@ -30970,10 +30970,10 @@
         <v/>
       </c>
       <c r="F105" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G105" s="27" t="n">
         <v>1</v>
-      </c>
-      <c r="G105" s="27" t="n">
-        <v>2</v>
       </c>
       <c r="H105" s="27" t="inlineStr">
         <is>
@@ -34738,10 +34738,10 @@
         <v/>
       </c>
       <c r="F105" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G105" s="27" t="n">
         <v>0</v>
-      </c>
-      <c r="G105" s="27" t="n">
-        <v>1</v>
       </c>
       <c r="H105" s="27" t="inlineStr">
         <is>

</xml_diff>